<commit_message>
Mise à jour auto - 2026-09-12 08:14
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bourse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33EDC66E-2092-4AA6-A8EC-B6C35DD916D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C94052-FB27-4366-A1D0-88B08924B7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{63CF4381-08A8-4F9A-BA0C-6F5F5274B36B}"/>
   </bookViews>
   <sheets>
     <sheet name="Donnees" sheetId="1" r:id="rId1"/>
     <sheet name="Suivi" sheetId="2" r:id="rId2"/>
+    <sheet name="Commentaires" sheetId="3" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Donnees!$A$2:$G$11</definedName>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="167">
   <si>
     <t>Code</t>
   </si>
@@ -546,6 +547,9 @@
   </si>
   <si>
     <t>SANOFI</t>
+  </si>
+  <si>
+    <t>Commentaire</t>
   </si>
 </sst>
 </file>
@@ -1194,7 +1198,7 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1355,7 +1359,7 @@
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1368,18 +1372,18 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="22" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="23" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1387,7 +1391,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1403,28 +1407,26 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="7" borderId="30" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="33" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="6" borderId="32" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1454,7 +1456,7 @@
     <xf numFmtId="10" fontId="6" fillId="8" borderId="39" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="32" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="8" fillId="8" borderId="40" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1475,142 +1477,7 @@
     <cellStyle name="Normal 4" xfId="3" xr:uid="{8A5525BB-3552-4FE6-A951-F5D328751787}"/>
     <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="214">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
+  <dxfs count="105">
     <dxf>
       <font>
         <condense val="0"/>
@@ -1644,16 +1511,6 @@
         <extend val="0"/>
         <color indexed="10"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1768,17 +1625,16 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
+        <color rgb="FF006100"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -1798,6 +1654,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -1814,82 +1672,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -1939,6 +1721,15 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <condense val="0"/>
@@ -1948,8 +1739,73 @@
     </dxf>
     <dxf>
       <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -1969,9 +1825,20 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
       </font>
     </dxf>
     <dxf>
@@ -2142,865 +2009,6 @@
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
       </font>
     </dxf>
     <dxf>
@@ -19282,7 +18290,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="112">
+      <c r="A1" s="110">
         <v>46276</v>
       </c>
       <c r="B1" s="93" t="s">
@@ -19294,13 +18302,13 @@
       <c r="D1" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="113" t="s">
+      <c r="E1" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="114" t="s">
+      <c r="F1" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="115" t="s">
+      <c r="G1" s="113" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="7" t="s">
@@ -19321,13 +18329,13 @@
       <c r="A2" s="96">
         <v>1</v>
       </c>
-      <c r="B2" s="105" t="s">
+      <c r="B2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="105" t="s">
+      <c r="C2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="106" t="s">
+      <c r="D2" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="16">
@@ -19336,7 +18344,7 @@
       <c r="F2" s="77">
         <v>0.35099999999999998</v>
       </c>
-      <c r="G2" s="116">
+      <c r="G2" s="114">
         <v>0</v>
       </c>
       <c r="I2" s="20"/>
@@ -19352,13 +18360,13 @@
       <c r="A3" s="98">
         <v>2</v>
       </c>
-      <c r="B3" s="105" t="s">
+      <c r="B3" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="105" t="s">
+      <c r="C3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="15" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="16">
@@ -19367,7 +18375,7 @@
       <c r="F3" s="77">
         <v>14.91</v>
       </c>
-      <c r="G3" s="116">
+      <c r="G3" s="114">
         <v>0</v>
       </c>
       <c r="H3" s="8"/>
@@ -19381,13 +18389,13 @@
       <c r="A4" s="96">
         <v>3</v>
       </c>
-      <c r="B4" s="105" t="s">
+      <c r="B4" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="105" t="s">
+      <c r="C4" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="106" t="s">
+      <c r="D4" s="15" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="16">
@@ -19396,7 +18404,7 @@
       <c r="F4" s="77">
         <v>78.77</v>
       </c>
-      <c r="G4" s="116">
+      <c r="G4" s="114">
         <v>0</v>
       </c>
       <c r="H4" s="8"/>
@@ -19410,13 +18418,13 @@
       <c r="A5" s="98">
         <v>4</v>
       </c>
-      <c r="B5" s="105" t="s">
+      <c r="B5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="105" t="s">
+      <c r="C5" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="106" t="s">
+      <c r="D5" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="16">
@@ -19425,7 +18433,7 @@
       <c r="F5" s="77">
         <v>140</v>
       </c>
-      <c r="G5" s="116">
+      <c r="G5" s="114">
         <v>0</v>
       </c>
       <c r="H5" s="8"/>
@@ -19439,13 +18447,13 @@
       <c r="A6" s="96">
         <v>5</v>
       </c>
-      <c r="B6" s="105" t="s">
+      <c r="B6" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="105" t="s">
+      <c r="C6" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="106" t="s">
+      <c r="D6" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="16">
@@ -19454,7 +18462,7 @@
       <c r="F6" s="77">
         <v>124.4</v>
       </c>
-      <c r="G6" s="116">
+      <c r="G6" s="114">
         <v>0</v>
       </c>
       <c r="H6" s="8"/>
@@ -19468,13 +18476,13 @@
       <c r="A7" s="98">
         <v>6</v>
       </c>
-      <c r="B7" s="105" t="s">
+      <c r="B7" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="105" t="s">
+      <c r="C7" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="106" t="s">
+      <c r="D7" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E7" s="16">
@@ -19483,7 +18491,7 @@
       <c r="F7" s="77">
         <v>47.5</v>
       </c>
-      <c r="G7" s="116">
+      <c r="G7" s="114">
         <v>0</v>
       </c>
       <c r="H7" s="8"/>
@@ -19497,13 +18505,13 @@
       <c r="A8" s="96">
         <v>7</v>
       </c>
-      <c r="B8" s="105" t="s">
+      <c r="B8" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="105" t="s">
+      <c r="C8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="106" t="s">
+      <c r="D8" s="15" t="s">
         <v>23</v>
       </c>
       <c r="E8" s="16">
@@ -19512,7 +18520,7 @@
       <c r="F8" s="77">
         <v>35.96</v>
       </c>
-      <c r="G8" s="116">
+      <c r="G8" s="114">
         <v>0</v>
       </c>
       <c r="H8" s="8"/>
@@ -19526,13 +18534,13 @@
       <c r="A9" s="98">
         <v>8</v>
       </c>
-      <c r="B9" s="105" t="s">
+      <c r="B9" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="105" t="s">
+      <c r="C9" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="106" t="s">
+      <c r="D9" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E9" s="16">
@@ -19541,7 +18549,7 @@
       <c r="F9" s="77">
         <v>216.2</v>
       </c>
-      <c r="G9" s="116">
+      <c r="G9" s="114">
         <v>0</v>
       </c>
       <c r="H9" s="8"/>
@@ -19555,13 +18563,13 @@
       <c r="A10" s="96">
         <v>9</v>
       </c>
-      <c r="B10" s="105" t="s">
+      <c r="B10" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="105" t="s">
+      <c r="C10" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D10" s="106" t="s">
+      <c r="D10" s="15" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="16">
@@ -19570,7 +18578,7 @@
       <c r="F10" s="77">
         <v>1.6E-2</v>
       </c>
-      <c r="G10" s="116">
+      <c r="G10" s="114">
         <v>0</v>
       </c>
       <c r="H10" s="8"/>
@@ -19584,13 +18592,13 @@
       <c r="A11" s="98">
         <v>10</v>
       </c>
-      <c r="B11" s="105" t="s">
+      <c r="B11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="105" t="s">
+      <c r="C11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="106" t="s">
+      <c r="D11" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E11" s="16">
@@ -19599,7 +18607,7 @@
       <c r="F11" s="77">
         <v>22.55</v>
       </c>
-      <c r="G11" s="116">
+      <c r="G11" s="114">
         <v>0</v>
       </c>
       <c r="H11" s="8"/>
@@ -19614,8 +18622,8 @@
       <c r="B12" s="100"/>
       <c r="C12" s="101"/>
       <c r="D12" s="102"/>
-      <c r="E12" s="117"/>
-      <c r="F12" s="118" t="s">
+      <c r="E12" s="115"/>
+      <c r="F12" s="116" t="s">
         <v>30</v>
       </c>
       <c r="G12" s="39">
@@ -19675,13 +18683,13 @@
       <c r="A16" s="96">
         <v>1</v>
       </c>
-      <c r="B16" s="105" t="s">
+      <c r="B16" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="105" t="s">
+      <c r="C16" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="106" t="s">
+      <c r="D16" s="15" t="s">
         <v>35</v>
       </c>
       <c r="E16" s="36">
@@ -19700,13 +18708,13 @@
       <c r="A17" s="98">
         <v>2</v>
       </c>
-      <c r="B17" s="105" t="s">
+      <c r="B17" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="105" t="s">
+      <c r="C17" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="106" t="s">
+      <c r="D17" s="15" t="s">
         <v>37</v>
       </c>
       <c r="E17" s="36">
@@ -19725,13 +18733,13 @@
       <c r="A18" s="96">
         <v>3</v>
       </c>
-      <c r="B18" s="105" t="s">
+      <c r="B18" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="105" t="s">
+      <c r="C18" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="106" t="s">
+      <c r="D18" s="15" t="s">
         <v>39</v>
       </c>
       <c r="E18" s="36">
@@ -19750,13 +18758,13 @@
       <c r="A19" s="98">
         <v>4</v>
       </c>
-      <c r="B19" s="105" t="s">
+      <c r="B19" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="105" t="s">
+      <c r="C19" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="106" t="s">
+      <c r="D19" s="15" t="s">
         <v>41</v>
       </c>
       <c r="E19" s="36">
@@ -19775,13 +18783,13 @@
       <c r="A20" s="96">
         <v>5</v>
       </c>
-      <c r="B20" s="105" t="s">
+      <c r="B20" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="105" t="s">
+      <c r="C20" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="106" t="s">
+      <c r="D20" s="15" t="s">
         <v>43</v>
       </c>
       <c r="E20" s="36">
@@ -19800,13 +18808,13 @@
       <c r="A21" s="98">
         <v>6</v>
       </c>
-      <c r="B21" s="105" t="s">
+      <c r="B21" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="105" t="s">
+      <c r="C21" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="106" t="s">
+      <c r="D21" s="15" t="s">
         <v>45</v>
       </c>
       <c r="E21" s="36">
@@ -19825,13 +18833,13 @@
       <c r="A22" s="96">
         <v>7</v>
       </c>
-      <c r="B22" s="105" t="s">
+      <c r="B22" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="105" t="s">
+      <c r="C22" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D22" s="106" t="s">
+      <c r="D22" s="15" t="s">
         <v>47</v>
       </c>
       <c r="E22" s="36">
@@ -19850,13 +18858,13 @@
       <c r="A23" s="98">
         <v>8</v>
       </c>
-      <c r="B23" s="105" t="s">
+      <c r="B23" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="105" t="s">
+      <c r="C23" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D23" s="106" t="s">
+      <c r="D23" s="15" t="s">
         <v>49</v>
       </c>
       <c r="E23" s="36">
@@ -19875,13 +18883,13 @@
       <c r="A24" s="96">
         <v>9</v>
       </c>
-      <c r="B24" s="105" t="s">
+      <c r="B24" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="105" t="s">
+      <c r="C24" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D24" s="106" t="s">
+      <c r="D24" s="15" t="s">
         <v>51</v>
       </c>
       <c r="E24" s="36">
@@ -19900,13 +18908,13 @@
       <c r="A25" s="98">
         <v>10</v>
       </c>
-      <c r="B25" s="105" t="s">
+      <c r="B25" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="105" t="s">
+      <c r="C25" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D25" s="106" t="s">
+      <c r="D25" s="15" t="s">
         <v>53</v>
       </c>
       <c r="E25" s="36">
@@ -19923,9 +18931,9 @@
     </row>
     <row r="26" spans="1:11" ht="15.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="96"/>
-      <c r="B26" s="105"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="76"/>
-      <c r="D26" s="107"/>
+      <c r="D26" s="105"/>
       <c r="E26" s="36"/>
       <c r="F26" s="38" t="s">
         <v>30</v>
@@ -19947,11 +18955,11 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A27" s="108"/>
-      <c r="B27" s="109"/>
+      <c r="A27" s="106"/>
+      <c r="B27" s="107"/>
       <c r="C27" s="100"/>
-      <c r="D27" s="110"/>
-      <c r="E27" s="111"/>
+      <c r="D27" s="108"/>
+      <c r="E27" s="109"/>
       <c r="F27" s="8"/>
       <c r="H27" s="8"/>
       <c r="I27"/>
@@ -19973,13 +18981,13 @@
       <c r="D29" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E29" s="113" t="s">
+      <c r="E29" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F29" s="114" t="s">
+      <c r="F29" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G29" s="115" t="s">
+      <c r="G29" s="113" t="s">
         <v>5</v>
       </c>
       <c r="H29" s="7" t="s">
@@ -19991,13 +18999,13 @@
       <c r="A30" s="96">
         <v>1</v>
       </c>
-      <c r="B30" s="105" t="s">
+      <c r="B30" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="105" t="s">
+      <c r="C30" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D30" s="106" t="s">
+      <c r="D30" s="15" t="s">
         <v>57</v>
       </c>
       <c r="E30" s="16">
@@ -20006,7 +19014,7 @@
       <c r="F30" s="77">
         <v>5.16</v>
       </c>
-      <c r="G30" s="116">
+      <c r="G30" s="114">
         <v>0</v>
       </c>
       <c r="H30"/>
@@ -20016,13 +19024,13 @@
       <c r="A31" s="98">
         <v>2</v>
       </c>
-      <c r="B31" s="105" t="s">
+      <c r="B31" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="105" t="s">
+      <c r="C31" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D31" s="106" t="s">
+      <c r="D31" s="15" t="s">
         <v>59</v>
       </c>
       <c r="E31" s="16">
@@ -20031,7 +19039,7 @@
       <c r="F31" s="77">
         <v>8.2000000000000003E-2</v>
       </c>
-      <c r="G31" s="116">
+      <c r="G31" s="114">
         <v>0</v>
       </c>
       <c r="H31"/>
@@ -20041,13 +19049,13 @@
       <c r="A32" s="96">
         <v>3</v>
       </c>
-      <c r="B32" s="105" t="s">
+      <c r="B32" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="C32" s="105" t="s">
+      <c r="C32" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D32" s="106" t="s">
+      <c r="D32" s="15" t="s">
         <v>61</v>
       </c>
       <c r="E32" s="16">
@@ -20056,7 +19064,7 @@
       <c r="F32" s="77">
         <v>5.86</v>
       </c>
-      <c r="G32" s="116">
+      <c r="G32" s="114">
         <v>0</v>
       </c>
       <c r="H32"/>
@@ -20066,13 +19074,13 @@
       <c r="A33" s="98">
         <v>4</v>
       </c>
-      <c r="B33" s="105" t="s">
+      <c r="B33" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="105" t="s">
+      <c r="C33" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D33" s="106" t="s">
+      <c r="D33" s="15" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="16">
@@ -20081,7 +19089,7 @@
       <c r="F33" s="77">
         <v>1.0549999999999999</v>
       </c>
-      <c r="G33" s="116">
+      <c r="G33" s="114">
         <v>0</v>
       </c>
       <c r="H33"/>
@@ -20091,13 +19099,13 @@
       <c r="A34" s="96">
         <v>5</v>
       </c>
-      <c r="B34" s="105" t="s">
+      <c r="B34" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C34" s="105" t="s">
+      <c r="C34" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D34" s="106" t="s">
+      <c r="D34" s="15" t="s">
         <v>65</v>
       </c>
       <c r="E34" s="16">
@@ -20106,7 +19114,7 @@
       <c r="F34" s="77">
         <v>8.6</v>
       </c>
-      <c r="G34" s="116">
+      <c r="G34" s="114">
         <v>0</v>
       </c>
       <c r="H34"/>
@@ -20116,13 +19124,13 @@
       <c r="A35" s="98">
         <v>6</v>
       </c>
-      <c r="B35" s="105" t="s">
+      <c r="B35" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="105" t="s">
+      <c r="C35" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D35" s="106" t="s">
+      <c r="D35" s="15" t="s">
         <v>67</v>
       </c>
       <c r="E35" s="16">
@@ -20131,7 +19139,7 @@
       <c r="F35" s="77">
         <v>20.3</v>
       </c>
-      <c r="G35" s="116">
+      <c r="G35" s="114">
         <v>0</v>
       </c>
       <c r="H35"/>
@@ -20141,13 +19149,13 @@
       <c r="A36" s="96">
         <v>7</v>
       </c>
-      <c r="B36" s="105" t="s">
+      <c r="B36" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C36" s="105" t="s">
+      <c r="C36" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="106" t="s">
+      <c r="D36" s="15" t="s">
         <v>69</v>
       </c>
       <c r="E36" s="16">
@@ -20156,7 +19164,7 @@
       <c r="F36" s="77">
         <v>0.28000000000000003</v>
       </c>
-      <c r="G36" s="116">
+      <c r="G36" s="114">
         <v>0</v>
       </c>
       <c r="H36"/>
@@ -20166,13 +19174,13 @@
       <c r="A37" s="98">
         <v>8</v>
       </c>
-      <c r="B37" s="105" t="s">
+      <c r="B37" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C37" s="105" t="s">
+      <c r="C37" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D37" s="106" t="s">
+      <c r="D37" s="15" t="s">
         <v>71</v>
       </c>
       <c r="E37" s="16">
@@ -20181,7 +19189,7 @@
       <c r="F37" s="77">
         <v>1.28</v>
       </c>
-      <c r="G37" s="116">
+      <c r="G37" s="114">
         <v>0</v>
       </c>
       <c r="H37"/>
@@ -20192,13 +19200,13 @@
       <c r="A38" s="96">
         <v>9</v>
       </c>
-      <c r="B38" s="105" t="s">
+      <c r="B38" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="105" t="s">
+      <c r="C38" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D38" s="106" t="s">
+      <c r="D38" s="15" t="s">
         <v>73</v>
       </c>
       <c r="E38" s="16">
@@ -20207,7 +19215,7 @@
       <c r="F38" s="77">
         <v>0.16</v>
       </c>
-      <c r="G38" s="116">
+      <c r="G38" s="114">
         <v>0</v>
       </c>
       <c r="H38"/>
@@ -20218,13 +19226,13 @@
       <c r="A39" s="98">
         <v>10</v>
       </c>
-      <c r="B39" s="105" t="s">
+      <c r="B39" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C39" s="105" t="s">
+      <c r="C39" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D39" s="106" t="s">
+      <c r="D39" s="15" t="s">
         <v>75</v>
       </c>
       <c r="E39" s="16">
@@ -20233,22 +19241,22 @@
       <c r="F39" s="77">
         <v>19.850000000000001</v>
       </c>
-      <c r="G39" s="116">
+      <c r="G39" s="114">
         <v>0</v>
       </c>
       <c r="H39"/>
       <c r="I39"/>
     </row>
     <row r="40" spans="1:16" ht="16.3" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A40" s="125"/>
-      <c r="B40" s="126"/>
-      <c r="C40" s="127"/>
-      <c r="D40" s="128"/>
-      <c r="E40" s="129"/>
-      <c r="F40" s="118" t="s">
+      <c r="A40" s="123"/>
+      <c r="B40" s="124"/>
+      <c r="C40" s="125"/>
+      <c r="D40" s="126"/>
+      <c r="E40" s="127"/>
+      <c r="F40" s="116" t="s">
         <v>30</v>
       </c>
-      <c r="G40" s="130">
+      <c r="G40" s="128">
         <v>0</v>
       </c>
       <c r="H40" s="31" t="s">
@@ -20287,13 +19295,13 @@
       <c r="D42" s="94" t="s">
         <v>2</v>
       </c>
-      <c r="E42" s="113" t="s">
+      <c r="E42" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="F42" s="114" t="s">
+      <c r="F42" s="112" t="s">
         <v>4</v>
       </c>
-      <c r="G42" s="121" t="s">
+      <c r="G42" s="119" t="s">
         <v>5</v>
       </c>
       <c r="H42" s="7" t="s">
@@ -20305,13 +19313,13 @@
       <c r="A43" s="96">
         <v>1</v>
       </c>
-      <c r="B43" s="105" t="s">
+      <c r="B43" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C43" s="105" t="s">
+      <c r="C43" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D43" s="106" t="s">
+      <c r="D43" s="15" t="s">
         <v>78</v>
       </c>
       <c r="E43" s="16">
@@ -20320,7 +19328,7 @@
       <c r="F43" s="77">
         <v>6.2549999999999999</v>
       </c>
-      <c r="G43" s="122">
+      <c r="G43" s="120">
         <v>0</v>
       </c>
       <c r="H43"/>
@@ -20330,13 +19338,13 @@
       <c r="A44" s="98">
         <v>2</v>
       </c>
-      <c r="B44" s="105" t="s">
+      <c r="B44" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C44" s="105" t="s">
+      <c r="C44" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D44" s="106" t="s">
+      <c r="D44" s="15" t="s">
         <v>80</v>
       </c>
       <c r="E44" s="16">
@@ -20345,7 +19353,7 @@
       <c r="F44" s="77">
         <v>5.22</v>
       </c>
-      <c r="G44" s="122">
+      <c r="G44" s="120">
         <v>0</v>
       </c>
       <c r="H44"/>
@@ -20355,13 +19363,13 @@
       <c r="A45" s="96">
         <v>3</v>
       </c>
-      <c r="B45" s="105" t="s">
+      <c r="B45" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="C45" s="105" t="s">
+      <c r="C45" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D45" s="106" t="s">
+      <c r="D45" s="15" t="s">
         <v>82</v>
       </c>
       <c r="E45" s="16">
@@ -20370,7 +19378,7 @@
       <c r="F45" s="77">
         <v>85.5</v>
       </c>
-      <c r="G45" s="122">
+      <c r="G45" s="120">
         <v>0</v>
       </c>
       <c r="H45"/>
@@ -20380,13 +19388,13 @@
       <c r="A46" s="98">
         <v>4</v>
       </c>
-      <c r="B46" s="105" t="s">
+      <c r="B46" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C46" s="105" t="s">
+      <c r="C46" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D46" s="106" t="s">
+      <c r="D46" s="15" t="s">
         <v>29</v>
       </c>
       <c r="E46" s="16">
@@ -20395,7 +19403,7 @@
       <c r="F46" s="77">
         <v>22.55</v>
       </c>
-      <c r="G46" s="122">
+      <c r="G46" s="120">
         <v>0</v>
       </c>
       <c r="H46"/>
@@ -20405,13 +19413,13 @@
       <c r="A47" s="96">
         <v>5</v>
       </c>
-      <c r="B47" s="105" t="s">
+      <c r="B47" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="C47" s="105" t="s">
+      <c r="C47" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D47" s="106" t="s">
+      <c r="D47" s="15" t="s">
         <v>84</v>
       </c>
       <c r="E47" s="16">
@@ -20420,7 +19428,7 @@
       <c r="F47" s="77">
         <v>21.6</v>
       </c>
-      <c r="G47" s="122">
+      <c r="G47" s="120">
         <v>0</v>
       </c>
       <c r="H47"/>
@@ -20430,13 +19438,13 @@
       <c r="A48" s="98">
         <v>6</v>
       </c>
-      <c r="B48" s="105" t="s">
+      <c r="B48" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="C48" s="105" t="s">
+      <c r="C48" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="106" t="s">
+      <c r="D48" s="15" t="s">
         <v>86</v>
       </c>
       <c r="E48" s="16">
@@ -20445,7 +19453,7 @@
       <c r="F48" s="77">
         <v>4.0060000000000002</v>
       </c>
-      <c r="G48" s="122">
+      <c r="G48" s="120">
         <v>0</v>
       </c>
       <c r="H48"/>
@@ -20455,13 +19463,13 @@
       <c r="A49" s="96">
         <v>7</v>
       </c>
-      <c r="B49" s="105" t="s">
+      <c r="B49" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C49" s="105" t="s">
+      <c r="C49" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D49" s="106" t="s">
+      <c r="D49" s="15" t="s">
         <v>88</v>
       </c>
       <c r="E49" s="16">
@@ -20470,7 +19478,7 @@
       <c r="F49" s="77">
         <v>90.4</v>
       </c>
-      <c r="G49" s="122">
+      <c r="G49" s="120">
         <v>0</v>
       </c>
       <c r="H49"/>
@@ -20480,13 +19488,13 @@
       <c r="A50" s="98">
         <v>8</v>
       </c>
-      <c r="B50" s="105" t="s">
+      <c r="B50" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="C50" s="105" t="s">
+      <c r="C50" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D50" s="106" t="s">
+      <c r="D50" s="15" t="s">
         <v>90</v>
       </c>
       <c r="E50" s="16">
@@ -20495,7 +19503,7 @@
       <c r="F50" s="77">
         <v>1.873</v>
       </c>
-      <c r="G50" s="122">
+      <c r="G50" s="120">
         <v>0</v>
       </c>
       <c r="H50"/>
@@ -20505,13 +19513,13 @@
       <c r="A51" s="96">
         <v>9</v>
       </c>
-      <c r="B51" s="105" t="s">
+      <c r="B51" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="C51" s="105" t="s">
+      <c r="C51" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D51" s="106" t="s">
+      <c r="D51" s="15" t="s">
         <v>91</v>
       </c>
       <c r="E51" s="16">
@@ -20520,7 +19528,7 @@
       <c r="F51" s="77">
         <v>35.200000000000003</v>
       </c>
-      <c r="G51" s="122">
+      <c r="G51" s="120">
         <v>0</v>
       </c>
       <c r="H51"/>
@@ -20530,13 +19538,13 @@
       <c r="A52" s="98">
         <v>10</v>
       </c>
-      <c r="B52" s="105" t="s">
+      <c r="B52" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="C52" s="105" t="s">
+      <c r="C52" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="D52" s="106" t="s">
+      <c r="D52" s="15" t="s">
         <v>93</v>
       </c>
       <c r="E52" s="16">
@@ -20545,7 +19553,7 @@
       <c r="F52" s="77">
         <v>222</v>
       </c>
-      <c r="G52" s="122">
+      <c r="G52" s="120">
         <v>0</v>
       </c>
       <c r="H52"/>
@@ -20556,11 +19564,11 @@
       <c r="B53" s="100"/>
       <c r="C53" s="101"/>
       <c r="D53" s="102"/>
-      <c r="E53" s="123"/>
-      <c r="F53" s="120" t="s">
+      <c r="E53" s="121"/>
+      <c r="F53" s="118" t="s">
         <v>30</v>
       </c>
-      <c r="G53" s="124">
+      <c r="G53" s="122">
         <v>0</v>
       </c>
       <c r="H53" s="31" t="s">
@@ -21079,7 +20087,7 @@
         <v>4</v>
       </c>
       <c r="B85" s="80"/>
-      <c r="C85" s="119"/>
+      <c r="C85" s="117"/>
       <c r="D85" s="80"/>
       <c r="E85" s="16"/>
       <c r="F85" s="77"/>
@@ -21094,7 +20102,7 @@
         <v>5</v>
       </c>
       <c r="B86" s="75"/>
-      <c r="C86" s="119"/>
+      <c r="C86" s="117"/>
       <c r="D86" s="75"/>
       <c r="E86" s="16"/>
       <c r="F86" s="77"/>
@@ -21109,7 +20117,7 @@
         <v>6</v>
       </c>
       <c r="B87" s="80"/>
-      <c r="C87" s="119"/>
+      <c r="C87" s="117"/>
       <c r="D87" s="80"/>
       <c r="E87" s="16"/>
       <c r="F87" s="77"/>
@@ -21139,7 +20147,7 @@
         <v>8</v>
       </c>
       <c r="B89" s="80"/>
-      <c r="C89" s="119"/>
+      <c r="C89" s="117"/>
       <c r="D89" s="80"/>
       <c r="E89" s="16"/>
       <c r="F89" s="77"/>
@@ -21185,7 +20193,7 @@
       <c r="C92" s="83"/>
       <c r="D92" s="54"/>
       <c r="E92" s="84"/>
-      <c r="F92" s="120" t="s">
+      <c r="F92" s="118" t="s">
         <v>30</v>
       </c>
       <c r="G92" s="50" t="e">
@@ -23629,431 +22637,451 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B56:B65">
-    <cfRule type="expression" dxfId="105" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="104" priority="5" stopIfTrue="1">
       <formula>IF(AO56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:B78">
-    <cfRule type="expression" dxfId="104" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="103" priority="3" stopIfTrue="1">
       <formula>IF(AO69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B81">
-    <cfRule type="expression" dxfId="103" priority="50" stopIfTrue="1">
+    <cfRule type="expression" dxfId="102" priority="50" stopIfTrue="1">
       <formula>IF(AN62&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82:B91">
-    <cfRule type="expression" dxfId="102" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="101" priority="9" stopIfTrue="1">
       <formula>IF(AL82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="expression" dxfId="101" priority="46" stopIfTrue="1">
+    <cfRule type="expression" dxfId="100" priority="46" stopIfTrue="1">
       <formula>IF(AL91&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="expression" dxfId="100" priority="49" stopIfTrue="1">
+    <cfRule type="expression" dxfId="99" priority="49" stopIfTrue="1">
       <formula>IF(AN75&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:B105">
-    <cfRule type="expression" dxfId="99" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="98" priority="7" stopIfTrue="1">
       <formula>IF(AO96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B106">
-    <cfRule type="expression" dxfId="98" priority="47" stopIfTrue="1">
+    <cfRule type="expression" dxfId="97" priority="47" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="expression" dxfId="97" priority="48" stopIfTrue="1">
+    <cfRule type="expression" dxfId="96" priority="48" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D56:D65">
-    <cfRule type="expression" dxfId="96" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="95" priority="4" stopIfTrue="1">
       <formula>IF(AQ56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D78">
-    <cfRule type="expression" dxfId="95" priority="2" stopIfTrue="1">
+    <cfRule type="expression" dxfId="94" priority="2" stopIfTrue="1">
       <formula>IF(AQ69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82:D91">
-    <cfRule type="expression" dxfId="94" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="93" priority="8" stopIfTrue="1">
       <formula>IF(AN82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D96:D105">
-    <cfRule type="expression" dxfId="93" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="92" priority="6" stopIfTrue="1">
       <formula>IF(AQ96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" dxfId="92" priority="19" stopIfTrue="1">
+    <cfRule type="expression" dxfId="91" priority="19" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="91" priority="20" stopIfTrue="1">
+    <cfRule type="expression" dxfId="90" priority="20" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="21" stopIfTrue="1">
+    <cfRule type="expression" dxfId="89" priority="21" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="89" priority="22" stopIfTrue="1">
+    <cfRule type="expression" dxfId="88" priority="22" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="88" priority="23" stopIfTrue="1">
+    <cfRule type="expression" dxfId="87" priority="23" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="87" priority="24" stopIfTrue="1">
+    <cfRule type="expression" dxfId="86" priority="24" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" dxfId="86" priority="80" stopIfTrue="1">
+    <cfRule type="expression" dxfId="85" priority="80" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="85" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="84" priority="85" stopIfTrue="1">
+      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="83" priority="84" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="82" stopIfTrue="1">
+    <cfRule type="expression" dxfId="82" priority="83" stopIfTrue="1">
+      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="81" priority="82" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="83" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="82" priority="84" stopIfTrue="1">
+    <cfRule type="expression" dxfId="80" priority="81" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="81" priority="85" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" dxfId="80" priority="86" stopIfTrue="1">
+    <cfRule type="expression" dxfId="79" priority="91" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="78" priority="89" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="77" priority="88" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="76" priority="87" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="75" priority="86" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="79" priority="87" stopIfTrue="1">
+    <cfRule type="expression" dxfId="74" priority="90" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="78" priority="88" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="77" priority="89" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="76" priority="90" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="75" priority="91" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F56">
-    <cfRule type="expression" dxfId="74" priority="76" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="73" priority="77" stopIfTrue="1">
-      <formula>IF($AN28="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="73" priority="79" stopIfTrue="1">
+      <formula>IF($U254="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="72" priority="78" stopIfTrue="1">
       <formula>IF($T254="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="79" stopIfTrue="1">
-      <formula>IF($U254="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="71" priority="77" stopIfTrue="1">
+      <formula>IF($AN28="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F67">
+    <cfRule type="expression" dxfId="70" priority="76" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F57:F67">
+    <cfRule type="expression" dxfId="69" priority="93" stopIfTrue="1">
+      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="68" priority="94" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="95" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69">
+    <cfRule type="expression" dxfId="66" priority="96" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="97" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="98" stopIfTrue="1">
+      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="63" priority="99" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="62" priority="100" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" dxfId="70" priority="1" stopIfTrue="1">
+    <cfRule type="expression" dxfId="61" priority="1" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F70:F78">
+    <cfRule type="expression" dxfId="60" priority="101" stopIfTrue="1">
+      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="59" priority="102" stopIfTrue="1">
+      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="58" priority="103" stopIfTrue="1">
+      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" dxfId="57" priority="104" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="56" priority="105" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="106" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" dxfId="69" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="54" priority="65" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" dxfId="68" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="53" priority="66" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="52" priority="68" stopIfTrue="1">
+      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="51" priority="67" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="66" priority="68" stopIfTrue="1">
-      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" dxfId="65" priority="73" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="50" priority="75" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="74" stopIfTrue="1">
+    <cfRule type="expression" dxfId="49" priority="74" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="75" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="48" priority="73" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" dxfId="62" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="47" priority="69" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" dxfId="61" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="46" priority="72" stopIfTrue="1">
+      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="71" stopIfTrue="1">
+      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="70" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="71" stopIfTrue="1">
-      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="59" priority="72" stopIfTrue="1">
-      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="58" priority="52" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" dxfId="43" priority="52" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="42" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G28 G2:G12">
-    <cfRule type="cellIs" dxfId="56" priority="25" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" dxfId="41" priority="25" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="55" priority="51" operator="greaterThan">
+  <conditionalFormatting sqref="G30:G41 G2:G12 G16:G26">
+    <cfRule type="cellIs" dxfId="40" priority="51" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54 G56:G67 G30:G41">
-    <cfRule type="cellIs" dxfId="54" priority="42" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G43:G54 G30:G41 G56:G67">
+    <cfRule type="cellIs" dxfId="39" priority="42" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" dxfId="53" priority="30" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="38" priority="33" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="37" priority="32" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="31" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="36" priority="31" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="32" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="35" priority="30" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="33" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" dxfId="49" priority="16" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="18" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="17" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="33" priority="17" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="18" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="32" priority="16" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" dxfId="46" priority="43" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="43" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="44" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="44" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" dxfId="43" priority="26" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="26" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="29" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="41" priority="28" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="26" priority="28" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="29" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="25" priority="27" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" dxfId="39" priority="38" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="24" priority="40" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="40" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="39" operator="greaterThan">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="38" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" dxfId="35" priority="34" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="20" priority="37" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="36" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="35" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="35" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="36" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="34" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="37" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
+    <cfRule type="cellIs" dxfId="16" priority="15" operator="greaterThan">
+      <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I12 I53 K53 I66 K66">
-    <cfRule type="cellIs" dxfId="31" priority="59" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="59" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26">
-    <cfRule type="cellIs" dxfId="30" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="14" priority="10" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I75">
-    <cfRule type="cellIs" dxfId="29" priority="60" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="13" priority="60" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I93:I94">
-    <cfRule type="cellIs" dxfId="28" priority="58" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="12" priority="58" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I107">
-    <cfRule type="cellIs" dxfId="27" priority="57" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="11" priority="57" operator="greaterThan">
       <formula>$K107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I109">
-    <cfRule type="cellIs" dxfId="26" priority="55" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="10" priority="55" operator="greaterThan">
       <formula>$K109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J97">
-    <cfRule type="cellIs" dxfId="25" priority="62" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="62" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J103">
-    <cfRule type="cellIs" dxfId="24" priority="61" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="61" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K12">
-    <cfRule type="cellIs" dxfId="23" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="13" operator="greaterThan">
       <formula>$K12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K26">
-    <cfRule type="cellIs" dxfId="22" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="12" operator="greaterThan">
       <formula>$K26</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K41">
-    <cfRule type="cellIs" dxfId="21" priority="11" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="11" operator="greaterThan">
       <formula>$K41</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" dxfId="20" priority="15" operator="greaterThan">
-      <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="K93:K94">
-    <cfRule type="cellIs" dxfId="19" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="14" operator="greaterThan">
       <formula>$K93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K104">
-    <cfRule type="cellIs" dxfId="18" priority="63" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="63" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K107">
-    <cfRule type="cellIs" dxfId="17" priority="56" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="56" operator="greaterThan">
       <formula>$I107</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K109">
-    <cfRule type="cellIs" dxfId="16" priority="54" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="54" operator="greaterThan">
       <formula>$I109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P37:P38">
-    <cfRule type="cellIs" dxfId="15" priority="64" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="64" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F57:F67">
-    <cfRule type="expression" dxfId="14" priority="92" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="93" stopIfTrue="1">
-      <formula>IF($AK29="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="94" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="11" priority="95" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69">
-    <cfRule type="expression" dxfId="10" priority="96" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="97" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="98" stopIfTrue="1">
-      <formula>IF($AJ43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="99" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="100" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F70:F78">
-    <cfRule type="expression" dxfId="5" priority="101" stopIfTrue="1">
-      <formula>IF($AJ42="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="102" stopIfTrue="1">
-      <formula>IF($T267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="103" stopIfTrue="1">
-      <formula>IF($U267="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" dxfId="2" priority="104" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="105" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="106" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA2E1525-4D7C-45EC-B8D4-E5AA18562442}">
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="2" max="2" width="65.4609375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-14 18:46
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19280,7 +19280,7 @@
         <v>0.333</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0</v>
+        <v>-0.05128205128205117</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" thickBot="1">
@@ -19338,7 +19338,7 @@
         <v>79.54000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0</v>
+        <v>0.009775295163133304</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" thickBot="1">
@@ -19367,7 +19367,7 @@
         <v>139</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.007142857142857143</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" thickBot="1">
@@ -19425,7 +19425,7 @@
         <v>47.6</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.002105263157894767</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" thickBot="1">
@@ -19454,7 +19454,7 @@
         <v>35.62</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0</v>
+        <v>-0.009454949944382743</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" thickBot="1">
@@ -19483,7 +19483,7 @@
         <v>214.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>-0.006475485661424502</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" thickBot="1">
@@ -19512,7 +19512,7 @@
         <v>0.015</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0</v>
+        <v>-0.06250000000000006</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" thickBot="1">
@@ -19541,7 +19541,7 @@
         <v>22.05</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>-0.02217294900221729</v>
       </c>
     </row>
     <row r="12" ht="15.45" customHeight="1">
@@ -19659,7 +19659,7 @@
         <v>3.255</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0</v>
+        <v>0.001538461538461506</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" thickBot="1">
@@ -19688,7 +19688,7 @@
         <v>5.685</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0</v>
+        <v>-0.0240343347639486</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" thickBot="1">
@@ -19717,7 +19717,7 @@
         <v>3.55</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0</v>
+        <v>-0.02686403508771938</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" thickBot="1">
@@ -19746,7 +19746,7 @@
         <v>7.43</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0</v>
+        <v>-0.002684563758389324</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" thickBot="1">
@@ -19775,7 +19775,7 @@
         <v>25.22</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0</v>
+        <v>0.01611603545527794</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" thickBot="1">
@@ -19804,7 +19804,7 @@
         <v>72.34</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0</v>
+        <v>0.0231966053748232</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" thickBot="1">
@@ -19833,7 +19833,7 @@
         <v>8.02</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>0.002499999999999947</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" thickBot="1">
@@ -19862,7 +19862,7 @@
         <v>8.199999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0</v>
+        <v>0.007371007371007213</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" thickBot="1">
@@ -19891,7 +19891,7 @@
         <v>21.94</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0</v>
+        <v>0.008272058823529398</v>
       </c>
     </row>
     <row r="26" ht="15.45" customHeight="1">
@@ -20012,7 +20012,7 @@
         <v>0.081</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.01219512195121952</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20041,7 +20041,7 @@
         <v>5.2</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0</v>
+        <v>-0.1126279863481229</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20070,7 +20070,7 @@
         <v>1.02</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>-0.03317535545023689</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20099,7 +20099,7 @@
         <v>8.279999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0</v>
+        <v>-0.03720930232558143</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20128,7 +20128,7 @@
         <v>20.4</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>0.004926108374384132</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20157,7 +20157,7 @@
         <v>0.263</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>-0.06071428571428576</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20186,7 +20186,7 @@
         <v>1.32</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>0.03125000000000003</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20244,7 +20244,7 @@
         <v>19.4</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.02267002518891702</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1">
@@ -20331,7 +20331,7 @@
         <v>5.785</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0</v>
+        <v>-0.07513988808952834</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20360,7 +20360,7 @@
         <v>5.284</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0</v>
+        <v>0.01226053639846744</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20418,7 +20418,7 @@
         <v>22.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0</v>
+        <v>-0.02217294900221729</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20447,7 +20447,7 @@
         <v>22.15</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0</v>
+        <v>0.02546296296296283</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20534,7 +20534,7 @@
         <v>1.821</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>-0.02776294714361989</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20592,7 +20592,7 @@
         <v>223</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0</v>
+        <v>0.004504504504504504</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1">
@@ -21799,7 +21799,7 @@
         <v>11.65</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.04000000000000004</v>
+        <v>-0.06799999999999998</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" thickBot="1">
@@ -21828,7 +21828,7 @@
         <v>214.8</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02077431539187913</v>
+        <v>0.0141643059490085</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" thickBot="1">
@@ -21886,7 +21886,7 @@
         <v>24.48</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01332223147377176</v>
+        <v>0.01915070774354708</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" thickBot="1">
@@ -21915,7 +21915,7 @@
         <v>9.369999999999999</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.01475409836065578</v>
+        <v>0.02404371584699441</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" thickBot="1">
@@ -21944,7 +21944,7 @@
         <v>13.76</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03891830018600662</v>
+        <v>-0.01559593647159822</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" thickBot="1">
@@ -21973,7 +21973,7 @@
         <v>47.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03260869565217384</v>
+        <v>0.0347826086956522</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" thickBot="1">
@@ -22002,7 +22002,7 @@
         <v>271.3</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.0352941176470587</v>
+        <v>-0.1009113504556752</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" thickBot="1">
@@ -22031,7 +22031,7 @@
         <v>5.42</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.01760563380281688</v>
+        <v>-0.04577464788732391</v>
       </c>
     </row>
     <row r="12" ht="15.45" customHeight="1">
@@ -22120,7 +22120,7 @@
         <v>61.22</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05981012658227847</v>
+        <v>-0.0313291139240507</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" thickBot="1">
@@ -22149,7 +22149,7 @@
         <v>99.7</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.04004106776180683</v>
+        <v>0.02361396303901434</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" thickBot="1">
@@ -22178,7 +22178,7 @@
         <v>18.95</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0100250626566416</v>
+        <v>-0.05012531328320802</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" thickBot="1">
@@ -22207,7 +22207,7 @@
         <v>1.547</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.06200122774708405</v>
+        <v>-0.05033763044812773</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" thickBot="1">
@@ -22236,7 +22236,7 @@
         <v>66.90000000000001</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01038575667655794</v>
+        <v>-0.007418397626112759</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" thickBot="1">
@@ -22265,7 +22265,7 @@
         <v>5.685</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1363973313565604</v>
+        <v>-0.1571534469977762</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" thickBot="1">
@@ -22294,7 +22294,7 @@
         <v>18.7</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.05639476334340388</v>
+        <v>-0.05840886203423969</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" thickBot="1">
@@ -22323,7 +22323,7 @@
         <v>8.02</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.096045197740113</v>
+        <v>-0.09378531073446329</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" thickBot="1">
@@ -22352,7 +22352,7 @@
         <v>2.128</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1162594776748106</v>
+        <v>-0.1036225779275484</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" thickBot="1">
@@ -22473,7 +22473,7 @@
         <v>3.87</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01308900523560208</v>
+        <v>0.01308900523560217</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22502,7 +22502,7 @@
         <v>0.57</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.05211726384364823</v>
+        <v>-0.07166123778501635</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22589,7 +22589,7 @@
         <v>9.34</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.01825557809330625</v>
+        <v>-0.0527383367139959</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22674,7 +22674,7 @@
         <v>2.44</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.01214574898785435</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22703,7 +22703,7 @@
         <v>17.4</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0</v>
+        <v>-0.0252100840336136</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22819,7 +22819,7 @@
         <v>139</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.04089219330855021</v>
+        <v>0.03345724907063197</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22848,7 +22848,7 @@
         <v>47.12</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.07495145631067957</v>
+        <v>-0.08504854368932044</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22906,7 +22906,7 @@
         <v>9.369999999999999</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01475409836065578</v>
+        <v>0.02404371584699441</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22935,7 +22935,7 @@
         <v>56.85</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.0436241610738255</v>
+        <v>-0.04614093959731543</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22964,7 +22964,7 @@
         <v>45.67</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01412368927883578</v>
+        <v>-0.02268350096297871</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22993,7 +22993,7 @@
         <v>35.62</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.06769596199524952</v>
+        <v>0.05760095011876478</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23022,7 +23022,7 @@
         <v>28.44</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02450331125827809</v>
+        <v>-0.05827814569536417</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23051,7 +23051,7 @@
         <v>21.36</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1234300563014292</v>
+        <v>-0.07492420961455178</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -23080,7 +23080,7 @@
         <v>24.48</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01332223147377176</v>
+        <v>0.01915070774354708</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-15 10:24
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17998,10 +17998,10 @@
         <v>24.54</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.54</v>
+        <v>14.88</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.393643031784841</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18058,10 +18058,10 @@
         <v>79.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79.53</v>
+        <v>91.15000000000001</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.1461083867722872</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18520,10 +18520,10 @@
         <v>18.95</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>18.85</v>
+        <v>93.42</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.005277044854881154</v>
+        <v>3.929815303430079</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18550,10 +18550,10 @@
         <v>184</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>184</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0</v>
+        <v>-0.5168478260869565</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19421,10 +19421,10 @@
         <v>79.53</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.53</v>
+        <v>91.15000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0</v>
+        <v>0.1461083867722872</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -19511,10 +19511,10 @@
         <v>15.42</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>15.42</v>
+        <v>2.775</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0</v>
+        <v>-0.8200389105058365</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -20650,10 +20650,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>15.42</v>
+        <v>2.775</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.04401735895846248</v>
+        <v>-0.8279603223806571</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20680,10 +20680,10 @@
         <v>24.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>24.54</v>
+        <v>14.88</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.02164862614487917</v>
+        <v>-0.3805162364696086</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20770,10 +20770,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>47.3</v>
+        <v>464.405</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02826086956521734</v>
+        <v>9.095760869565217</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20800,10 +20800,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>271.1</v>
+        <v>68.73</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.1015741507870753</v>
+        <v>-0.7722286661143331</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20962,10 +20962,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>96.95</v>
+        <v>113.59</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.00462012320328545</v>
+        <v>0.1662217659137577</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20992,10 +20992,10 @@
         <v>19.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>18.85</v>
+        <v>93.42</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.05513784461152871</v>
+        <v>3.682706766917293</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21022,10 +21022,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.55</v>
+        <v>11.875</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.04849600982197666</v>
+        <v>6.28974831184776</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21052,10 +21052,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>66.90000000000001</v>
+        <v>7.76</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.007418397626112759</v>
+        <v>-0.88486646884273</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21690,10 +21690,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.96</v>
+        <v>30.02</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.08815533980582524</v>
+        <v>-0.4170873786407767</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21864,10 +21864,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>28.36</v>
+        <v>4.375</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.06092715231788082</v>
+        <v>-0.8551324503311258</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21893,10 +21893,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>21.25</v>
+        <v>3.755</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.07968817669987005</v>
+        <v>-0.8373754872239065</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21922,10 +21922,10 @@
         <v>24.02</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.54</v>
+        <v>14.88</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02164862614487917</v>
+        <v>-0.3805162364696086</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-15 10:41
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17908,10 +17908,10 @@
         <v>105.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>105.7</v>
+        <v>108.7</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0</v>
+        <v>0.02838221381267739</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17938,10 +17938,10 @@
         <v>15.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>15.26</v>
+        <v>15.18</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0</v>
+        <v>-0.005242463958060293</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17968,10 +17968,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>8.35</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.00654372397382507</v>
+        <v>-0.001784651992861248</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -17998,10 +17998,10 @@
         <v>24.54</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.88</v>
+        <v>24.4</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.393643031784841</v>
+        <v>-0.005704971475142648</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18028,10 +18028,10 @@
         <v>314.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>314.5</v>
+        <v>315</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0</v>
+        <v>0.001589825119236884</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18058,10 +18058,10 @@
         <v>79.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>91.15000000000001</v>
+        <v>79.39</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1461083867722872</v>
+        <v>-0.001760342009304672</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18118,10 +18118,10 @@
         <v>124.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>124.4</v>
+        <v>124.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>-0.0008038585209003901</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18148,10 +18148,10 @@
         <v>71.58</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>71.58</v>
+        <v>69.94</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0</v>
+        <v>-0.02291142777312099</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18178,10 +18178,10 @@
         <v>32.8</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>32.7</v>
+        <v>32.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.003048780487804705</v>
+        <v>-0.009146341463414549</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18280,10 +18280,10 @@
         <v>1.69</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1.678</v>
+        <v>1.684</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.007100591715976338</v>
+        <v>-0.003550295857988169</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -18310,10 +18310,10 @@
         <v>22.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>22.25</v>
+        <v>22</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0</v>
+        <v>-0.01123595505617977</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18340,10 +18340,10 @@
         <v>3.546</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.546</v>
+        <v>3.67</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0</v>
+        <v>0.03496897913141572</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18370,10 +18370,10 @@
         <v>5.695</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>5.695</v>
+        <v>5.532</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0</v>
+        <v>-0.02862159789288854</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18400,10 +18400,10 @@
         <v>4.87</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.78</v>
+        <v>4.75</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01848049281314166</v>
+        <v>-0.02464065708418893</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18430,10 +18430,10 @@
         <v>5.7</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.7</v>
+        <v>5.72</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0</v>
+        <v>0.003508771929824486</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18460,10 +18460,10 @@
         <v>0.51</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>0.512</v>
+        <v>0.511</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.003921568627450984</v>
+        <v>0.001960784313725492</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18490,10 +18490,10 @@
         <v>116</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>116</v>
+        <v>115.4</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>-0.0051724137931034</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18520,10 +18520,10 @@
         <v>18.95</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>93.42</v>
+        <v>18.8</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>3.929815303430079</v>
+        <v>-0.007915567282321826</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18550,10 +18550,10 @@
         <v>184</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>88.90000000000001</v>
+        <v>185.2</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.5168478260869565</v>
+        <v>0.006521739130434721</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18655,10 +18655,10 @@
         <v>5.278</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.278</v>
+        <v>5.071</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0</v>
+        <v>-0.03921940128836678</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18684,10 +18684,10 @@
         <v>0.083</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.083</v>
+        <v>0.091</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>0.09638554216867461</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18713,10 +18713,10 @@
         <v>2.94</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>2.94</v>
+        <v>2.9</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0</v>
+        <v>-0.01360544217687076</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18800,10 +18800,10 @@
         <v>1.13</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.13</v>
+        <v>1.1</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>-0.02654867256637151</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18829,10 +18829,10 @@
         <v>1.68</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.65</v>
+        <v>1.78</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.01785714285714287</v>
+        <v>0.05952380952380958</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18858,10 +18858,10 @@
         <v>0.133</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.133</v>
+        <v>0.127</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.04511278195488726</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18887,10 +18887,10 @@
         <v>1.32</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.32</v>
+        <v>1.29</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0</v>
+        <v>-0.02272727272727275</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18916,10 +18916,10 @@
         <v>20.4</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.004901960784313621</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19421,10 +19421,10 @@
         <v>79.53</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>91.15000000000001</v>
+        <v>79.39</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.1461083867722872</v>
+        <v>-0.001760342009304672</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -19451,10 +19451,10 @@
         <v>16.61</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>16.65</v>
+        <v>16.705</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.002408187838651364</v>
+        <v>0.005719446116797042</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -19481,10 +19481,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.35</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.00654372397382507</v>
+        <v>-0.001784651992861248</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -19511,10 +19511,10 @@
         <v>15.42</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>2.775</v>
+        <v>14.98</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.8200389105058365</v>
+        <v>-0.02853437094682228</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -19541,10 +19541,10 @@
         <v>100.35</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>100.35</v>
+        <v>98.62</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0</v>
+        <v>-0.01723966118584943</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -19571,10 +19571,10 @@
         <v>71.58</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>71.58</v>
+        <v>69.94</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0</v>
+        <v>-0.02291142777312099</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -19601,10 +19601,10 @@
         <v>109.7</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>109.7</v>
+        <v>107.05</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0</v>
+        <v>-0.02415679124886058</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -19631,10 +19631,10 @@
         <v>72.16</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>72.16</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0</v>
+        <v>0.006097560975609725</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -19691,10 +19691,10 @@
         <v>27.93</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>27.93</v>
+        <v>27.66</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0</v>
+        <v>-0.009667024704618674</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -20560,10 +20560,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>105.7</v>
+        <v>108.7</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.3146766169154229</v>
+        <v>0.3519900497512437</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20590,10 +20590,10 @@
         <v>12.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>11.65</v>
+        <v>11.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.06799999999999995</v>
+        <v>-0.08</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20620,10 +20620,10 @@
         <v>211.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>215.6</v>
+        <v>216.6</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01794145420207735</v>
+        <v>0.02266288951841352</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20650,10 +20650,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>2.775</v>
+        <v>14.98</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.8279603223806571</v>
+        <v>-0.07129572225666451</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20680,10 +20680,10 @@
         <v>24.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>14.88</v>
+        <v>24.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.3805162364696086</v>
+        <v>0.01582014987510404</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20740,10 +20740,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.848</v>
+        <v>13.56</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.009300329088567705</v>
+        <v>-0.02990413506939471</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20770,10 +20770,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>464.405</v>
+        <v>47.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>9.095760869565217</v>
+        <v>0.02826086956521733</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20800,10 +20800,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>68.73</v>
+        <v>271.8</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.7722286661143331</v>
+        <v>-0.09925434962717478</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20830,10 +20830,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.42</v>
+        <v>5.4</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.04577464788732388</v>
+        <v>-0.04929577464788722</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20932,10 +20932,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>60.66</v>
+        <v>60.62</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04018987341772162</v>
+        <v>-0.04082278481012667</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -20962,10 +20962,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>113.59</v>
+        <v>97.3</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1662217659137577</v>
+        <v>-0.001026694045174625</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20992,10 +20992,10 @@
         <v>19.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>93.42</v>
+        <v>18.8</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>3.682706766917293</v>
+        <v>-0.05764411027568915</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21022,10 +21022,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>11.875</v>
+        <v>1.543</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>6.28974831184776</v>
+        <v>-0.05279312461632908</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21052,10 +21052,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.76</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.88486646884273</v>
+        <v>-0.007418397626112759</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21082,10 +21082,10 @@
         <v>6.745</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.695</v>
+        <v>5.532</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1556708673091178</v>
+        <v>-0.1798369162342476</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21112,10 +21112,10 @@
         <v>19.86</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.76</v>
+        <v>18.56</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.05538771399798581</v>
+        <v>-0.0654582074521652</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21142,10 +21142,10 @@
         <v>8.85</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.98</v>
+        <v>7.59</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.09830508474576261</v>
+        <v>-0.1423728813559322</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21172,10 +21172,10 @@
         <v>2.374</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>2.128</v>
+        <v>2.14</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1036225779275484</v>
+        <v>-0.09856781802864363</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21202,10 +21202,10 @@
         <v>27.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.25</v>
+        <v>22</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1981981981981982</v>
+        <v>-0.2072072072072072</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21310,7 +21310,7 @@
         <v>3.87</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01308900523560208</v>
+        <v>0.01308900523560217</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21365,10 +21365,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>27.4</v>
+        <v>27.1</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.00363636363636366</v>
+        <v>-0.01454545454545449</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21394,10 +21394,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.151</v>
+        <v>0.148</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05625000000000002</v>
+        <v>-0.07500000000000007</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21452,10 +21452,10 @@
         <v>8.880000000000001</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.52</v>
+        <v>8.5</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04054054054054068</v>
+        <v>-0.04279279279279288</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21567,7 +21567,7 @@
         <v>3.81</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.08851674641148322</v>
+        <v>-0.08851674641148317</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21661,10 +21661,10 @@
         <v>134.5</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0483271375464684</v>
+        <v>0.03345724907063197</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21690,10 +21690,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>30.02</v>
+        <v>46.14</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.4170873786407767</v>
+        <v>-0.1040776699029126</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21719,10 +21719,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>105.7</v>
+        <v>108.7</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.3146766169154229</v>
+        <v>0.3519900497512437</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -21777,10 +21777,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>56.95</v>
+        <v>55.8</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.04446308724832215</v>
+        <v>-0.06375838926174504</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21806,10 +21806,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.73</v>
+        <v>45.35</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02139952921035737</v>
+        <v>-0.02953135031029308</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21835,10 +21835,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.54</v>
+        <v>35.4</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05522565320665085</v>
+        <v>0.05106888361045128</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21864,10 +21864,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>4.375</v>
+        <v>28.7</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.8551324503311258</v>
+        <v>-0.04966887417218543</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21893,10 +21893,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.755</v>
+        <v>20.67</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.8373754872239065</v>
+        <v>-0.1048072758770029</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21922,10 +21922,10 @@
         <v>24.02</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>14.88</v>
+        <v>24.4</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.3805162364696086</v>
+        <v>0.01582014987510404</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-15 12:34
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17908,10 +17908,10 @@
         <v>105.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>108.7</v>
+        <v>109.4</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.02838221381267739</v>
+        <v>0.0350047303689688</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17938,10 +17938,10 @@
         <v>15.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>15.18</v>
+        <v>15.21</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.005242463958060293</v>
+        <v>-0.00327653997378761</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17968,10 +17968,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>8.390000000000001</v>
+        <v>8.31</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.001784651992861248</v>
+        <v>-0.01130279595478868</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -17998,10 +17998,10 @@
         <v>24.54</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.4</v>
+        <v>24.44</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.005704971475142648</v>
+        <v>-0.004074979625101787</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18028,10 +18028,10 @@
         <v>314.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>315</v>
+        <v>317.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.001589825119236884</v>
+        <v>0.009538950715421303</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18058,10 +18058,10 @@
         <v>79.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79.39</v>
+        <v>79.25</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.001760342009304672</v>
+        <v>-0.003520684018609344</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18088,10 +18088,10 @@
         <v>9.385</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>9.355</v>
+        <v>9.275</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.003196590303676011</v>
+        <v>-0.0117208311134789</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18148,10 +18148,10 @@
         <v>71.58</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>69.94</v>
+        <v>69.52</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.02291142777312099</v>
+        <v>-0.02877898854428615</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18178,10 +18178,10 @@
         <v>32.8</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.009146341463414549</v>
+        <v>-0.006097560975609627</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18280,10 +18280,10 @@
         <v>1.69</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1.684</v>
+        <v>1.668</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.003550295857988169</v>
+        <v>-0.01301775147928995</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -18310,10 +18310,10 @@
         <v>22.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>22</v>
+        <v>21.45</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01123595505617977</v>
+        <v>-0.03595505617977531</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18340,10 +18340,10 @@
         <v>3.546</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.67</v>
+        <v>3.66</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.03496897913141572</v>
+        <v>0.03214890016920483</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18370,10 +18370,10 @@
         <v>5.695</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>5.532</v>
+        <v>5.51</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02862159789288854</v>
+        <v>-0.03248463564530298</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18400,10 +18400,10 @@
         <v>4.87</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.75</v>
+        <v>4.745</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02464065708418893</v>
+        <v>-0.02566735112936345</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18430,10 +18430,10 @@
         <v>5.7</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.72</v>
+        <v>5.74</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.003508771929824486</v>
+        <v>0.007017543859649129</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18460,10 +18460,10 @@
         <v>0.51</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>0.511</v>
+        <v>0.51</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.001960784313725492</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18490,10 +18490,10 @@
         <v>116</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>115.4</v>
+        <v>115.8</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.0051724137931034</v>
+        <v>-0.001724137931034507</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18520,10 +18520,10 @@
         <v>18.95</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>18.8</v>
+        <v>19.05</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.007915567282321826</v>
+        <v>0.005277044854881342</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18550,10 +18550,10 @@
         <v>184</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>185.2</v>
+        <v>184.9</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.006521739130434721</v>
+        <v>0.004891304347826118</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18655,10 +18655,10 @@
         <v>5.278</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.071</v>
+        <v>5.026</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.03921940128836678</v>
+        <v>-0.04774535809018564</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18684,10 +18684,10 @@
         <v>0.083</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.091</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.09638554216867461</v>
+        <v>0.06024096385542157</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18887,10 +18887,10 @@
         <v>1.32</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.29</v>
+        <v>1.25</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.02272727272727275</v>
+        <v>-0.05303030303030307</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19421,10 +19421,10 @@
         <v>79.53</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.39</v>
+        <v>79.25</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.001760342009304672</v>
+        <v>-0.003520684018609344</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -19451,10 +19451,10 @@
         <v>16.61</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>16.705</v>
+        <v>16.67</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.005719446116797042</v>
+        <v>0.003612281757977259</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -19481,10 +19481,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.390000000000001</v>
+        <v>8.31</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.001784651992861248</v>
+        <v>-0.01130279595478868</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -19511,10 +19511,10 @@
         <v>15.42</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>14.98</v>
+        <v>14.89</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.02853437094682228</v>
+        <v>-0.03437094682230865</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -19571,10 +19571,10 @@
         <v>71.58</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>69.94</v>
+        <v>69.52</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.02291142777312099</v>
+        <v>-0.02877898854428615</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -19601,10 +19601,10 @@
         <v>109.7</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>107.05</v>
+        <v>107.1</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.02415679124886058</v>
+        <v>-0.02370100273473116</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -19631,10 +19631,10 @@
         <v>72.16</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>72.59999999999999</v>
+        <v>72.72</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.006097560975609725</v>
+        <v>0.007760532150776085</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -19661,10 +19661,10 @@
         <v>9.385</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>9.355</v>
+        <v>9.275</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.003196590303676011</v>
+        <v>-0.0117208311134789</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -19691,10 +19691,10 @@
         <v>27.93</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>27.66</v>
+        <v>27.55</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.009667024704618674</v>
+        <v>-0.01360544217687071</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -20560,10 +20560,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>108.7</v>
+        <v>109.4</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.3519900497512437</v>
+        <v>0.3606965174129353</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20590,10 +20590,10 @@
         <v>12.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>11.5</v>
+        <v>11.75</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.08</v>
+        <v>-0.06</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20620,10 +20620,10 @@
         <v>211.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>216.6</v>
+        <v>215.2</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02266288951841352</v>
+        <v>0.01605288007554286</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20650,10 +20650,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.98</v>
+        <v>14.89</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.07129572225666451</v>
+        <v>-0.07687538747675131</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20680,10 +20680,10 @@
         <v>24.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>24.4</v>
+        <v>24.44</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01582014987510404</v>
+        <v>0.01748542880932564</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20710,10 +20710,10 @@
         <v>9.15</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>9.355</v>
+        <v>9.275</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02240437158469946</v>
+        <v>0.01366120218579235</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20740,10 +20740,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.56</v>
+        <v>13.742</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02990413506939471</v>
+        <v>-0.01688367434539984</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20770,10 +20770,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>47.3</v>
+        <v>46.9</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02826086956521733</v>
+        <v>0.01956521739130432</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20800,10 +20800,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>271.8</v>
+        <v>273.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.09925434962717478</v>
+        <v>-0.0936205468102734</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20830,10 +20830,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.4</v>
+        <v>5.38</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.04929577464788722</v>
+        <v>-0.05281690140845068</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20932,10 +20932,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>60.62</v>
+        <v>60.4</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04082278481012667</v>
+        <v>-0.04430379746835449</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -20962,10 +20962,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>97.3</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.001026694045174625</v>
+        <v>0</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20992,10 +20992,10 @@
         <v>19.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>18.8</v>
+        <v>19.05</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.05764411027568915</v>
+        <v>-0.04511278195488715</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21022,10 +21022,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.543</v>
+        <v>1.545</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.05279312461632908</v>
+        <v>-0.05156537753222841</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21052,10 +21052,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>66.90000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.007418397626112759</v>
+        <v>-0.002967359050445146</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21082,10 +21082,10 @@
         <v>6.745</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.532</v>
+        <v>5.51</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1798369162342476</v>
+        <v>-0.1830985915492958</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21112,10 +21112,10 @@
         <v>19.86</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.56</v>
+        <v>18.58</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.0654582074521652</v>
+        <v>-0.06445115810674729</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21142,10 +21142,10 @@
         <v>8.85</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.59</v>
+        <v>7.64</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.1423728813559322</v>
+        <v>-0.1367231638418079</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21172,10 +21172,10 @@
         <v>2.374</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>2.14</v>
+        <v>2.142</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.09856781802864363</v>
+        <v>-0.09772535804549293</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21202,10 +21202,10 @@
         <v>27.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22</v>
+        <v>21.45</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2072072072072072</v>
+        <v>-0.227027027027027</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21365,10 +21365,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>27.1</v>
+        <v>27.4</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.01454545454545449</v>
+        <v>-0.003636363636363688</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21394,10 +21394,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.148</v>
+        <v>0.149</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07500000000000007</v>
+        <v>-0.06875000000000006</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21452,10 +21452,10 @@
         <v>8.880000000000001</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.5</v>
+        <v>8.48</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04279279279279288</v>
+        <v>-0.04504504504504508</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21535,10 +21535,10 @@
         <v>17.85</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>17.25</v>
+        <v>17.2</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03361344537815134</v>
+        <v>-0.03641456582633065</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21564,10 +21564,10 @@
         <v>4.18</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>3.81</v>
+        <v>3.78</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.08851674641148317</v>
+        <v>-0.09569377990430621</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21690,10 +21690,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.14</v>
+        <v>46.3</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.1040776699029126</v>
+        <v>-0.1009708737864078</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21719,10 +21719,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>108.7</v>
+        <v>109.4</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.3519900497512437</v>
+        <v>0.3606965174129353</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -21748,10 +21748,10 @@
         <v>9.15</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>9.355</v>
+        <v>9.275</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.02240437158469946</v>
+        <v>0.01366120218579235</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21777,10 +21777,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>55.8</v>
+        <v>56.4</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.06375838926174504</v>
+        <v>-0.05369127516778528</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21806,10 +21806,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.35</v>
+        <v>45.36</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02953135031029308</v>
+        <v>-0.02931735501818955</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21835,10 +21835,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.4</v>
+        <v>35.44</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05106888361045128</v>
+        <v>0.05225653206650825</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21864,10 +21864,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>28.7</v>
+        <v>28.99</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.04966887417218543</v>
+        <v>-0.04006622516556294</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21893,10 +21893,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>20.67</v>
+        <v>20.68</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1048072758770029</v>
+        <v>-0.1043741879601559</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21922,10 +21922,10 @@
         <v>24.02</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.4</v>
+        <v>24.44</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01582014987510404</v>
+        <v>0.01748542880932564</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-15 14:52
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17908,10 +17908,10 @@
         <v>105.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>109.4</v>
+        <v>109</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.0350047303689688</v>
+        <v>0.0312204351939451</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17938,10 +17938,10 @@
         <v>15.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>15.21</v>
+        <v>15.25</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.00327653997378761</v>
+        <v>-0.0006553079947575221</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17968,10 +17968,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>8.31</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01130279595478868</v>
+        <v>-0.005353955978584168</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18028,10 +18028,10 @@
         <v>314.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>317.5</v>
+        <v>317</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.009538950715421303</v>
+        <v>0.007949125596184419</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18058,10 +18058,10 @@
         <v>79.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79.25</v>
+        <v>79.34</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.003520684018609344</v>
+        <v>-0.002389035584056302</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18088,10 +18088,10 @@
         <v>9.385</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>9.275</v>
+        <v>9.35</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0117208311134789</v>
+        <v>-0.003729355354288774</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18118,10 +18118,10 @@
         <v>124.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>124.3</v>
+        <v>124.4</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0008038585209003901</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18148,10 +18148,10 @@
         <v>71.58</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>69.52</v>
+        <v>69.48</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.02877898854428615</v>
+        <v>-0.02933780385582557</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18178,10 +18178,10 @@
         <v>32.8</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>32.6</v>
+        <v>32.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.006097560975609627</v>
+        <v>-0.009146341463414549</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18280,10 +18280,10 @@
         <v>1.69</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1.668</v>
+        <v>1.678</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01301775147928995</v>
+        <v>-0.007100591715976338</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -18310,10 +18310,10 @@
         <v>22.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>21.45</v>
+        <v>21.1</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.03595505617977531</v>
+        <v>-0.0516853932584269</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18340,10 +18340,10 @@
         <v>3.546</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.66</v>
+        <v>3.71</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.03214890016920483</v>
+        <v>0.04624929498025949</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18370,10 +18370,10 @@
         <v>5.695</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>5.51</v>
+        <v>5.515</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.03248463564530298</v>
+        <v>-0.03160667251975428</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18400,10 +18400,10 @@
         <v>4.87</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.745</v>
+        <v>4.75</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02566735112936345</v>
+        <v>-0.02464065708418893</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18430,10 +18430,10 @@
         <v>5.7</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.74</v>
+        <v>5.68</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.007017543859649129</v>
+        <v>-0.003508771929824642</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18460,10 +18460,10 @@
         <v>0.51</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>0.51</v>
+        <v>0.515</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0</v>
+        <v>0.00980392156862746</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18490,10 +18490,10 @@
         <v>116</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>115.8</v>
+        <v>115.5</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.001724137931034507</v>
+        <v>-0.004310344827586207</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18520,10 +18520,10 @@
         <v>18.95</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>19.05</v>
+        <v>18.8</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.005277044854881342</v>
+        <v>-0.007915567282321826</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18550,10 +18550,10 @@
         <v>184</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>184.9</v>
+        <v>187.7</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.004891304347826118</v>
+        <v>0.02010869565217385</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18655,10 +18655,10 @@
         <v>5.278</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.026</v>
+        <v>4.99</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.04774535809018564</v>
+        <v>-0.05456612353164066</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18684,10 +18684,10 @@
         <v>0.083</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.06024096385542157</v>
+        <v>0.01204819277108435</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18713,10 +18713,10 @@
         <v>2.94</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>2.9</v>
+        <v>2.925</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.01360544217687076</v>
+        <v>-0.005102040816326573</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18800,10 +18800,10 @@
         <v>1.13</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.1</v>
+        <v>1.085</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.02654867256637151</v>
+        <v>-0.03982300884955747</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18829,10 +18829,10 @@
         <v>1.68</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.78</v>
+        <v>1.7</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.05952380952380958</v>
+        <v>0.01190476190476192</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18858,10 +18858,10 @@
         <v>0.133</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.127</v>
+        <v>0.125</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04511278195488726</v>
+        <v>-0.06015037593984968</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18916,10 +18916,10 @@
         <v>20.4</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.004901960784313621</v>
+        <v>-0.009803921568627416</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19421,10 +19421,10 @@
         <v>79.53</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.25</v>
+        <v>79.34</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.003520684018609344</v>
+        <v>-0.002389035584056302</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -19451,10 +19451,10 @@
         <v>16.61</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>16.67</v>
+        <v>16.76</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.003612281757977259</v>
+        <v>0.009030704394942935</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -19481,10 +19481,10 @@
         <v>8.404999999999999</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.31</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.01130279595478868</v>
+        <v>-0.005353955978584168</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -19511,10 +19511,10 @@
         <v>15.42</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>14.89</v>
+        <v>14.9</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03437094682230865</v>
+        <v>-0.03372243839169906</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -19541,10 +19541,10 @@
         <v>100.35</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>98.62</v>
+        <v>98.64</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01723966118584943</v>
+        <v>-0.01704035874439456</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -19571,10 +19571,10 @@
         <v>71.58</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>69.52</v>
+        <v>69.48</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.02877898854428615</v>
+        <v>-0.02933780385582557</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -19601,10 +19601,10 @@
         <v>109.7</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>107.1</v>
+        <v>106.65</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.02370100273473116</v>
+        <v>-0.02780309936189605</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -19631,10 +19631,10 @@
         <v>72.16</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>72.72</v>
+        <v>72.34</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.007760532150776085</v>
+        <v>0.00249445676274954</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -19661,10 +19661,10 @@
         <v>9.385</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>9.275</v>
+        <v>9.35</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.0117208311134789</v>
+        <v>-0.003729355354288774</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -19691,10 +19691,10 @@
         <v>27.93</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>27.55</v>
+        <v>27.65</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.01360544217687071</v>
+        <v>-0.01002506265664165</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -20560,10 +20560,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>109.4</v>
+        <v>109</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.3606965174129353</v>
+        <v>0.3557213930348258</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20590,10 +20590,10 @@
         <v>12.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>11.75</v>
+        <v>11.9</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.06</v>
+        <v>-0.04799999999999997</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20620,10 +20620,10 @@
         <v>211.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>215.2</v>
+        <v>216.8</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01605288007554286</v>
+        <v>0.02360717658168083</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20650,10 +20650,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.89</v>
+        <v>14.9</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.07687538747675131</v>
+        <v>-0.07625542467451946</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20710,10 +20710,10 @@
         <v>9.15</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>9.275</v>
+        <v>9.35</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.01366120218579235</v>
+        <v>0.02185792349726768</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20740,10 +20740,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.742</v>
+        <v>13.67</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01688367434539984</v>
+        <v>-0.02203462584060666</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20770,10 +20770,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>46.9</v>
+        <v>47.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01956521739130432</v>
+        <v>0.03260869565217391</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20800,10 +20800,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>273.5</v>
+        <v>275.8</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.0936205468102734</v>
+        <v>-0.08599834299917146</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20830,10 +20830,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.38</v>
+        <v>5.28</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05281690140845068</v>
+        <v>-0.07042253521126751</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20932,10 +20932,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>60.4</v>
+        <v>60.62</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04430379746835449</v>
+        <v>-0.04082278481012667</v>
       </c>
       <c r="H16" s="50" t="n"/>
     </row>
@@ -20962,10 +20962,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>97.40000000000001</v>
+        <v>97.75</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0</v>
+        <v>0.003593429158110824</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20992,10 +20992,10 @@
         <v>19.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>19.05</v>
+        <v>18.8</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.04511278195488715</v>
+        <v>-0.05764411027568915</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21022,10 +21022,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.545</v>
+        <v>1.538</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.05156537753222841</v>
+        <v>-0.05586249232658071</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21052,10 +21052,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.002967359050445146</v>
+        <v>0</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21082,10 +21082,10 @@
         <v>6.745</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.51</v>
+        <v>5.515</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1830985915492958</v>
+        <v>-0.1823573017049667</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21112,10 +21112,10 @@
         <v>19.86</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.58</v>
+        <v>18.64</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.06445115810674729</v>
+        <v>-0.0614300100704934</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21142,10 +21142,10 @@
         <v>8.85</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.64</v>
+        <v>7.66</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.1367231638418079</v>
+        <v>-0.1344632768361581</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21172,10 +21172,10 @@
         <v>2.374</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>2.142</v>
+        <v>2.132</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.09772535804549293</v>
+        <v>-0.1019376579612468</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21202,10 +21202,10 @@
         <v>27.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.45</v>
+        <v>21.1</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.227027027027027</v>
+        <v>-0.2396396396396396</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21307,10 +21307,10 @@
         <v>3.82</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>3.87</v>
+        <v>3.92</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01308900523560217</v>
+        <v>0.02617801047120421</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21365,10 +21365,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>27.4</v>
+        <v>27.5</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.003636363636363688</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21394,10 +21394,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.149</v>
+        <v>0.15</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.06875000000000006</v>
+        <v>-0.06250000000000006</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21452,10 +21452,10 @@
         <v>8.880000000000001</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.48</v>
+        <v>8.5</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04504504504504508</v>
+        <v>-0.04279279279279288</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21535,10 +21535,10 @@
         <v>17.85</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>17.2</v>
+        <v>17.25</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03641456582633065</v>
+        <v>-0.03361344537815134</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21661,10 +21661,10 @@
         <v>134.5</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>139</v>
+        <v>139.5</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.03345724907063197</v>
+        <v>0.03717472118959108</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21690,10 +21690,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.3</v>
+        <v>46.66</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.1009708737864078</v>
+        <v>-0.09398058252427191</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21719,10 +21719,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>109.4</v>
+        <v>109</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.3606965174129353</v>
+        <v>0.3557213930348258</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -21748,10 +21748,10 @@
         <v>9.15</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>9.275</v>
+        <v>9.35</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01366120218579235</v>
+        <v>0.02185792349726768</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21777,10 +21777,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>56.4</v>
+        <v>56.9</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.05369127516778528</v>
+        <v>-0.04530201342281884</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21806,10 +21806,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.36</v>
+        <v>45.68</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02931735501818955</v>
+        <v>-0.02246950567087518</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21835,10 +21835,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.44</v>
+        <v>35.4</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05225653206650825</v>
+        <v>0.05106888361045128</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21864,10 +21864,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>28.99</v>
+        <v>29.44</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.04006622516556294</v>
+        <v>-0.02516556291390722</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21893,10 +21893,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>20.68</v>
+        <v>20.57</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1043741879601559</v>
+        <v>-0.1091381550454742</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-16 11:04
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 11:00</t>
+          <t>16/09/2026 11:04</t>
         </is>
       </c>
     </row>
@@ -19381,10 +19381,10 @@
         <v>110</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>107.2</v>
+        <v>107.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02545454545454543</v>
+        <v>-0.02636363636363642</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19411,10 +19411,10 @@
         <v>275.3</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>277.5</v>
+        <v>277.6</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.007991282237558985</v>
+        <v>0.008354522339266295</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19441,10 +19441,10 @@
         <v>124.3</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>124.5</v>
+        <v>124.4</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.001609010458568004</v>
+        <v>0.0008045052292840589</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19561,10 +19561,10 @@
         <v>15.3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>16.17</v>
+        <v>16.16</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.05686274509803928</v>
+        <v>0.05620915032679735</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19603,10 +19603,10 @@
         <v>406.45</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>403.7</v>
+        <v>404.05</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.006765899864682003</v>
+        <v>-0.005904785336449692</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19735,10 +19735,10 @@
         <v>93.84999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>92.2</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01758124667021834</v>
+        <v>-0.0159829515183804</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -19795,10 +19795,10 @@
         <v>3.664</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.602</v>
+        <v>3.6</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.01692139737991274</v>
+        <v>-0.01746724890829696</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19855,10 +19855,10 @@
         <v>45.11</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>45.46</v>
+        <v>45.51</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.007758811793393957</v>
+        <v>0.008867213478164455</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19915,10 +19915,10 @@
         <v>166.24</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>166.28</v>
+        <v>166.32</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.0002406159769008183</v>
+        <v>0.0004812319538016367</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19945,10 +19945,10 @@
         <v>11.26</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>11.23</v>
+        <v>11.24</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.002664298401420902</v>
+        <v>-0.001776198934280602</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19987,10 +19987,10 @@
         <v>5.9</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.94</v>
+        <v>5.72</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.006779661016949158</v>
+        <v>-0.03050847457627129</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20868,10 +20868,10 @@
         <v>80.48999999999999</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>80.87</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.004721083364393213</v>
+        <v>0.004472605292582922</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>8.5</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.515000000000001</v>
+        <v>8.505000000000001</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.001764705882353008</v>
+        <v>0.0005882352941177391</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>16.77</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>16.575</v>
+        <v>16.595</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.0116279069767442</v>
+        <v>-0.0104353011329756</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>22.4</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>22.45</v>
+        <v>22.35</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.002232142857142889</v>
+        <v>-0.00223214285714273</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21937,7 +21937,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 11:00</t>
+          <t>16/09/2026 11:04</t>
         </is>
       </c>
     </row>
@@ -21964,10 +21964,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>107.2</v>
+        <v>107.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3320895522388058</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22054,10 +22054,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.82</v>
+        <v>14.81</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.08121512709237438</v>
+        <v>-0.08183508989460624</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22114,10 +22114,10 @@
         <v>9.15</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>8.99</v>
+        <v>8.975</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01748633879781422</v>
+        <v>-0.01912568306010937</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22144,10 +22144,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.356</v>
+        <v>13.408</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.04449849763914723</v>
+        <v>-0.04077836600372015</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22204,10 +22204,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>277.5</v>
+        <v>277.6</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.08036454018227009</v>
+        <v>-0.08003314001656993</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22234,10 +22234,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.32</v>
+        <v>5.38</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.06338028169014075</v>
+        <v>-0.05281690140845068</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22336,10 +22336,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>60.24</v>
+        <v>60.28</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.0468354430379747</v>
+        <v>-0.04620253164556964</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -22366,10 +22366,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>92.2</v>
+        <v>92.34999999999999</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.053388090349076</v>
+        <v>-0.05184804928131428</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22396,10 +22396,10 @@
         <v>19.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>18.75</v>
+        <v>18.7</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.06015037593984959</v>
+        <v>-0.06265664160401002</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22740,10 +22740,10 @@
         <v>0.614</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.57</v>
+        <v>0.59</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.07166123778501635</v>
+        <v>-0.03908794788273619</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22769,10 +22769,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>27.72</v>
+        <v>27.75</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.007999999999999959</v>
+        <v>0.00909090909090909</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22798,10 +22798,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.149</v>
+        <v>0.148</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.06875000000000006</v>
+        <v>-0.07500000000000007</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23094,10 +23094,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.58</v>
+        <v>46.64</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.09553398058252431</v>
+        <v>-0.09436893203883494</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23123,10 +23123,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>107.2</v>
+        <v>107.1</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3320895522388058</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23152,10 +23152,10 @@
         <v>9.15</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>8.99</v>
+        <v>8.975</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.01748633879781422</v>
+        <v>-0.01912568306010937</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23181,10 +23181,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>57.05</v>
+        <v>57.15</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.04278523489932893</v>
+        <v>-0.04110738255033562</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23210,10 +23210,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.46</v>
+        <v>45.51</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02717740209715378</v>
+        <v>-0.02610742563663597</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23239,10 +23239,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.84</v>
+        <v>35.88</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.0641330166270785</v>
+        <v>0.06532066508313547</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23268,10 +23268,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>30.22</v>
+        <v>30.16</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.000662251655629125</v>
+        <v>-0.00132450331125825</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-16 18:31
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 11:04</t>
+          <t>16/09/2026 18:31</t>
         </is>
       </c>
     </row>
@@ -19381,10 +19381,10 @@
         <v>110</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>107.1</v>
+        <v>106.2</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02636363636363642</v>
+        <v>-0.03454545454545452</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19411,10 +19411,10 @@
         <v>275.3</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>277.6</v>
+        <v>279.4</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.008354522339266295</v>
+        <v>0.01489284416999624</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19441,10 +19441,10 @@
         <v>124.3</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>124.4</v>
+        <v>124.6</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.0008045052292840589</v>
+        <v>0.002413515687851948</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19471,10 +19471,10 @@
         <v>38.3</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>38.3</v>
+        <v>38</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.007832898172323686</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19561,10 +19561,10 @@
         <v>15.3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>16.16</v>
+        <v>16.7</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.05620915032679735</v>
+        <v>0.09150326797385611</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19603,10 +19603,10 @@
         <v>406.45</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>404.05</v>
+        <v>410.7</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.005904785336449692</v>
+        <v>0.0104563906999631</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19633,10 +19633,10 @@
         <v>25.65</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>25.6</v>
+        <v>25.7</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.001949317738791312</v>
+        <v>0.001949317738791451</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19735,10 +19735,10 @@
         <v>93.84999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>92.34999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.0159829515183804</v>
+        <v>-0.03782631859350024</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -19765,10 +19765,10 @@
         <v>0.703</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.711</v>
+        <v>0.716</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.01137980085348507</v>
+        <v>0.01849217638691325</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19795,10 +19795,10 @@
         <v>3.664</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.6</v>
+        <v>3.638</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.01746724890829696</v>
+        <v>-0.0070960698689957</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19825,10 +19825,10 @@
         <v>5.34</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>5.33</v>
+        <v>5.37</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.001872659176029923</v>
+        <v>0.005617977528089934</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19855,10 +19855,10 @@
         <v>45.11</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>45.51</v>
+        <v>45.75</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.008867213478164455</v>
+        <v>0.01418754156506319</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19885,10 +19885,10 @@
         <v>3.155</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>3.125</v>
+        <v>3.19</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.009508716323296293</v>
+        <v>0.01109350237717913</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19915,10 +19915,10 @@
         <v>166.24</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>166.32</v>
+        <v>166.62</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.0004812319538016367</v>
+        <v>0.002285851780558202</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19945,10 +19945,10 @@
         <v>11.26</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>11.24</v>
+        <v>11.425</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.001776198934280602</v>
+        <v>0.01465364120781536</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19987,10 +19987,10 @@
         <v>5.9</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.72</v>
+        <v>5.96</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.03050847457627129</v>
+        <v>0.01016949152542366</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20092,10 +20092,10 @@
         <v>6.86</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>6.84</v>
+        <v>6.7</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.002915451895043799</v>
+        <v>-0.02332361516034987</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20150,10 +20150,10 @@
         <v>0.21</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.209</v>
+        <v>0.203</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.004761904761904767</v>
+        <v>-0.03333333333333323</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20179,10 +20179,10 @@
         <v>0.39</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>0.02564102564102566</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20208,10 +20208,10 @@
         <v>4.86</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>5.25</v>
+        <v>4.86</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08024691358024684</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20248,10 +20248,10 @@
         <v>1.155</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.16</v>
+        <v>1.19</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.004329004329004236</v>
+        <v>0.03030303030303023</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20277,10 +20277,10 @@
         <v>3.63</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.785</v>
+        <v>3.82</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.04269972451790641</v>
+        <v>0.05234159779614324</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20306,10 +20306,10 @@
         <v>0.8080000000000001</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.795</v>
+        <v>0.779</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.0160891089108911</v>
+        <v>-0.03589108910891092</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20335,10 +20335,10 @@
         <v>0.625</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.625</v>
+        <v>0.618</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.01120000000000001</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20868,10 +20868,10 @@
         <v>80.48999999999999</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>80.84999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.004472605292582922</v>
+        <v>-0.007330103118399668</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -20898,10 +20898,10 @@
         <v>73.48</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>73.42</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.0008165487207403684</v>
+        <v>0.01252041371801853</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>8.5</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.505000000000001</v>
+        <v>8.365</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.0005882352941177391</v>
+        <v>-0.01588235294117644</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>16.77</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>16.595</v>
+        <v>16.8</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.0104353011329756</v>
+        <v>0.00178890876565302</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>22.4</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>22.35</v>
+        <v>22.2</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.00223214285714273</v>
+        <v>-0.008928571428571397</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21048,10 +21048,10 @@
         <v>22.95</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>22.85</v>
+        <v>23.25</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.004357298474945441</v>
+        <v>0.01307189542483663</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21937,7 +21937,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 11:04</t>
+          <t>16/09/2026 18:31</t>
         </is>
       </c>
     </row>
@@ -21964,10 +21964,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>107.1</v>
+        <v>106.2</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.3320895522388058</v>
+        <v>0.3208955223880596</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22024,10 +22024,10 @@
         <v>211.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>220.6</v>
+        <v>222.8</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.04154863078375818</v>
+        <v>0.05193578847969783</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22054,10 +22054,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.81</v>
+        <v>15.06</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.08183508989460624</v>
+        <v>-0.06633601983880959</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22084,10 +22084,10 @@
         <v>24.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>24.22</v>
+        <v>24.44</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.008326394671107381</v>
+        <v>0.01748542880932564</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22114,10 +22114,10 @@
         <v>9.15</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>8.975</v>
+        <v>9.1</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01912568306010937</v>
+        <v>-0.005464480874317017</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22144,10 +22144,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.408</v>
+        <v>13.6</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.04077836600372015</v>
+        <v>-0.02704249534983547</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22174,10 +22174,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>46.9</v>
+        <v>47.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01956521739130432</v>
+        <v>0.03260869565217391</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22204,10 +22204,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>277.6</v>
+        <v>279.4</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.08003314001656993</v>
+        <v>-0.07406793703396859</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22234,10 +22234,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.38</v>
+        <v>5.36</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05281690140845068</v>
+        <v>-0.05633802816901398</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22336,10 +22336,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>60.28</v>
+        <v>60.7</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04620253164556964</v>
+        <v>-0.03955696202531645</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -22366,10 +22366,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>92.34999999999999</v>
+        <v>90.3</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.05184804928131428</v>
+        <v>-0.07289527720739228</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22426,10 +22426,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.54</v>
+        <v>1.553</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.05463474524248003</v>
+        <v>-0.0466543891958257</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22456,10 +22456,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>66.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.0103857566765579</v>
+        <v>0.002967359050444935</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22486,10 +22486,10 @@
         <v>6.745</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.455</v>
+        <v>5.45</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1912527798369162</v>
+        <v>-0.1919940696812454</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22516,10 +22516,10 @@
         <v>19.86</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.62</v>
+        <v>18.68</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.0624370594159113</v>
+        <v>-0.05941591137965759</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22546,10 +22546,10 @@
         <v>8.85</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.64</v>
+        <v>7.41</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.1367231638418079</v>
+        <v>-0.1627118644067796</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22576,10 +22576,10 @@
         <v>2.374</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>2.12</v>
+        <v>2.096</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1069924178601516</v>
+        <v>-0.1171019376579613</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22606,10 +22606,10 @@
         <v>27.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.4</v>
+        <v>20.95</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2288288288288289</v>
+        <v>-0.2450450450450451</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22740,10 +22740,10 @@
         <v>0.614</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03908794788273619</v>
+        <v>-0.08794788273615625</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22769,10 +22769,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>27.75</v>
+        <v>28.92</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.00909090909090909</v>
+        <v>0.0516363636363637</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22798,10 +22798,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.148</v>
+        <v>0.15</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07500000000000007</v>
+        <v>-0.06250000000000006</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22884,8 +22884,12 @@
       <c r="E36" s="11" t="n">
         <v>0.33</v>
       </c>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="13" t="n"/>
+      <c r="F36" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>-0.09090909090909098</v>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
       <c r="A37" s="15" t="n">
@@ -22910,10 +22914,10 @@
         <v>2.47</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.38</v>
+        <v>2.37</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03643724696356287</v>
+        <v>-0.04048582995951421</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22939,10 +22943,10 @@
         <v>17.85</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>17.15</v>
+        <v>17.1</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03921568627450996</v>
+        <v>-0.04201680672268907</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22968,10 +22972,10 @@
         <v>4.18</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>3.73</v>
+        <v>3.72</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.1076555023923444</v>
+        <v>-0.110047846889952</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23065,10 +23069,10 @@
         <v>134.5</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>141.5</v>
+        <v>140</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05204460966542751</v>
+        <v>0.04089219330855019</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23094,10 +23098,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.64</v>
+        <v>46.62</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.09436893203883494</v>
+        <v>-0.0947572815533981</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23123,10 +23127,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>107.1</v>
+        <v>106.2</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.3320895522388058</v>
+        <v>0.3208955223880596</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23152,10 +23156,10 @@
         <v>9.15</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>8.975</v>
+        <v>9.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.01912568306010937</v>
+        <v>-0.005464480874317017</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23181,10 +23185,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>57.15</v>
+        <v>56.95</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.04110738255033562</v>
+        <v>-0.04446308724832213</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23210,10 +23214,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.51</v>
+        <v>45.75</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02610742563663597</v>
+        <v>-0.02097153862615016</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23239,10 +23243,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.88</v>
+        <v>35.92</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.06532066508313547</v>
+        <v>0.06650831353919245</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23297,10 +23301,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>20.64</v>
+        <v>20.92</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1061065396275444</v>
+        <v>-0.09398007795582496</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -23326,10 +23330,10 @@
         <v>24.02</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.22</v>
+        <v>24.44</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.008326394671107381</v>
+        <v>0.01748542880932564</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-16 19:41
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -1364,6 +1364,54 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1791,54 +1839,6 @@
       <font>
         <b val="1"/>
         <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
         <color indexed="18"/>
         <extend val="0"/>
       </font>
@@ -1952,6 +1952,13 @@
     <dxf>
       <font>
         <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
         <color rgb="FF006100"/>
         <extend val="0"/>
       </font>
@@ -1993,13 +2000,6 @@
     <dxf>
       <font>
         <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
         <color rgb="FF006100"/>
         <extend val="0"/>
       </font>
@@ -2020,13 +2020,6 @@
     <dxf>
       <font>
         <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
         <color rgb="FF006100"/>
         <extend val="0"/>
       </font>
@@ -2048,6 +2041,13 @@
         <b val="1"/>
         <condense val="0"/>
         <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
         <extend val="0"/>
       </font>
     </dxf>
@@ -19314,7 +19314,7 @@
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>15/09/2026</t>
+          <t>16/09/2026</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -19349,12 +19349,12 @@
       </c>
       <c r="H1" s="47" t="inlineStr">
         <is>
-          <t>Les valeurs qui montent 📈 avec des volumes 👍:</t>
+          <t>Les valeurs qui montent avec des volumes 👍:</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 18:31</t>
+          <t>16/09/2026 19:41</t>
         </is>
       </c>
     </row>
@@ -19364,27 +19364,27 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>NAE</t>
+          <t>OVH</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>NORTH ATLANTIC</t>
+          <t>OVH GROUPE</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>110</v>
+        <v>16.52</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>106.2</v>
+        <v>16.7</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.03454545454545452</v>
+        <v>0.01089588377723969</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19394,27 +19394,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>SU</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>SCHNEIDER ELECTRIC</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>275.3</v>
+        <v>12.4</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>279.4</v>
+        <v>12.45</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01489284416999624</v>
+        <v>0.004032258064516043</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19424,7 +19424,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>EXA</t>
+          <t>SCHP</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -19434,17 +19434,17 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>EXAIL TECH</t>
+          <t>SECHE ENVIRONNEMENT</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>124.3</v>
+        <v>86.2</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>124.6</v>
+        <v>86.5</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.002413515687851948</v>
+        <v>0.003480278422273749</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19454,7 +19454,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>74SW</t>
+          <t>VK</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -19464,17 +19464,17 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>74SOFTWARE</t>
+          <t>VALLOUREC</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>38.3</v>
+        <v>19.9</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>38</v>
+        <v>19.81</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.007832898172323686</v>
+        <v>-0.004522613065326626</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19484,7 +19484,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>GDS</t>
+          <t>EDEN</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -19494,17 +19494,17 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>RAMSAY GENERALE</t>
+          <t>EDENRED</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>11</v>
+        <v>29.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>11</v>
+        <v>29.19</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0</v>
+        <v>-0.0003424657534245894</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19514,27 +19514,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>DKUPL</t>
+          <t>GTT</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>DEKUPLE</t>
+          <t>GAZTRANS TECHN</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>24</v>
+        <v>221.6</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>24</v>
+        <v>222.8</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.005415162454873723</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19544,27 +19544,27 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>OVH</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>OVH GROUPE</t>
+          <t>VALEO</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>15.3</v>
+        <v>14.79</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>16.7</v>
+        <v>14.74</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.09150326797385611</v>
+        <v>-0.003380662609871463</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19572,12 +19572,30 @@
       <c r="A9" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="13" t="n"/>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>BAIN</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>BAINS MER MONACO</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>140</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="H9" s="6" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" thickBot="1">
@@ -19586,7 +19604,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>MC</t>
+          <t>KER</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -19596,17 +19614,17 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>LVMH</t>
+          <t>KERING</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>406.45</v>
+        <v>238</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>410.7</v>
+        <v>237.45</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.0104563906999631</v>
+        <v>-0.002310924369747947</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19616,27 +19634,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>LBIRD</t>
+          <t>UBI</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>LUMIBIRD</t>
+          <t>UBISOFT</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>25.65</v>
+        <v>5.634</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>25.7</v>
+        <v>5.666</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.001949317738791451</v>
+        <v>0.005679801206957761</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19651,8 +19669,8 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G12" s="20" t="e">
-        <v>#VALUE!</v>
+      <c r="G12" s="20" t="n">
+        <v>0</v>
       </c>
       <c r="H12" s="48" t="inlineStr">
         <is>
@@ -19708,7 +19726,7 @@
       </c>
       <c r="H15" s="47" t="inlineStr">
         <is>
-          <t>Les valeurs qui baissent 📉 avec des volumes 👎:</t>
+          <t>Les valeurs qui baissent avec des volumes 👎:</t>
         </is>
       </c>
     </row>
@@ -19718,7 +19736,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>ABVX</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -19728,17 +19746,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>ABIVAX</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>93.84999999999999</v>
+        <v>20.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>90.3</v>
+        <v>20.95</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.03782631859350024</v>
+        <v>0.007211538461538393</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -19748,7 +19766,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>ANTIN</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -19758,17 +19776,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>AB SCIENCE</t>
+          <t>ANTIN INFRA</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>0.703</v>
+        <v>7.4</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.716</v>
+        <v>7.41</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.01849217638691325</v>
+        <v>0.001351351351351323</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19792,13 +19810,13 @@
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>3.664</v>
+        <v>3.604</v>
       </c>
       <c r="F18" s="12" t="n">
         <v>3.638</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0070960698689957</v>
+        <v>0.009433962264150889</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19808,7 +19826,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ABCA</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -19818,17 +19836,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>ABC ARBITRAGE</t>
+          <t>ABIVAX</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>5.34</v>
+        <v>90.45</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>5.37</v>
+        <v>90.3</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.005617977528089934</v>
+        <v>-0.001658374792703214</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19838,7 +19856,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>STLAP</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -19848,17 +19866,17 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>ACCOR</t>
+          <t>STELLANTIS</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>45.11</v>
+        <v>4.334</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>45.75</v>
+        <v>4.352</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.01418754156506319</v>
+        <v>0.004153207198892636</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19868,7 +19886,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ARAMI</t>
+          <t>TFF</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -19878,17 +19896,17 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>ARAMIS</t>
+          <t>TFF GROUP</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>3.155</v>
+        <v>15</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>3.19</v>
+        <v>15</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01109350237717913</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19898,7 +19916,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -19908,17 +19926,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>AIR LIQUIDE</t>
+          <t>L'OREAL</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>166.24</v>
+        <v>381.9</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>166.62</v>
+        <v>383.2</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.002285851780558202</v>
+        <v>0.003404032469232814</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19928,27 +19946,27 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>AF</t>
+          <t>BASS</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>AIR FRANCE-KLM</t>
+          <t>BASSAC</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>11.26</v>
+        <v>39.8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>11.425</v>
+        <v>39.9</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01465364120781536</v>
+        <v>0.002512562814070388</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19956,12 +19974,30 @@
       <c r="A24" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="22" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="13" t="n"/>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>ELIOR</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>ELIOR GROUP</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="n">
+        <v>1.917</v>
+      </c>
+      <c r="F24" s="12" t="n">
+        <v>1.914</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>-0.001564945226917117</v>
+      </c>
       <c r="H24" s="6" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" thickBot="1">
@@ -19970,27 +20006,27 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>AKW</t>
+          <t>PEUG</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>AKWEL</t>
+          <t>PEUGEOT INVEST</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>5.9</v>
+        <v>53.4</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.96</v>
+        <v>53.2</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.01016949152542366</v>
+        <v>-0.003745318352059845</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20005,8 +20041,8 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G26" s="24" t="e">
-        <v>#VALUE!</v>
+      <c r="G26" s="24" t="n">
+        <v>0</v>
       </c>
       <c r="H26" s="48" t="inlineStr">
         <is>
@@ -20065,7 +20101,7 @@
       </c>
       <c r="H29" s="47" t="inlineStr">
         <is>
-          <t>Les Smallcaps qui montent 📈 avec des volumes 👍:</t>
+          <t>Les Smallcaps qui montent avec des volumes 👍:</t>
         </is>
       </c>
     </row>
@@ -20075,27 +20111,27 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>ALSMA</t>
+          <t>DPT</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>SMAIO</t>
+          <t>ST DUPONT</t>
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>6.86</v>
+        <v>0.089</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>6.7</v>
+        <v>0.081</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.02332361516034987</v>
+        <v>-0.08988764044943813</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20104,7 +20140,7 @@
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>ALEXP</t>
+          <t>AL2SI</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
@@ -20114,17 +20150,17 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>ONE EXPERIENCE</t>
+          <t>2CRSI</t>
         </is>
       </c>
       <c r="E31" s="11" t="n">
-        <v>0.428</v>
+        <v>29.06</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.424</v>
+        <v>28.92</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.009345794392523372</v>
+        <v>-0.004817618719889781</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20133,7 +20169,7 @@
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>ALFOR</t>
+          <t>ALSTW</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
@@ -20143,17 +20179,17 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>FORSEE POWER</t>
+          <t>STREAMWIDE</t>
         </is>
       </c>
       <c r="E32" s="11" t="n">
-        <v>0.21</v>
+        <v>87.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.203</v>
+        <v>87</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03333333333333323</v>
+        <v>-0.009111617312072861</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20162,7 +20198,7 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>ALNMG</t>
+          <t>ALDEL</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
@@ -20172,17 +20208,17 @@
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>NETMEDIA</t>
+          <t>DELFINGEN</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>0.39</v>
+        <v>33.1</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.4</v>
+        <v>33.1</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.02564102564102566</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20191,7 +20227,7 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>ALGTR</t>
+          <t>ALESE</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
@@ -20201,29 +20237,47 @@
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>TERA GROUPE</t>
+          <t>ENTECH</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>4.86</v>
+        <v>10.3</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.86</v>
+        <v>10.22</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0</v>
+        <v>-0.007766990291262143</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
       <c r="A35" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="10" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="12" t="n"/>
-      <c r="G35" s="13" t="n"/>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>ALNXT</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>EG</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>NEXTEDIA</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="F35" s="12" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="n">
@@ -20231,7 +20285,7 @@
       </c>
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>ALPAU</t>
+          <t>ALCAF</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
@@ -20241,17 +20295,17 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>PAULIC MEUNERIE</t>
+          <t>CAFOM</t>
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>1.155</v>
+        <v>13.25</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.19</v>
+        <v>13.25</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.03030303030303023</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20260,7 +20314,7 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>ALMDT</t>
+          <t>ALHG</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
@@ -20270,17 +20324,17 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>MEDIAN TECHNOLOGIES</t>
+          <t>LOUIS HACHETTE</t>
         </is>
       </c>
       <c r="E37" s="11" t="n">
-        <v>3.63</v>
+        <v>1.77</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.82</v>
+        <v>1.766</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.05234159779614324</v>
+        <v>-0.002259887005649719</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20289,7 +20343,7 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>ALNFL</t>
+          <t>ALPAU</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
@@ -20299,17 +20353,17 @@
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>NFL BIOSCIENCES</t>
+          <t>PAULIC MEUNERIE</t>
         </is>
       </c>
       <c r="E38" s="11" t="n">
-        <v>0.8080000000000001</v>
+        <v>1.19</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.779</v>
+        <v>1.19</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03589108910891092</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20318,27 +20372,27 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>ALCLA</t>
+          <t>FMONC</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>CLARANOVA</t>
+          <t>FINANCIERE MONCEY</t>
         </is>
       </c>
       <c r="E39" s="11" t="n">
-        <v>0.625</v>
+        <v>116.5</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.618</v>
+        <v>116.5</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.01120000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20351,8 +20405,8 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G40" s="29" t="e">
-        <v>#VALUE!</v>
+      <c r="G40" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="H40" s="48" t="inlineStr">
         <is>
@@ -20418,7 +20472,7 @@
       <c r="D43" s="10" t="n"/>
       <c r="E43" s="11" t="n"/>
       <c r="F43" s="12" t="n">
-        <v>15.3</v>
+        <v>23.2</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0</v>
@@ -20433,7 +20487,7 @@
       <c r="D44" s="10" t="n"/>
       <c r="E44" s="11" t="n"/>
       <c r="F44" s="12" t="n">
-        <v>11</v>
+        <v>44.21</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>0</v>
@@ -20448,7 +20502,7 @@
       <c r="D45" s="10" t="n"/>
       <c r="E45" s="11" t="n"/>
       <c r="F45" s="12" t="n">
-        <v>24</v>
+        <v>5.37</v>
       </c>
       <c r="G45" s="13" t="n">
         <v>0</v>
@@ -20463,7 +20517,7 @@
       <c r="D46" s="10" t="n"/>
       <c r="E46" s="11" t="n"/>
       <c r="F46" s="12" t="n">
-        <v>110</v>
+        <v>5.634</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>0</v>
@@ -20478,7 +20532,7 @@
       <c r="D47" s="10" t="n"/>
       <c r="E47" s="11" t="n"/>
       <c r="F47" s="12" t="n">
-        <v>25.65</v>
+        <v>31.86</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>0</v>
@@ -20492,8 +20546,12 @@
       <c r="C48" s="9" t="n"/>
       <c r="D48" s="10" t="n"/>
       <c r="E48" s="11" t="n"/>
-      <c r="F48" s="12" t="n"/>
-      <c r="G48" s="13" t="n"/>
+      <c r="F48" s="12" t="n">
+        <v>27.89</v>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
       <c r="A49" s="8" t="n">
@@ -20504,7 +20562,7 @@
       <c r="D49" s="10" t="n"/>
       <c r="E49" s="11" t="n"/>
       <c r="F49" s="12" t="n">
-        <v>275.3</v>
+        <v>29.2</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>0</v>
@@ -20519,7 +20577,7 @@
       <c r="D50" s="10" t="n"/>
       <c r="E50" s="11" t="n"/>
       <c r="F50" s="12" t="n">
-        <v>124.3</v>
+        <v>1308</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>0</v>
@@ -20534,7 +20592,7 @@
       <c r="D51" s="10" t="n"/>
       <c r="E51" s="11" t="n"/>
       <c r="F51" s="12" t="n">
-        <v>1.548</v>
+        <v>47.2</v>
       </c>
       <c r="G51" s="13" t="n">
         <v>0</v>
@@ -20549,7 +20607,7 @@
       <c r="D52" s="10" t="n"/>
       <c r="E52" s="11" t="n"/>
       <c r="F52" s="12" t="n">
-        <v>771</v>
+        <v>36.98</v>
       </c>
       <c r="G52" s="13" t="n">
         <v>0</v>
@@ -20565,8 +20623,8 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G53" s="34" t="e">
-        <v>#VALUE!</v>
+      <c r="G53" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="H53" s="48" t="inlineStr">
         <is>
@@ -20633,7 +20691,7 @@
       <c r="D56" s="36" t="n"/>
       <c r="E56" s="18" t="n"/>
       <c r="F56" s="12" t="n">
-        <v>80.48999999999999</v>
+        <v>80.03</v>
       </c>
       <c r="G56" s="37" t="n">
         <v>0</v>
@@ -20649,7 +20707,7 @@
       <c r="D57" s="36" t="n"/>
       <c r="E57" s="18" t="n"/>
       <c r="F57" s="12" t="n">
-        <v>16.77</v>
+        <v>16.81</v>
       </c>
       <c r="G57" s="37" t="n">
         <v>0</v>
@@ -20665,7 +20723,7 @@
       <c r="D58" s="36" t="n"/>
       <c r="E58" s="18" t="n"/>
       <c r="F58" s="12" t="n">
-        <v>73.48</v>
+        <v>74.7</v>
       </c>
       <c r="G58" s="37" t="n">
         <v>0</v>
@@ -20681,7 +20739,7 @@
       <c r="D59" s="36" t="n"/>
       <c r="E59" s="18" t="n"/>
       <c r="F59" s="12" t="n">
-        <v>22.4</v>
+        <v>19.9</v>
       </c>
       <c r="G59" s="37" t="n">
         <v>0</v>
@@ -20697,7 +20755,7 @@
       <c r="D60" s="36" t="n"/>
       <c r="E60" s="18" t="n"/>
       <c r="F60" s="12" t="n">
-        <v>22.95</v>
+        <v>23.2</v>
       </c>
       <c r="G60" s="37" t="n">
         <v>0</v>
@@ -20713,7 +20771,7 @@
       <c r="D61" s="36" t="n"/>
       <c r="E61" s="18" t="n"/>
       <c r="F61" s="12" t="n">
-        <v>8.5</v>
+        <v>14.79</v>
       </c>
       <c r="G61" s="37" t="n">
         <v>0</v>
@@ -20728,9 +20786,11 @@
       <c r="C62" s="30" t="n"/>
       <c r="D62" s="36" t="n"/>
       <c r="E62" s="18" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="F62" s="12" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="G62" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -20742,9 +20802,11 @@
       <c r="C63" s="30" t="n"/>
       <c r="D63" s="36" t="n"/>
       <c r="E63" s="18" t="n"/>
-      <c r="F63" s="12" t="n"/>
-      <c r="G63" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="F63" s="12" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="G63" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -20756,9 +20818,11 @@
       <c r="C64" s="30" t="n"/>
       <c r="D64" s="36" t="n"/>
       <c r="E64" s="18" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="F64" s="12" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="G64" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -20851,7 +20915,7 @@
       </c>
       <c r="B69" s="36" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>ERF</t>
         </is>
       </c>
       <c r="C69" s="30" t="inlineStr">
@@ -20861,17 +20925,17 @@
       </c>
       <c r="D69" s="36" t="inlineStr">
         <is>
-          <t>TOTALENERGIES</t>
+          <t>EUROFINS SCIENTIFIC</t>
         </is>
       </c>
       <c r="E69" s="18" t="n">
-        <v>80.48999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.90000000000001</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.007330103118399668</v>
+        <v>-0.004016064257028074</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -20881,7 +20945,7 @@
       </c>
       <c r="B70" s="36" t="inlineStr">
         <is>
-          <t>ERF</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="C70" s="30" t="inlineStr">
@@ -20891,17 +20955,17 @@
       </c>
       <c r="D70" s="36" t="inlineStr">
         <is>
-          <t>EUROFINS SCIENTIFIC</t>
+          <t>TOTALENERGIES</t>
         </is>
       </c>
       <c r="E70" s="18" t="n">
-        <v>73.48</v>
+        <v>80.03</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>74.40000000000001</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.01252041371801853</v>
+        <v>-0.001624390853429907</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -20911,7 +20975,7 @@
       </c>
       <c r="B71" s="36" t="inlineStr">
         <is>
-          <t>MAU</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="C71" s="30" t="inlineStr">
@@ -20921,17 +20985,17 @@
       </c>
       <c r="D71" s="36" t="inlineStr">
         <is>
-          <t>MAUREL ET PROM</t>
+          <t>CARREFOUR</t>
         </is>
       </c>
       <c r="E71" s="18" t="n">
-        <v>8.5</v>
+        <v>16.81</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>8.365</v>
+        <v>16.8</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.01588235294117644</v>
+        <v>-0.0005948839976203458</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -20941,7 +21005,7 @@
       </c>
       <c r="B72" s="36" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>VK</t>
         </is>
       </c>
       <c r="C72" s="30" t="inlineStr">
@@ -20951,17 +21015,17 @@
       </c>
       <c r="D72" s="36" t="inlineStr">
         <is>
-          <t>CARREFOUR</t>
+          <t>VALLOUREC</t>
         </is>
       </c>
       <c r="E72" s="18" t="n">
-        <v>16.77</v>
+        <v>19.9</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>16.8</v>
+        <v>19.81</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.00178890876565302</v>
+        <v>-0.004522613065326626</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -20971,27 +21035,27 @@
       </c>
       <c r="B73" s="36" t="inlineStr">
         <is>
-          <t>JCQ</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="C73" s="30" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D73" s="36" t="inlineStr">
         <is>
-          <t>JACQUET METAL</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="E73" s="18" t="n">
-        <v>22.4</v>
+        <v>12.4</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>22.2</v>
+        <v>12.45</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.008928571428571397</v>
+        <v>0.004032258064516043</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21001,27 +21065,27 @@
       </c>
       <c r="B74" s="36" t="inlineStr">
         <is>
-          <t>ATEME</t>
+          <t>MTU</t>
         </is>
       </c>
       <c r="C74" s="30" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D74" s="36" t="inlineStr">
         <is>
-          <t>ATEME</t>
+          <t>MANITOU</t>
         </is>
       </c>
       <c r="E74" s="18" t="n">
-        <v>12.4</v>
+        <v>23.2</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>12.45</v>
+        <v>23.25</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.004032258064516043</v>
+        <v>0.002155172413793134</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21031,7 +21095,7 @@
       </c>
       <c r="B75" s="36" t="inlineStr">
         <is>
-          <t>MTU</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="C75" s="30" t="inlineStr">
@@ -21041,17 +21105,17 @@
       </c>
       <c r="D75" s="36" t="inlineStr">
         <is>
-          <t>MANITOU</t>
+          <t>VALEO</t>
         </is>
       </c>
       <c r="E75" s="18" t="n">
-        <v>22.95</v>
+        <v>14.79</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>23.25</v>
+        <v>14.74</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.01307189542483663</v>
+        <v>-0.003380662609871463</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21059,13 +21123,29 @@
       <c r="A76" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="36" t="n"/>
-      <c r="C76" s="30" t="n"/>
-      <c r="D76" s="36" t="n"/>
-      <c r="E76" s="18" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>EDEN</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D76" s="36" t="inlineStr">
+        <is>
+          <t>EDENRED</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="F76" s="12" t="n">
+        <v>29.19</v>
+      </c>
+      <c r="G76" s="37" t="n">
+        <v>-0.0003424657534245894</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21073,13 +21153,29 @@
       <c r="A77" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B77" s="36" t="n"/>
-      <c r="C77" s="30" t="n"/>
-      <c r="D77" s="36" t="n"/>
-      <c r="E77" s="18" t="n"/>
-      <c r="F77" s="12" t="n"/>
-      <c r="G77" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>SCHP</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D77" s="36" t="inlineStr">
+        <is>
+          <t>SECHE ENVIRONNEMENT</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="F77" s="12" t="n">
+        <v>86.5</v>
+      </c>
+      <c r="G77" s="37" t="n">
+        <v>0.003480278422273749</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21087,13 +21183,29 @@
       <c r="A78" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B78" s="36" t="n"/>
-      <c r="C78" s="30" t="n"/>
-      <c r="D78" s="36" t="n"/>
-      <c r="E78" s="18" t="n"/>
-      <c r="F78" s="12" t="n"/>
-      <c r="G78" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B78" s="36" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D78" s="36" t="inlineStr">
+        <is>
+          <t>BIC</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="F78" s="12" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="G78" s="37" t="n">
+        <v>-0.001477104874446212</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -21104,8 +21216,8 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G79" s="34" t="e">
-        <v>#VALUE!</v>
+      <c r="G79" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="H79" s="6" t="n"/>
     </row>
@@ -21535,108 +21647,88 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B56:B65">
-    <cfRule type="expression" priority="16" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="22" dxfId="77" stopIfTrue="1">
       <formula>IF(AO56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:B78">
-    <cfRule type="expression" priority="14" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="20" dxfId="77" stopIfTrue="1">
       <formula>IF(AO69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B81">
-    <cfRule type="expression" priority="56" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="62" dxfId="77" stopIfTrue="1">
       <formula>IF(AN62&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82:B91">
-    <cfRule type="expression" priority="20" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="26" dxfId="77" stopIfTrue="1">
       <formula>IF(AL82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="expression" priority="52" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="58" dxfId="77" stopIfTrue="1">
       <formula>IF(AL91&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="expression" priority="55" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="61" dxfId="77" stopIfTrue="1">
       <formula>IF(AN75&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:B105">
-    <cfRule type="expression" priority="18" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="24" dxfId="77" stopIfTrue="1">
       <formula>IF(AO96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B106">
-    <cfRule type="expression" priority="53" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="59" dxfId="77" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="expression" priority="54" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="60" dxfId="77" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D56:D65">
-    <cfRule type="expression" priority="15" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="21" dxfId="77" stopIfTrue="1">
       <formula>IF(AQ56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D78">
-    <cfRule type="expression" priority="13" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="19" dxfId="77" stopIfTrue="1">
       <formula>IF(AQ69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82:D91">
-    <cfRule type="expression" priority="19" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="25" dxfId="77" stopIfTrue="1">
       <formula>IF(AN82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D96:D105">
-    <cfRule type="expression" priority="17" dxfId="77" stopIfTrue="1">
+    <cfRule type="expression" priority="23" dxfId="77" stopIfTrue="1">
       <formula>IF(AQ96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="32" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="34" dxfId="0" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
@@ -21660,149 +21752,149 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="60" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="61" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="63" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
       <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
       <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="64" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="65" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="18">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="18">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="17" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="17" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
+    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="16" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="15">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="15">
       <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>
@@ -21832,43 +21924,63 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
     <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
+  <conditionalFormatting sqref="F30:F39">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21937,7 +22049,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/09/2026 18:31</t>
+          <t>16/09/2026 19:41</t>
         </is>
       </c>
     </row>
@@ -22253,7 +22365,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>0.02001849504745926</v>
+        <v>0.01624759718445673</v>
       </c>
       <c r="H12" s="48" t="inlineStr">
         <is>
@@ -22625,7 +22737,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.0949579911811978</v>
+        <v>-0.09963012330341871</v>
       </c>
       <c r="H26" s="48" t="inlineStr">
         <is>
@@ -22989,7 +23101,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.04634063154680584</v>
+        <v>-0.04198879593316946</v>
       </c>
       <c r="H40" s="48" t="inlineStr">
         <is>
@@ -23347,7 +23459,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>0.02087476589203252</v>
+        <v>0.01825492822143965</v>
       </c>
       <c r="H53" s="48" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-18 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19354,7 +19354,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>18/09/2026 10:18</t>
+          <t>18/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -19381,10 +19381,10 @@
         <v>141.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>139.2</v>
+        <v>138.85</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01764290755116443</v>
+        <v>-0.02011291460832742</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19411,10 +19411,10 @@
         <v>17.69</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>17.39</v>
+        <v>17.23</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.0169587337478802</v>
+        <v>-0.02600339174674962</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19441,10 +19441,10 @@
         <v>227</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>223.8</v>
+        <v>223.2</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01409691629955942</v>
+        <v>-0.01674008810572692</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19471,10 +19471,10 @@
         <v>15.495</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>15.385</v>
+        <v>15.375</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.007099064214262629</v>
+        <v>-0.007744433688286494</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19501,10 +19501,10 @@
         <v>24.8</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>24.48</v>
+        <v>24.62</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.01290322580645162</v>
+        <v>-0.00725806451612902</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19531,10 +19531,10 @@
         <v>58.9</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>60.3</v>
+        <v>60.95</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02376910016977926</v>
+        <v>0.03480475382003403</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19561,10 +19561,10 @@
         <v>58.05</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>57.25</v>
+        <v>57.6</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01378122308354862</v>
+        <v>-0.007751937984496051</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19591,10 +19591,10 @@
         <v>239.6</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>237.7</v>
+        <v>238.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.007929883138564298</v>
+        <v>-0.00459098497495824</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19621,10 +19621,10 @@
         <v>314.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>308</v>
+        <v>299.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.02066772655007949</v>
+        <v>-0.04769475357710652</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19651,10 +19651,10 @@
         <v>36.2</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>35.58</v>
+        <v>35.18</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.01712707182320454</v>
+        <v>-0.02817679558011058</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19753,10 +19753,10 @@
         <v>5.45</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.405</v>
+        <v>5.355</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.008256880733944941</v>
+        <v>-0.01743119266055041</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -19783,10 +19783,10 @@
         <v>49.35</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>50.7</v>
+        <v>51.5</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02735562310030398</v>
+        <v>0.04356636271529885</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19813,10 +19813,10 @@
         <v>14.86</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>14.6</v>
+        <v>14.2</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.01749663526244952</v>
+        <v>-0.04441453566621804</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19843,10 +19843,10 @@
         <v>53.1</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>53.1</v>
+        <v>53.2</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0</v>
+        <v>0.001883239171374791</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19873,10 +19873,10 @@
         <v>105.08</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>105</v>
+        <v>104.9</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.0007613247049866606</v>
+        <v>-0.001712980586219953</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19903,10 +19903,10 @@
         <v>377.4</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>373</v>
+        <v>372.8</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.01165871754107042</v>
+        <v>-0.01218865924748269</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19933,10 +19933,10 @@
         <v>43.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>43.2</v>
+        <v>43.1</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.002320185614849221</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19963,10 +19963,10 @@
         <v>141.45</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>139.45</v>
+        <v>139.8</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01413927182750089</v>
+        <v>-0.01166489925768807</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19993,10 +19993,10 @@
         <v>67.84999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>67.59999999999999</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.003684598378776714</v>
+        <v>-0.002947678703021203</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20023,10 +20023,10 @@
         <v>0.712</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.713</v>
+        <v>0.724</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.001404494382022473</v>
+        <v>0.01685393258426968</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20128,10 +20128,10 @@
         <v>5.293</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.49</v>
+        <v>5.5</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.03721896844889478</v>
+        <v>0.03910825618741731</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20157,10 +20157,10 @@
         <v>0.074</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.073</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.01351351351351353</v>
+        <v>-0.02702702702702705</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20186,10 +20186,10 @@
         <v>2.96</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>3</v>
+        <v>2.98</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.01351351351351353</v>
+        <v>0.006756756756756763</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20215,10 +20215,10 @@
         <v>89</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>89</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>-0.01797752808988758</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20331,10 +20331,10 @@
         <v>25.1</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>25.1</v>
+        <v>25.2</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>0.003984063745019835</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20360,10 +20360,10 @@
         <v>2.58</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>2.56</v>
+        <v>2.48</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.007751937984496131</v>
+        <v>-0.03875968992248065</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20486,10 +20486,10 @@
         <v>75.26000000000001</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>74.92</v>
+        <v>75.11</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.004517672070156835</v>
+        <v>-0.001993090619186894</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20515,10 +20515,10 @@
         <v>47.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>47.4</v>
+        <v>48.2</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0</v>
+        <v>0.01687763713080178</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20544,10 +20544,10 @@
         <v>108.7</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>108.9</v>
+        <v>108.8</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.001839926402943908</v>
+        <v>0.0009199632014718889</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20602,10 +20602,10 @@
         <v>19.12</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.1</v>
+        <v>19.13</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.001046025104602488</v>
+        <v>0.0005230125523011511</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20631,10 +20631,10 @@
         <v>16.81</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>16.635</v>
+        <v>16.56</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01041046995835795</v>
+        <v>-0.0148720999405116</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20660,10 +20660,10 @@
         <v>72.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>72</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.005524861878453117</v>
+        <v>-0.006906077348066298</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20689,10 +20689,10 @@
         <v>239.6</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>237.7</v>
+        <v>238.5</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.007929883138564298</v>
+        <v>-0.00459098497495824</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20718,10 +20718,10 @@
         <v>18.64</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>18.5</v>
+        <v>18.44</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.007510729613733936</v>
+        <v>-0.01072961373390554</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20747,10 +20747,10 @@
         <v>16.06</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>15.96</v>
+        <v>15.93</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.006226650062266369</v>
+        <v>-0.008094645080946389</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22045,7 +22045,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>18/09/2026 10:18</t>
+          <t>18/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22072,10 +22072,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>104.2</v>
+        <v>102.3</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.2960199004975124</v>
+        <v>0.2723880597014924</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22102,10 +22102,10 @@
         <v>12.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>12.3</v>
+        <v>12.45</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.01599999999999994</v>
+        <v>-0.004000000000000056</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22132,10 +22132,10 @@
         <v>211.8</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>223.8</v>
+        <v>223.2</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.05665722379603399</v>
+        <v>0.05382436260623218</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22162,10 +22162,10 @@
         <v>16.13</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.96</v>
+        <v>14.95</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.07253564786112822</v>
+        <v>-0.07315561066336018</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22192,10 +22192,10 @@
         <v>24.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>24.48</v>
+        <v>24.62</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01915070774354708</v>
+        <v>0.02497918401332229</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22222,10 +22222,10 @@
         <v>9.15</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>8.970000000000001</v>
+        <v>8.92</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01967213114754095</v>
+        <v>-0.02513661202185797</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22252,10 +22252,10 @@
         <v>13.978</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>13.468</v>
+        <v>13.116</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03648590642438115</v>
+        <v>-0.06166833595650308</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22282,10 +22282,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>47.4</v>
+        <v>48.2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03043478260869562</v>
+        <v>0.0478260869565218</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22312,10 +22312,10 @@
         <v>301.75</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>289.05</v>
+        <v>287.95</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.04208782104391048</v>
+        <v>-0.04573322286661147</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22342,10 +22342,10 @@
         <v>5.68</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.38</v>
+        <v>5.36</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05281690140845068</v>
+        <v>-0.05633802816901398</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22444,10 +22444,10 @@
         <v>63.2</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>59.62</v>
+        <v>59.9</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05664556962025324</v>
+        <v>-0.05221518987341778</v>
       </c>
       <c r="H16" s="49" t="n"/>
     </row>
@@ -22474,10 +22474,10 @@
         <v>97.40000000000001</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>93.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.03696098562628345</v>
+        <v>-0.03388090349075987</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22534,10 +22534,10 @@
         <v>1.629</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.529</v>
+        <v>1.515</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.06138735420503381</v>
+        <v>-0.06998158379373855</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22564,10 +22564,10 @@
         <v>67.40000000000001</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>67.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.001483679525222678</v>
+        <v>0</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22594,10 +22594,10 @@
         <v>6.745</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>5.405</v>
+        <v>5.355</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1986656782802075</v>
+        <v>-0.2060785767234988</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22624,10 +22624,10 @@
         <v>19.86</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>18.8</v>
+        <v>18.72</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.05337361530714999</v>
+        <v>-0.05740181268882178</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22654,10 +22654,10 @@
         <v>8.85</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.3</v>
+        <v>7.35</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.1751412429378531</v>
+        <v>-0.1694915254237288</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22684,10 +22684,10 @@
         <v>2.374</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>2.214</v>
+        <v>2.256</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.06739679865206408</v>
+        <v>-0.04970513900589735</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22714,10 +22714,10 @@
         <v>27.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.55</v>
+        <v>21.35</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2234234234234234</v>
+        <v>-0.2306306306306306</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22819,10 +22819,10 @@
         <v>3.82</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>3.89</v>
+        <v>3.85</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01832460732984301</v>
+        <v>0.007853403141361322</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22877,10 +22877,10 @@
         <v>27.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>29.34</v>
+        <v>29</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.0669090909090909</v>
+        <v>0.05454545454545454</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22906,10 +22906,10 @@
         <v>0.16</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.147</v>
+        <v>0.146</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.08125000000000007</v>
+        <v>-0.08750000000000008</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22935,10 +22935,10 @@
         <v>9.859999999999999</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.06</v>
+        <v>9.08</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.08113590263691674</v>
+        <v>-0.07910750507099386</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22964,10 +22964,10 @@
         <v>8.880000000000001</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.0540540540540541</v>
+        <v>-0.04279279279279288</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23018,10 +23018,10 @@
         <v>2.47</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.42</v>
+        <v>2.5</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02024291497975719</v>
+        <v>0.01214574898785417</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23047,10 +23047,10 @@
         <v>17.85</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>16.9</v>
+        <v>17</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.05322128851540632</v>
+        <v>-0.04761904761904769</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23076,10 +23076,10 @@
         <v>4.18</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>3.94</v>
+        <v>3.86</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05741626794258368</v>
+        <v>-0.07655502392344495</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23176,7 +23176,7 @@
         <v>136</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.01115241635687725</v>
+        <v>0.01115241635687732</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23202,10 +23202,10 @@
         <v>51.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>46.5</v>
+        <v>46.64</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.0970873786407767</v>
+        <v>-0.09436893203883494</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23231,10 +23231,10 @@
         <v>80.40000000000001</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>104.2</v>
+        <v>102.3</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.2960199004975124</v>
+        <v>0.2723880597014924</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23260,10 +23260,10 @@
         <v>9.15</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>8.970000000000001</v>
+        <v>8.92</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.01967213114754095</v>
+        <v>-0.02513661202185797</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23289,10 +23289,10 @@
         <v>59.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>56.9</v>
+        <v>56.7</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.04530201342281884</v>
+        <v>-0.04865771812080535</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23318,10 +23318,10 @@
         <v>46.73</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.77</v>
+        <v>46.02</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02054354804194294</v>
+        <v>-0.0151936657393536</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23347,10 +23347,10 @@
         <v>33.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>35.58</v>
+        <v>35.18</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.0564133016627078</v>
+        <v>0.04453681710213777</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23376,10 +23376,10 @@
         <v>30.2</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>29.36</v>
+        <v>29.02</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02781456953642384</v>
+        <v>-0.0390728476821192</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23405,10 +23405,10 @@
         <v>23.09</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>20.61</v>
+        <v>20.7</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1074058033780858</v>
+        <v>-0.1035080121264617</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -23434,10 +23434,10 @@
         <v>24.02</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.48</v>
+        <v>24.62</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01915070774354708</v>
+        <v>0.02497918401332229</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-21 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>19/09/2026 11:10</t>
+          <t>21/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>17.62</v>
+        <v>17.03</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.007432818753573617</v>
+        <v>-0.02630074328187521</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.54</v>
+        <v>24.58</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02850356294536827</v>
+        <v>-0.02692003167062562</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12.55</v>
+        <v>12.9</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01619433198380575</v>
+        <v>0.04453441295546565</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8.27</v>
+        <v>8.205</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.007859733978234524</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>60.3</v>
+        <v>60.1</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.005770816158285267</v>
+        <v>-0.009068425391591049</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.915</v>
+        <v>1.925</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.005221932114882511</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>48.4</v>
+        <v>53.4</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0</v>
+        <v>0.1033057851239669</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.64</v>
+        <v>3.56</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.002739726027397202</v>
+        <v>-0.0246575342465753</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.5</v>
+        <v>34.55</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>0.001449275362318758</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.62</v>
+        <v>4.745</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.004310344827586115</v>
+        <v>0.02262931034482768</v>
       </c>
       <c r="H16" s="48" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>5.265</v>
+        <v>5.215</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.001902949571836306</v>
+        <v>-0.007611798287345393</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.17</v>
+        <v>4.259</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.00690640628721122</v>
+        <v>0.01428911645629924</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01424979044425817</v>
+        <v>0.001676445934618573</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21</v>
+        <v>21.65</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0</v>
+        <v>0.03095238095238088</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.522</v>
+        <v>0.523</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01754385964912282</v>
+        <v>0.01949317738791425</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.35</v>
+        <v>7.44</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0</v>
+        <v>0.01224489795918378</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>28.95</v>
+        <v>30.15</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>0.04145077720207251</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52</v>
+        <v>52.6</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02564102564102558</v>
+        <v>0.03747534516765283</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0</v>
+        <v>-0.01449275362318842</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.802</v>
+        <v>5.92</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01968365553602798</v>
+        <v>0.04042179261862909</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.113</v>
+        <v>0.111</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.008771929824561412</v>
+        <v>-0.02631578947368423</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.92</v>
+        <v>3.82</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>-0.02551020408163268</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18776,10 +18776,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>21.4</v>
+        <v>21</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.01834862385321111</v>
+        <v>-0.03669724770642205</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.88</v>
+        <v>4.86</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>-0.004098360655737618</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.95</v>
+        <v>3.09</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01006711409395967</v>
+        <v>0.03691275167785231</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.135</v>
+        <v>0.153</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>0.1333333333333332</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>8.27</v>
+        <v>8.205</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0</v>
+        <v>-0.007859733978234524</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>48.4</v>
+        <v>53.4</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0</v>
+        <v>0.1033057851239669</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.55</v>
+        <v>12.9</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.01619433198380575</v>
+        <v>0.04453441295546565</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>97.22</v>
+        <v>97.64</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.003076292042657887</v>
+        <v>0.001230516817063213</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>9.18</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0</v>
+        <v>0.002178649237472721</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.3</v>
+        <v>60.1</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.005770816158285267</v>
+        <v>-0.009068425391591049</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.915</v>
+        <v>1.925</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>0.005221932114882511</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.64</v>
+        <v>3.56</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.002739726027397202</v>
+        <v>-0.0246575342465753</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.54</v>
+        <v>24.58</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02850356294536827</v>
+        <v>-0.02692003167062562</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20557,7 +20557,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>19/09/2026 11:10</t>
+          <t>21/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20584,10 +20584,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.313</v>
+        <v>0.305</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1082621082621082</v>
+        <v>-0.131054131054131</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20614,10 +20614,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.76</v>
+        <v>18.34</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1240778001341383</v>
+        <v>0.2300469483568075</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20644,10 +20644,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.3</v>
+        <v>79.13</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.00672844991748129</v>
+        <v>0.00457026786847784</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20674,10 +20674,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02857142857142857</v>
+        <v>-0.01428571428571429</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20734,10 +20734,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>48.4</v>
+        <v>53.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0189473684210526</v>
+        <v>0.1242105263157894</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20764,10 +20764,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.72</v>
+        <v>35.08</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03448275862068971</v>
+        <v>-0.02447163515016692</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20794,10 +20794,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>225.6</v>
+        <v>224</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.04347826086956524</v>
+        <v>0.03607770582793715</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20854,10 +20854,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>22.2</v>
+        <v>21.75</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.01552106430155217</v>
+        <v>-0.0354767184035477</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20956,10 +20956,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04166666666666651</v>
+        <v>-0.05555555555555541</v>
       </c>
       <c r="H16" s="48" t="n"/>
     </row>
@@ -20986,10 +20986,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.64</v>
+        <v>3.56</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.12</v>
+        <v>0.0953846153846154</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21016,10 +21016,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.265</v>
+        <v>5.215</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.09613733905579408</v>
+        <v>-0.1047210300429185</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21046,10 +21046,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.658</v>
+        <v>3.61</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.00274122807017538</v>
+        <v>-0.01041666666666674</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21076,10 +21076,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.4</v>
+        <v>7.27</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.00671140939597313</v>
+        <v>-0.02416107382550343</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21106,10 +21106,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>24.2</v>
+        <v>23.9</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02497985495568094</v>
+        <v>-0.03706688154713947</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21136,10 +21136,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>76.81999999999999</v>
+        <v>77.42</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.08656294200848642</v>
+        <v>0.09504950495049502</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21166,10 +21166,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.35</v>
+        <v>7.44</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.08125000000000004</v>
+        <v>-0.06999999999999995</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21196,10 +21196,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.1</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.004914004914005028</v>
+        <v>-0.003685503685503825</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21226,10 +21226,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.86</v>
+        <v>21.62</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.00459558823529402</v>
+        <v>-0.00643382352941179</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21331,10 +21331,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.802</v>
+        <v>5.92</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1244186046511627</v>
+        <v>0.1472868217054263</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21360,10 +21360,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.065</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1585365853658536</v>
+        <v>-0.2073170731707317</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21389,10 +21389,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.08</v>
+        <v>5.26</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1331058020477816</v>
+        <v>-0.1023890784982936</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21418,10 +21418,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.954</v>
+        <v>0.96</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.09573459715639809</v>
+        <v>-0.0900473933649289</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21447,10 +21447,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>8.58</v>
+        <v>9.07</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.002325581395348788</v>
+        <v>0.05465116279069775</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21476,10 +21476,10 @@
         <v>20.3</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2413793103448275</v>
+        <v>0.2364532019704434</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21505,10 +21505,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.27</v>
+        <v>0.265</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03571428571428574</v>
+        <v>-0.05357142857142862</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21534,10 +21534,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.21</v>
+        <v>1.215</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.05468750000000005</v>
+        <v>-0.05078124999999996</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21563,10 +21563,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.1187500000000001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21591,9 +21591,11 @@
       <c r="E39" s="11" t="n">
         <v>19.85</v>
       </c>
-      <c r="F39" s="12" t="n"/>
-      <c r="G39" s="13" t="e">
-        <v>#VALUE!</v>
+      <c r="F39" s="12" t="n">
+        <v>19.35</v>
+      </c>
+      <c r="G39" s="13" t="n">
+        <v>-0.0251889168765743</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21687,10 +21689,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.08</v>
+        <v>6.56</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.02797761790567543</v>
+        <v>0.04876099120703433</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21716,10 +21718,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.27</v>
+        <v>5.32</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.009578544061302648</v>
+        <v>0.01915708812260547</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21774,10 +21776,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>22.2</v>
+        <v>21.75</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.01552106430155217</v>
+        <v>-0.0354767184035477</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21803,10 +21805,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.4</v>
+        <v>21.45</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.009259259259259391</v>
+        <v>-0.006944444444444543</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21832,10 +21834,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.828</v>
+        <v>3.92</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04443334997503753</v>
+        <v>-0.02146779830254626</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21861,10 +21863,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>92.84999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.0271017699115043</v>
+        <v>0.02654867256637158</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21890,10 +21892,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.76</v>
+        <v>1.776</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.06033101975440469</v>
+        <v>-0.05178857447944473</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21919,10 +21921,10 @@
         <v>35.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.005681818181818262</v>
+        <v>-0.03409090909090917</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21948,10 +21950,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-21 18:45
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/09/2026 13:00</t>
+          <t>21/09/2026 18:45</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>17.03</v>
+        <v>17.16</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02630074328187521</v>
+        <v>-0.01886792452830179</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.58</v>
+        <v>24.64</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02692003167062562</v>
+        <v>-0.02454473475851152</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.04453441295546565</v>
+        <v>0.03643724696356284</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8.205</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.007859733978234524</v>
+        <v>-0.02781136638452242</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>60.1</v>
+        <v>60.55</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.009068425391591049</v>
+        <v>-0.00164880461665295</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.925</v>
+        <v>1.915</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.005221932114882511</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.56</v>
+        <v>3.78</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0246575342465753</v>
+        <v>0.03561643835616436</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.55</v>
+        <v>34.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.001449275362318758</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.745</v>
+        <v>4.71</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.02262931034482768</v>
+        <v>0.01508620689655179</v>
       </c>
       <c r="H16" s="48" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>5.215</v>
+        <v>5.085</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.007611798287345393</v>
+        <v>-0.03235014272121788</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.259</v>
+        <v>4.227</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01428911645629924</v>
+        <v>0.006668254346273034</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>23.9</v>
+        <v>23.46</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.001676445934618573</v>
+        <v>-0.01676445934618603</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21.65</v>
+        <v>20</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.03095238095238088</v>
+        <v>-0.04761904761904762</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.523</v>
+        <v>0.532</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01949317738791425</v>
+        <v>0.03703703703703707</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.44</v>
+        <v>7.38</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.01224489795918378</v>
+        <v>0.004081632653061259</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>30.15</v>
+        <v>29.7</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.04145077720207251</v>
+        <v>0.02590673575129534</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.01449275362318842</v>
+        <v>0</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.92</v>
+        <v>6.019</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.04042179261862909</v>
+        <v>0.05782073813708255</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.111</v>
+        <v>0.11</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02631578947368423</v>
+        <v>-0.03508771929824565</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.82</v>
+        <v>3.91</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02551020408163268</v>
+        <v>-0.002551020408163211</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18776,10 +18776,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>21</v>
+        <v>21.2</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.03669724770642205</v>
+        <v>-0.02752293577981658</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.06</v>
+        <v>1.07</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.0701754385964911</v>
+        <v>-0.06140350877192969</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.86</v>
+        <v>4.88</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.004098360655737618</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.09</v>
+        <v>3.13</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.03691275167785231</v>
+        <v>0.05033557046979863</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>5.07</v>
+        <v>5.06</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.009765624999999965</v>
+        <v>-0.0117187500000001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.153</v>
+        <v>0.164</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1333333333333332</v>
+        <v>0.2148148148148148</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>8.205</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.007859733978234524</v>
+        <v>-0.02781136638452242</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.04453441295546565</v>
+        <v>0.03643724696356284</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>97.64</v>
+        <v>97.94</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.001230516817063213</v>
+        <v>0.0043068088597211</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.1</v>
+        <v>60.55</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.009068425391591049</v>
+        <v>-0.00164880461665295</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.925</v>
+        <v>1.915</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.005221932114882511</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.56</v>
+        <v>3.78</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.0246575342465753</v>
+        <v>0.03561643835616436</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.58</v>
+        <v>24.64</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02692003167062562</v>
+        <v>-0.02454473475851152</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20557,7 +20557,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/09/2026 13:00</t>
+          <t>21/09/2026 18:45</t>
         </is>
       </c>
     </row>
@@ -20584,10 +20584,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.305</v>
+        <v>0.302</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.131054131054131</v>
+        <v>-0.1396011396011396</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20614,10 +20614,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.34</v>
+        <v>18.01</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.2300469483568075</v>
+        <v>0.2079141515761235</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20644,10 +20644,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.13</v>
+        <v>78.43000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.00457026786847784</v>
+        <v>-0.004316364098006719</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20674,10 +20674,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>138</v>
+        <v>138.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01428571428571429</v>
+        <v>-0.01071428571428571</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20764,10 +20764,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.08</v>
+        <v>35.7</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02447163515016692</v>
+        <v>-0.007230255839821969</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20794,10 +20794,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>224</v>
+        <v>223.4</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03607770582793715</v>
+        <v>0.03330249768732663</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20854,10 +20854,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.75</v>
+        <v>21.7</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0354767184035477</v>
+        <v>-0.03769401330376947</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20956,10 +20956,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05555555555555541</v>
+        <v>-0.04166666666666651</v>
       </c>
       <c r="H16" s="48" t="n"/>
     </row>
@@ -20986,10 +20986,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.56</v>
+        <v>3.78</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.0953846153846154</v>
+        <v>0.163076923076923</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21016,10 +21016,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.215</v>
+        <v>5.085</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1047210300429185</v>
+        <v>-0.1270386266094421</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21046,10 +21046,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.61</v>
+        <v>3.586</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01041666666666674</v>
+        <v>-0.01699561403508779</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21076,10 +21076,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.27</v>
+        <v>7.21</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02416107382550343</v>
+        <v>-0.03221476510067117</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21106,10 +21106,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.9</v>
+        <v>23.46</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.03706688154713947</v>
+        <v>-0.05479452054794518</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21136,10 +21136,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>77.42</v>
+        <v>78.04000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.09504950495049502</v>
+        <v>0.1038189533239039</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21166,10 +21166,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.44</v>
+        <v>7.38</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.06999999999999995</v>
+        <v>-0.07750000000000001</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21196,10 +21196,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.109999999999999</v>
+        <v>8.02</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.003685503685503825</v>
+        <v>-0.01474201474201486</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21226,10 +21226,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.62</v>
+        <v>21.6</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.00643382352941179</v>
+        <v>-0.007352941176470594</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21331,10 +21331,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.92</v>
+        <v>6.019</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1472868217054263</v>
+        <v>0.1664728682170543</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21360,10 +21360,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.065</v>
+        <v>0.064</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2073170731707317</v>
+        <v>-0.2195121951219512</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21389,10 +21389,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.26</v>
+        <v>5.38</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1023890784982936</v>
+        <v>-0.08191126279863488</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21418,10 +21418,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.96</v>
+        <v>0.962</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0900473933649289</v>
+        <v>-0.08815165876777249</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21447,10 +21447,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.07</v>
+        <v>8.98</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.05465116279069775</v>
+        <v>0.044186046511628</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21505,10 +21505,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.265</v>
+        <v>0.269</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05357142857142862</v>
+        <v>-0.03928571428571432</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21534,10 +21534,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.215</v>
+        <v>1.24</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.05078124999999996</v>
+        <v>-0.03125000000000003</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21563,10 +21563,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.141</v>
+        <v>0.139</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1187500000000001</v>
+        <v>-0.13125</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21592,10 +21592,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.35</v>
+        <v>19.8</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.0251889168765743</v>
+        <v>-0.002518891687657466</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21689,10 +21689,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.56</v>
+        <v>6.55</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.04876099120703433</v>
+        <v>0.0471622701838529</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21718,10 +21718,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.32</v>
+        <v>5.348</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.01915708812260547</v>
+        <v>0.02452107279693489</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21776,10 +21776,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.75</v>
+        <v>21.7</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.0354767184035477</v>
+        <v>-0.03769401330376947</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21805,10 +21805,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.45</v>
+        <v>21.5</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.006944444444444543</v>
+        <v>-0.004629629629629695</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21834,10 +21834,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.92</v>
+        <v>3.962</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02146779830254626</v>
+        <v>-0.01098352471293061</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21863,10 +21863,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>92.8</v>
+        <v>93.7</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.02654867256637158</v>
+        <v>0.03650442477876103</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21892,10 +21892,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.776</v>
+        <v>1.802</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05178857447944473</v>
+        <v>-0.03790710090763479</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-22 19:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19347,7 +19347,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/09/2026 13:01</t>
+          <t>22/09/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -19374,10 +19374,10 @@
         <v>154.85</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>152.55</v>
+        <v>152.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01485308362931859</v>
+        <v>-0.01775912173070714</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19404,10 +19404,10 @@
         <v>18.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.39</v>
+        <v>18.15</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.0188365650969529</v>
+        <v>0.005540166204986032</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19434,10 +19434,10 @@
         <v>44.65</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>45.44</v>
+        <v>46.61</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01769316909294511</v>
+        <v>0.04389697648376262</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19464,10 +19464,10 @@
         <v>12.85</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.003891050583657505</v>
+        <v>0.02723735408560309</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19524,10 +19524,10 @@
         <v>6.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>6.715</v>
+        <v>6.81</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0251908396946565</v>
+        <v>0.03969465648854958</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19554,10 +19554,10 @@
         <v>60.85</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0106820049301561</v>
+        <v>-0.009038619556286018</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19584,10 +19584,10 @@
         <v>94.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>91.40000000000001</v>
+        <v>94.05</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.02972399150743097</v>
+        <v>-0.00159235668789815</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19644,10 +19644,10 @@
         <v>72.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>72.7</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.00553250345781474</v>
+        <v>0.01175656984785627</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19746,10 +19746,10 @@
         <v>5.075</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.235</v>
+        <v>5.28</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.03152709359605914</v>
+        <v>0.04039408866995075</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19776,10 +19776,10 @@
         <v>21.74</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>21.92</v>
+        <v>22.3</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.008279668813247621</v>
+        <v>0.02575896964121446</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19806,10 +19806,10 @@
         <v>20.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>20.7</v>
+        <v>20.3</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.02985074626865661</v>
+        <v>0.009950248756218869</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19836,10 +19836,10 @@
         <v>23.5</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>24.3</v>
+        <v>23.92</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03404255319148939</v>
+        <v>0.01787234042553199</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19866,10 +19866,10 @@
         <v>12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>12.44</v>
+        <v>12.254</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.03666666666666663</v>
+        <v>0.02116666666666663</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19896,10 +19896,10 @@
         <v>20.98</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.2</v>
+        <v>22.34</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.05815061963775018</v>
+        <v>0.06482364156339368</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19926,10 +19926,10 @@
         <v>14.46</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>14.3</v>
+        <v>14.16</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01106500691562933</v>
+        <v>-0.02074688796680503</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19986,10 +19986,10 @@
         <v>21.1</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>21.35</v>
+        <v>21.45</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.01184834123222749</v>
+        <v>0.01658767772511838</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20016,10 +20016,10 @@
         <v>102.14</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>102.16</v>
+        <v>99.55</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0001958096729978071</v>
+        <v>-0.0253573526532211</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20121,10 +20121,10 @@
         <v>6.004</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.904</v>
+        <v>5.887</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.01665556295802792</v>
+        <v>-0.01948700866089274</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20150,10 +20150,10 @@
         <v>5.4</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>5.2</v>
+        <v>5.17</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03703703703703707</v>
+        <v>-0.04259259259259267</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20179,10 +20179,10 @@
         <v>9.01</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.23</v>
+        <v>9.32</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.02441731409544957</v>
+        <v>0.03440621531631526</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20208,10 +20208,10 @@
         <v>0.166</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.163</v>
+        <v>0.159</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01807228915662652</v>
+        <v>-0.04216867469879522</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20237,10 +20237,10 @@
         <v>28.56</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>29.4</v>
+        <v>29.36</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.02941176470588235</v>
+        <v>0.02801120448179274</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20295,10 +20295,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.92</v>
+        <v>4.9</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.008196721311475417</v>
+        <v>0.0040983606557378</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20324,10 +20324,10 @@
         <v>33</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>32.8</v>
+        <v>32.9</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.006060606060606146</v>
+        <v>-0.003030303030303073</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20353,10 +20353,10 @@
         <v>41</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>43.65</v>
+        <v>43.1</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.06463414634146337</v>
+        <v>0.05121951219512198</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20382,10 +20382,10 @@
         <v>0.455</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.412</v>
+        <v>0.43</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.09450549450549459</v>
+        <v>-0.05494505494505499</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20479,10 +20479,10 @@
         <v>35.7</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>35.26</v>
+        <v>35.46</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.01232492997198893</v>
+        <v>-0.006722689075630307</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20508,10 +20508,10 @@
         <v>167.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165.4</v>
+        <v>165.8</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01194743130227001</v>
+        <v>-0.009557945041815976</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20537,10 +20537,10 @@
         <v>4.26</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>4.24</v>
+        <v>4.22</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.004694835680751074</v>
+        <v>-0.009389671361502356</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20566,10 +20566,10 @@
         <v>94.2</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>91.40000000000001</v>
+        <v>94.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02972399150743097</v>
+        <v>-0.00159235668789815</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20595,10 +20595,10 @@
         <v>16.72</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>16.74</v>
+        <v>16.22</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.001196172248803802</v>
+        <v>-0.0299043062200957</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20624,10 +20624,10 @@
         <v>72.2</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>73.2</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.01385041551246537</v>
+        <v>0.005540166204986032</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20653,10 +20653,10 @@
         <v>60.85</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.0106820049301561</v>
+        <v>-0.009038619556286018</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20740,10 +20740,10 @@
         <v>4.878</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>4.858</v>
+        <v>4.778</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.004100041000410099</v>
+        <v>-0.02050020500205013</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20838,10 +20838,10 @@
         <v>44.65</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>45.44</v>
+        <v>46.61</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>0.01769316909294511</v>
+        <v>0.04389697648376262</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -20868,10 +20868,10 @@
         <v>78.56</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>77.37</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.0151476578411405</v>
+        <v>-0.003436863543788137</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -20898,10 +20898,10 @@
         <v>78.06</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>78.59999999999999</v>
+        <v>78.95999999999999</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>0.006917755572636331</v>
+        <v>0.01152959262106061</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>6.55</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>6.715</v>
+        <v>6.81</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.0251908396946565</v>
+        <v>0.03969465648854958</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>3.78</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>3.74</v>
+        <v>3.75</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>-0.01058201058201047</v>
+        <v>-0.007936507936507886</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>38.06</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>40.56</v>
+        <v>40.98</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>0.06568575932737782</v>
+        <v>0.07672096689437716</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -21018,10 +21018,10 @@
         <v>46.5</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>47.12</v>
+        <v>46.78</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>0.01333333333333328</v>
+        <v>0.00602150537634411</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -21048,10 +21048,10 @@
         <v>140.8</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>143</v>
+        <v>143.7</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.01562499999999992</v>
+        <v>0.02059659090909075</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -21078,10 +21078,10 @@
         <v>138.85</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>141.45</v>
+        <v>141.05</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>0.01872524306805902</v>
+        <v>0.01584443644220394</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -21191,10 +21191,10 @@
         <v>38.06</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>40.56</v>
+        <v>40.98</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.06568575932737782</v>
+        <v>0.07672096689437716</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21221,10 +21221,10 @@
         <v>44.65</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>45.44</v>
+        <v>46.61</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.01769316909294511</v>
+        <v>0.04389697648376262</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21251,10 +21251,10 @@
         <v>12.85</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>12.8</v>
+        <v>13.2</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.003891050583657505</v>
+        <v>0.02723735408560309</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21281,10 +21281,10 @@
         <v>78.06</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>78.59999999999999</v>
+        <v>78.95999999999999</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.006917755572636331</v>
+        <v>0.01152959262106061</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21311,10 +21311,10 @@
         <v>78.56</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>77.37</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.0151476578411405</v>
+        <v>-0.003436863543788137</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21341,10 +21341,10 @@
         <v>94.2</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>91.40000000000001</v>
+        <v>94.05</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.02972399150743097</v>
+        <v>-0.00159235668789815</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21371,10 +21371,10 @@
         <v>6.55</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>6.715</v>
+        <v>6.81</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.0251908396946565</v>
+        <v>0.03969465648854958</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21401,10 +21401,10 @@
         <v>3.78</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>3.74</v>
+        <v>3.75</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.01058201058201047</v>
+        <v>-0.007936507936507886</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21461,10 +21461,10 @@
         <v>46.5</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>47.12</v>
+        <v>46.78</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.01333333333333328</v>
+        <v>0.00602150537634411</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/09/2026 13:01</t>
+          <t>22/09/2026 19:00</t>
         </is>
       </c>
     </row>
@@ -22333,10 +22333,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.297</v>
+        <v>0.302</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1538461538461538</v>
+        <v>-0.1396011396011396</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22363,10 +22363,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.39</v>
+        <v>18.15</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.233400402414487</v>
+        <v>0.2173038229376257</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22393,10 +22393,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>77.37</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.0177732639329693</v>
+        <v>-0.006093690491303666</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22453,10 +22453,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>124.3</v>
+        <v>124.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.0008038585209003901</v>
+        <v>0</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22513,10 +22513,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.26</v>
+        <v>35.46</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01946607341490553</v>
+        <v>-0.01390433815350389</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22543,10 +22543,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>222.2</v>
+        <v>223</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02775208140610546</v>
+        <v>0.03145235892691958</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22603,10 +22603,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.85</v>
+        <v>21.7</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.03104212860310418</v>
+        <v>-0.03769401330376947</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22705,10 +22705,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.02777777777777761</v>
+        <v>-0.05555555555555541</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -22735,10 +22735,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.74</v>
+        <v>3.75</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1507692307692308</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22765,10 +22765,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.235</v>
+        <v>5.28</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1012875536480686</v>
+        <v>-0.09356223175965664</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22795,10 +22795,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.572</v>
+        <v>3.608</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02083333333333335</v>
+        <v>-0.01096491228070176</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22825,10 +22825,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.2</v>
+        <v>7.25</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03355704697986577</v>
+        <v>-0.02684563758389264</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22855,10 +22855,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>24.3</v>
+        <v>23.92</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02095084609186139</v>
+        <v>-0.03626107977437545</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22885,10 +22885,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>78.59999999999999</v>
+        <v>78.95999999999999</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.1117397454031116</v>
+        <v>0.1168316831683167</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22915,10 +22915,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.49</v>
+        <v>7.38</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.06374999999999997</v>
+        <v>-0.07750000000000001</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22945,10 +22945,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.15</v>
+        <v>8.08</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.001228501228501202</v>
+        <v>-0.007371007371007432</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22975,10 +22975,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>21.92</v>
+        <v>22.3</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.007352941176470594</v>
+        <v>0.0248161764705882</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23080,10 +23080,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.904</v>
+        <v>5.887</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1441860465116279</v>
+        <v>0.1408914728682169</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23109,10 +23109,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.065</v>
+        <v>0.064</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2073170731707317</v>
+        <v>-0.2195121951219512</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23138,10 +23138,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.2</v>
+        <v>5.17</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1126279863481229</v>
+        <v>-0.1177474402730376</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23196,10 +23196,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.23</v>
+        <v>9.32</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.07325581395348847</v>
+        <v>0.08372093023255822</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23225,10 +23225,10 @@
         <v>20.3</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.1</v>
+        <v>25.2</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2364532019704434</v>
+        <v>0.2413793103448275</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23254,10 +23254,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.259</v>
+        <v>0.262</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.07500000000000005</v>
+        <v>-0.06428571428571433</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23283,10 +23283,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.21</v>
+        <v>1.215</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.05468750000000005</v>
+        <v>-0.05078124999999996</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23312,10 +23312,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.139</v>
+        <v>0.14</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.13125</v>
+        <v>-0.1249999999999999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23341,10 +23341,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.75</v>
+        <v>19.45</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.005037783375314932</v>
+        <v>-0.02015113350125955</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23438,10 +23438,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.715</v>
+        <v>6.81</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.07354116706634692</v>
+        <v>0.08872901678657071</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23467,10 +23467,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.538</v>
+        <v>5.378</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.06091954022988515</v>
+        <v>0.03026819923371655</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23525,10 +23525,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.85</v>
+        <v>21.7</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.03104212860310418</v>
+        <v>-0.03769401330376947</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23583,10 +23583,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.94</v>
+        <v>3.97</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01647528706939598</v>
+        <v>-0.008986520219670502</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23612,10 +23612,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>91.40000000000001</v>
+        <v>94.05</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01106194690265487</v>
+        <v>0.04037610619469017</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23641,10 +23641,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.79</v>
+        <v>1.758</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.04431393486385476</v>
+        <v>-0.06139882541377469</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23699,10 +23699,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>222.5</v>
+        <v>220.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.002252252252252252</v>
+        <v>-0.006756756756756757</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-23 16:37
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19347,7 +19347,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/09/2026 19:00</t>
+          <t>23/09/2026 16:37</t>
         </is>
       </c>
     </row>
@@ -19374,10 +19374,10 @@
         <v>154.85</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>152.1</v>
+        <v>151.25</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01775912173070714</v>
+        <v>-0.02324830481110749</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19404,10 +19404,10 @@
         <v>18.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.15</v>
+        <v>18.04</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.005540166204986032</v>
+        <v>-0.0005540166204987015</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19434,10 +19434,10 @@
         <v>44.65</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>46.61</v>
+        <v>45.75</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.04389697648376262</v>
+        <v>0.02463605823068312</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19494,10 +19494,10 @@
         <v>53.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01498127340823978</v>
+        <v>0.0112359550561798</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19524,10 +19524,10 @@
         <v>6.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>6.81</v>
+        <v>6.695</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.03969465648854958</v>
+        <v>0.02213740458015274</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19554,10 +19554,10 @@
         <v>60.85</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>60.3</v>
+        <v>63.8</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.009038619556286018</v>
+        <v>0.04847986852917002</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19584,10 +19584,10 @@
         <v>94.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>94.05</v>
+        <v>95.05</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.00159235668789815</v>
+        <v>0.009023354564755778</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19614,10 +19614,10 @@
         <v>140</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>140</v>
+        <v>141.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0</v>
+        <v>0.01071428571428571</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19644,10 +19644,10 @@
         <v>72.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>73.15000000000001</v>
+        <v>74.75</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01175656984785627</v>
+        <v>0.03388658367911484</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19746,10 +19746,10 @@
         <v>5.075</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.28</v>
+        <v>5.13</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.04039408866995075</v>
+        <v>0.01083743842364526</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19776,10 +19776,10 @@
         <v>21.74</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>22.3</v>
+        <v>23.4</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02575896964121446</v>
+        <v>0.07635694572217112</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19806,10 +19806,10 @@
         <v>20.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>20.3</v>
+        <v>20.55</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.009950248756218869</v>
+        <v>0.0223880597014925</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19836,10 +19836,10 @@
         <v>23.5</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>23.92</v>
+        <v>23.38</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01787234042553199</v>
+        <v>-0.005106382978723446</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19866,10 +19866,10 @@
         <v>12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>12.254</v>
+        <v>11.96</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.02116666666666663</v>
+        <v>-0.003333333333333262</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19896,10 +19896,10 @@
         <v>20.98</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.34</v>
+        <v>22.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.06482364156339368</v>
+        <v>0.07244995233555765</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19926,10 +19926,10 @@
         <v>14.46</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>14.16</v>
+        <v>13.98</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02074688796680503</v>
+        <v>-0.03319502074688799</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19956,10 +19956,10 @@
         <v>0.083</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.083</v>
+        <v>0.082</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>-0.01204819277108435</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19986,10 +19986,10 @@
         <v>21.1</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>21.45</v>
+        <v>20.9</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.01658767772511838</v>
+        <v>-0.009478672985782125</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20016,10 +20016,10 @@
         <v>102.14</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>99.55</v>
+        <v>96.39</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0253573526532211</v>
+        <v>-0.05629528098688075</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20121,10 +20121,10 @@
         <v>6.004</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.887</v>
+        <v>5.599</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.01948700866089274</v>
+        <v>-0.06745502998001322</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20150,10 +20150,10 @@
         <v>5.4</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>5.17</v>
+        <v>5.32</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.04259259259259267</v>
+        <v>-0.01481481481481483</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20179,10 +20179,10 @@
         <v>9.01</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.32</v>
+        <v>9.42</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.03440621531631526</v>
+        <v>0.04550499445061045</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20208,10 +20208,10 @@
         <v>0.166</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.159</v>
+        <v>0.15</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04216867469879522</v>
+        <v>-0.09638554216867477</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20237,10 +20237,10 @@
         <v>28.56</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>29.36</v>
+        <v>29.94</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.02801120448179274</v>
+        <v>0.04831932773109253</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20295,10 +20295,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.9</v>
+        <v>4.89</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.0040983606557378</v>
+        <v>0.002049180327868809</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20353,10 +20353,10 @@
         <v>41</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>43.1</v>
+        <v>48.75</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.05121951219512198</v>
+        <v>0.1890243902439024</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20382,10 +20382,10 @@
         <v>0.455</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05494505494505499</v>
+        <v>-0.1428571428571428</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20479,10 +20479,10 @@
         <v>35.7</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>35.46</v>
+        <v>34.8</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.006722689075630307</v>
+        <v>-0.0252100840336136</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20508,10 +20508,10 @@
         <v>167.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165.8</v>
+        <v>165.6</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.009557945041815976</v>
+        <v>-0.01075268817204308</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20537,10 +20537,10 @@
         <v>4.26</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>4.22</v>
+        <v>4.14</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.009389671361502356</v>
+        <v>-0.02816901408450707</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20566,10 +20566,10 @@
         <v>94.2</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>94.05</v>
+        <v>95.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.00159235668789815</v>
+        <v>0.009023354564755778</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20595,10 +20595,10 @@
         <v>16.72</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>16.22</v>
+        <v>16.64</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.0299043062200957</v>
+        <v>-0.004784688995215209</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20624,10 +20624,10 @@
         <v>72.2</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>72.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.005540166204986032</v>
+        <v>-0.004155124653739573</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20653,10 +20653,10 @@
         <v>60.85</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.3</v>
+        <v>63.8</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.009038619556286018</v>
+        <v>0.04847986852917002</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20682,10 +20682,10 @@
         <v>140</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>140</v>
+        <v>141.5</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>0.01071428571428571</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20740,10 +20740,10 @@
         <v>4.878</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>4.778</v>
+        <v>4.69</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02050020500205013</v>
+        <v>-0.03854038540385398</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20838,10 +20838,10 @@
         <v>44.65</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>46.61</v>
+        <v>45.75</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>0.04389697648376262</v>
+        <v>0.02463605823068312</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -20868,10 +20868,10 @@
         <v>78.56</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>78.29000000000001</v>
+        <v>79.45999999999999</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.003436863543788137</v>
+        <v>0.01145621181262718</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -20898,10 +20898,10 @@
         <v>78.06</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>78.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>0.01152959262106061</v>
+        <v>-0.0105047399436332</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>6.55</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>6.81</v>
+        <v>6.695</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.03969465648854958</v>
+        <v>0.02213740458015274</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>3.78</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>3.75</v>
+        <v>3.82</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>-0.007936507936507886</v>
+        <v>0.01058201058201059</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>38.06</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>40.98</v>
+        <v>41.64</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>0.07672096689437716</v>
+        <v>0.09406200735680499</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -21018,10 +21018,10 @@
         <v>46.5</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>46.78</v>
+        <v>46.31</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>0.00602150537634411</v>
+        <v>-0.004086021505376295</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -21048,10 +21048,10 @@
         <v>140.8</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>143.7</v>
+        <v>141.6</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.02059659090909075</v>
+        <v>0.005681818181818061</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -21078,10 +21078,10 @@
         <v>138.85</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>141.05</v>
+        <v>139.25</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>0.01584443644220394</v>
+        <v>0.00288080662585528</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -21191,10 +21191,10 @@
         <v>38.06</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>40.98</v>
+        <v>41.64</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.07672096689437716</v>
+        <v>0.09406200735680499</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21221,10 +21221,10 @@
         <v>44.65</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>46.61</v>
+        <v>45.75</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.04389697648376262</v>
+        <v>0.02463605823068312</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21281,10 +21281,10 @@
         <v>78.06</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>78.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.01152959262106061</v>
+        <v>-0.0105047399436332</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21311,10 +21311,10 @@
         <v>78.56</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>78.29000000000001</v>
+        <v>79.45999999999999</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.003436863543788137</v>
+        <v>0.01145621181262718</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21341,10 +21341,10 @@
         <v>94.2</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>94.05</v>
+        <v>95.05</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.00159235668789815</v>
+        <v>0.009023354564755778</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21371,10 +21371,10 @@
         <v>6.55</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>6.81</v>
+        <v>6.695</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.03969465648854958</v>
+        <v>0.02213740458015274</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21401,10 +21401,10 @@
         <v>3.78</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>3.75</v>
+        <v>3.82</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.007936507936507886</v>
+        <v>0.01058201058201059</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21431,10 +21431,10 @@
         <v>53.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.01498127340823978</v>
+        <v>0.0112359550561798</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21461,10 +21461,10 @@
         <v>46.5</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>46.78</v>
+        <v>46.31</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.00602150537634411</v>
+        <v>-0.004086021505376295</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/09/2026 19:00</t>
+          <t>23/09/2026 16:37</t>
         </is>
       </c>
     </row>
@@ -22333,10 +22333,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.302</v>
+        <v>0.308</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1396011396011396</v>
+        <v>-0.1225071225071225</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22363,10 +22363,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.15</v>
+        <v>18.04</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.2173038229376257</v>
+        <v>0.209926224010731</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22393,10 +22393,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>78.29000000000001</v>
+        <v>79.45999999999999</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.006093690491303666</v>
+        <v>0.008759680081249178</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22423,10 +22423,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>140</v>
+        <v>141.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>0.01071428571428571</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22453,10 +22453,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>124.4</v>
+        <v>124.8</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0</v>
+        <v>0.003215434083601218</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22483,10 +22483,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.2</v>
+        <v>54</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1410526315789474</v>
+        <v>0.1368421052631579</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22513,10 +22513,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.46</v>
+        <v>34.8</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01390433815350389</v>
+        <v>-0.03225806451612914</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22573,10 +22573,10 @@
         <v>0.016</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.06250000000000006</v>
+        <v>-0.1875000000000001</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22603,10 +22603,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.7</v>
+        <v>21.1</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.03769401330376947</v>
+        <v>-0.06430155210643013</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22705,10 +22705,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.068</v>
+        <v>0.067</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05555555555555541</v>
+        <v>-0.06944444444444432</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -22735,10 +22735,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.75</v>
+        <v>3.82</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1538461538461539</v>
+        <v>0.1753846153846153</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22765,10 +22765,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.28</v>
+        <v>5.13</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.09356223175965664</v>
+        <v>-0.1193133047210301</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22795,10 +22795,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.608</v>
+        <v>3.54</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01096491228070176</v>
+        <v>-0.02960526315789476</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22825,10 +22825,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.25</v>
+        <v>7.2</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02684563758389264</v>
+        <v>-0.03355704697986577</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22855,10 +22855,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.92</v>
+        <v>23.38</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.03626107977437545</v>
+        <v>-0.05801772763900086</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22885,10 +22885,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>78.95999999999999</v>
+        <v>77.23999999999999</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.1168316831683167</v>
+        <v>0.09250353606789238</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22915,10 +22915,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.38</v>
+        <v>7.405</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.07750000000000001</v>
+        <v>-0.07437499999999997</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22945,10 +22945,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.08</v>
+        <v>8.1</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.007371007371007432</v>
+        <v>-0.004914004914005028</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22975,10 +22975,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.3</v>
+        <v>23.4</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0248161764705882</v>
+        <v>0.07536764705882339</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23080,10 +23080,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.887</v>
+        <v>5.599</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1408914728682169</v>
+        <v>0.08507751937984497</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23109,10 +23109,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.064</v>
+        <v>0.061</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2195121951219512</v>
+        <v>-0.2560975609756098</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23138,10 +23138,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.17</v>
+        <v>5.32</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1177474402730376</v>
+        <v>-0.09215017064846416</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23167,10 +23167,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.964</v>
+        <v>0.952</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.08625592417061609</v>
+        <v>-0.09763033175355448</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23196,10 +23196,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.32</v>
+        <v>9.42</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08372093023255822</v>
+        <v>0.09534883720930236</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23225,10 +23225,10 @@
         <v>20.3</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2413793103448275</v>
+        <v>0.2364532019704434</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23254,10 +23254,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.262</v>
+        <v>0.257</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06428571428571433</v>
+        <v>-0.08214285714285721</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23283,10 +23283,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.215</v>
+        <v>1.24</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.05078124999999996</v>
+        <v>-0.03125000000000003</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23312,10 +23312,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.14</v>
+        <v>0.139</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.13125</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23341,10 +23341,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.45</v>
+        <v>19.2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.02015113350125955</v>
+        <v>-0.0327455919395467</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23438,10 +23438,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.81</v>
+        <v>6.695</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.08872901678657071</v>
+        <v>0.07034372501998408</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23467,10 +23467,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.378</v>
+        <v>5.392</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.03026819923371655</v>
+        <v>0.03295019157088134</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23525,10 +23525,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.7</v>
+        <v>21.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.03769401330376947</v>
+        <v>-0.06430155210643013</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23554,10 +23554,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.5</v>
+        <v>21.45</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.004629629629629695</v>
+        <v>-0.006944444444444543</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23583,10 +23583,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.97</v>
+        <v>3.934</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.008986520219670502</v>
+        <v>-0.017973040439341</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23612,10 +23612,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>94.05</v>
+        <v>95.05</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04037610619469017</v>
+        <v>0.05143805309734503</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23641,10 +23641,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.758</v>
+        <v>1.781</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.06139882541377469</v>
+        <v>-0.0491190603310198</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23699,10 +23699,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>220.5</v>
+        <v>220</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.006756756756756757</v>
+        <v>-0.009009009009009009</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-23 16:45
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19347,7 +19347,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 16:37</t>
+          <t>23/09/2026 16:45</t>
         </is>
       </c>
     </row>
@@ -19374,10 +19374,10 @@
         <v>154.85</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>151.25</v>
+        <v>149.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02324830481110749</v>
+        <v>-0.03261220536002572</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19404,10 +19404,10 @@
         <v>18.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.04</v>
+        <v>18.01</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.0005540166204987015</v>
+        <v>-0.002216066481994412</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19434,10 +19434,10 @@
         <v>44.65</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>45.75</v>
+        <v>45.405</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02463605823068312</v>
+        <v>0.016909294512878</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19464,10 +19464,10 @@
         <v>12.85</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>13.2</v>
+        <v>13.05</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02723735408560309</v>
+        <v>0.01556420233463043</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19524,10 +19524,10 @@
         <v>6.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>6.695</v>
+        <v>6.66</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02213740458015274</v>
+        <v>0.01679389312977104</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19554,10 +19554,10 @@
         <v>60.85</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>63.8</v>
+        <v>63.75</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.04847986852917002</v>
+        <v>0.04765817584223498</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19584,10 +19584,10 @@
         <v>94.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>95.05</v>
+        <v>95.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.009023354564755778</v>
+        <v>0.01167728237791926</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19644,10 +19644,10 @@
         <v>72.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>74.75</v>
+        <v>74.55</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.03388658367911484</v>
+        <v>0.03112033195020747</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19746,10 +19746,10 @@
         <v>5.075</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.13</v>
+        <v>5.155</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.01083743842364526</v>
+        <v>0.01576354679802957</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19776,10 +19776,10 @@
         <v>21.74</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07635694572217112</v>
+        <v>0.08555657773689067</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19806,10 +19806,10 @@
         <v>20.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>20.55</v>
+        <v>20.5</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.0223880597014925</v>
+        <v>0.01990049751243774</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19836,10 +19836,10 @@
         <v>23.5</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>23.38</v>
+        <v>23.24</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.005106382978723446</v>
+        <v>-0.01106382978723411</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19866,10 +19866,10 @@
         <v>12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>11.96</v>
+        <v>11.888</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.003333333333333262</v>
+        <v>-0.009333333333333341</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19896,10 +19896,10 @@
         <v>20.98</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.5</v>
+        <v>22.48</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.07244995233555765</v>
+        <v>0.07149666348903717</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19926,10 +19926,10 @@
         <v>14.46</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>13.98</v>
+        <v>13.62</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.03319502074688799</v>
+        <v>-0.05809128630705405</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19986,10 +19986,10 @@
         <v>21.1</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>20.9</v>
+        <v>20.85</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.009478672985782125</v>
+        <v>-0.01184834123222749</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20016,10 +20016,10 @@
         <v>102.14</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>96.39</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.05629528098688075</v>
+        <v>-0.05913452124534958</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20121,10 +20121,10 @@
         <v>6.004</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.599</v>
+        <v>5.545</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06745502998001322</v>
+        <v>-0.07644903397734838</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20150,10 +20150,10 @@
         <v>5.4</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>5.32</v>
+        <v>5.22</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.01481481481481483</v>
+        <v>-0.03333333333333344</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20179,10 +20179,10 @@
         <v>9.01</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.42</v>
+        <v>9.34</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.04550499445061045</v>
+        <v>0.03662597114317426</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20208,10 +20208,10 @@
         <v>0.166</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.15</v>
+        <v>0.144</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.09638554216867477</v>
+        <v>-0.1325301204819278</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20237,10 +20237,10 @@
         <v>28.56</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>29.94</v>
+        <v>30</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.04831932773109253</v>
+        <v>0.05042016806722694</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20353,10 +20353,10 @@
         <v>41</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>48.75</v>
+        <v>48.7</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.1890243902439024</v>
+        <v>0.1878048780487805</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20479,10 +20479,10 @@
         <v>35.7</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>34.8</v>
+        <v>34.78</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.0252100840336136</v>
+        <v>-0.02577030812324935</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20508,10 +20508,10 @@
         <v>167.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165.6</v>
+        <v>165.2</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01075268817204308</v>
+        <v>-0.01314217443249711</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20566,10 +20566,10 @@
         <v>94.2</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.05</v>
+        <v>95.3</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.009023354564755778</v>
+        <v>0.01167728237791926</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20595,10 +20595,10 @@
         <v>16.72</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>16.64</v>
+        <v>16.6</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.004784688995215209</v>
+        <v>-0.007177033492822814</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20653,10 +20653,10 @@
         <v>60.85</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>63.8</v>
+        <v>63.75</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04847986852917002</v>
+        <v>0.04765817584223498</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20740,10 +20740,10 @@
         <v>4.878</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>4.69</v>
+        <v>4.704</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03854038540385398</v>
+        <v>-0.03567035670356711</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20838,10 +20838,10 @@
         <v>44.65</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>45.75</v>
+        <v>45.405</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>0.02463605823068312</v>
+        <v>0.016909294512878</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -20868,10 +20868,10 @@
         <v>78.56</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>79.45999999999999</v>
+        <v>79.61</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>0.01145621181262718</v>
+        <v>0.01336558044806514</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -20898,10 +20898,10 @@
         <v>78.06</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>77.23999999999999</v>
+        <v>76.52</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.0105047399436332</v>
+        <v>-0.01972841404048176</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>6.55</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>6.695</v>
+        <v>6.66</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.02213740458015274</v>
+        <v>0.01679389312977104</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>3.78</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>3.82</v>
+        <v>3.785</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.01058201058201059</v>
+        <v>0.001322751322751412</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>38.06</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>41.64</v>
+        <v>41.68</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>0.09406200735680499</v>
+        <v>0.09511297950604301</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -21018,10 +21018,10 @@
         <v>46.5</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>46.31</v>
+        <v>46.42</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.004086021505376295</v>
+        <v>-0.001720430107526845</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -21048,10 +21048,10 @@
         <v>140.8</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>141.6</v>
+        <v>141.3</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.005681818181818061</v>
+        <v>0.003551136363636364</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -21078,10 +21078,10 @@
         <v>138.85</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>139.25</v>
+        <v>138.75</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>0.00288080662585528</v>
+        <v>-0.0007202016564637689</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -21191,10 +21191,10 @@
         <v>38.06</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>41.64</v>
+        <v>41.68</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.09406200735680499</v>
+        <v>0.09511297950604301</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21221,10 +21221,10 @@
         <v>44.65</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>45.75</v>
+        <v>45.405</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.02463605823068312</v>
+        <v>0.016909294512878</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21251,10 +21251,10 @@
         <v>12.85</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>13.2</v>
+        <v>13.05</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.02723735408560309</v>
+        <v>0.01556420233463043</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21281,10 +21281,10 @@
         <v>78.06</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>77.23999999999999</v>
+        <v>76.52</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.0105047399436332</v>
+        <v>-0.01972841404048176</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21311,10 +21311,10 @@
         <v>78.56</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>79.45999999999999</v>
+        <v>79.61</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.01145621181262718</v>
+        <v>0.01336558044806514</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21341,10 +21341,10 @@
         <v>94.2</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>95.05</v>
+        <v>95.3</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.009023354564755778</v>
+        <v>0.01167728237791926</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21371,10 +21371,10 @@
         <v>6.55</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>6.695</v>
+        <v>6.66</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.02213740458015274</v>
+        <v>0.01679389312977104</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21401,10 +21401,10 @@
         <v>3.78</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>3.82</v>
+        <v>3.785</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.01058201058201059</v>
+        <v>0.001322751322751412</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21461,10 +21461,10 @@
         <v>46.5</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>46.31</v>
+        <v>46.42</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.004086021505376295</v>
+        <v>-0.001720430107526845</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 16:37</t>
+          <t>23/09/2026 16:45</t>
         </is>
       </c>
     </row>
@@ -22363,10 +22363,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.04</v>
+        <v>18.01</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.209926224010731</v>
+        <v>0.2079141515761235</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22393,10 +22393,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.45999999999999</v>
+        <v>79.61</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.008759680081249178</v>
+        <v>0.01066395835978169</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22453,10 +22453,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>124.8</v>
+        <v>124.7</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.003215434083601218</v>
+        <v>0.002411575562700942</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22513,10 +22513,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.8</v>
+        <v>34.78</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03225806451612914</v>
+        <v>-0.03281423804226918</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22543,10 +22543,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>223</v>
+        <v>224.2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03145235892691958</v>
+        <v>0.03700277520814061</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22603,10 +22603,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.1</v>
+        <v>21.05</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.06430155210643013</v>
+        <v>-0.06651884700665188</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22705,10 +22705,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.067</v>
+        <v>0.066</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.06944444444444432</v>
+        <v>-0.08333333333333322</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -22735,10 +22735,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.82</v>
+        <v>3.785</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1753846153846153</v>
+        <v>0.1646153846153847</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22765,10 +22765,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.13</v>
+        <v>5.155</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1193133047210301</v>
+        <v>-0.1150214592274678</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22795,10 +22795,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.54</v>
+        <v>3.566</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02960526315789476</v>
+        <v>-0.02247807017543868</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22855,10 +22855,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.38</v>
+        <v>23.24</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.05801772763900086</v>
+        <v>-0.06365834004834818</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22885,10 +22885,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>77.23999999999999</v>
+        <v>76.52</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.09250353606789238</v>
+        <v>0.08231966053748221</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22915,10 +22915,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.405</v>
+        <v>7.38</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.07437499999999997</v>
+        <v>-0.07750000000000001</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22945,10 +22945,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.1</v>
+        <v>8.08</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.004914004914005028</v>
+        <v>-0.007371007371007432</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22975,10 +22975,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.07536764705882339</v>
+        <v>0.08455882352941176</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23080,10 +23080,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.599</v>
+        <v>5.545</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.08507751937984497</v>
+        <v>0.07461240310077515</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23109,10 +23109,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.061</v>
+        <v>0.06</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2560975609756098</v>
+        <v>-0.2682926829268293</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23138,10 +23138,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.32</v>
+        <v>5.22</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.09215017064846416</v>
+        <v>-0.1092150170648465</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23167,10 +23167,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.952</v>
+        <v>0.982</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.09763033175355448</v>
+        <v>-0.0691943127962085</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23196,10 +23196,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.42</v>
+        <v>9.34</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.09534883720930236</v>
+        <v>0.08604651162790701</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23438,10 +23438,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.695</v>
+        <v>6.66</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.07034372501998408</v>
+        <v>0.06474820143884896</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23467,10 +23467,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.392</v>
+        <v>5.37</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.03295019157088134</v>
+        <v>0.02873563218390811</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23525,10 +23525,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.1</v>
+        <v>21.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.06430155210643013</v>
+        <v>-0.06651884700665188</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23554,10 +23554,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.45</v>
+        <v>21.5</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.006944444444444543</v>
+        <v>-0.004629629629629695</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23583,10 +23583,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.934</v>
+        <v>3.94</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.017973040439341</v>
+        <v>-0.01647528706939598</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23612,10 +23612,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>95.05</v>
+        <v>95.3</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05143805309734503</v>
+        <v>0.05420353982300875</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23641,10 +23641,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.781</v>
+        <v>1.773</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0491190603310198</v>
+        <v>-0.05339028296849978</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-23 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19347,7 +19347,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 16:45</t>
+          <t>23/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -19374,10 +19374,10 @@
         <v>154.85</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>149.8</v>
+        <v>149.45</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.03261220536002572</v>
+        <v>-0.03487245721666132</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19404,10 +19404,10 @@
         <v>18.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.01</v>
+        <v>17.9</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.002216066481994412</v>
+        <v>-0.008310249307479343</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19434,10 +19434,10 @@
         <v>44.65</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>45.405</v>
+        <v>46.17</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.016909294512878</v>
+        <v>0.03404255319148943</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19464,10 +19464,10 @@
         <v>12.85</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>13.05</v>
+        <v>13.2</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01556420233463043</v>
+        <v>0.02723735408560309</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19524,10 +19524,10 @@
         <v>6.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>6.66</v>
+        <v>6.735</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.01679389312977104</v>
+        <v>0.02824427480916038</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19554,10 +19554,10 @@
         <v>60.85</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>63.75</v>
+        <v>63.55</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.04765817584223498</v>
+        <v>0.04437140509449459</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19584,10 +19584,10 @@
         <v>94.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>95.3</v>
+        <v>95.95</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01167728237791926</v>
+        <v>0.01857749469214437</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19644,10 +19644,10 @@
         <v>72.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>74.55</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.03112033195020747</v>
+        <v>0.03181189488243426</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19746,10 +19746,10 @@
         <v>5.075</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.155</v>
+        <v>5.21</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.01576354679802957</v>
+        <v>0.02660098522167484</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19776,10 +19776,10 @@
         <v>21.74</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>23.6</v>
+        <v>23.38</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.08555657773689067</v>
+        <v>0.07543698252069921</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19806,10 +19806,10 @@
         <v>20.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>20.5</v>
+        <v>20.7</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01990049751243774</v>
+        <v>0.02985074626865661</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19836,10 +19836,10 @@
         <v>23.5</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>23.24</v>
+        <v>23.48</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01106382978723411</v>
+        <v>-0.0008510638297872159</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19866,10 +19866,10 @@
         <v>12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>11.888</v>
+        <v>11.988</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.009333333333333341</v>
+        <v>-0.001000000000000038</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19896,10 +19896,10 @@
         <v>20.98</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.48</v>
+        <v>22.44</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.07149666348903717</v>
+        <v>0.06959008579599622</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19926,10 +19926,10 @@
         <v>14.46</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>13.62</v>
+        <v>13.7</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.05809128630705405</v>
+        <v>-0.05255878284923939</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19956,10 +19956,10 @@
         <v>0.083</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01204819277108435</v>
+        <v>-0.02409638554216869</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19986,10 +19986,10 @@
         <v>21.1</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>20.85</v>
+        <v>20.9</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01184834123222749</v>
+        <v>-0.009478672985782125</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20016,10 +20016,10 @@
         <v>102.14</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>96.09999999999999</v>
+        <v>96.05</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.05913452124534958</v>
+        <v>-0.05962404542784417</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20121,10 +20121,10 @@
         <v>6.004</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.545</v>
+        <v>5.6</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.07644903397734838</v>
+        <v>-0.06728847435043303</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20150,10 +20150,10 @@
         <v>5.4</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>5.22</v>
+        <v>5.28</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03333333333333344</v>
+        <v>-0.02222222222222224</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20179,10 +20179,10 @@
         <v>9.01</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.34</v>
+        <v>9.5</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.03662597114317426</v>
+        <v>0.05438401775804664</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20208,10 +20208,10 @@
         <v>0.166</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.144</v>
+        <v>0.143</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.1325301204819278</v>
+        <v>-0.13855421686747</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20237,10 +20237,10 @@
         <v>28.56</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>30</v>
+        <v>30.86</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.05042016806722694</v>
+        <v>0.08053221288515409</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20266,10 +20266,10 @@
         <v>8.380000000000001</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.380000000000001</v>
+        <v>8.34</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>-0.00477326968973758</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20324,10 +20324,10 @@
         <v>33</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>32.9</v>
+        <v>33</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.003030303030303073</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20353,10 +20353,10 @@
         <v>41</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>48.7</v>
+        <v>48.55</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.1878048780487805</v>
+        <v>0.1841463414634146</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20479,10 +20479,10 @@
         <v>35.7</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>34.78</v>
+        <v>35.02</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.02577030812324935</v>
+        <v>-0.01904761904761904</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20508,10 +20508,10 @@
         <v>167.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165.2</v>
+        <v>165</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01314217443249711</v>
+        <v>-0.01433691756272405</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20537,10 +20537,10 @@
         <v>4.26</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>4.14</v>
+        <v>4.19</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.02816901408450707</v>
+        <v>-0.01643192488262897</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20566,10 +20566,10 @@
         <v>94.2</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.3</v>
+        <v>95.95</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01167728237791926</v>
+        <v>0.01857749469214437</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20624,10 +20624,10 @@
         <v>72.2</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>71.90000000000001</v>
+        <v>72</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.004155124653739573</v>
+        <v>-0.002770083102493114</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20653,10 +20653,10 @@
         <v>60.85</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>63.75</v>
+        <v>63.55</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04765817584223498</v>
+        <v>0.04437140509449459</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20740,10 +20740,10 @@
         <v>4.878</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>4.704</v>
+        <v>4.71</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03567035670356711</v>
+        <v>-0.03444034440344407</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20838,10 +20838,10 @@
         <v>44.65</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>45.405</v>
+        <v>46.17</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>0.016909294512878</v>
+        <v>0.03404255319148943</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -20868,10 +20868,10 @@
         <v>78.56</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>79.61</v>
+        <v>79.69</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>0.01336558044806514</v>
+        <v>0.01438391038696532</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -20898,10 +20898,10 @@
         <v>78.06</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>76.52</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.01972841404048176</v>
+        <v>-0.02331539841147844</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -20928,10 +20928,10 @@
         <v>6.55</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>6.66</v>
+        <v>6.735</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.01679389312977104</v>
+        <v>0.02824427480916038</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -20958,10 +20958,10 @@
         <v>3.78</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>3.785</v>
+        <v>3.81</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.001322751322751412</v>
+        <v>0.007936507936508002</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -20988,10 +20988,10 @@
         <v>38.06</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>41.68</v>
+        <v>41.76</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>0.09511297950604301</v>
+        <v>0.09721492380451906</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -21018,10 +21018,10 @@
         <v>46.5</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>46.42</v>
+        <v>46.27</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.001720430107526845</v>
+        <v>-0.004946236559139718</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -21048,10 +21048,10 @@
         <v>140.8</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>141.3</v>
+        <v>140.9</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.003551136363636364</v>
+        <v>0.0007102272727272323</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -21078,10 +21078,10 @@
         <v>138.85</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>138.75</v>
+        <v>138.55</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.0007202016564637689</v>
+        <v>-0.002160604969391307</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -21191,10 +21191,10 @@
         <v>38.06</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>41.68</v>
+        <v>41.76</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.09511297950604301</v>
+        <v>0.09721492380451906</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21221,10 +21221,10 @@
         <v>44.65</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>45.405</v>
+        <v>46.17</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.016909294512878</v>
+        <v>0.03404255319148943</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21251,10 +21251,10 @@
         <v>12.85</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>13.05</v>
+        <v>13.2</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.01556420233463043</v>
+        <v>0.02723735408560309</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21281,10 +21281,10 @@
         <v>78.06</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>76.52</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.01972841404048176</v>
+        <v>-0.02331539841147844</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21311,10 +21311,10 @@
         <v>78.56</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>79.61</v>
+        <v>79.69</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.01336558044806514</v>
+        <v>0.01438391038696532</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21341,10 +21341,10 @@
         <v>94.2</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>95.3</v>
+        <v>95.95</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.01167728237791926</v>
+        <v>0.01857749469214437</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21371,10 +21371,10 @@
         <v>6.55</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>6.66</v>
+        <v>6.735</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.01679389312977104</v>
+        <v>0.02824427480916038</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21401,10 +21401,10 @@
         <v>3.78</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>3.785</v>
+        <v>3.81</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.001322751322751412</v>
+        <v>0.007936507936508002</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21461,10 +21461,10 @@
         <v>46.5</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>46.42</v>
+        <v>46.27</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.001720430107526845</v>
+        <v>-0.004946236559139718</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22306,7 +22306,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 16:45</t>
+          <t>23/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22333,10 +22333,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.308</v>
+        <v>0.305</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1225071225071225</v>
+        <v>-0.131054131054131</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22363,10 +22363,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>18.01</v>
+        <v>17.9</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.2079141515761235</v>
+        <v>0.2005365526492286</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22393,10 +22393,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.61</v>
+        <v>79.69</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01066395835978169</v>
+        <v>0.01167957344166563</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22513,10 +22513,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.78</v>
+        <v>35.02</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03281423804226918</v>
+        <v>-0.02614015572858725</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22543,10 +22543,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>224.2</v>
+        <v>225</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03700277520814061</v>
+        <v>0.04070305272895473</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22573,10 +22573,10 @@
         <v>0.016</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.1875000000000001</v>
+        <v>-0.125</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22603,10 +22603,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.05</v>
+        <v>21.25</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.06651884700665188</v>
+        <v>-0.057649667405765</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22735,10 +22735,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.785</v>
+        <v>3.81</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1646153846153847</v>
+        <v>0.1723076923076923</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22765,10 +22765,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.155</v>
+        <v>5.21</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1150214592274678</v>
+        <v>-0.1055793991416309</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22795,10 +22795,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.566</v>
+        <v>3.542</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02247807017543868</v>
+        <v>-0.02905701754385974</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22825,10 +22825,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.2</v>
+        <v>7.18</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03355704697986577</v>
+        <v>-0.0362416107382551</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22855,10 +22855,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.24</v>
+        <v>23.48</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.06365834004834818</v>
+        <v>-0.0539887187751813</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22885,10 +22885,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>76.52</v>
+        <v>76.23999999999999</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.08231966053748221</v>
+        <v>0.07835926449787825</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22915,10 +22915,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.38</v>
+        <v>7.45</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.07750000000000001</v>
+        <v>-0.06874999999999998</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22945,10 +22945,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.08</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.007371007371007432</v>
+        <v>0</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22975,10 +22975,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.6</v>
+        <v>23.38</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.08455882352941176</v>
+        <v>0.07444852941176458</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23080,10 +23080,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.545</v>
+        <v>5.6</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.07461240310077515</v>
+        <v>0.08527131782945727</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23109,10 +23109,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.06</v>
+        <v>0.061</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2682926829268293</v>
+        <v>-0.2560975609756098</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23138,10 +23138,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.22</v>
+        <v>5.28</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1092150170648465</v>
+        <v>-0.09897610921501707</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23167,10 +23167,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.982</v>
+        <v>0.98</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0691943127962085</v>
+        <v>-0.07109004739336489</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23196,10 +23196,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.34</v>
+        <v>9.5</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08604651162790701</v>
+        <v>0.1046511627906977</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23254,10 +23254,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.257</v>
+        <v>0.264</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.08214285714285721</v>
+        <v>-0.05714285714285719</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23283,10 +23283,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.24</v>
+        <v>1.19</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03125000000000003</v>
+        <v>-0.07031250000000006</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23341,10 +23341,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.2</v>
+        <v>18.2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.0327455919395467</v>
+        <v>-0.08312342569269532</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23438,10 +23438,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.66</v>
+        <v>6.735</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.06474820143884896</v>
+        <v>0.0767386091127099</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23467,10 +23467,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.37</v>
+        <v>5.414</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.02873563218390811</v>
+        <v>0.0371647509578544</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23525,10 +23525,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.05</v>
+        <v>21.25</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.06651884700665188</v>
+        <v>-0.057649667405765</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23583,10 +23583,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.94</v>
+        <v>3.98</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01647528706939598</v>
+        <v>-0.006490264603095418</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23612,10 +23612,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>95.3</v>
+        <v>95.95</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05420353982300875</v>
+        <v>0.06139380530973448</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23641,10 +23641,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.773</v>
+        <v>1.779</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05339028296849978</v>
+        <v>-0.0501868659903898</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23699,10 +23699,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>220</v>
+        <v>221.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.009009009009009009</v>
+        <v>-0.002252252252252252</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-24 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -24,8 +24,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="000000"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="9">
@@ -336,7 +336,7 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -465,7 +465,6 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
@@ -1944,14 +1943,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -1978,6 +1969,29 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <color rgb="FF006100"/>
         <extend val="0"/>
@@ -1997,14 +2011,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -2031,13 +2037,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="1"/>
         <condense val="0"/>
         <color auto="1"/>
@@ -2100,14 +2099,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -2134,6 +2125,14 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -2160,16 +2159,16 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
         <extend val="0"/>
       </font>
     </dxf>
@@ -19307,7 +19306,7 @@
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="54" t="inlineStr">
         <is>
-          <t>21/09/2026</t>
+          <t>23/09/2026</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -19347,7 +19346,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 19:05</t>
+          <t>24/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -19357,7 +19356,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>SOI</t>
+          <t>MRN</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -19367,17 +19366,17 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOITEC </t>
+          <t>MERSEN</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>154.85</v>
+        <v>42.04</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>149.45</v>
+        <v>41.18</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.03487245721666132</v>
+        <v>-0.02045670789724071</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19387,27 +19386,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>OVH</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>OVH GROUPE</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>18.05</v>
+        <v>13.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>17.9</v>
+        <v>13.25</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.008310249307479343</v>
+        <v>0.01532567049808424</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19417,27 +19416,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>STMPA</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>STMICROELECTRONICS</t>
+          <t>LINEDATA</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>44.65</v>
+        <v>54</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>46.17</v>
+        <v>54.4</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.03404255319148943</v>
+        <v>0.007407407407407381</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19447,27 +19446,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>ATEME</t>
+          <t>EXENS</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>ATEME</t>
+          <t>EXOSENS</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>12.85</v>
+        <v>63.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>13.2</v>
+        <v>61</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02723735408560309</v>
+        <v>-0.03785488958990534</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19477,27 +19476,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>LINEDATA</t>
+          <t>JCDECAUX</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>53.4</v>
+        <v>25.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54</v>
+        <v>25.06</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.0112359550561798</v>
+        <v>-0.001593625498008076</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19507,7 +19506,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>ABCA</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -19517,17 +19516,17 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>X-FAB SILICON</t>
+          <t>ABC ARBITRAGE</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>6.55</v>
+        <v>5.81</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>6.735</v>
+        <v>5.83</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02824427480916038</v>
+        <v>0.003442340791738462</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19537,7 +19536,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>EXENS</t>
+          <t>BAIN</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -19547,17 +19546,17 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>EXOSENS</t>
+          <t>BAINS MER MONACO</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>60.85</v>
+        <v>141.5</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>63.55</v>
+        <v>141</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.04437140509449459</v>
+        <v>-0.00353356890459364</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19581,13 +19580,13 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>94.2</v>
+        <v>96.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>95.95</v>
+        <v>98.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01857749469214437</v>
+        <v>0.02390852390852388</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19597,7 +19596,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -19607,17 +19606,17 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>BIOMERIEUX</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>140</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>141.5</v>
+        <v>77.65000000000001</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01071428571428571</v>
+        <v>0.03671562082777036</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19627,27 +19626,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>BSD</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>BIOMERIEUX</t>
+          <t>BOURSE DIRECT</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>72.3</v>
+        <v>5.48</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>74.59999999999999</v>
+        <v>5.44</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.03181189488243426</v>
+        <v>-0.007299270072992707</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19729,7 +19728,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>NXI</t>
+          <t>NACON</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -19739,17 +19738,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>NEXITY</t>
+          <t>NACON</t>
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>5.075</v>
+        <v>0.064</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>5.21</v>
+        <v>0.058</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.02660098522167484</v>
+        <v>-0.09374999999999997</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19759,27 +19758,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>MEDCL</t>
+          <t>LAT</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>MEDINCELL</t>
+          <t>LATECOERE</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>21.74</v>
+        <v>0.013</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>23.38</v>
+        <v>0.013</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07543698252069921</v>
+        <v>0</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19789,7 +19788,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>FDE</t>
+          <t>ATO</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -19799,17 +19798,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>FRANCAISE ENER</t>
+          <t>ATOS</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>20.1</v>
+        <v>23.66</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>20.7</v>
+        <v>23.04</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.02985074626865661</v>
+        <v>-0.02620456466610317</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19819,7 +19818,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ATO</t>
+          <t>EXA</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -19829,17 +19828,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>EXAIL TECH</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>23.5</v>
+        <v>125</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>23.48</v>
+        <v>124.8</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.0008510638297872159</v>
+        <v>-0.001600000000000023</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19849,27 +19848,27 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>WLN</t>
+          <t>NXI</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>WORLDLINE</t>
+          <t>NEXITY</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>12</v>
+        <v>5.185</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>11.988</v>
+        <v>5.195</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.001000000000000038</v>
+        <v>0.00192864030858258</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19879,7 +19878,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ELIS</t>
+          <t>TFF</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -19889,17 +19888,17 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>ELIS</t>
+          <t>TFF GROUP</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>20.98</v>
+        <v>13.66</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.44</v>
+        <v>13.82</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.06959008579599622</v>
+        <v>0.01171303074670572</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19909,7 +19908,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>TFF</t>
+          <t>EQS</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -19919,17 +19918,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>TFF GROUP</t>
+          <t>EQUASENS</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>14.46</v>
+        <v>29.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>13.7</v>
+        <v>29.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.05255878284923939</v>
+        <v>0.01030927835051537</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19939,27 +19938,27 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>VANTI</t>
+          <t>WLN</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>VANTIVA</t>
+          <t>WORLDLINE</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.083</v>
+        <v>12</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.081</v>
+        <v>11.802</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.02409638554216869</v>
+        <v>-0.01650000000000003</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19969,27 +19968,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>KOF</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>KAUFMAN ET BROAD</t>
+          <t>CA PARIS IDF</t>
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>21.1</v>
+        <v>96.06</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>20.9</v>
+        <v>96.06</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.009478672985782125</v>
+        <v>0</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19999,27 +19998,27 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>ADOC</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>CA PARIS IDF</t>
+          <t>ADOCIA</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>102.14</v>
+        <v>3.534</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>96.05</v>
+        <v>3.51</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.05962404542784417</v>
+        <v>-0.006791171477079802</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20104,7 +20103,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>ALCPB</t>
+          <t>ALHAF</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -20114,17 +20113,17 @@
       </c>
       <c r="D30" s="51" t="inlineStr">
         <is>
-          <t>CAPITAL B</t>
+          <t>HAFFNER ENERGY</t>
         </is>
       </c>
       <c r="E30" s="18" t="n">
-        <v>6.004</v>
+        <v>0.717</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.6</v>
+        <v>0.77</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06728847435043303</v>
+        <v>0.07391910739191081</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20133,7 +20132,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>ALKAL</t>
+          <t>AL2SI</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -20143,17 +20142,17 @@
       </c>
       <c r="D31" s="51" t="inlineStr">
         <is>
-          <t>KALRAY</t>
+          <t>2CRSI</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>5.4</v>
+        <v>30.88</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>5.28</v>
+        <v>30</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02222222222222224</v>
+        <v>-0.02849740932642484</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20176,13 +20175,13 @@
         </is>
       </c>
       <c r="E32" s="18" t="n">
-        <v>9.01</v>
+        <v>9.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.5</v>
+        <v>9.33</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.05438401775804664</v>
+        <v>-0.01789473684210525</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20191,7 +20190,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>ALCBI</t>
+          <t>ALSEM</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -20201,17 +20200,17 @@
       </c>
       <c r="D33" s="51" t="inlineStr">
         <is>
-          <t>CBI</t>
+          <t>SEMCO TECHNOLOGIES</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>0.166</v>
+        <v>48.6</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.143</v>
+        <v>46.95</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.13855421686747</v>
+        <v>-0.03395061728395059</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20220,7 +20219,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>AL2SI</t>
+          <t>ALINV</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -20230,17 +20229,17 @@
       </c>
       <c r="D34" s="51" t="inlineStr">
         <is>
-          <t>2CRSI</t>
+          <t>INVIBES ADVERTISING</t>
         </is>
       </c>
       <c r="E34" s="18" t="n">
-        <v>28.56</v>
+        <v>1.55</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>30.86</v>
+        <v>1.58</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08053221288515409</v>
+        <v>0.01935483870967744</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20249,7 +20248,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ALLEX</t>
+          <t>ALNRG</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -20259,17 +20258,17 @@
       </c>
       <c r="D35" s="51" t="inlineStr">
         <is>
-          <t>LEXIBOOK LINGUIST.</t>
+          <t>ENERGISME</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>8.380000000000001</v>
+        <v>3.86</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>8.34</v>
+        <v>3.8</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.00477326968973758</v>
+        <v>-0.01554404145077722</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20278,27 +20277,27 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>ALGLD</t>
+          <t>ALCBX</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D36" s="51" t="inlineStr">
         <is>
-          <t>GOLD BY GOLD</t>
+          <t>CIBOX INTERACTIVE</t>
         </is>
       </c>
       <c r="E36" s="18" t="n">
-        <v>4.88</v>
+        <v>0.013</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.89</v>
+        <v>0.012</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.002049180327868809</v>
+        <v>-0.07692307692307686</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20307,27 +20306,27 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>ALDEL</t>
+          <t>MEMS</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D37" s="51" t="inlineStr">
         <is>
-          <t>DELFINGEN</t>
+          <t>MEMSCAP REPGT</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>33</v>
+        <v>5.16</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>33</v>
+        <v>5.06</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.01937984496124041</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20336,27 +20335,27 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>ALSEM</t>
+          <t>ARTE</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D38" s="51" t="inlineStr">
         <is>
-          <t>SEMCO TECHNOLOGIES</t>
+          <t>ARTEA</t>
         </is>
       </c>
       <c r="E38" s="18" t="n">
-        <v>41</v>
+        <v>6.45</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>48.55</v>
+        <v>6.45</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.1841463414634146</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -20365,7 +20364,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>ALEXP</t>
+          <t>ALESE</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -20375,17 +20374,17 @@
       </c>
       <c r="D39" s="51" t="inlineStr">
         <is>
-          <t>ONE EXPERIENCE</t>
+          <t>ENTECH</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>0.455</v>
+        <v>10.34</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.39</v>
+        <v>10.2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.1428571428571428</v>
+        <v>-0.01353965183752423</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20462,7 +20461,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>RUI</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -20472,17 +20471,17 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>RUBIS</t>
+          <t>AIR LIQUIDE</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>35.7</v>
+        <v>168.18</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>35.02</v>
+        <v>168.22</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.01904761904761904</v>
+        <v>0.0002378404090854563</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20491,27 +20490,27 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>ELEC</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>ELECTICITE DE STRASBOURG</t>
+          <t>BIOMERIEUX</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>167.4</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165</v>
+        <v>77.65000000000001</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01433691756272405</v>
+        <v>0.03671562082777036</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20520,27 +20519,27 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>GUI</t>
+          <t>ARAMI</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>GUILLEMOT</t>
+          <t>ARAMIS</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
-        <v>4.26</v>
+        <v>3.82</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>4.19</v>
+        <v>3.805</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01643192488262897</v>
+        <v>-0.003926701570680545</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20549,27 +20548,27 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>VIRI</t>
+          <t>AKE</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>VIRIDIEN</t>
+          <t>ARKEMA</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>94.2</v>
+        <v>57.5</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.95</v>
+        <v>57.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01857749469214437</v>
+        <v>-0.007826086956521788</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20578,7 +20577,7 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>TKO</t>
+          <t>ATE</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -20588,17 +20587,17 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>TIKEHAU CAPITAL</t>
+          <t>ALTEN</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>16.72</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>16.6</v>
+        <v>71.3</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.007177033492822814</v>
+        <v>-0.01790633608815423</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20607,7 +20606,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>THEP</t>
+          <t>PUB</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -20617,17 +20616,17 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>THERMADOR GROUPE</t>
+          <t>PUBLICIS GRP</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>72.2</v>
+        <v>97.54000000000001</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>72</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.002770083102493114</v>
+        <v>0.001435308591347145</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20636,7 +20635,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>EXENS</t>
+          <t>PLNW</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -20646,17 +20645,17 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>EXOSENS</t>
+          <t>PLANISWARE</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>60.85</v>
+        <v>24.4</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>63.55</v>
+        <v>23.95</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04437140509449459</v>
+        <v>-0.01844262295081964</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20665,7 +20664,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>ENX</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -20675,17 +20674,17 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>EURONEXT</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
-        <v>140</v>
+        <v>160.4</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>141.5</v>
+        <v>160.7</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.01071428571428571</v>
+        <v>0.001870324189526078</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20694,7 +20693,7 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>GAM</t>
+          <t>VIRI</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -20704,17 +20703,17 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>GAUMONT</t>
+          <t>VIRIDIEN</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>103</v>
+        <v>96.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>103</v>
+        <v>98.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0</v>
+        <v>0.02390852390852388</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20723,27 +20722,27 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>SESG</t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">SES </t>
+          <t>ATEME</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>4.878</v>
+        <v>13.05</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>4.71</v>
+        <v>13.25</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03444034440344407</v>
+        <v>0.01532567049808424</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20819,270 +20818,108 @@
       <c r="A56" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="inlineStr">
-        <is>
-          <t>STMPA</t>
-        </is>
-      </c>
-      <c r="C56" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D56" s="36" t="inlineStr">
-        <is>
-          <t>STMICROELECTRONICS</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="n">
-        <v>44.65</v>
-      </c>
-      <c r="F56" s="12" t="n">
-        <v>46.17</v>
-      </c>
-      <c r="G56" s="37" t="n">
-        <v>0.03404255319148943</v>
-      </c>
+      <c r="B56" s="36" t="n"/>
+      <c r="C56" s="30" t="n"/>
+      <c r="D56" s="36" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="37" t="n"/>
       <c r="H56" s="6" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" thickBot="1">
       <c r="A57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="inlineStr">
-        <is>
-          <t>TTE</t>
-        </is>
-      </c>
-      <c r="C57" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D57" s="36" t="inlineStr">
-        <is>
-          <t>TOTALENERGIES</t>
-        </is>
-      </c>
-      <c r="E57" s="18" t="n">
-        <v>78.56</v>
-      </c>
-      <c r="F57" s="12" t="n">
-        <v>79.69</v>
-      </c>
-      <c r="G57" s="37" t="n">
-        <v>0.01438391038696532</v>
-      </c>
+      <c r="B57" s="36" t="n"/>
+      <c r="C57" s="30" t="n"/>
+      <c r="D57" s="36" t="n"/>
+      <c r="E57" s="18" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="37" t="n"/>
       <c r="H57" s="6" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" thickBot="1">
       <c r="A58" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="36" t="inlineStr">
-        <is>
-          <t>ERF</t>
-        </is>
-      </c>
-      <c r="C58" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D58" s="36" t="inlineStr">
-        <is>
-          <t>EUROFINS SCIENTIFIC</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="n">
-        <v>78.06</v>
-      </c>
-      <c r="F58" s="12" t="n">
-        <v>76.23999999999999</v>
-      </c>
-      <c r="G58" s="37" t="n">
-        <v>-0.02331539841147844</v>
-      </c>
+      <c r="B58" s="36" t="n"/>
+      <c r="C58" s="30" t="n"/>
+      <c r="D58" s="36" t="n"/>
+      <c r="E58" s="18" t="n"/>
+      <c r="F58" s="12" t="n"/>
+      <c r="G58" s="37" t="n"/>
       <c r="H58" s="6" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" thickBot="1">
       <c r="A59" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B59" s="36" t="inlineStr">
-        <is>
-          <t>XFAB</t>
-        </is>
-      </c>
-      <c r="C59" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D59" s="36" t="inlineStr">
-        <is>
-          <t>X-FAB SILICON</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="F59" s="12" t="n">
-        <v>6.735</v>
-      </c>
-      <c r="G59" s="37" t="n">
-        <v>0.02824427480916038</v>
-      </c>
+      <c r="B59" s="36" t="n"/>
+      <c r="C59" s="30" t="n"/>
+      <c r="D59" s="36" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="12" t="n"/>
+      <c r="G59" s="37" t="n"/>
       <c r="H59" s="6" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" thickBot="1">
       <c r="A60" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B60" s="36" t="inlineStr">
-        <is>
-          <t>ARAMI</t>
-        </is>
-      </c>
-      <c r="C60" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D60" s="36" t="inlineStr">
-        <is>
-          <t>ARAMIS</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="F60" s="12" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="G60" s="37" t="n">
-        <v>0.007936507936508002</v>
-      </c>
+      <c r="B60" s="36" t="n"/>
+      <c r="C60" s="30" t="n"/>
+      <c r="D60" s="36" t="n"/>
+      <c r="E60" s="18" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="37" t="n"/>
       <c r="H60" s="6" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" thickBot="1">
       <c r="A61" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B61" s="36" t="inlineStr">
-        <is>
-          <t>MRN</t>
-        </is>
-      </c>
-      <c r="C61" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D61" s="36" t="inlineStr">
-        <is>
-          <t>MERSEN</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="n">
-        <v>38.06</v>
-      </c>
-      <c r="F61" s="12" t="n">
-        <v>41.76</v>
-      </c>
-      <c r="G61" s="37" t="n">
-        <v>0.09721492380451906</v>
-      </c>
+      <c r="B61" s="36" t="n"/>
+      <c r="C61" s="30" t="n"/>
+      <c r="D61" s="36" t="n"/>
+      <c r="E61" s="18" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="37" t="n"/>
       <c r="H61" s="6" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" thickBot="1">
       <c r="A62" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B62" s="36" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="C62" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D62" s="36" t="inlineStr">
-        <is>
-          <t>ACCOR</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="F62" s="12" t="n">
-        <v>46.27</v>
-      </c>
-      <c r="G62" s="37" t="n">
-        <v>-0.004946236559139718</v>
-      </c>
+      <c r="B62" s="36" t="n"/>
+      <c r="C62" s="30" t="n"/>
+      <c r="D62" s="36" t="n"/>
+      <c r="E62" s="18" t="n"/>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="37" t="n"/>
       <c r="H62" s="6" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" thickBot="1">
       <c r="A63" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B63" s="36" t="inlineStr">
-        <is>
-          <t>NEX</t>
-        </is>
-      </c>
-      <c r="C63" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D63" s="36" t="inlineStr">
-        <is>
-          <t>NEXANS</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="n">
-        <v>140.8</v>
-      </c>
-      <c r="F63" s="12" t="n">
-        <v>140.9</v>
-      </c>
-      <c r="G63" s="37" t="n">
-        <v>0.0007102272727272323</v>
-      </c>
+      <c r="B63" s="36" t="n"/>
+      <c r="C63" s="30" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="18" t="n"/>
+      <c r="F63" s="12" t="n"/>
+      <c r="G63" s="37" t="n"/>
       <c r="H63" s="6" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" thickBot="1">
       <c r="A64" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B64" s="36" t="inlineStr">
-        <is>
-          <t>LR</t>
-        </is>
-      </c>
-      <c r="C64" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D64" s="36" t="inlineStr">
-        <is>
-          <t>LEGRAND SA</t>
-        </is>
-      </c>
-      <c r="E64" s="18" t="n">
-        <v>138.85</v>
-      </c>
-      <c r="F64" s="12" t="n">
-        <v>138.55</v>
-      </c>
-      <c r="G64" s="37" t="n">
-        <v>-0.002160604969391307</v>
-      </c>
+      <c r="B64" s="36" t="n"/>
+      <c r="C64" s="30" t="n"/>
+      <c r="D64" s="36" t="n"/>
+      <c r="E64" s="18" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="37" t="n"/>
       <c r="H64" s="6" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" thickBot="1">
@@ -21094,9 +20931,7 @@
       <c r="D65" s="36" t="n"/>
       <c r="E65" s="18" t="n"/>
       <c r="F65" s="12" t="n"/>
-      <c r="G65" s="37" t="e">
-        <v>#VALUE!</v>
-      </c>
+      <c r="G65" s="37" t="n"/>
       <c r="H65" s="6" t="n"/>
     </row>
     <row r="66" ht="15.45" customHeight="1">
@@ -21109,9 +20944,7 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G66" s="34" t="e">
-        <v>#VALUE!</v>
-      </c>
+      <c r="G66" s="34" t="n"/>
       <c r="H66" s="48" t="inlineStr">
         <is>
           <t>nb &gt; 0</t>
@@ -21172,300 +21005,120 @@
       <c r="A69" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="36" t="inlineStr">
-        <is>
-          <t>MRN</t>
-        </is>
-      </c>
-      <c r="C69" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D69" s="36" t="inlineStr">
-        <is>
-          <t>MERSEN</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="n">
-        <v>38.06</v>
-      </c>
-      <c r="F69" s="12" t="n">
-        <v>41.76</v>
-      </c>
-      <c r="G69" s="37" t="n">
-        <v>0.09721492380451906</v>
-      </c>
+      <c r="B69" s="36" t="n"/>
+      <c r="C69" s="30" t="n"/>
+      <c r="D69" s="36" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="37" t="n"/>
       <c r="H69" s="6" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" thickBot="1">
       <c r="A70" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B70" s="36" t="inlineStr">
-        <is>
-          <t>STMPA</t>
-        </is>
-      </c>
-      <c r="C70" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D70" s="36" t="inlineStr">
-        <is>
-          <t>STMICROELECTRONICS</t>
-        </is>
-      </c>
-      <c r="E70" s="18" t="n">
-        <v>44.65</v>
-      </c>
-      <c r="F70" s="12" t="n">
-        <v>46.17</v>
-      </c>
-      <c r="G70" s="37" t="n">
-        <v>0.03404255319148943</v>
-      </c>
+      <c r="B70" s="36" t="n"/>
+      <c r="C70" s="30" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="18" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="37" t="n"/>
       <c r="H70" s="6" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" thickBot="1">
       <c r="A71" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B71" s="36" t="inlineStr">
-        <is>
-          <t>ATEME</t>
-        </is>
-      </c>
-      <c r="C71" s="30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D71" s="36" t="inlineStr">
-        <is>
-          <t>ATEME</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="n">
-        <v>12.85</v>
-      </c>
-      <c r="F71" s="12" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G71" s="37" t="n">
-        <v>0.02723735408560309</v>
-      </c>
+      <c r="B71" s="36" t="n"/>
+      <c r="C71" s="30" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="18" t="n"/>
+      <c r="F71" s="12" t="n"/>
+      <c r="G71" s="37" t="n"/>
       <c r="H71" s="6" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" thickBot="1">
       <c r="A72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="36" t="inlineStr">
-        <is>
-          <t>ERF</t>
-        </is>
-      </c>
-      <c r="C72" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D72" s="36" t="inlineStr">
-        <is>
-          <t>EUROFINS SCIENTIFIC</t>
-        </is>
-      </c>
-      <c r="E72" s="18" t="n">
-        <v>78.06</v>
-      </c>
-      <c r="F72" s="12" t="n">
-        <v>76.23999999999999</v>
-      </c>
-      <c r="G72" s="37" t="n">
-        <v>-0.02331539841147844</v>
-      </c>
+      <c r="B72" s="36" t="n"/>
+      <c r="C72" s="30" t="n"/>
+      <c r="D72" s="36" t="n"/>
+      <c r="E72" s="18" t="n"/>
+      <c r="F72" s="12" t="n"/>
+      <c r="G72" s="37" t="n"/>
       <c r="H72" s="6" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" thickBot="1">
       <c r="A73" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="36" t="inlineStr">
-        <is>
-          <t>TTE</t>
-        </is>
-      </c>
-      <c r="C73" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D73" s="36" t="inlineStr">
-        <is>
-          <t>TOTALENERGIES</t>
-        </is>
-      </c>
-      <c r="E73" s="18" t="n">
-        <v>78.56</v>
-      </c>
-      <c r="F73" s="12" t="n">
-        <v>79.69</v>
-      </c>
-      <c r="G73" s="37" t="n">
-        <v>0.01438391038696532</v>
-      </c>
+      <c r="B73" s="36" t="n"/>
+      <c r="C73" s="30" t="n"/>
+      <c r="D73" s="36" t="n"/>
+      <c r="E73" s="18" t="n"/>
+      <c r="F73" s="12" t="n"/>
+      <c r="G73" s="37" t="n"/>
       <c r="H73" s="6" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" thickBot="1">
       <c r="A74" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B74" s="36" t="inlineStr">
-        <is>
-          <t>VIRI</t>
-        </is>
-      </c>
-      <c r="C74" s="30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D74" s="36" t="inlineStr">
-        <is>
-          <t>VIRIDIEN</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="F74" s="12" t="n">
-        <v>95.95</v>
-      </c>
-      <c r="G74" s="37" t="n">
-        <v>0.01857749469214437</v>
-      </c>
+      <c r="B74" s="36" t="n"/>
+      <c r="C74" s="30" t="n"/>
+      <c r="D74" s="36" t="n"/>
+      <c r="E74" s="18" t="n"/>
+      <c r="F74" s="12" t="n"/>
+      <c r="G74" s="37" t="n"/>
       <c r="H74" s="6" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" thickBot="1">
       <c r="A75" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B75" s="36" t="inlineStr">
-        <is>
-          <t>XFAB</t>
-        </is>
-      </c>
-      <c r="C75" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D75" s="36" t="inlineStr">
-        <is>
-          <t>X-FAB SILICON</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="n">
-        <v>6.55</v>
-      </c>
-      <c r="F75" s="12" t="n">
-        <v>6.735</v>
-      </c>
-      <c r="G75" s="37" t="n">
-        <v>0.02824427480916038</v>
-      </c>
+      <c r="B75" s="36" t="n"/>
+      <c r="C75" s="30" t="n"/>
+      <c r="D75" s="36" t="n"/>
+      <c r="E75" s="18" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="37" t="n"/>
       <c r="H75" s="6" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" thickBot="1">
       <c r="A76" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="36" t="inlineStr">
-        <is>
-          <t>ARAMI</t>
-        </is>
-      </c>
-      <c r="C76" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D76" s="36" t="inlineStr">
-        <is>
-          <t>ARAMIS</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="n">
-        <v>3.78</v>
-      </c>
-      <c r="F76" s="12" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="G76" s="37" t="n">
-        <v>0.007936507936508002</v>
-      </c>
+      <c r="B76" s="36" t="n"/>
+      <c r="C76" s="30" t="n"/>
+      <c r="D76" s="36" t="n"/>
+      <c r="E76" s="18" t="n"/>
+      <c r="F76" s="12" t="n"/>
+      <c r="G76" s="37" t="n"/>
       <c r="H76" s="6" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" thickBot="1">
       <c r="A77" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B77" s="36" t="inlineStr">
-        <is>
-          <t>LIN</t>
-        </is>
-      </c>
-      <c r="C77" s="30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D77" s="36" t="inlineStr">
-        <is>
-          <t>LINEDATA</t>
-        </is>
-      </c>
-      <c r="E77" s="18" t="n">
-        <v>53.4</v>
-      </c>
-      <c r="F77" s="12" t="n">
-        <v>54</v>
-      </c>
-      <c r="G77" s="37" t="n">
-        <v>0.0112359550561798</v>
-      </c>
+      <c r="B77" s="36" t="n"/>
+      <c r="C77" s="30" t="n"/>
+      <c r="D77" s="36" t="n"/>
+      <c r="E77" s="18" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="37" t="n"/>
       <c r="H77" s="6" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" thickBot="1">
       <c r="A78" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B78" s="36" t="inlineStr">
-        <is>
-          <t>AC</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D78" s="36" t="inlineStr">
-        <is>
-          <t>ACCOR</t>
-        </is>
-      </c>
-      <c r="E78" s="18" t="n">
-        <v>46.5</v>
-      </c>
-      <c r="F78" s="12" t="n">
-        <v>46.27</v>
-      </c>
-      <c r="G78" s="37" t="n">
-        <v>-0.004946236559139718</v>
-      </c>
+      <c r="B78" s="36" t="n"/>
+      <c r="C78" s="30" t="n"/>
+      <c r="D78" s="36" t="n"/>
+      <c r="E78" s="18" t="n"/>
+      <c r="F78" s="12" t="n"/>
+      <c r="G78" s="37" t="n"/>
       <c r="H78" s="6" t="n"/>
     </row>
     <row r="79" ht="15.45" customHeight="1">
@@ -21475,9 +21128,7 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="G79" s="34" t="n">
-        <v>0</v>
-      </c>
+      <c r="G79" s="34" t="n"/>
       <c r="H79" s="6" t="n"/>
     </row>
     <row r="80" ht="15.45" customHeight="1">
@@ -21523,7 +21174,7 @@
         </is>
       </c>
       <c r="H81" s="49" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" thickBot="1">
@@ -22266,7 +21917,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="55" t="n">
+      <c r="A1" s="52" t="n">
         <v>46335</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -22306,7 +21957,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/09/2026 19:05</t>
+          <t>24/09/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22333,10 +21984,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.305</v>
+        <v>0.306</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.131054131054131</v>
+        <v>-0.1282051282051282</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22363,10 +22014,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>17.9</v>
+        <v>16.65</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.2005365526492286</v>
+        <v>0.1167002012072434</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22393,10 +22044,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.69</v>
+        <v>80.3</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01167957344166563</v>
+        <v>0.01942363844103086</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22423,10 +22074,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>141.5</v>
+        <v>141</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01071428571428571</v>
+        <v>0.007142857142857143</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22453,10 +22104,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>124.7</v>
+        <v>124.8</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.002411575562700942</v>
+        <v>0.003215434083601218</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22483,10 +22134,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54</v>
+        <v>54.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1368421052631579</v>
+        <v>0.1452631578947368</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22513,10 +22164,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.02</v>
+        <v>34.98</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02614015572858725</v>
+        <v>-0.02725250278086774</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22543,10 +22194,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.04070305272895473</v>
+        <v>0.03607770582793715</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22573,10 +22224,10 @@
         <v>0.016</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.125</v>
+        <v>-0.1875000000000001</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22603,10 +22254,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.25</v>
+        <v>21.05</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.057649667405765</v>
+        <v>-0.06651884700665188</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22622,7 +22273,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>0.01226293151009987</v>
+        <v>-0.001203634829822797</v>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
@@ -22705,10 +22356,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.066</v>
+        <v>0.058</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.08333333333333322</v>
+        <v>-0.1944444444444443</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -22735,10 +22386,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.81</v>
+        <v>3.805</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1723076923076923</v>
+        <v>0.1707692307692308</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22765,10 +22416,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.21</v>
+        <v>5.195</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1055793991416309</v>
+        <v>-0.1081545064377682</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22795,10 +22446,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.542</v>
+        <v>3.51</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02905701754385974</v>
+        <v>-0.03782894736842114</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22825,10 +22476,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.18</v>
+        <v>7.05</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.0362416107382551</v>
+        <v>-0.05369127516778528</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22855,10 +22506,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.48</v>
+        <v>23.04</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.0539887187751813</v>
+        <v>-0.07171635777598716</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22885,10 +22536,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>76.23999999999999</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.07835926449787825</v>
+        <v>0.0916548797736917</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22915,10 +22566,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.45</v>
+        <v>7.33</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.06874999999999998</v>
+        <v>-0.08374999999999999</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22945,10 +22596,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.140000000000001</v>
+        <v>8.125</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0</v>
+        <v>-0.001842751842751912</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22975,10 +22626,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.38</v>
+        <v>23.6</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.07444852941176458</v>
+        <v>0.08455882352941176</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22994,7 +22645,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.005169954798889787</v>
+        <v>-0.009142166055973799</v>
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
@@ -23080,10 +22731,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.6</v>
+        <v>5.454</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.08527131782945727</v>
+        <v>0.05697674418604643</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23109,10 +22760,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.061</v>
+        <v>0.062</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2560975609756098</v>
+        <v>-0.2439024390243903</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23138,10 +22789,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.28</v>
+        <v>5.15</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.09897610921501707</v>
+        <v>-0.121160409556314</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23167,10 +22818,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.98</v>
+        <v>0.972</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07109004739336489</v>
+        <v>-0.07867298578199049</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23196,10 +22847,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.5</v>
+        <v>9.33</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.1046511627906977</v>
+        <v>0.08488372093023261</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23254,10 +22905,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.264</v>
+        <v>0.26</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05714285714285719</v>
+        <v>-0.07142857142857148</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23283,10 +22934,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.19</v>
+        <v>1.22</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.07031250000000006</v>
+        <v>-0.04687500000000004</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23312,10 +22963,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.139</v>
+        <v>0.136</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.13125</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23341,10 +22992,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>18.2</v>
+        <v>18.6</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.08312342569269532</v>
+        <v>-0.06297229219143577</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23358,7 +23009,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.01267018127590628</v>
+        <v>-0.03443060221939261</v>
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
@@ -23438,10 +23089,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.735</v>
+        <v>6.58</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0767386091127099</v>
+        <v>0.05195843325339731</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23467,10 +23118,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.414</v>
+        <v>5.378</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.0371647509578544</v>
+        <v>0.03026819923371655</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23525,10 +23176,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.25</v>
+        <v>21.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.057649667405765</v>
+        <v>-0.06651884700665188</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23554,10 +23205,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.5</v>
+        <v>21.35</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.004629629629629695</v>
+        <v>-0.01157407407407407</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23583,10 +23234,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.98</v>
+        <v>3.938</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.006490264603095418</v>
+        <v>-0.01697453819271095</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23612,10 +23263,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>95.95</v>
+        <v>98.5</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.06139380530973448</v>
+        <v>0.08960176991150436</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23641,10 +23292,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.779</v>
+        <v>1.707</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0501868659903898</v>
+        <v>-0.08862786972770952</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23670,10 +23321,10 @@
         <v>35.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>34</v>
+        <v>34.2</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.03409090909090917</v>
+        <v>-0.02840909090909091</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -23699,10 +23350,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>221.5</v>
+        <v>221</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.002252252252252252</v>
+        <v>-0.004504504504504504</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -23716,7 +23367,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>-0.0008238530156982948</v>
+        <v>0.002134113848817021</v>
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-24 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19346,7 +19346,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>24/09/2026 13:00</t>
+          <t>24/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -19373,10 +19373,10 @@
         <v>42.04</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>41.18</v>
+        <v>41.24</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02045670789724071</v>
+        <v>-0.0190294957183634</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19403,10 +19403,10 @@
         <v>13.05</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>13.25</v>
+        <v>13</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01532567049808424</v>
+        <v>-0.003831417624521127</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19463,10 +19463,10 @@
         <v>63.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.03785488958990534</v>
+        <v>-0.02208201892744477</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19493,10 +19493,10 @@
         <v>25.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>25.06</v>
+        <v>24.74</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.001593625498008076</v>
+        <v>-0.01434262948207183</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19523,10 +19523,10 @@
         <v>5.81</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>5.83</v>
+        <v>5.86</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.003442340791738462</v>
+        <v>0.008605851979346078</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19553,10 +19553,10 @@
         <v>141.5</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>141</v>
+        <v>141.5</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.00353356890459364</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19583,10 +19583,10 @@
         <v>96.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>98.5</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02390852390852388</v>
+        <v>0.02234927234927226</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -19613,10 +19613,10 @@
         <v>74.90000000000001</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>77.65000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.03671562082777036</v>
+        <v>0.03471295060080099</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19643,10 +19643,10 @@
         <v>5.48</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>5.44</v>
+        <v>5.32</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.007299270072992707</v>
+        <v>-0.02919708029197083</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -19745,10 +19745,10 @@
         <v>0.064</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.058</v>
+        <v>0.06</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.09374999999999997</v>
+        <v>-0.06250000000000006</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19805,10 +19805,10 @@
         <v>23.66</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>23.04</v>
+        <v>22.7</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02620456466610317</v>
+        <v>-0.04057480980557907</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19865,10 +19865,10 @@
         <v>5.185</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.195</v>
+        <v>5.135</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.00192864030858258</v>
+        <v>-0.009643201542912214</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19895,10 +19895,10 @@
         <v>13.66</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.82</v>
+        <v>14</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01171303074670572</v>
+        <v>0.02489019033674962</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19925,10 +19925,10 @@
         <v>29.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>29.4</v>
+        <v>29.15</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.01030927835051537</v>
+        <v>0.001718213058419146</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19955,10 +19955,10 @@
         <v>12</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>11.802</v>
+        <v>11.934</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01650000000000003</v>
+        <v>-0.00550000000000006</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19985,10 +19985,10 @@
         <v>96.06</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>96.06</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0</v>
+        <v>-0.003123048094940632</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20015,10 +20015,10 @@
         <v>3.534</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>3.51</v>
+        <v>3.492</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.006791171477079802</v>
+        <v>-0.01188455008488959</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20120,10 +20120,10 @@
         <v>0.717</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.77</v>
+        <v>0.791</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.07391910739191081</v>
+        <v>0.1032078103207811</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20149,10 +20149,10 @@
         <v>30.88</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>30</v>
+        <v>29.8</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02849740932642484</v>
+        <v>-0.03497409326424865</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20178,10 +20178,10 @@
         <v>9.5</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.33</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.01789473684210525</v>
+        <v>-0.01157894736842099</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20207,10 +20207,10 @@
         <v>48.6</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>46.95</v>
+        <v>46.9</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.03395061728395059</v>
+        <v>-0.03497942386831281</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20236,10 +20236,10 @@
         <v>1.55</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>1.58</v>
+        <v>1.5</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.01935483870967744</v>
+        <v>-0.03225806451612906</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20323,10 +20323,10 @@
         <v>5.16</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>5.06</v>
+        <v>5.1</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01937984496124041</v>
+        <v>-0.01162790697674428</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20381,10 +20381,10 @@
         <v>10.34</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>10.2</v>
+        <v>10.14</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.01353965183752423</v>
+        <v>-0.01934235976789161</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20478,10 +20478,10 @@
         <v>168.18</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>168.22</v>
+        <v>168.2</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0002378404090854563</v>
+        <v>0.0001189202045426437</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20507,10 +20507,10 @@
         <v>74.90000000000001</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>77.65000000000001</v>
+        <v>77.5</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.03671562082777036</v>
+        <v>0.03471295060080099</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -20536,10 +20536,10 @@
         <v>3.82</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>3.805</v>
+        <v>3.625</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.003926701570680545</v>
+        <v>-0.05104712041884813</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20565,10 +20565,10 @@
         <v>57.5</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>57.05</v>
+        <v>56.9</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.007826086956521788</v>
+        <v>-0.01043478260869568</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20594,10 +20594,10 @@
         <v>72.59999999999999</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>71.3</v>
+        <v>70.7</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01790633608815423</v>
+        <v>-0.02617079889807151</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -20623,10 +20623,10 @@
         <v>97.54000000000001</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>97.68000000000001</v>
+        <v>97.94</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.001435308591347145</v>
+        <v>0.004100881689563169</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20652,10 +20652,10 @@
         <v>24.4</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>23.95</v>
+        <v>23.8</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01844262295081964</v>
+        <v>-0.02459016393442614</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20681,10 +20681,10 @@
         <v>160.4</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>160.7</v>
+        <v>160.1</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.001870324189526078</v>
+        <v>-0.001870324189526255</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20710,10 +20710,10 @@
         <v>96.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>98.5</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.02390852390852388</v>
+        <v>0.02234927234927226</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20739,10 +20739,10 @@
         <v>13.05</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>13.25</v>
+        <v>13</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01532567049808424</v>
+        <v>-0.003831417624521127</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21957,7 +21957,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>24/09/2026 13:00</t>
+          <t>24/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22014,10 +22014,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.65</v>
+        <v>17.01</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1167002012072434</v>
+        <v>0.1408450704225353</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22044,10 +22044,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>80.3</v>
+        <v>81.18000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01942363844103086</v>
+        <v>0.03059540434175461</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22074,10 +22074,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>141</v>
+        <v>141.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.007142857142857143</v>
+        <v>0.01071428571428571</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22164,10 +22164,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.98</v>
+        <v>34.82</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02725250278086774</v>
+        <v>-0.03170189098998889</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22194,10 +22194,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>224</v>
+        <v>223.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03607770582793715</v>
+        <v>0.03422756706753009</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22254,10 +22254,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>21.05</v>
+        <v>20.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.06651884700665188</v>
+        <v>-0.07760532150776053</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22356,10 +22356,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.058</v>
+        <v>0.06</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1944444444444443</v>
+        <v>-0.1666666666666666</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -22386,10 +22386,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.805</v>
+        <v>3.625</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1707692307692308</v>
+        <v>0.1153846153846154</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22416,10 +22416,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.195</v>
+        <v>5.135</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1081545064377682</v>
+        <v>-0.1184549356223177</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22446,10 +22446,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>3.51</v>
+        <v>3.492</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.03782894736842114</v>
+        <v>-0.04276315789473688</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22476,10 +22476,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.05</v>
+        <v>7.01</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.05369127516778528</v>
+        <v>-0.05906040268456381</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22506,10 +22506,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>23.04</v>
+        <v>22.7</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.07171635777598716</v>
+        <v>-0.08541498791297344</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22536,10 +22536,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>77.18000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.0916548797736917</v>
+        <v>0.1018387553041019</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22566,10 +22566,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.33</v>
+        <v>7.35</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.08374999999999999</v>
+        <v>-0.08125000000000004</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22596,10 +22596,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.125</v>
+        <v>7.85</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.001842751842751912</v>
+        <v>-0.03562653562653574</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22626,10 +22626,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.6</v>
+        <v>23.56</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.08455882352941176</v>
+        <v>0.08272058823529398</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22731,10 +22731,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.454</v>
+        <v>5.569</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.05697674418604643</v>
+        <v>0.07926356589147283</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22760,10 +22760,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2439024390243903</v>
+        <v>-0.2317073170731708</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22789,10 +22789,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.15</v>
+        <v>5.46</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.121160409556314</v>
+        <v>-0.06825938566552907</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22818,10 +22818,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.972</v>
+        <v>0.97</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07867298578199049</v>
+        <v>-0.08056872037914689</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22847,10 +22847,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.33</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08488372093023261</v>
+        <v>0.09186046511627918</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22905,10 +22905,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.26</v>
+        <v>0.263</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.07142857142857148</v>
+        <v>-0.06071428571428576</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22934,10 +22934,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04687500000000004</v>
+        <v>-0.06250000000000006</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22963,10 +22963,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.136</v>
+        <v>0.142</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.15</v>
+        <v>-0.1125000000000001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22992,10 +22992,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>18.6</v>
+        <v>19.35</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.06297229219143577</v>
+        <v>-0.0251889168765743</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23089,10 +23089,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.58</v>
+        <v>6.535</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05195843325339731</v>
+        <v>0.04476418864908078</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23118,10 +23118,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.378</v>
+        <v>5.384</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.03026819923371655</v>
+        <v>0.03141762452107291</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23176,10 +23176,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>21.05</v>
+        <v>20.8</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.06651884700665188</v>
+        <v>-0.07760532150776053</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23205,10 +23205,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.35</v>
+        <v>21.4</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01157407407407407</v>
+        <v>-0.009259259259259391</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23234,10 +23234,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.938</v>
+        <v>3.902</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01697453819271095</v>
+        <v>-0.02596105841238145</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23263,10 +23263,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>98.5</v>
+        <v>98.34999999999999</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.08960176991150436</v>
+        <v>0.08794247787610607</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23292,10 +23292,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.707</v>
+        <v>1.699</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.08862786972770952</v>
+        <v>-0.09289909236518951</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23350,10 +23350,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>221</v>
+        <v>222.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.004504504504504504</v>
+        <v>0.002252252252252252</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-25 14:11
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>25/09/2026 13:52</t>
+          <t>25/09/2026 14:11</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>13.05</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>12.85</v>
+        <v>12.7</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01532567049808437</v>
+        <v>-0.02681992337164762</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>1.95</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>1.92</v>
+        <v>1.895</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.0153846153846154</v>
+        <v>-0.02820512820512817</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>81.05</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>79.55</v>
+        <v>79.58</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.01850709438618137</v>
+        <v>-0.01813695249845773</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>19.415</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>19.07</v>
+        <v>19.05</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01776976564511969</v>
+        <v>-0.01879989698686575</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>97.8</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>92.15000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.05777096114519419</v>
+        <v>-0.05316973415132927</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>224</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>228</v>
+        <v>228.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02008928571428572</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>0.057</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.055</v>
+        <v>0.063</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.03508771929824565</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>1.45</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1.416</v>
+        <v>1.404</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.02344827586206899</v>
+        <v>-0.03172413793103451</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>4.52</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.55</v>
+        <v>4.53</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.006637168141592976</v>
+        <v>0.002212389380531123</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>22.72</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.48</v>
+        <v>22.46</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01056338028169007</v>
+        <v>-0.0114436619718309</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>3.97</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.978</v>
+        <v>3.973</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.002015113350125946</v>
+        <v>0.0007556675062971459</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>81.45</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>82.95</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01841620626151013</v>
+        <v>0.01718845917740935</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>5.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>5.17</v>
+        <v>5.165</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.003883495145630985</v>
+        <v>0.002912621359223239</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>1.783</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>1.819</v>
+        <v>1.82</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02019068984856984</v>
+        <v>0.02075154234436351</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>11.882</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>11.806</v>
+        <v>11.872</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.006396229590977993</v>
+        <v>-0.0008416091567076071</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>11.78</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>11.44</v>
+        <v>11.3</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.02886247877758912</v>
+        <v>-0.04074702886247866</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18718,10 +18718,10 @@
         <v>1.33</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.384</v>
+        <v>1.386</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.04060150375939836</v>
+        <v>0.0421052631578946</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>116.78</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>112.86</v>
+        <v>112.42</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.03356739167665698</v>
+        <v>-0.03733516013015927</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>31.2</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>31.4</v>
+        <v>31</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.006410256410256387</v>
+        <v>-0.006410256410256387</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>1.79</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>1.782</v>
+        <v>1.78</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.004469273743016764</v>
+        <v>-0.005586592178770954</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>81.05</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>79.55</v>
+        <v>79.58</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.01850709438618137</v>
+        <v>-0.01813695249845773</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>13.05</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.85</v>
+        <v>12.7</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01532567049808437</v>
+        <v>-0.02681992337164762</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>224</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>228</v>
+        <v>228.5</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02008928571428572</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>97.66</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>97.40000000000001</v>
+        <v>97.36</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.002662297767765625</v>
+        <v>-0.003071882039729646</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>18.3</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>18.1</v>
+        <v>18.14</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01092896174863384</v>
+        <v>-0.008743169398907111</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>97.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>92.15000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05777096114519419</v>
+        <v>-0.05316973415132927</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>1.86</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>1.864</v>
+        <v>1.862</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.002150537634408604</v>
+        <v>0.001075268817204302</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20467,7 +20467,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>25/09/2026 13:52</t>
+          <t>25/09/2026 14:11</t>
         </is>
       </c>
     </row>
@@ -20524,10 +20524,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>17.47</v>
+        <v>17.42</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1716968477531857</v>
+        <v>0.1683433936955065</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20554,10 +20554,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.55</v>
+        <v>79.58</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.009902247048368683</v>
+        <v>0.01028310270407518</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20674,10 +20674,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.7</v>
+        <v>34.66</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03503893214682975</v>
+        <v>-0.03615127919911024</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20704,10 +20704,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>222.2</v>
+        <v>222.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02775208140610546</v>
+        <v>0.02960222016651252</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20866,10 +20866,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.055</v>
+        <v>0.063</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.236111111111111</v>
+        <v>-0.1249999999999999</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20896,10 +20896,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.72</v>
+        <v>3.705</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.1446153846153847</v>
+        <v>0.14</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20926,10 +20926,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.17</v>
+        <v>5.165</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1124463519313305</v>
+        <v>-0.1133047210300429</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20986,10 +20986,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.07</v>
+        <v>7.09</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.05100671140939596</v>
+        <v>-0.04832214765100675</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21016,10 +21016,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.48</v>
+        <v>22.46</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.0942788074133763</v>
+        <v>-0.09508460918614019</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21046,10 +21046,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>77.23999999999999</v>
+        <v>77.28</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.09250353606789238</v>
+        <v>0.09306930693069304</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21136,10 +21136,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.94</v>
+        <v>22.92</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.05422794117647057</v>
+        <v>0.05330882352941177</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21241,10 +21241,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.679</v>
+        <v>5.65</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1005813953488372</v>
+        <v>0.09496124031007756</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21270,10 +21270,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.061</v>
+        <v>0.06</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2560975609756098</v>
+        <v>-0.2682926829268293</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21299,10 +21299,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.825</v>
+        <v>4.85</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1766211604095563</v>
+        <v>-0.1723549488054608</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21357,10 +21357,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.130000000000001</v>
+        <v>9.09</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.06162790697674432</v>
+        <v>0.05697674418604654</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21599,10 +21599,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.62</v>
+        <v>6.61</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05835331734612314</v>
+        <v>0.05675459632294171</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21628,10 +21628,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.25</v>
+        <v>5.272</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.005747126436781657</v>
+        <v>0.009961685823754883</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21715,10 +21715,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.3</v>
+        <v>21.25</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01388888888888892</v>
+        <v>-0.01620370370370377</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21744,10 +21744,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.922</v>
+        <v>3.916</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02096854717923117</v>
+        <v>-0.02246630054917631</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21773,10 +21773,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>92.15000000000001</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01935840707964602</v>
+        <v>0.02433628318584058</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21802,10 +21802,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.713</v>
+        <v>1.706</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.08542445274959953</v>
+        <v>-0.08916177255739458</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21860,10 +21860,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>228</v>
+        <v>228.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02927927927927928</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-25 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>25/09/2026 14:11</t>
+          <t>25/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>13.05</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02681992337164762</v>
+        <v>-0.01915708812260536</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>54.4</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>54.2</v>
+        <v>54.6</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.003676470588235216</v>
+        <v>0.003676470588235347</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>5.86</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>5.8</v>
+        <v>5.79</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01023890784982944</v>
+        <v>-0.01194539249146762</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>81.05</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>79.58</v>
+        <v>80.2</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.01813695249845773</v>
+        <v>-0.01048735348550271</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>19.415</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>19.05</v>
+        <v>18.93</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01879989698686575</v>
+        <v>-0.02498068503734223</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>97.8</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>92.59999999999999</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.05316973415132927</v>
+        <v>-0.05777096114519419</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>141.5</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>144</v>
+        <v>143.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.0176678445229682</v>
+        <v>0.01413427561837456</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18153,10 +18153,10 @@
         <v>77.15000000000001</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>76.90000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.003240440699935191</v>
+        <v>0.008425145819831385</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>224</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>228.5</v>
+        <v>227.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.02008928571428572</v>
+        <v>0.015625</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>0.057</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.1052631578947368</v>
+        <v>0.05263157894736834</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>1.45</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1.404</v>
+        <v>1.448</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.03172413793103451</v>
+        <v>-0.001379310344827587</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>4.52</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.53</v>
+        <v>4.495</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.002212389380531123</v>
+        <v>-0.005530973451327316</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>22.72</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.46</v>
+        <v>22.24</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.0114436619718309</v>
+        <v>-0.0211267605633803</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>3.97</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.973</v>
+        <v>4.03</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.0007556675062971459</v>
+        <v>0.0151133501259446</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>81.45</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>82.84999999999999</v>
+        <v>82.25</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01718845917740935</v>
+        <v>0.009821976672805367</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>5.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>5.165</v>
+        <v>5.11</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.002912621359223239</v>
+        <v>-0.007766990291262143</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>1.783</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>1.82</v>
+        <v>1.822</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02075154234436351</v>
+        <v>0.02187324733595073</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>28.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>29.35</v>
+        <v>29.4</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.01557093425605546</v>
+        <v>0.01730103806228374</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>11.882</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>11.872</v>
+        <v>11.808</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0008416091567076071</v>
+        <v>-0.006227907759636411</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>11.78</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>11.3</v>
+        <v>11.48</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.04074702886247866</v>
+        <v>-0.02546689303904915</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>4.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.9</v>
+        <v>4.82</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.01632653061224491</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18718,10 +18718,10 @@
         <v>1.33</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.386</v>
+        <v>1.32</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.0421052631578946</v>
+        <v>-0.00751879699248121</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>116.78</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>112.42</v>
+        <v>113.5</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.03733516013015927</v>
+        <v>-0.02808700119883543</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>31.2</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>31</v>
+        <v>31.4</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.006410256410256387</v>
+        <v>0.006410256410256387</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>6.45</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>6.45</v>
+        <v>6.35</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>-0.01550387596899233</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>33</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>33</v>
+        <v>32.4</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.01818181818181823</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>3.64</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>3.58</v>
+        <v>3.64</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.0164835164835165</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>1.79</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>1.78</v>
+        <v>1.758</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.005586592178770954</v>
+        <v>-0.01787709497206705</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>81.05</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>79.58</v>
+        <v>80.2</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.01813695249845773</v>
+        <v>-0.01048735348550271</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>54.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>54.2</v>
+        <v>54.6</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.003676470588235216</v>
+        <v>0.003676470588235347</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>13.05</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.7</v>
+        <v>12.8</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.02681992337164762</v>
+        <v>-0.01915708812260536</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>224</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>228.5</v>
+        <v>227.5</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.02008928571428572</v>
+        <v>0.015625</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19134,10 +19134,10 @@
         <v>77.15000000000001</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>76.90000000000001</v>
+        <v>77.8</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.003240440699935191</v>
+        <v>0.008425145819831385</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>97.66</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>97.36</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.003071882039729646</v>
+        <v>0.002457505631783833</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>18.3</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>18.14</v>
+        <v>18.02</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.008743169398907111</v>
+        <v>-0.01530054644808749</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>97.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>92.59999999999999</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05316973415132927</v>
+        <v>-0.05777096114519419</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>1.86</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>1.862</v>
+        <v>1.86</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.001075268817204302</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>141.5</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>144</v>
+        <v>143.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.0176678445229682</v>
+        <v>0.01413427561837456</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20467,7 +20467,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>25/09/2026 14:11</t>
+          <t>25/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20494,10 +20494,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.307</v>
+        <v>0.305</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1253561253561253</v>
+        <v>-0.131054131054131</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20524,10 +20524,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>17.42</v>
+        <v>16.81</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1683433936955065</v>
+        <v>0.1274312541918175</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20554,10 +20554,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>79.58</v>
+        <v>80.2</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01028310270407518</v>
+        <v>0.01815411958867598</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20584,10 +20584,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>144</v>
+        <v>143.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02857142857142857</v>
+        <v>0.025</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20614,10 +20614,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>124.6</v>
+        <v>124.8</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.001607717041800552</v>
+        <v>0.003215434083601218</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20644,10 +20644,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.2</v>
+        <v>54.6</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1410526315789474</v>
+        <v>0.1494736842105263</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20674,10 +20674,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.66</v>
+        <v>34.56</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03615127919911024</v>
+        <v>-0.03893214682981086</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20704,10 +20704,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>222.6</v>
+        <v>220.2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02960222016651252</v>
+        <v>0.01850138760407031</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20764,10 +20764,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.8</v>
+        <v>20.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.07760532150776053</v>
+        <v>-0.08647450110864742</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20866,10 +20866,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.063</v>
+        <v>0.06</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.1666666666666666</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20896,10 +20896,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.705</v>
+        <v>3.7</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.14</v>
+        <v>0.1384615384615385</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20926,10 +20926,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.165</v>
+        <v>5.11</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1133047210300429</v>
+        <v>-0.1227467811158798</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20956,10 +20956,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.6</v>
+        <v>2.64</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.287280701754386</v>
+        <v>-0.2763157894736842</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20986,10 +20986,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.09</v>
+        <v>7.07</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.04832214765100675</v>
+        <v>-0.05100671140939596</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21016,10 +21016,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.46</v>
+        <v>22.24</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.09508460918614019</v>
+        <v>-0.1039484286865432</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21046,10 +21046,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>77.28</v>
+        <v>77.08</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.09306930693069304</v>
+        <v>0.09024045261669017</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21076,10 +21076,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.41</v>
+        <v>7.38</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.07374999999999998</v>
+        <v>-0.07750000000000001</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21106,10 +21106,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.9</v>
+        <v>7.86</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.02948402948402951</v>
+        <v>-0.03439803439803443</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21136,10 +21136,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.92</v>
+        <v>22.98</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.05330882352941177</v>
+        <v>0.05606617647058818</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21241,10 +21241,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.65</v>
+        <v>5.48</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.09496124031007756</v>
+        <v>0.06201550387596905</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21270,10 +21270,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.06</v>
+        <v>0.061</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.2682926829268293</v>
+        <v>-0.2560975609756098</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21299,10 +21299,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.85</v>
+        <v>5.04</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1723549488054608</v>
+        <v>-0.1399317406143345</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21328,10 +21328,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.964</v>
+        <v>0.98</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.08625592417061609</v>
+        <v>-0.07109004739336489</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21357,10 +21357,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.09</v>
+        <v>8.92</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.05697674418604654</v>
+        <v>0.03720930232558143</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21415,10 +21415,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.256</v>
+        <v>0.255</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.08571428571428578</v>
+        <v>-0.08928571428571436</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21502,10 +21502,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>20</v>
+        <v>20.8</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.00755667506297222</v>
+        <v>0.04785894206549114</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21599,10 +21599,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.61</v>
+        <v>6.555</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05675459632294171</v>
+        <v>0.04796163069544362</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21628,10 +21628,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.272</v>
+        <v>5.338</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.009961685823754883</v>
+        <v>0.02260536398467439</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21657,10 +21657,10 @@
         <v>85.5</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>86</v>
+        <v>86.5</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.005847953216374269</v>
+        <v>0.01169590643274854</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -21686,10 +21686,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.8</v>
+        <v>20.6</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.07760532150776053</v>
+        <v>-0.08647450110864742</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21715,10 +21715,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>21.25</v>
+        <v>20.75</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01620370370370377</v>
+        <v>-0.03935185185185192</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21744,10 +21744,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.916</v>
+        <v>3.904</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02246630054917631</v>
+        <v>-0.02546180728906648</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21773,10 +21773,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>92.59999999999999</v>
+        <v>92.15000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.02433628318584058</v>
+        <v>0.01935840707964602</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21802,10 +21802,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.706</v>
+        <v>1.709</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.08916177255739458</v>
+        <v>-0.08756006406833952</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21860,10 +21860,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>228.5</v>
+        <v>227.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02927927927927928</v>
+        <v>0.02477477477477477</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise a jour auto - 2026-09-26 08:30
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bourse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A86E3C7-3915-4761-A8EA-FB7A41E8880E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC7A3D5F-FA5B-4B0E-AC8E-9A5E987B9544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Donnees" sheetId="1" r:id="rId1"/>
@@ -512,11 +512,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="000000"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -954,14 +953,276 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 4" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="356">
+  <dxfs count="178">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -1131,268 +1392,6 @@
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
       </font>
     </dxf>
     <dxf>
@@ -1775,6 +1774,268 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <condense val="0"/>
@@ -1996,268 +2257,6 @@
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
       </font>
     </dxf>
     <dxf>
@@ -2579,1464 +2578,6 @@
       <font>
         <b/>
         <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color auto="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="12"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="18"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -21948,277 +20489,277 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" dxfId="164" priority="31" stopIfTrue="1">
+    <cfRule type="expression" dxfId="164" priority="36" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="163" priority="35" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="162" priority="34" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="161" priority="33" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="160" priority="32" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="159" priority="31" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="163" priority="32" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F30:F39">
+    <cfRule type="expression" dxfId="158" priority="3" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="162" priority="33" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="157" priority="4" stopIfTrue="1">
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="161" priority="34" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="156" priority="5" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="160" priority="35" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="155" priority="1" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="159" priority="36" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="154" priority="6" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="153" priority="2" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" dxfId="158" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="152" priority="82" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="151" priority="81" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="150" priority="80" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="149" priority="77" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="157" priority="78" stopIfTrue="1">
+    <cfRule type="expression" dxfId="148" priority="78" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="156" priority="79" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="155" priority="80" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="154" priority="81" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="153" priority="82" stopIfTrue="1">
+    <cfRule type="expression" dxfId="147" priority="79" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" dxfId="146" priority="18" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="145" priority="17" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="144" priority="16" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="143" priority="15" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="142" priority="14" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="141" priority="13" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" dxfId="140" priority="83" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="139" priority="84" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="138" priority="85" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="137" priority="86" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" dxfId="136" priority="11" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="135" priority="10" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="134" priority="9" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="133" priority="8" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="132" priority="7" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="131" priority="12" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" dxfId="130" priority="89" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="129" priority="87" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="128" priority="88" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" dxfId="152" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="127" priority="66" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" dxfId="151" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="126" priority="67" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="150" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="125" priority="68" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="149" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="124" priority="69" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" dxfId="148" priority="74" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="123" priority="76" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="147" priority="75" stopIfTrue="1">
+    <cfRule type="expression" dxfId="122" priority="75" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="146" priority="76" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="121" priority="74" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" dxfId="145" priority="70" stopIfTrue="1">
+    <cfRule type="expression" dxfId="120" priority="70" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" dxfId="144" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="119" priority="71" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="143" priority="72" stopIfTrue="1">
+    <cfRule type="expression" dxfId="118" priority="72" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="142" priority="73" stopIfTrue="1">
+    <cfRule type="expression" dxfId="117" priority="73" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="141" priority="64" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" dxfId="116" priority="65" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="115" priority="64" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="65" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" dxfId="114" priority="37" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:G41 G2:G12 G16:G26">
+    <cfRule type="cellIs" dxfId="113" priority="63" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G28 G2:G12">
-    <cfRule type="cellIs" dxfId="139" priority="37" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="138" priority="63" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54 G56:G67 G30:G41">
-    <cfRule type="cellIs" dxfId="137" priority="54" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G43:G54 G30:G41 G56:G67">
+    <cfRule type="cellIs" dxfId="112" priority="54" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" dxfId="136" priority="42" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="111" priority="44" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="43" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="110" priority="43" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="134" priority="44" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="109" priority="42" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="108" priority="45" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" dxfId="132" priority="28" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="107" priority="30" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="29" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="106" priority="29" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="30" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="105" priority="28" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" dxfId="129" priority="55" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="104" priority="55" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="128" priority="56" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="103" priority="56" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="127" priority="57" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="102" priority="57" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" dxfId="126" priority="38" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="101" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="100" priority="40" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="125" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="99" priority="39" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="40" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="98" priority="38" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="41" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" dxfId="122" priority="50" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="97" priority="52" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="51" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="96" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="52" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="95" priority="50" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="119" priority="53" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="94" priority="51" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" dxfId="118" priority="46" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="93" priority="46" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="47" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="92" priority="47" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="116" priority="48" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="91" priority="48" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="115" priority="49" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="90" priority="49" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" dxfId="114" priority="27" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="89" priority="27" operator="greaterThan">
       <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" dxfId="113" priority="83" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="112" priority="84" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="111" priority="85" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="110" priority="86" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" dxfId="109" priority="87" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="108" priority="88" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="107" priority="89" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" dxfId="106" priority="13" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="105" priority="14" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="104" priority="15" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="103" priority="16" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="102" priority="17" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="101" priority="18" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" dxfId="100" priority="7" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="99" priority="8" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="98" priority="9" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="97" priority="10" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="96" priority="11" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="95" priority="12" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" dxfId="94" priority="1" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="93" priority="2" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="92" priority="3" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="91" priority="4" stopIfTrue="1">
-      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="90" priority="5" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="89" priority="6" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22243,7 +20784,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="52">
-        <v>46335</v>
+        <v>46276</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -24201,277 +22742,277 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" dxfId="75" priority="25" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" dxfId="75" priority="27" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="74" priority="26" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="27" stopIfTrue="1">
+    <cfRule type="expression" dxfId="73" priority="25" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="72" priority="29" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="71" priority="30" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="28" stopIfTrue="1">
+    <cfRule type="expression" dxfId="70" priority="28" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="71" priority="29" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="70" priority="30" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" dxfId="69" priority="71" stopIfTrue="1">
+    <cfRule type="expression" dxfId="69" priority="75" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="68" priority="74" stopIfTrue="1">
+      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="72" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="66" priority="71" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="72" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="67" priority="73" stopIfTrue="1">
+    <cfRule type="expression" dxfId="65" priority="73" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="66" priority="74" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="65" priority="75" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" dxfId="64" priority="76" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" dxfId="63" priority="77" stopIfTrue="1">
+    <cfRule type="expression" dxfId="63" priority="79" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="62" priority="77" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="78" stopIfTrue="1">
+    <cfRule type="expression" dxfId="61" priority="81" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="79" stopIfTrue="1">
+    <cfRule type="expression" dxfId="60" priority="82" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="80" stopIfTrue="1">
+    <cfRule type="expression" dxfId="59" priority="80" stopIfTrue="1">
       <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="81" stopIfTrue="1">
+    <cfRule type="expression" dxfId="58" priority="78" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="58" priority="82" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" dxfId="57" priority="12" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="56" priority="10" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="55" priority="9" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="54" priority="8" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="53" priority="11" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="7" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" dxfId="51" priority="83" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="50" priority="84" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="85" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="86" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" dxfId="47" priority="2" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="3" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="4" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="44" priority="6" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="1" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="42" priority="5" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" dxfId="41" priority="89" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="40" priority="87" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="39" priority="88" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" dxfId="57" priority="60" stopIfTrue="1">
+    <cfRule type="expression" dxfId="38" priority="60" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" dxfId="56" priority="61" stopIfTrue="1">
+    <cfRule type="expression" dxfId="37" priority="61" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="62" stopIfTrue="1">
+    <cfRule type="expression" dxfId="36" priority="62" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="63" stopIfTrue="1">
+    <cfRule type="expression" dxfId="35" priority="63" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" dxfId="53" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="34" priority="70" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="33" priority="68" stopIfTrue="1">
       <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="32" priority="69" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="51" priority="70" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" dxfId="50" priority="64" stopIfTrue="1">
+    <cfRule type="expression" dxfId="31" priority="64" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" dxfId="49" priority="65" stopIfTrue="1">
+    <cfRule type="expression" dxfId="30" priority="66" stopIfTrue="1">
+      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="29" priority="67" stopIfTrue="1">
+      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="65" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="66" stopIfTrue="1">
-      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="47" priority="67" stopIfTrue="1">
-      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="46" priority="58" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" dxfId="27" priority="58" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="45" priority="59" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="26" priority="59" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G28 G2:G12">
-    <cfRule type="cellIs" dxfId="44" priority="31" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" dxfId="25" priority="31" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:G26 G2:G12 G30:G41">
-    <cfRule type="cellIs" dxfId="43" priority="57" operator="greaterThan">
+  <conditionalFormatting sqref="G30:G41 G2:G12 G16:G26">
+    <cfRule type="cellIs" dxfId="24" priority="57" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54 G56:G67 G30:G41">
-    <cfRule type="cellIs" dxfId="42" priority="48" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G43:G54 G30:G41 G56:G67">
+    <cfRule type="cellIs" dxfId="23" priority="48" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" dxfId="41" priority="36" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="39" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="38" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="37" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="37" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="38" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="36" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="39" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" dxfId="37" priority="22" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="18" priority="24" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="23" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="17" priority="23" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="24" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="16" priority="22" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" dxfId="34" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="15" priority="49" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="50" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="14" priority="50" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="51" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="13" priority="51" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" dxfId="31" priority="32" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="12" priority="35" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="33" operator="greaterThan">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="32" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="33" operator="greaterThan">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="34" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="9" priority="34" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="35" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" dxfId="27" priority="44" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="44" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="45" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="45" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="46" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="46" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="47" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="5" priority="47" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" dxfId="23" priority="40" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="43" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="42" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="41" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="2" priority="41" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="42" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="40" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="43" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" dxfId="19" priority="21" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="21" operator="greaterThan">
       <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" dxfId="18" priority="83" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="17" priority="84" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="85" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="86" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" dxfId="14" priority="87" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="88" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="89" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="8" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="9" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="10" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="11" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="12" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" dxfId="5" priority="1" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="5" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="6" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-29 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>29/09/2026 13:00</t>
+          <t>29/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>47.28</v>
+        <v>46.89</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.04822081809112082</v>
+        <v>0.03957432657133364</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>79.75</v>
+        <v>78.7</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.02638352638352635</v>
+        <v>0.01287001287001287</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.94</v>
+        <v>24.88</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.0008012820512820341</v>
+        <v>-0.003205128205128279</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>145</v>
+        <v>142.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.006944444444444444</v>
+        <v>-0.01041666666666667</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>80.15000000000001</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.05114754098360663</v>
+        <v>0.06426229508196729</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>60.6</v>
+        <v>60.3</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.02728731942215082</v>
+        <v>-0.03210272873194222</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>6.88</v>
+        <v>6.92</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.05038167938931299</v>
+        <v>0.05648854961832063</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>56.9</v>
+        <v>56.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.007846556233653058</v>
+        <v>-0.01830863121185709</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18153,10 +18153,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.006622516556291391</v>
+        <v>-0.004415011037527594</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.76</v>
+        <v>18.67</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.003717472118958935</v>
+        <v>-0.008497079129049208</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.792</v>
+        <v>2.674</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.06564885496183195</v>
+        <v>0.0206106870229007</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>976</v>
+        <v>985</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.006185567010309278</v>
+        <v>0.0154639175257732</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.473</v>
+        <v>0.47</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.02674897119341566</v>
+        <v>-0.03292181069958851</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.395</v>
+        <v>4.335</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01897321428571448</v>
+        <v>-0.03236607142857153</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.16</v>
+        <v>20.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.05366726296958852</v>
+        <v>-0.08318425760286223</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.406</v>
+        <v>1.352</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02496532593619975</v>
+        <v>-0.06241331484049921</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.077</v>
+        <v>0.078</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.6</v>
+        <v>0.605</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1228070175438598</v>
+        <v>-0.1154970760233919</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.909</v>
+        <v>0.897</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.2609756097560975</v>
+        <v>-0.2707317073170731</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>48.55</v>
+        <v>47.85</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.02318229715489977</v>
+        <v>0.008429926238145386</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18718,10 +18718,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.984</v>
+        <v>0.978</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.004081632653061228</v>
+        <v>-0.002040816326530614</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.08</v>
+        <v>3.96</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>-0.02941176470588238</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>5</v>
+        <v>4.76</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>-0.04800000000000004</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>31.3</v>
+        <v>31.4</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.00318471337579611</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.275</v>
+        <v>1.265</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01923076923076933</v>
+        <v>-0.02692307692307703</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.02400000000000002</v>
+        <v>0.008000000000000007</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>6.72</v>
+        <v>6.8</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05617977528089892</v>
+        <v>-0.04494382022471914</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>164.1</v>
+        <v>161.6</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.007259528130671609</v>
+        <v>-0.02238354506957058</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>24</v>
+        <v>23.95</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.008264462809917326</v>
+        <v>-0.01033057851239669</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.864</v>
+        <v>1.866</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.002150537634408604</v>
+        <v>0.003225806451612906</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.76</v>
+        <v>18.67</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.003717472118958935</v>
+        <v>-0.008497079129049208</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19134,10 +19134,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.94</v>
+        <v>24.88</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.0008012820512820341</v>
+        <v>-0.003205128205128279</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>47.28</v>
+        <v>46.89</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.04822081809112082</v>
+        <v>0.03957432657133364</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>96.28</v>
+        <v>96.08</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01614551399959124</v>
+        <v>-0.01818924994890661</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>109.3</v>
+        <v>109.6</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.01353790613718412</v>
+        <v>-0.01083032490974732</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>60.6</v>
+        <v>60.3</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02728731942215082</v>
+        <v>-0.03210272873194222</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>79.75</v>
+        <v>78.7</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02638352638352635</v>
+        <v>0.01287001287001287</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>29/09/2026 13:00</t>
+          <t>29/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20528,10 +20528,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.309</v>
+        <v>0.301</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1196581196581196</v>
+        <v>-0.1424501424501424</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20558,10 +20558,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.71</v>
+        <v>16.92</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1207243460764588</v>
+        <v>0.1348088531187124</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20588,10 +20588,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>78.55</v>
+        <v>78.14</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.002792941475180892</v>
+        <v>-0.007997968769836175</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20618,10 +20618,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>145</v>
+        <v>142.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.01785714285714286</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20708,10 +20708,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.98</v>
+        <v>34.9</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02725250278086774</v>
+        <v>-0.02947719688542831</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20738,10 +20738,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>218.4</v>
+        <v>215.4</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01017576318223875</v>
+        <v>-0.003700277520813982</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20798,10 +20798,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.08647450110864742</v>
+        <v>-0.08203991130820405</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20900,10 +20900,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.062</v>
+        <v>0.063</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1388888888888888</v>
+        <v>-0.1249999999999999</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20930,10 +20930,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.57</v>
+        <v>3.48</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.09846153846153841</v>
+        <v>0.07076923076923076</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20960,10 +20960,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>5.045</v>
+        <v>4.91</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1339055793991417</v>
+        <v>-0.1570815450643777</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20990,10 +20990,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.792</v>
+        <v>2.674</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.2346491228070176</v>
+        <v>-0.2669956140350878</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21020,10 +21020,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.95</v>
+        <v>6.94</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.06711409395973154</v>
+        <v>-0.06845637583892615</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21050,10 +21050,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.16</v>
+        <v>20.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1474617244157937</v>
+        <v>-0.1740531829170024</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21080,10 +21080,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>76.84</v>
+        <v>76.5</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.08684582743988685</v>
+        <v>0.082036775106082</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21110,10 +21110,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.35</v>
+        <v>7.27</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.08125000000000004</v>
+        <v>-0.09125000000000005</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21140,10 +21140,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.71</v>
+        <v>7.7</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.05282555282555289</v>
+        <v>-0.0540540540540541</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21170,10 +21170,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>24.06</v>
+        <v>23.96</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.1056985294117646</v>
+        <v>0.1011029411764705</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21275,10 +21275,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.79</v>
+        <v>5.646</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1220930232558139</v>
+        <v>0.09418604651162786</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21304,10 +21304,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.074</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.09756097560975618</v>
+        <v>-0.1219512195121952</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21333,10 +21333,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.895</v>
+        <v>4.46</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.1646757679180889</v>
+        <v>-0.2389078498293516</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21362,10 +21362,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.984</v>
+        <v>0.978</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.06729857819905209</v>
+        <v>-0.07298578199052129</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21391,10 +21391,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.5</v>
+        <v>9.42</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.1046511627906977</v>
+        <v>0.09534883720930236</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21420,10 +21420,10 @@
         <v>20.3</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.1</v>
+        <v>25.2</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2364532019704434</v>
+        <v>0.2413793103448275</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21449,10 +21449,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.244</v>
+        <v>0.249</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1285714285714287</v>
+        <v>-0.1107142857142858</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21478,10 +21478,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04687500000000004</v>
+        <v>-0.01562500000000001</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21507,10 +21507,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.131</v>
+        <v>0.124</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.18125</v>
+        <v>-0.225</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21536,10 +21536,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.95</v>
+        <v>20.1</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.005037783375314754</v>
+        <v>0.01259445843828715</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21633,10 +21633,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.88</v>
+        <v>6.92</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.09992006394884093</v>
+        <v>0.1063149480415668</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21662,10 +21662,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.404</v>
+        <v>5.374</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.0352490421455939</v>
+        <v>0.02950191570881225</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21720,10 +21720,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.08647450110864742</v>
+        <v>-0.08203991130820405</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21749,10 +21749,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.06481481481481491</v>
+        <v>-0.06944444444444443</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21778,10 +21778,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.828</v>
+        <v>3.818</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04443334997503753</v>
+        <v>-0.04692960559161262</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21807,10 +21807,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>89.55</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.009402654867256732</v>
+        <v>0.01106194690265487</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21836,10 +21836,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.648</v>
+        <v>1.605</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1201281366791244</v>
+        <v>-0.1430859583555793</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21894,10 +21894,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01576576576576576</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-30 13:46
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>29/09/2026 19:05</t>
+          <t>30/09/2026 13:46</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>46.89</v>
+        <v>46.95</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.03957432657133364</v>
+        <v>0.04090455603591633</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>78.7</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01287001287001287</v>
+        <v>0.01801801801801791</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.88</v>
+        <v>24.64</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.003205128205128279</v>
+        <v>-0.01282051282051283</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>142.5</v>
+        <v>144</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01041666666666667</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>81.15000000000001</v>
+        <v>81</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06426229508196729</v>
+        <v>0.06229508196721312</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>60.3</v>
+        <v>60.5</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.03210272873194222</v>
+        <v>-0.02889245585874795</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>6.92</v>
+        <v>6.885</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.05648854961832063</v>
+        <v>0.05114503816793893</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>56.3</v>
+        <v>55.9</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01830863121185709</v>
+        <v>-0.02528334786399307</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.67</v>
+        <v>18.43</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.008497079129049208</v>
+        <v>-0.0212426978226234</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.674</v>
+        <v>2.412</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.0206106870229007</v>
+        <v>-0.07938931297709931</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>985</v>
+        <v>1008</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.0154639175257732</v>
+        <v>0.03917525773195876</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.47</v>
+        <v>0.463</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.03292181069958851</v>
+        <v>-0.04732510288065837</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.335</v>
+        <v>4.31</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03236607142857153</v>
+        <v>-0.03794642857142875</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.5</v>
+        <v>20.66</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.08318425760286223</v>
+        <v>-0.07602862254025042</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.352</v>
+        <v>1.374</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.06241331484049921</v>
+        <v>-0.04715672676837714</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.605</v>
+        <v>0.599</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1154970760233919</v>
+        <v>-0.1242690058479533</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>38</v>
+        <v>39.2</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0410958904109589</v>
+        <v>0.07397260273972611</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.897</v>
+        <v>0.968</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.2707317073170731</v>
+        <v>-0.2130081300813008</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>47.85</v>
+        <v>48.15</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.008429926238145386</v>
+        <v>0.01475237091675439</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18718,10 +18718,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.978</v>
+        <v>0.998</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.002040816326530614</v>
+        <v>0.01836734693877553</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.96</v>
+        <v>3.99</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02941176470588238</v>
+        <v>-0.02205882352941173</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18776,10 +18776,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>5.01</v>
+        <v>5</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.02906976744186053</v>
+        <v>-0.03100775193798452</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.76</v>
+        <v>4.82</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04800000000000004</v>
+        <v>-0.03599999999999994</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>-0.006369426751592334</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.265</v>
+        <v>1.25</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02692307692307703</v>
+        <v>-0.03846153846153849</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.26</v>
+        <v>1.225</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.008000000000000007</v>
+        <v>-0.01999999999999993</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.04494382022471914</v>
+        <v>-0.03089887640449435</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>161.6</v>
+        <v>161</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.02238354506957058</v>
+        <v>-0.0260133091349063</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>23.95</v>
+        <v>23.65</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01033057851239669</v>
+        <v>-0.02272727272727276</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.866</v>
+        <v>1.87</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.003225806451612906</v>
+        <v>0.00537634408602151</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.67</v>
+        <v>18.43</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.008497079129049208</v>
+        <v>-0.0212426978226234</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19134,10 +19134,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.88</v>
+        <v>24.64</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.003205128205128279</v>
+        <v>-0.01282051282051283</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>46.89</v>
+        <v>46.95</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.03957432657133364</v>
+        <v>0.04090455603591633</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>96.08</v>
+        <v>93.54000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01818924994890661</v>
+        <v>-0.04414469650521146</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>109.6</v>
+        <v>108.5</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.01083032490974732</v>
+        <v>-0.02075812274368229</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>60.3</v>
+        <v>60.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.03210272873194222</v>
+        <v>-0.02889245585874795</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>78.7</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01287001287001287</v>
+        <v>0.01801801801801791</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>29/09/2026 19:05</t>
+          <t>30/09/2026 13:46</t>
         </is>
       </c>
     </row>
@@ -20528,10 +20528,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.301</v>
+        <v>0.31</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1424501424501424</v>
+        <v>-0.1168091168091168</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20558,10 +20558,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.92</v>
+        <v>16.52</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1348088531187124</v>
+        <v>0.107981220657277</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20588,10 +20588,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>78.14</v>
+        <v>76.09</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.007997968769836175</v>
+        <v>-0.03402310524311277</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20618,10 +20618,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>142.5</v>
+        <v>144</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02857142857142857</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20648,10 +20648,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.3</v>
+        <v>125.2</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.007234726688102825</v>
+        <v>0.006430868167202549</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20708,10 +20708,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.9</v>
+        <v>35.12</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02947719688542831</v>
+        <v>-0.02335928809788664</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20738,10 +20738,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>215.4</v>
+        <v>216.2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.003700277520813982</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20798,10 +20798,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.7</v>
+        <v>20.65</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.08203991130820405</v>
+        <v>-0.08425720620842582</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20900,10 +20900,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.063</v>
+        <v>0.064</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.111111111111111</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20930,10 +20930,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.48</v>
+        <v>3.405</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07076923076923076</v>
+        <v>0.04769230769230763</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20960,10 +20960,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.91</v>
+        <v>4.826</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1570815450643777</v>
+        <v>-0.1715021459227469</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20990,10 +20990,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.674</v>
+        <v>2.412</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.2669956140350878</v>
+        <v>-0.3388157894736842</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21020,10 +21020,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.94</v>
+        <v>7.03</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.06845637583892615</v>
+        <v>-0.05637583892617449</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21050,10 +21050,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.5</v>
+        <v>20.66</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1740531829170024</v>
+        <v>-0.1676067687348912</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21080,10 +21080,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>76.5</v>
+        <v>75.45999999999999</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.082036775106082</v>
+        <v>0.06732673267326719</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21110,10 +21110,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.27</v>
+        <v>7.42</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.09125000000000005</v>
+        <v>-0.07250000000000001</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21140,10 +21140,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.7</v>
+        <v>7.61</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.0540540540540541</v>
+        <v>-0.06511056511056514</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21170,10 +21170,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.96</v>
+        <v>23.74</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.1011029411764705</v>
+        <v>0.09099264705882337</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21275,10 +21275,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.646</v>
+        <v>5.731</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.09418604651162786</v>
+        <v>0.1106589147286821</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21304,10 +21304,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.075</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1219512195121952</v>
+        <v>-0.08536585365853666</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21333,10 +21333,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.46</v>
+        <v>4.71</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2389078498293516</v>
+        <v>-0.196245733788396</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21362,10 +21362,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.978</v>
+        <v>0.998</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07298578199052129</v>
+        <v>-0.05402843601895729</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21391,10 +21391,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.42</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.09534883720930236</v>
+        <v>0.09069767441860478</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21420,10 +21420,10 @@
         <v>20.3</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.2</v>
+        <v>25.1</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2413793103448275</v>
+        <v>0.2364532019704434</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21449,10 +21449,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.249</v>
+        <v>0.244</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1107142857142858</v>
+        <v>-0.1285714285714287</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21478,10 +21478,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.26</v>
+        <v>1.225</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01562500000000001</v>
+        <v>-0.04296874999999995</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21507,10 +21507,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.124</v>
+        <v>0.127</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.225</v>
+        <v>-0.20625</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21633,10 +21633,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.92</v>
+        <v>6.885</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.1063149480415668</v>
+        <v>0.1007194244604316</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21662,10 +21662,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.374</v>
+        <v>5.332</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.02950191570881225</v>
+        <v>0.02145593869731803</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21720,10 +21720,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.7</v>
+        <v>20.65</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.08203991130820405</v>
+        <v>-0.08425720620842582</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21749,10 +21749,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>20.1</v>
+        <v>20.3</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.06944444444444443</v>
+        <v>-0.06018518518518522</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21778,10 +21778,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.818</v>
+        <v>3.842</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04692960559161262</v>
+        <v>-0.04093859211183228</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21807,10 +21807,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>91.40000000000001</v>
+        <v>86.05</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01106194690265487</v>
+        <v>-0.04811946902654876</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21836,10 +21836,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.605</v>
+        <v>1.607</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1430859583555793</v>
+        <v>-0.1420181526962093</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-09-30 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>30/09/2026 13:46</t>
+          <t>30/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>46.95</v>
+        <v>46.97</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.04090455603591633</v>
+        <v>0.04134796585744379</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>79.09999999999999</v>
+        <v>78.34999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01801801801801791</v>
+        <v>0.008365508365508256</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.64</v>
+        <v>24.68</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>-0.01121794871794876</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.02083333333333333</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>81</v>
+        <v>82.65000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06229508196721312</v>
+        <v>0.08393442622950827</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>60.5</v>
+        <v>59.95</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.02889245585874795</v>
+        <v>-0.03772070626003202</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18093,10 +18093,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>6.885</v>
+        <v>6.87</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.05114503816793893</v>
+        <v>0.04885496183206112</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.9</v>
+        <v>55.35</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.02528334786399307</v>
+        <v>-0.03487358326068003</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18153,10 +18153,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.004415011037527594</v>
+        <v>-0.002207505518763797</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18183,10 +18183,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.43</v>
+        <v>18.47</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0212426978226234</v>
+        <v>-0.0191184280403611</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.412</v>
+        <v>2.484</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.07938931297709931</v>
+        <v>-0.05190839694656493</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1008</v>
+        <v>1002</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.03917525773195876</v>
+        <v>0.03298969072164949</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>0.012</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0</v>
+        <v>-0.08333333333333341</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.463</v>
+        <v>0.475</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.04732510288065837</v>
+        <v>-0.0226337448559671</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.31</v>
+        <v>4.4</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03794642857142875</v>
+        <v>-0.01785714285714287</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.66</v>
+        <v>20.94</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.07602862254025042</v>
+        <v>-0.0635062611806797</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.374</v>
+        <v>1.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.04715672676837714</v>
+        <v>-0.02912621359223303</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.078</v>
+        <v>0.077</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>-0.01282051282051283</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.599</v>
+        <v>0.592</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1242690058479533</v>
+        <v>-0.1345029239766083</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>39.2</v>
+        <v>39.5</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.07397260273972611</v>
+        <v>0.0821917808219178</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.968</v>
+        <v>1.05</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.2130081300813008</v>
+        <v>-0.1463414634146341</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>48.15</v>
+        <v>48.25</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.01475237091675439</v>
+        <v>0.01685985247629077</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18718,10 +18718,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.998</v>
+        <v>0.986</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.01836734693877553</v>
+        <v>0.006122448979591842</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.99</v>
+        <v>4.03</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02205882352941173</v>
+        <v>-0.01225490196078427</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18776,10 +18776,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>5</v>
+        <v>5.13</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.03100775193798452</v>
+        <v>-0.005813953488372141</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>31.2</v>
+        <v>31</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.006369426751592334</v>
+        <v>-0.01273885350318467</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.25</v>
+        <v>1.245</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03846153846153849</v>
+        <v>-0.04230769230769226</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.225</v>
+        <v>1.215</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.01999999999999993</v>
+        <v>-0.02799999999999993</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18921,10 +18921,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>6.9</v>
+        <v>6.76</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.03089887640449435</v>
+        <v>-0.05056179775280904</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19018,10 +19018,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.0260133091349063</v>
+        <v>-0.007864488808227533</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>23.65</v>
+        <v>24.05</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.02272727272727276</v>
+        <v>-0.006198347107437958</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.87</v>
+        <v>1.868</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.00537634408602151</v>
+        <v>0.004301075268817208</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.43</v>
+        <v>18.47</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.0212426978226234</v>
+        <v>-0.0191184280403611</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19134,10 +19134,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.64</v>
+        <v>24.68</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>-0.01121794871794876</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19163,10 +19163,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>46.95</v>
+        <v>46.97</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.04090455603591633</v>
+        <v>0.04134796585744379</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>93.54000000000001</v>
+        <v>94.64</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.04414469650521146</v>
+        <v>-0.0329041487839771</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>108.5</v>
+        <v>107.6</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02075812274368229</v>
+        <v>-0.02888086642599281</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>60.5</v>
+        <v>59.95</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02889245585874795</v>
+        <v>-0.03772070626003202</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>79.09999999999999</v>
+        <v>78.34999999999999</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01801801801801791</v>
+        <v>0.008365508365508256</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20501,7 +20501,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>30/09/2026 13:46</t>
+          <t>30/09/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20528,10 +20528,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1168091168091168</v>
+        <v>-0.1452991452991453</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20558,10 +20558,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.52</v>
+        <v>16.63</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.107981220657277</v>
+        <v>0.1153588195841716</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20588,10 +20588,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>76.09</v>
+        <v>75.59</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.03402310524311277</v>
+        <v>-0.04037069950488756</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20618,10 +20618,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02857142857142857</v>
+        <v>0.007142857142857143</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20648,10 +20648,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.2</v>
+        <v>125.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.006430868167202549</v>
+        <v>0.008038585209003215</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20678,10 +20678,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.4</v>
+        <v>54.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1452631578947368</v>
+        <v>0.1410526315789474</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20708,10 +20708,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.12</v>
+        <v>35.14</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02335928809788664</v>
+        <v>-0.02280311457174639</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20738,10 +20738,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>216.2</v>
+        <v>216</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>-0.0009250693802034627</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20768,10 +20768,10 @@
         <v>0.016</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.25</v>
+        <v>-0.3125000000000001</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20798,10 +20798,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.65</v>
+        <v>20.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.08425720620842582</v>
+        <v>-0.09090909090909094</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20900,10 +20900,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.064</v>
+        <v>0.065</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.111111111111111</v>
+        <v>-0.09722222222222213</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20930,10 +20930,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.405</v>
+        <v>3.44</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.04769230769230763</v>
+        <v>0.05846153846153845</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20990,10 +20990,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.412</v>
+        <v>2.484</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3388157894736842</v>
+        <v>-0.3190789473684211</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21020,10 +21020,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>7.03</v>
+        <v>6.95</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.05637583892617449</v>
+        <v>-0.06711409395973154</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21050,10 +21050,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.66</v>
+        <v>20.94</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1676067687348912</v>
+        <v>-0.1563255439161966</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21080,10 +21080,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>75.45999999999999</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.06732673267326719</v>
+        <v>0.06449787835926453</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21110,10 +21110,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.42</v>
+        <v>7.29</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.07250000000000001</v>
+        <v>-0.08875</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21170,10 +21170,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.74</v>
+        <v>24.08</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.09099264705882337</v>
+        <v>0.1066176470588234</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21275,10 +21275,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.731</v>
+        <v>5.671</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1106589147286821</v>
+        <v>0.099031007751938</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21333,10 +21333,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.71</v>
+        <v>4.8</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.196245733788396</v>
+        <v>-0.180887372013652</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21362,10 +21362,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.998</v>
+        <v>0.986</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05402843601895729</v>
+        <v>-0.06540284360189569</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21391,10 +21391,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.380000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.09069767441860478</v>
+        <v>0.08255813953488382</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21449,10 +21449,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.244</v>
+        <v>0.243</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1285714285714287</v>
+        <v>-0.1321428571428573</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21478,10 +21478,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.225</v>
+        <v>1.215</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04296874999999995</v>
+        <v>-0.05078124999999996</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21507,10 +21507,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.127</v>
+        <v>0.13</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.20625</v>
+        <v>-0.1875</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21536,10 +21536,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>20.1</v>
+        <v>19.85</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.01259445843828715</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21633,10 +21633,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.885</v>
+        <v>6.87</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.1007194244604316</v>
+        <v>0.09832134292565951</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21662,10 +21662,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.332</v>
+        <v>5.282</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.02145593869731803</v>
+        <v>0.01187739463601538</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21720,10 +21720,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.65</v>
+        <v>20.5</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.08425720620842582</v>
+        <v>-0.09090909090909094</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21749,10 +21749,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>20.3</v>
+        <v>20.35</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.06018518518518522</v>
+        <v>-0.05787037037037036</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21778,10 +21778,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.842</v>
+        <v>3.75</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04093859211183228</v>
+        <v>-0.06390414378432356</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21807,10 +21807,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>86.05</v>
+        <v>87.45</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.04811946902654876</v>
+        <v>-0.03263274336283189</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21836,10 +21836,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.607</v>
+        <v>1.583</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1420181526962093</v>
+        <v>-0.1548318206086493</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21865,10 +21865,10 @@
         <v>35.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>34.4</v>
+        <v>34.8</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02272727272727285</v>
+        <v>-0.01136363636363652</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21894,10 +21894,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01576576576576576</v>
+        <v>0.01801801801801802</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-01 15:08
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1886" yWindow="1886" windowWidth="24685" windowHeight="13054" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Donnees" sheetId="1" state="visible" r:id="rId1"/>
@@ -17846,7 +17846,7 @@
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="53" t="inlineStr">
         <is>
-          <t>25/09/2026</t>
+          <t>30/09/2026</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>30/09/2026 19:05</t>
+          <t>01/10/2026 15:08</t>
         </is>
       </c>
     </row>
@@ -17896,7 +17896,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>STMPA</t>
+          <t>SOI</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -17906,17 +17906,17 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>STMICROELECTRONICS</t>
+          <t xml:space="preserve">SOITEC </t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>45.105</v>
+        <v>155.95</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>46.97</v>
+        <v>155.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.04134796585744379</v>
+        <v>-0.005450464892593744</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17926,7 +17926,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>ATE</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -17936,17 +17936,17 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>BIOMERIEUX</t>
+          <t>ALTEN</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>77.7</v>
+        <v>82</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>78.34999999999999</v>
+        <v>83.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.008365508365508256</v>
+        <v>0.01829268292682927</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17956,27 +17956,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>VMX</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>JCDECAUX</t>
+          <t>VERIMATRIX</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>24.96</v>
+        <v>0.314</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.68</v>
+        <v>0.314</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01121794871794876</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -17986,7 +17986,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -17996,17 +17996,17 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>144</v>
+        <v>6.895</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>141</v>
+        <v>6.73</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02083333333333333</v>
+        <v>-0.02393038433647559</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18016,7 +18016,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>ATE</t>
+          <t>QDT</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -18026,17 +18026,17 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>ALTEN</t>
+          <t>QUADIENT</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>76.25</v>
+        <v>14.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>82.65000000000001</v>
+        <v>13.92</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.08393442622950827</v>
+        <v>-0.007132667617688991</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18046,7 +18046,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>EXENS</t>
+          <t>ABCA</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -18056,17 +18056,17 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>EXOSENS</t>
+          <t>ABC ARBITRAGE</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>62.3</v>
+        <v>5.91</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>59.95</v>
+        <v>5.83</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.03772070626003202</v>
+        <v>-0.01353637901861253</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18076,7 +18076,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>BAIN</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -18086,17 +18086,17 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>X-FAB SILICON</t>
+          <t>BAINS MER MONACO</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>6.55</v>
+        <v>144</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>6.87</v>
+        <v>142</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.04885496183206112</v>
+        <v>-0.01388888888888889</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18106,7 +18106,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>RCO</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -18116,17 +18116,17 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>SODEXO</t>
+          <t>REMY COINTREAU</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>57.35</v>
+        <v>43.88</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.35</v>
+        <v>43.22</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03487358326068003</v>
+        <v>-0.01504102096627173</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18150,13 +18150,13 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>226.5</v>
+        <v>225.5</v>
       </c>
       <c r="F10" s="12" t="n">
         <v>226</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.002207505518763797</v>
+        <v>0.002217294900221729</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18166,27 +18166,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>GETLINK SE</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>18.83</v>
+        <v>34.8</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.47</v>
+        <v>34.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0191184280403611</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18282,13 +18282,13 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>2.62</v>
+        <v>2.47</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.484</v>
+        <v>2.262</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05190839694656493</v>
+        <v>-0.08421052631578954</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18298,27 +18298,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>ODET</t>
+          <t>SIGHT</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>COMP. ODET</t>
+          <t>GENSIGHT BIOLO</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>970</v>
+        <v>0.099</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1002</v>
+        <v>0.091</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.03298969072164949</v>
+        <v>-0.08080808080808087</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18328,27 +18328,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>LAT</t>
+          <t>MEDCL</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>LATECOERE</t>
+          <t>MEDINCELL</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>0.012</v>
+        <v>24.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>0.011</v>
+        <v>23.08</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.08333333333333341</v>
+        <v>-0.04232365145228228</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18358,7 +18358,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>NXI</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -18368,17 +18368,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>SOLUTIONS 30</t>
+          <t>NEXITY</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>0.486</v>
+        <v>4.816</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.475</v>
+        <v>4.612</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.0226337448559671</v>
+        <v>-0.04235880398671091</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18388,7 +18388,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>VLTSA</t>
+          <t>STLAP</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -18398,17 +18398,17 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>VOLTALIA</t>
+          <t>STELLANTIS</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>4.48</v>
+        <v>3.901</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.4</v>
+        <v>3.861</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01785714285714287</v>
+        <v>-0.0102537810817738</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18418,7 +18418,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ATO</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -18428,17 +18428,17 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>22.36</v>
+        <v>19.8</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.94</v>
+        <v>18.7</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.0635062611806797</v>
+        <v>-0.05555555555555563</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18448,7 +18448,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>IPH</t>
+          <t>EMEIS</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -18458,17 +18458,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>INNATE PHARMA</t>
+          <t>EMEIS</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>1.442</v>
+        <v>10.83</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.4</v>
+        <v>10.45</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02912621359223303</v>
+        <v>-0.03508771929824569</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18478,27 +18478,27 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>VANTI</t>
+          <t>ETL</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>VANTIVA</t>
+          <t>EUTELSAT COMMUNICATION</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.078</v>
+        <v>1.582</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.077</v>
+        <v>1.565</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>-0.01074589127686481</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18508,27 +18508,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>AB SCIENCE</t>
+          <t>CA PARIS IDF</t>
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>0.6840000000000001</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.592</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1345029239766083</v>
+        <v>-0.02685284640171859</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18538,27 +18538,27 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>BASS</t>
+          <t>ASY</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>BASSAC</t>
+          <t>ASSYSTEM</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="F25" s="12" t="n">
         <v>36.5</v>
       </c>
-      <c r="F25" s="12" t="n">
-        <v>39.5</v>
-      </c>
       <c r="G25" s="13" t="n">
-        <v>0.0821917808219178</v>
+        <v>-0.005449591280654028</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18643,7 +18643,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>ALHRS</t>
+          <t>ALDBT</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -18653,17 +18653,17 @@
       </c>
       <c r="D30" s="51" t="inlineStr">
         <is>
-          <t>HYDROGEN-REFUELING</t>
+          <t>DBT</t>
         </is>
       </c>
       <c r="E30" s="18" t="n">
-        <v>1.23</v>
+        <v>0.076</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>1.05</v>
+        <v>0.102</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1463414634146341</v>
+        <v>0.3421052631578947</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18672,7 +18672,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>ALSEM</t>
+          <t>ALHRS</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -18682,17 +18682,17 @@
       </c>
       <c r="D31" s="51" t="inlineStr">
         <is>
-          <t>SEMCO TECHNOLOGIES</t>
+          <t>HYDROGEN-REFUELING</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>47.45</v>
+        <v>1.064</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>48.25</v>
+        <v>0.963</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.01685985247629077</v>
+        <v>-0.09492481203007527</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18701,7 +18701,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>ALNTG</t>
+          <t>ALAMA</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -18711,17 +18711,17 @@
       </c>
       <c r="D32" s="51" t="inlineStr">
         <is>
-          <t>NETGEM</t>
+          <t>ALMA CORP</t>
         </is>
       </c>
       <c r="E32" s="18" t="n">
-        <v>0.98</v>
+        <v>0.167</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.986</v>
+        <v>0.155</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.006122448979591842</v>
+        <v>-0.07185628742514975</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18730,27 +18730,27 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>ALATI</t>
+          <t>ALSTI</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D33" s="51" t="inlineStr">
         <is>
-          <t>ACTIA GROUP</t>
+          <t>STIF</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>4.08</v>
+        <v>46.6</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.03</v>
+        <v>46.38</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01225490196078427</v>
+        <v>-0.00472103004291843</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18759,27 +18759,27 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>MEMS</t>
+          <t>ALICA</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D34" s="51" t="inlineStr">
         <is>
-          <t>MEMSCAP REPGT</t>
+          <t>ICAP HOLDING</t>
         </is>
       </c>
       <c r="E34" s="18" t="n">
-        <v>5.16</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>5.13</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.005813953488372141</v>
+        <v>0.04827586206896551</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18788,7 +18788,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ALPAS</t>
+          <t>ALESE</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -18798,17 +18798,17 @@
       </c>
       <c r="D35" s="51" t="inlineStr">
         <is>
-          <t>PASSAT</t>
+          <t>ENTECH</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>5</v>
+        <v>10.44</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.82</v>
+        <v>10</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.03599999999999994</v>
+        <v>-0.04214559386973175</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18817,27 +18817,27 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>ALSOG</t>
+          <t>ALATI</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D36" s="51" t="inlineStr">
         <is>
-          <t>SOGECLAIR</t>
+          <t>ACTIA GROUP</t>
         </is>
       </c>
       <c r="E36" s="18" t="n">
-        <v>31.4</v>
+        <v>4.03</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>31</v>
+        <v>3.99</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.01273885350318467</v>
+        <v>-0.009925558312655096</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18846,27 +18846,27 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>DEEZR</t>
+          <t>ALCWE</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D37" s="51" t="inlineStr">
         <is>
-          <t>DEEZER</t>
+          <t>CHARWOOD ENERGY</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>1.3</v>
+        <v>3.36</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.245</v>
+        <v>3.34</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04230769230769226</v>
+        <v>-0.005952380952380958</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18875,27 +18875,27 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>ALNN6</t>
+          <t>FMONC</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D38" s="51" t="inlineStr">
         <is>
-          <t>ENENSYS TECHNO</t>
+          <t>FINANCIERE MONCEY</t>
         </is>
       </c>
       <c r="E38" s="18" t="n">
-        <v>1.25</v>
+        <v>120</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.215</v>
+        <v>119</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.02799999999999993</v>
+        <v>-0.008333333333333333</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18904,7 +18904,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>ALSMA</t>
+          <t>ALMCE</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -18914,17 +18914,17 @@
       </c>
       <c r="D39" s="51" t="inlineStr">
         <is>
-          <t>SMAIO</t>
+          <t>MON COURTIER ENERGIE</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>7.12</v>
+        <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>6.76</v>
+        <v>5.6</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05056179775280904</v>
+        <v>-0.0175438596491229</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19001,7 +19001,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>SOP</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -19011,17 +19011,17 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>SOPRA STERIA GROUP</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>165.3</v>
+        <v>225.5</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>164</v>
+        <v>226</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.007864488808227533</v>
+        <v>0.002217294900221729</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19030,7 +19030,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>PLNW</t>
+          <t>RUI</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
@@ -19040,17 +19040,17 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>PLANISWARE</t>
+          <t>RUBIS</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>24.2</v>
+        <v>35.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>24.05</v>
+        <v>34.84</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.006198347107437958</v>
+        <v>-0.01078932424758647</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19059,7 +19059,7 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>VAC</t>
+          <t>VIRP</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -19069,17 +19069,17 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>PIERRE &amp; VACANCES</t>
+          <t>VIRBAC</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
-        <v>1.86</v>
+        <v>311.5</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.868</v>
+        <v>309</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.004301075268817208</v>
+        <v>-0.008025682182985553</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19088,7 +19088,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>SOI</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
@@ -19098,17 +19098,17 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>GETLINK SE</t>
+          <t xml:space="preserve">SOITEC </t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>18.83</v>
+        <v>155.95</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.47</v>
+        <v>155.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.0191184280403611</v>
+        <v>-0.005450464892593744</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19117,27 +19117,27 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>DKUPL</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>JCDECAUX</t>
+          <t>DEKUPLE</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>24.96</v>
+        <v>24.9</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.68</v>
+        <v>24.2</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01121794871794876</v>
+        <v>-0.02811244979919676</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19146,7 +19146,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>STMPA</t>
+          <t>BAIN</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -19156,17 +19156,17 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>STMICROELECTRONICS</t>
+          <t>BAINS MER MONACO</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>45.105</v>
+        <v>144</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>46.97</v>
+        <v>142</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.04134796585744379</v>
+        <v>-0.01388888888888889</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19175,7 +19175,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>PUB</t>
+          <t>ABCA</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -19185,17 +19185,17 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>PUBLICIS GRP</t>
+          <t>ABC ARBITRAGE</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>97.86</v>
+        <v>5.91</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>94.64</v>
+        <v>5.83</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.0329041487839771</v>
+        <v>-0.01353637901861253</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19204,27 +19204,27 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>VMX</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>VERIMATRIX</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
-        <v>110.8</v>
+        <v>0.314</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>107.6</v>
+        <v>0.314</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02888086642599281</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19233,7 +19233,7 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>EXENS</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -19243,17 +19243,17 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>EXOSENS</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>62.3</v>
+        <v>6.895</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>59.95</v>
+        <v>6.73</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.03772070626003202</v>
+        <v>-0.02393038433647559</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>BIM</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
@@ -19272,17 +19272,17 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>BIOMERIEUX</t>
+          <t>AIR LIQUIDE</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>77.7</v>
+        <v>170.88</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>78.34999999999999</v>
+        <v>169.52</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.008365508365508256</v>
+        <v>-0.007958801498127254</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -19363,7 +19363,9 @@
       <c r="D56" s="36" t="n"/>
       <c r="E56" s="18" t="n"/>
       <c r="F56" s="12" t="n"/>
-      <c r="G56" s="37" t="n"/>
+      <c r="G56" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H56" s="6" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" thickBot="1">
@@ -19375,7 +19377,9 @@
       <c r="D57" s="36" t="n"/>
       <c r="E57" s="18" t="n"/>
       <c r="F57" s="12" t="n"/>
-      <c r="G57" s="37" t="n"/>
+      <c r="G57" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H57" s="6" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" thickBot="1">
@@ -19387,7 +19391,9 @@
       <c r="D58" s="36" t="n"/>
       <c r="E58" s="18" t="n"/>
       <c r="F58" s="12" t="n"/>
-      <c r="G58" s="37" t="n"/>
+      <c r="G58" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H58" s="6" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" thickBot="1">
@@ -19399,7 +19405,9 @@
       <c r="D59" s="36" t="n"/>
       <c r="E59" s="18" t="n"/>
       <c r="F59" s="12" t="n"/>
-      <c r="G59" s="37" t="n"/>
+      <c r="G59" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H59" s="6" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" thickBot="1">
@@ -19411,7 +19419,9 @@
       <c r="D60" s="36" t="n"/>
       <c r="E60" s="18" t="n"/>
       <c r="F60" s="12" t="n"/>
-      <c r="G60" s="37" t="n"/>
+      <c r="G60" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H60" s="6" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" thickBot="1">
@@ -19423,7 +19433,9 @@
       <c r="D61" s="36" t="n"/>
       <c r="E61" s="18" t="n"/>
       <c r="F61" s="12" t="n"/>
-      <c r="G61" s="37" t="n"/>
+      <c r="G61" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H61" s="6" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" thickBot="1">
@@ -19435,7 +19447,9 @@
       <c r="D62" s="36" t="n"/>
       <c r="E62" s="18" t="n"/>
       <c r="F62" s="12" t="n"/>
-      <c r="G62" s="37" t="n"/>
+      <c r="G62" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H62" s="6" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" thickBot="1">
@@ -19447,7 +19461,9 @@
       <c r="D63" s="36" t="n"/>
       <c r="E63" s="18" t="n"/>
       <c r="F63" s="12" t="n"/>
-      <c r="G63" s="37" t="n"/>
+      <c r="G63" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H63" s="6" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" thickBot="1">
@@ -19459,7 +19475,9 @@
       <c r="D64" s="36" t="n"/>
       <c r="E64" s="18" t="n"/>
       <c r="F64" s="12" t="n"/>
-      <c r="G64" s="37" t="n"/>
+      <c r="G64" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H64" s="6" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" thickBot="1">
@@ -19471,7 +19489,9 @@
       <c r="D65" s="36" t="n"/>
       <c r="E65" s="18" t="n"/>
       <c r="F65" s="12" t="n"/>
-      <c r="G65" s="37" t="n"/>
+      <c r="G65" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H65" s="6" t="n"/>
     </row>
     <row r="66" ht="15.45" customHeight="1">
@@ -19552,7 +19572,9 @@
       <c r="D69" s="36" t="n"/>
       <c r="E69" s="18" t="n"/>
       <c r="F69" s="12" t="n"/>
-      <c r="G69" s="37" t="n"/>
+      <c r="G69" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H69" s="6" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" thickBot="1">
@@ -19564,7 +19586,9 @@
       <c r="D70" s="36" t="n"/>
       <c r="E70" s="18" t="n"/>
       <c r="F70" s="12" t="n"/>
-      <c r="G70" s="37" t="n"/>
+      <c r="G70" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H70" s="6" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" thickBot="1">
@@ -19576,7 +19600,9 @@
       <c r="D71" s="36" t="n"/>
       <c r="E71" s="18" t="n"/>
       <c r="F71" s="12" t="n"/>
-      <c r="G71" s="37" t="n"/>
+      <c r="G71" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H71" s="6" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" thickBot="1">
@@ -19588,7 +19614,9 @@
       <c r="D72" s="36" t="n"/>
       <c r="E72" s="18" t="n"/>
       <c r="F72" s="12" t="n"/>
-      <c r="G72" s="37" t="n"/>
+      <c r="G72" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H72" s="6" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" thickBot="1">
@@ -19600,7 +19628,9 @@
       <c r="D73" s="36" t="n"/>
       <c r="E73" s="18" t="n"/>
       <c r="F73" s="12" t="n"/>
-      <c r="G73" s="37" t="n"/>
+      <c r="G73" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H73" s="6" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" thickBot="1">
@@ -19612,7 +19642,9 @@
       <c r="D74" s="36" t="n"/>
       <c r="E74" s="18" t="n"/>
       <c r="F74" s="12" t="n"/>
-      <c r="G74" s="37" t="n"/>
+      <c r="G74" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H74" s="6" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" thickBot="1">
@@ -19624,7 +19656,9 @@
       <c r="D75" s="36" t="n"/>
       <c r="E75" s="18" t="n"/>
       <c r="F75" s="12" t="n"/>
-      <c r="G75" s="37" t="n"/>
+      <c r="G75" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H75" s="6" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" thickBot="1">
@@ -19636,7 +19670,9 @@
       <c r="D76" s="36" t="n"/>
       <c r="E76" s="18" t="n"/>
       <c r="F76" s="12" t="n"/>
-      <c r="G76" s="37" t="n"/>
+      <c r="G76" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H76" s="6" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" thickBot="1">
@@ -19648,7 +19684,9 @@
       <c r="D77" s="36" t="n"/>
       <c r="E77" s="18" t="n"/>
       <c r="F77" s="12" t="n"/>
-      <c r="G77" s="37" t="n"/>
+      <c r="G77" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H77" s="6" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" thickBot="1">
@@ -19660,7 +19698,9 @@
       <c r="D78" s="36" t="n"/>
       <c r="E78" s="18" t="n"/>
       <c r="F78" s="12" t="n"/>
-      <c r="G78" s="37" t="n"/>
+      <c r="G78" s="37" t="n">
+        <v>0</v>
+      </c>
       <c r="H78" s="6" t="n"/>
     </row>
     <row r="79" ht="15.45" customHeight="1">
@@ -19718,7 +19758,7 @@
         </is>
       </c>
       <c r="H81" s="49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" thickBot="1">
@@ -20462,7 +20502,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="52" t="n">
-        <v>46276</v>
+        <v>46335</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -20501,7 +20541,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>30/09/2026 19:05</t>
+          <t>01/10/2026 15:08</t>
         </is>
       </c>
     </row>
@@ -20528,10 +20568,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.3</v>
+        <v>0.314</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1452991452991453</v>
+        <v>-0.1054131054131053</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20558,10 +20598,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.63</v>
+        <v>16.8</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1153588195841716</v>
+        <v>0.1267605633802817</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20588,10 +20628,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>75.59</v>
+        <v>74.67</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.04037069950488756</v>
+        <v>-0.05205027294655318</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20618,10 +20658,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.007142857142857143</v>
+        <v>0.01428571428571429</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20648,10 +20688,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.4</v>
+        <v>125.05</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.008038585209003215</v>
+        <v>0.005225080385852021</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20678,10 +20718,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.2</v>
+        <v>54.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1410526315789474</v>
+        <v>0.1452631578947368</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20708,10 +20748,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.14</v>
+        <v>34.84</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02280311457174639</v>
+        <v>-0.03114571746384865</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20738,10 +20778,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>216</v>
+        <v>208.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0009250693802034627</v>
+        <v>-0.03422756706752996</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20798,10 +20838,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.09090909090909094</v>
+        <v>-0.1086474501108647</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20817,7 +20857,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.01697281143519945</v>
+        <v>-0.02980891507715736</v>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
@@ -20930,10 +20970,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.44</v>
+        <v>3.49</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.05846153846153845</v>
+        <v>0.07384615384615391</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20960,10 +21000,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.826</v>
+        <v>4.612</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.1715021459227469</v>
+        <v>-0.2082403433476395</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20990,10 +21030,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.484</v>
+        <v>2.262</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3190789473684211</v>
+        <v>-0.3799342105263158</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21020,10 +21060,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.95</v>
+        <v>6.74</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.06711409395973154</v>
+        <v>-0.09530201342281878</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21050,10 +21090,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>20.94</v>
+        <v>22.58</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1563255439161966</v>
+        <v>-0.09024979854955689</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21080,10 +21120,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>75.26000000000001</v>
+        <v>75.56</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.06449787835926453</v>
+        <v>0.06874115983026872</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21110,10 +21150,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.29</v>
+        <v>7.23</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.08875</v>
+        <v>-0.09624999999999995</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21140,10 +21180,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.61</v>
+        <v>7.56</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.06511056511056514</v>
+        <v>-0.07125307125307137</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21170,10 +21210,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>24.08</v>
+        <v>23.08</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.1066176470588234</v>
+        <v>0.0606617647058822</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21189,7 +21229,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.05339032762494453</v>
+        <v>-0.07229153257140972</v>
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
@@ -21275,10 +21315,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.671</v>
+        <v>5.768</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.099031007751938</v>
+        <v>0.117829457364341</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21304,10 +21344,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.075</v>
+        <v>0.102</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.08536585365853666</v>
+        <v>0.2439024390243901</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21333,10 +21373,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.8</v>
+        <v>4.66</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.180887372013652</v>
+        <v>-0.2047781569965871</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21362,10 +21402,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.986</v>
+        <v>0.994</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.06540284360189569</v>
+        <v>-0.05781990521327009</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21391,10 +21431,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.31</v>
+        <v>9.27</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08255813953488382</v>
+        <v>0.07790697674418604</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21449,10 +21489,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.243</v>
+        <v>0.249</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1321428571428573</v>
+        <v>-0.1107142857142858</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21478,10 +21518,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.215</v>
+        <v>1.245</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.05078124999999996</v>
+        <v>-0.02734374999999994</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21507,10 +21547,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1875</v>
+        <v>-0.1249999999999999</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21536,10 +21576,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.85</v>
+        <v>19.4</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.02267002518891702</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21553,7 +21593,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.03201169390599398</v>
+        <v>-0.02368454312373558</v>
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
@@ -21633,10 +21673,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.87</v>
+        <v>6.73</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.09832134292565951</v>
+        <v>0.0759392486011192</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21662,10 +21702,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.282</v>
+        <v>5.328</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.01187739463601538</v>
+        <v>0.0206896551724139</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21720,10 +21760,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.5</v>
+        <v>20.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.09090909090909094</v>
+        <v>-0.1086474501108647</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21749,10 +21789,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>20.35</v>
+        <v>19.98</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.05787037037037036</v>
+        <v>-0.07500000000000004</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21778,10 +21818,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.75</v>
+        <v>3.484</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.06390414378432356</v>
+        <v>-0.1303045431852222</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21807,10 +21847,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>87.45</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.03263274336283189</v>
+        <v>-0.06360619469026549</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21836,10 +21876,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.583</v>
+        <v>1.565</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1548318206086493</v>
+        <v>-0.1644420715429792</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21911,7 +21951,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>-0.01450246300213581</v>
+        <v>-0.02759156780805985</v>
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-01 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17886,7 +17886,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>01/10/2026 15:08</t>
+          <t>01/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -17913,10 +17913,10 @@
         <v>155.95</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>155.1</v>
+        <v>160.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.005450464892593744</v>
+        <v>0.02661109329913438</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17943,10 +17943,10 @@
         <v>82</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>83.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01829268292682927</v>
+        <v>-0.004878048780487874</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17973,10 +17973,10 @@
         <v>0.314</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.314</v>
+        <v>0.313</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0</v>
+        <v>-0.003184713375796181</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18003,10 +18003,10 @@
         <v>6.895</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.73</v>
+        <v>6.77</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02393038433647559</v>
+        <v>-0.01812907904278463</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18033,10 +18033,10 @@
         <v>14.02</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>13.92</v>
+        <v>13.88</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.007132667617688991</v>
+        <v>-0.009985734664764536</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18063,10 +18063,10 @@
         <v>5.91</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>5.83</v>
+        <v>5.81</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01353637901861253</v>
+        <v>-0.01692047377326574</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18123,10 +18123,10 @@
         <v>43.88</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>43.22</v>
+        <v>42.2</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01504102096627173</v>
+        <v>-0.03828623518687328</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18285,10 +18285,10 @@
         <v>2.47</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.262</v>
+        <v>2.25</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.08421052631578954</v>
+        <v>-0.08906882591093125</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18315,10 +18315,10 @@
         <v>0.099</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.091</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.08080808080808087</v>
+        <v>-0.1111111111111112</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18345,10 +18345,10 @@
         <v>24.1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>23.08</v>
+        <v>23.22</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.04232365145228228</v>
+        <v>-0.03651452282157687</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18375,10 +18375,10 @@
         <v>4.816</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.612</v>
+        <v>4.462</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.04235880398671091</v>
+        <v>-0.07350498338870434</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18405,10 +18405,10 @@
         <v>3.901</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.861</v>
+        <v>3.849</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.0102537810817738</v>
+        <v>-0.01332991540630597</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18435,10 +18435,10 @@
         <v>19.8</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>18.7</v>
+        <v>18.06</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.05555555555555563</v>
+        <v>-0.08787878787878797</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18465,10 +18465,10 @@
         <v>10.83</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.45</v>
+        <v>10.39</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.03508771929824569</v>
+        <v>-0.04062788550323172</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18495,10 +18495,10 @@
         <v>1.582</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>1.565</v>
+        <v>1.545</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01074589127686481</v>
+        <v>-0.02338811630847038</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18525,10 +18525,10 @@
         <v>93.09999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>90.59999999999999</v>
+        <v>90.12</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.02685284640171859</v>
+        <v>-0.03200859291084844</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18555,10 +18555,10 @@
         <v>36.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.005449591280654028</v>
+        <v>-0.008174386920981042</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18660,10 +18660,10 @@
         <v>0.076</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.102</v>
+        <v>0.097</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.3421052631578947</v>
+        <v>0.2763157894736843</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18689,10 +18689,10 @@
         <v>1.064</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.963</v>
+        <v>0.96</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.09492481203007527</v>
+        <v>-0.09774436090225572</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18747,10 +18747,10 @@
         <v>46.6</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>46.38</v>
+        <v>45.62</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.00472103004291843</v>
+        <v>-0.02103004291845502</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18776,10 +18776,10 @@
         <v>8.699999999999999</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.119999999999999</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.04827586206896551</v>
+        <v>0.05977011494252889</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18805,10 +18805,10 @@
         <v>10.44</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>10</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04214559386973175</v>
+        <v>-0.04597701149425275</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18834,10 +18834,10 @@
         <v>4.03</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>3.99</v>
+        <v>3.88</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.009925558312655096</v>
+        <v>-0.03722084367245666</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18863,10 +18863,10 @@
         <v>3.36</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.34</v>
+        <v>3.48</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.005952380952380958</v>
+        <v>0.03571428571428575</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18892,10 +18892,10 @@
         <v>120</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>119</v>
+        <v>118.5</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.008333333333333333</v>
+        <v>-0.0125</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19047,10 +19047,10 @@
         <v>35.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>34.84</v>
+        <v>34.96</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01078932424758647</v>
+        <v>-0.00738216922203288</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19076,10 +19076,10 @@
         <v>311.5</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>309</v>
+        <v>306.5</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.008025682182985553</v>
+        <v>-0.01605136436597111</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19105,10 +19105,10 @@
         <v>155.95</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>155.1</v>
+        <v>160.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.005450464892593744</v>
+        <v>0.02661109329913438</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19192,10 +19192,10 @@
         <v>5.91</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>5.83</v>
+        <v>5.81</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01353637901861253</v>
+        <v>-0.01692047377326574</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19221,10 +19221,10 @@
         <v>0.314</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>0.314</v>
+        <v>0.313</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>-0.003184713375796181</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19250,10 +19250,10 @@
         <v>6.895</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>6.73</v>
+        <v>6.77</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02393038433647559</v>
+        <v>-0.01812907904278463</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19279,10 +19279,10 @@
         <v>170.88</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>169.52</v>
+        <v>167.2</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.007958801498127254</v>
+        <v>-0.02153558052434461</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -20541,7 +20541,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>01/10/2026 15:08</t>
+          <t>01/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20568,10 +20568,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.314</v>
+        <v>0.313</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1054131054131053</v>
+        <v>-0.1082621082621082</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20598,10 +20598,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.8</v>
+        <v>16.6</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1267605633802817</v>
+        <v>0.1133467471495641</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20628,10 +20628,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.67</v>
+        <v>74.75</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05205027294655318</v>
+        <v>-0.05103465786466924</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20688,10 +20688,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.05</v>
+        <v>125.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.005225080385852021</v>
+        <v>0.008038585209003215</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20718,10 +20718,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.4</v>
+        <v>54</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1452631578947368</v>
+        <v>0.1368421052631579</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20748,10 +20748,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.84</v>
+        <v>34.96</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.03114571746384865</v>
+        <v>-0.02780867630700778</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20778,10 +20778,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>208.8</v>
+        <v>210.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03422756706752996</v>
+        <v>-0.0259019426456984</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20838,10 +20838,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.1</v>
+        <v>19.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.1086474501108647</v>
+        <v>-0.1219512195121951</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20940,10 +20940,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.065</v>
+        <v>0.063</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.09722222222222213</v>
+        <v>-0.1249999999999999</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20970,10 +20970,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.49</v>
+        <v>3.46</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07384615384615391</v>
+        <v>0.0646153846153846</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21000,10 +21000,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.612</v>
+        <v>4.462</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.2082403433476395</v>
+        <v>-0.2339914163090129</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21030,10 +21030,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.262</v>
+        <v>2.25</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3799342105263158</v>
+        <v>-0.3832236842105263</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21060,10 +21060,10 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.74</v>
+        <v>6.7</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.09530201342281878</v>
+        <v>-0.1006711409395973</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21090,10 +21090,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.58</v>
+        <v>22</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.09024979854955689</v>
+        <v>-0.1136180499597099</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21120,10 +21120,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>75.56</v>
+        <v>74.72</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.06874115983026872</v>
+        <v>0.0568599717114568</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21150,10 +21150,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.23</v>
+        <v>7.15</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.09624999999999995</v>
+        <v>-0.10625</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21180,10 +21180,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.56</v>
+        <v>7.4</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.07125307125307137</v>
+        <v>-0.09090909090909093</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21210,10 +21210,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.08</v>
+        <v>23.22</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0606617647058822</v>
+        <v>0.06709558823529399</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21315,10 +21315,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.768</v>
+        <v>5.735</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.117829457364341</v>
+        <v>0.1114341085271318</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21344,10 +21344,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.102</v>
+        <v>0.097</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.2439024390243901</v>
+        <v>0.1829268292682927</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21373,10 +21373,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.66</v>
+        <v>4.6</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2047781569965871</v>
+        <v>-0.2150170648464165</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21402,10 +21402,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.994</v>
+        <v>0.998</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05781990521327009</v>
+        <v>-0.05402843601895729</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21489,10 +21489,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.249</v>
+        <v>0.243</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1107142857142858</v>
+        <v>-0.1321428571428573</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21547,10 +21547,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.14</v>
+        <v>0.136</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21576,10 +21576,10 @@
         <v>19.85</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.4</v>
+        <v>19.45</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.02267002518891702</v>
+        <v>-0.02015113350125955</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21673,10 +21673,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.73</v>
+        <v>6.77</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0759392486011192</v>
+        <v>0.08233413269384487</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21702,10 +21702,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.328</v>
+        <v>5.122</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.0206896551724139</v>
+        <v>-0.01877394636015323</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21760,10 +21760,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.1</v>
+        <v>19.8</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1086474501108647</v>
+        <v>-0.1219512195121951</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21789,10 +21789,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.98</v>
+        <v>19.8</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.07500000000000004</v>
+        <v>-0.08333333333333336</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21818,10 +21818,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.484</v>
+        <v>3.418</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1303045431852222</v>
+        <v>-0.1467798302546181</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21847,10 +21847,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>84.65000000000001</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.06360619469026549</v>
+        <v>-0.04756637168141605</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21876,10 +21876,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.565</v>
+        <v>1.545</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1644420715429792</v>
+        <v>-0.1751201281366792</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 10:09
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1886" yWindow="1886" windowWidth="24685" windowHeight="13054" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Donnees" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="000000"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -332,10 +333,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -463,14 +464,1473 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
     <cellStyle name="Normal 4" xfId="2"/>
   </cellStyles>
-  <dxfs count="178">
+  <dxfs count="356">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -17844,10 +19304,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="53" t="inlineStr">
-        <is>
-          <t>30/09/2026</t>
-        </is>
+      <c r="A1" s="54" t="n">
+        <v>46296</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -17886,7 +19344,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>01/10/2026 19:05</t>
+          <t>02/10/2026 10:09</t>
         </is>
       </c>
     </row>
@@ -17910,13 +19368,13 @@
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>155.95</v>
+        <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>160.1</v>
+        <v>164.1</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.02661109329913438</v>
+        <v>0.03500473036896867</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17926,7 +19384,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>ATE</t>
+          <t>STMPA</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -17936,17 +19394,17 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>ALTEN</t>
+          <t>STMICROELECTRONICS</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>82</v>
+        <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>81.59999999999999</v>
+        <v>48.26</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.004878048780487874</v>
+        <v>0.02137566137566133</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17956,27 +19414,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>VMX</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>VERIMATRIX</t>
+          <t>JCDECAUX</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>0.314</v>
+        <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.313</v>
+        <v>24.82</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.003184713375796181</v>
+        <v>0.005672609400324173</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -17986,7 +19444,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>SAVE</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -17996,17 +19454,17 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>X-FAB SILICON</t>
+          <t>SAVENCIA</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>6.895</v>
+        <v>59.2</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.77</v>
+        <v>57.4</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01812907904278463</v>
+        <v>-0.03040540540540548</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18016,7 +19474,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>QDT</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -18026,17 +19484,17 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>QUADIENT</t>
+          <t>CAP GEMINI</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>14.02</v>
+        <v>112.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>13.88</v>
+        <v>113.85</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.009985734664764536</v>
+        <v>0.01561106155218555</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18046,7 +19504,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>ABCA</t>
+          <t>PLNW</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -18056,17 +19514,17 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>ABC ARBITRAGE</t>
+          <t>PLANISWARE</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>5.91</v>
+        <v>24.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>5.81</v>
+        <v>24.55</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01692047377326574</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18076,7 +19534,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -18086,17 +19544,17 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>144</v>
+        <v>226</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>142</v>
+        <v>228.5</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01388888888888889</v>
+        <v>0.01106194690265487</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18106,7 +19564,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>RCO</t>
+          <t>SOP</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -18116,17 +19574,17 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>REMY COINTREAU</t>
+          <t>SOPRA STERIA GROUP</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>43.88</v>
+        <v>165.8</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>42.2</v>
+        <v>166.9</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03828623518687328</v>
+        <v>0.006634499396863657</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18136,27 +19594,27 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>225.5</v>
+        <v>34.8</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>226</v>
+        <v>34.8</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.002217294900221729</v>
+        <v>0</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18166,7 +19624,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>FNAC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -18176,14 +19634,14 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>FNAC DARTY</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>34.8</v>
+        <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.8</v>
+        <v>34.5</v>
       </c>
       <c r="G11" s="13" t="n">
         <v>0</v>
@@ -18282,13 +19740,13 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>2.47</v>
+        <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.25</v>
+        <v>2.248</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.08906882591093125</v>
+        <v>-0.000888888888888791</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18298,27 +19756,27 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>SIGHT</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>GENSIGHT BIOLO</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>0.099</v>
+        <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.08799999999999999</v>
+        <v>18.02</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1111111111111112</v>
+        <v>-0.002214839424141703</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18328,7 +19786,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>MEDCL</t>
+          <t>NXI</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -18338,17 +19796,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>MEDINCELL</t>
+          <t>NEXITY</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>24.1</v>
+        <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>23.22</v>
+        <v>4.502</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.03651452282157687</v>
+        <v>0.001780151312861595</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18358,7 +19816,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>NXI</t>
+          <t>MEDCL</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -18368,17 +19826,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>NEXITY</t>
+          <t>MEDINCELL</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>4.816</v>
+        <v>23.18</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.462</v>
+        <v>22.8</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.07350498338870434</v>
+        <v>-0.01639344262295078</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18388,7 +19846,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>STLAP</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -18398,17 +19856,17 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>STELLANTIS</t>
+          <t>AB SCIENCE</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>3.901</v>
+        <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.849</v>
+        <v>0.583</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01332991540630597</v>
+        <v>0.001718213058419246</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18418,27 +19876,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>FDE</t>
+          <t>WLN</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>FRANCAISE ENER</t>
+          <t>WORLDLINE</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>19.8</v>
+        <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>18.06</v>
+        <v>10.742</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.08787878787878797</v>
+        <v>0.002052238805970172</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18448,7 +19906,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>EMEIS</t>
+          <t>OR</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -18458,17 +19916,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>EMEIS</t>
+          <t>L'OREAL</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>10.83</v>
+        <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.39</v>
+        <v>373.85</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.04062788550323172</v>
+        <v>0.005648957632817815</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18478,7 +19936,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -18488,17 +19946,17 @@
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>EUTELSAT COMMUNICATION</t>
+          <t>SOLUTIONS 30</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>1.582</v>
+        <v>0.467</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>1.545</v>
+        <v>0.461</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.02338811630847038</v>
+        <v>-0.01284796573875804</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18508,27 +19966,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>CAF</t>
+          <t>CLARI</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>CA PARIS IDF</t>
+          <t>CLARIANE</t>
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>93.09999999999999</v>
+        <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>90.12</v>
+        <v>3.348</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.03200859291084844</v>
+        <v>-0.01760563380281692</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18538,7 +19996,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ASY</t>
+          <t>EMEIS</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -18548,17 +20006,17 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>ASSYSTEM</t>
+          <t>EMEIS</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>36.7</v>
+        <v>10.32</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>36.4</v>
+        <v>10.16</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.008174386920981042</v>
+        <v>-0.01550387596899226</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18657,13 +20115,13 @@
         </is>
       </c>
       <c r="E30" s="18" t="n">
-        <v>0.076</v>
+        <v>0.094</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.2763157894736843</v>
+        <v>0.1170212765957446</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18672,7 +20130,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>ALHRS</t>
+          <t>ALWIT</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -18682,17 +20140,17 @@
       </c>
       <c r="D31" s="51" t="inlineStr">
         <is>
-          <t>HYDROGEN-REFUELING</t>
+          <t>WITBE</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>1.064</v>
+        <v>4.5</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.96</v>
+        <v>4.4</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.09774436090225572</v>
+        <v>-0.02222222222222214</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18701,7 +20159,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>ALAMA</t>
+          <t>ALSEM</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -18711,17 +20169,17 @@
       </c>
       <c r="D32" s="51" t="inlineStr">
         <is>
-          <t>ALMA CORP</t>
+          <t>SEMCO TECHNOLOGIES</t>
         </is>
       </c>
       <c r="E32" s="18" t="n">
-        <v>0.167</v>
+        <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.155</v>
+        <v>49.3</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.07185628742514975</v>
+        <v>0.00817995910020447</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18730,7 +20188,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>ALSTI</t>
+          <t>ALICA</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -18740,17 +20198,17 @@
       </c>
       <c r="D33" s="51" t="inlineStr">
         <is>
-          <t>STIF</t>
+          <t>ICAP HOLDING</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>46.6</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>45.62</v>
+        <v>9.24</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02103004291845502</v>
+        <v>-0.004310344827586115</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18759,7 +20217,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>ALICA</t>
+          <t>ALIMP</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -18769,17 +20227,17 @@
       </c>
       <c r="D34" s="51" t="inlineStr">
         <is>
-          <t>ICAP HOLDING</t>
+          <t>IMPLANET</t>
         </is>
       </c>
       <c r="E34" s="18" t="n">
-        <v>8.699999999999999</v>
+        <v>0.162</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.220000000000001</v>
+        <v>0.158</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.05977011494252889</v>
+        <v>-0.02469135802469138</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18788,7 +20246,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ALESE</t>
+          <t>ALCWE</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -18798,17 +20256,17 @@
       </c>
       <c r="D35" s="51" t="inlineStr">
         <is>
-          <t>ENTECH</t>
+          <t>CHARWOOD ENERGY</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>10.44</v>
+        <v>3.48</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.960000000000001</v>
+        <v>3.47</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04597701149425275</v>
+        <v>-0.002873563218390743</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18817,27 +20275,27 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>ALATI</t>
+          <t>ALNTG</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D36" s="51" t="inlineStr">
         <is>
-          <t>ACTIA GROUP</t>
+          <t>NETGEM</t>
         </is>
       </c>
       <c r="E36" s="18" t="n">
-        <v>4.03</v>
+        <v>0.998</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>3.88</v>
+        <v>1.005</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03722084367245666</v>
+        <v>0.00701402805611212</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18846,27 +20304,27 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>ALCWE</t>
+          <t>FMONC</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D37" s="51" t="inlineStr">
         <is>
-          <t>CHARWOOD ENERGY</t>
+          <t>FINANCIERE MONCEY</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>3.36</v>
+        <v>122</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.48</v>
+        <v>121</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.03571428571428575</v>
+        <v>-0.00819672131147541</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18875,27 +20333,27 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>FMONC</t>
+          <t>ALNLF</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D38" s="51" t="inlineStr">
         <is>
-          <t>FINANCIERE MONCEY</t>
+          <t>NEOLIFE</t>
         </is>
       </c>
       <c r="E38" s="18" t="n">
-        <v>120</v>
+        <v>0.062</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>118.5</v>
+        <v>0.062</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.0125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -18904,7 +20362,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>ALMCE</t>
+          <t>ALECO</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -18914,17 +20372,17 @@
       </c>
       <c r="D39" s="51" t="inlineStr">
         <is>
-          <t>MON COURTIER ENERGIE</t>
+          <t>ECOMIAM</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>5.7</v>
+        <v>2.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.6</v>
+        <v>2.12</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.0175438596491229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19001,7 +20459,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>STMPA</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -19011,17 +20469,17 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>STMICROELECTRONICS</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>225.5</v>
+        <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>226</v>
+        <v>48.26</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.002217294900221729</v>
+        <v>0.02137566137566133</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19030,27 +20488,27 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>RUI</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>RUBIS</t>
+          <t>FREY</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>35.22</v>
+        <v>34.8</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>34.96</v>
+        <v>34.8</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.00738216922203288</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19059,7 +20517,7 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>VIRP</t>
+          <t>PLNW</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -19069,17 +20527,17 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>VIRBAC</t>
+          <t>PLANISWARE</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
-        <v>311.5</v>
+        <v>24.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>306.5</v>
+        <v>24.55</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01605136436597111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19088,7 +20546,7 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>SOI</t>
+          <t>IPS</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
@@ -19098,17 +20556,17 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOITEC </t>
+          <t>IPSOS</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>155.95</v>
+        <v>35.46</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>160.1</v>
+        <v>35.34</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.02661109329913438</v>
+        <v>-0.003384094754653058</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19117,27 +20575,27 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>DKUPL</t>
+          <t>SOP</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>DEKUPLE</t>
+          <t>SOPRA STERIA GROUP</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>24.9</v>
+        <v>165.8</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.2</v>
+        <v>166.9</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.02811244979919676</v>
+        <v>0.006634499396863657</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19146,7 +20604,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>SOI</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -19156,17 +20614,17 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t xml:space="preserve">SOITEC </t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>144</v>
+        <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>142</v>
+        <v>164.1</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01388888888888889</v>
+        <v>0.03500473036896867</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19175,7 +20633,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>ABCA</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -19185,17 +20643,17 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>ABC ARBITRAGE</t>
+          <t>JCDECAUX</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>5.91</v>
+        <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>5.81</v>
+        <v>24.82</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.01692047377326574</v>
+        <v>0.005672609400324173</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19204,27 +20662,27 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>VMX</t>
+          <t>VAC</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>VERIMATRIX</t>
+          <t>PIERRE &amp; VACANCES</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
-        <v>0.314</v>
+        <v>1.87</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>0.313</v>
+        <v>1.87</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.003184713375796181</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19233,7 +20691,7 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -19243,17 +20701,17 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>X-FAB SILICON</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>6.895</v>
+        <v>226</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>6.77</v>
+        <v>228.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01812907904278463</v>
+        <v>0.01106194690265487</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19262,7 +20720,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>CAP</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
@@ -19272,17 +20730,17 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>AIR LIQUIDE</t>
+          <t>CAP GEMINI</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>170.88</v>
+        <v>112.1</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>167.2</v>
+        <v>113.85</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02153558052434461</v>
+        <v>0.01561106155218555</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -19475,8 +20933,8 @@
       <c r="D64" s="36" t="n"/>
       <c r="E64" s="18" t="n"/>
       <c r="F64" s="12" t="n"/>
-      <c r="G64" s="37" t="n">
-        <v>0</v>
+      <c r="G64" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -19489,8 +20947,8 @@
       <c r="D65" s="36" t="n"/>
       <c r="E65" s="18" t="n"/>
       <c r="F65" s="12" t="n"/>
-      <c r="G65" s="37" t="n">
-        <v>0</v>
+      <c r="G65" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H65" s="6" t="n"/>
     </row>
@@ -19698,8 +21156,8 @@
       <c r="D78" s="36" t="n"/>
       <c r="E78" s="18" t="n"/>
       <c r="F78" s="12" t="n"/>
-      <c r="G78" s="37" t="n">
-        <v>0</v>
+      <c r="G78" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -20206,275 +21664,275 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="36" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="0" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="35" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="34" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="34" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="33" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="32" dxfId="28" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="31" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="18" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="17" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="15" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="13" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="21" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="21" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="19">
       <formula>$H81</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F30:F39">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20541,7 +21999,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>01/10/2026 19:05</t>
+          <t>02/10/2026 10:09</t>
         </is>
       </c>
     </row>
@@ -20568,10 +22026,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.313</v>
+        <v>0.306</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1082621082621082</v>
+        <v>-0.1282051282051282</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20598,10 +22056,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.6</v>
+        <v>16.54</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1133467471495641</v>
+        <v>0.1093226022803487</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20628,10 +22086,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.75</v>
+        <v>74.3</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05103465786466924</v>
+        <v>-0.05674749270026658</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20658,10 +22116,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01428571428571429</v>
+        <v>0.02857142857142857</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20688,10 +22146,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.4</v>
+        <v>125.3</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.008038585209003215</v>
+        <v>0.007234726688102825</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20718,10 +22176,10 @@
         <v>47.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54</v>
+        <v>54.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1368421052631579</v>
+        <v>0.1410526315789474</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20748,10 +22206,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>34.96</v>
+        <v>35</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02780867630700778</v>
+        <v>-0.0266963292547275</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20778,10 +22236,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>210.6</v>
+        <v>209.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0259019426456984</v>
+        <v>-0.03052728954671598</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20838,10 +22296,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.8</v>
+        <v>20.05</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.1219512195121951</v>
+        <v>-0.1108647450110865</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20857,7 +22315,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.02980891507715736</v>
+        <v>-0.03977493163122617</v>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
@@ -20970,10 +22428,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.46</v>
+        <v>3.48</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.0646153846153846</v>
+        <v>0.07076923076923076</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21000,10 +22458,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.462</v>
+        <v>4.502</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.2339914163090129</v>
+        <v>-0.2271244635193134</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21030,10 +22488,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.25</v>
+        <v>2.248</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3832236842105263</v>
+        <v>-0.3837719298245614</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21090,10 +22548,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22</v>
+        <v>21.9</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1136180499597099</v>
+        <v>-0.1176470588235295</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21120,10 +22578,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>74.72</v>
+        <v>74.44</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.0568599717114568</v>
+        <v>0.05289957567185283</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21150,10 +22608,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.15</v>
+        <v>7.16</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.10625</v>
+        <v>-0.105</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21180,10 +22638,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.4</v>
+        <v>7.53</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.09090909090909093</v>
+        <v>-0.07493857493857498</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21210,10 +22668,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.22</v>
+        <v>22.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.06709558823529399</v>
+        <v>0.04779411764705878</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21229,7 +22687,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.07229153257140972</v>
+        <v>-0.09337206841239842</v>
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
@@ -21315,10 +22773,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.735</v>
+        <v>5.855</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1114341085271318</v>
+        <v>0.1346899224806202</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21344,10 +22802,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.097</v>
+        <v>0.105</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.1829268292682927</v>
+        <v>0.2804878048780487</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21373,10 +22831,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.6</v>
+        <v>4.645</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2150170648464165</v>
+        <v>-0.2073378839590445</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21402,10 +22860,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.998</v>
+        <v>1.005</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05402843601895729</v>
+        <v>-0.04739336492891</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21431,10 +22889,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.27</v>
+        <v>9.4</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.07790697674418604</v>
+        <v>0.09302325581395357</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21489,10 +22947,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.243</v>
+        <v>0.255</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1321428571428573</v>
+        <v>-0.08928571428571436</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21518,10 +22976,10 @@
         <v>1.28</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.245</v>
+        <v>1.22</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02734374999999994</v>
+        <v>-0.04687500000000004</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21547,10 +23005,10 @@
         <v>0.16</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.136</v>
+        <v>0.139</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.15</v>
+        <v>-0.13125</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21593,7 +23051,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.02368454312373558</v>
+        <v>-0.007487657864445452</v>
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
@@ -21673,10 +23131,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.77</v>
+        <v>6.9</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.08233413269384487</v>
+        <v>0.1031175059952039</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21702,10 +23160,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.122</v>
+        <v>5.1</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01877394636015323</v>
+        <v>-0.02298850574712646</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21734,7 +23192,7 @@
         <v>86.5</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.01169590643274854</v>
+        <v>0.01169590643274865</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -21760,10 +23218,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.8</v>
+        <v>20.05</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1219512195121951</v>
+        <v>-0.1108647450110865</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21818,10 +23276,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.418</v>
+        <v>3.348</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1467798302546181</v>
+        <v>-0.1642536195706441</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21847,10 +23305,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>86.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.04756637168141605</v>
+        <v>-0.06084070796460177</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21876,10 +23334,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.545</v>
+        <v>1.549</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1751201281366792</v>
+        <v>-0.1729845168179392</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21908,7 +23366,7 @@
         <v>34.8</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01136363636363652</v>
+        <v>-0.01136363636363658</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -21934,10 +23392,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>226</v>
+        <v>228.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01801801801801802</v>
+        <v>0.02927927927927928</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21951,7 +23409,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>-0.02759156780805985</v>
+        <v>-0.05141568298676826</v>
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>
@@ -22861,275 +24319,275 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="27" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="29" dxfId="28" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="28" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
+      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
       <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="60" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="60" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="61" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="61" dxfId="0" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="62" dxfId="0" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="63" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="63" dxfId="0" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
       <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="64" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="64" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="65" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="65" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="21" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="21" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="2">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
+    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="21" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="22">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="21" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
       <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="19">
       <formula>$H81</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 11:29
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Donnees" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,17 +16,16 @@
   <definedNames>
     <definedName name="cours">[1]Cours!$A$2:$H$3000</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="000000"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -333,10 +332,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -464,1473 +463,14 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
     <cellStyle name="Normal 4" xfId="2"/>
   </cellStyles>
-  <dxfs count="356">
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color rgb="FF006100"/>
-        <extend val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="12"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color indexed="18"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
+  <dxfs count="178">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -19304,7 +17844,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="54" t="n">
+      <c r="A1" s="53" t="n">
         <v>46296</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -19344,7 +17884,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 10:09</t>
+          <t>02/10/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -19371,10 +17911,10 @@
         <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>164.1</v>
+        <v>166.5</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.03500473036896867</v>
+        <v>0.04541154210028375</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -19401,10 +17941,10 @@
         <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.26</v>
+        <v>48.82</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.02137566137566133</v>
+        <v>0.0280423280423281</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -19431,10 +17971,10 @@
         <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.82</v>
+        <v>24.88</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.005672609400324173</v>
+        <v>0.01134521880064835</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -19461,10 +18001,10 @@
         <v>59.2</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>57.4</v>
+        <v>55.6</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.03040540540540548</v>
+        <v>-0.05743243243243253</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -19491,10 +18031,10 @@
         <v>112.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>113.85</v>
+        <v>113.65</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01561106155218555</v>
+        <v>0.01427297056199829</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -19521,10 +18061,10 @@
         <v>24.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>24.55</v>
+        <v>24.7</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.002036659877800436</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -19551,10 +18091,10 @@
         <v>226</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>228.5</v>
+        <v>225</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.01106194690265487</v>
+        <v>0.008849557522123894</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -19581,7 +18121,7 @@
         <v>165.8</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>166.9</v>
+        <v>167</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -19743,10 +18283,10 @@
         <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.248</v>
+        <v>2.208</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.000888888888888791</v>
+        <v>-0.01155555555555547</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19773,10 +18313,10 @@
         <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>18.02</v>
+        <v>17.88</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.002214839424141703</v>
+        <v>-0.01771871539313401</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19803,10 +18343,10 @@
         <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.502</v>
+        <v>4.524</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.001780151312861595</v>
+        <v>0.008010680907877276</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19833,10 +18373,10 @@
         <v>23.18</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.8</v>
+        <v>22.84</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01639344262295078</v>
+        <v>-0.01466781708369283</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19863,10 +18403,10 @@
         <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.583</v>
+        <v>0.578</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.001718213058419246</v>
+        <v>-0.001718213058419246</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19893,10 +18433,10 @@
         <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.742</v>
+        <v>10.766</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.002052238805970172</v>
+        <v>0.007462686567164185</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19923,10 +18463,10 @@
         <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>373.85</v>
+        <v>374.75</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.005648957632817815</v>
+        <v>0.01116341627437788</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19953,10 +18493,10 @@
         <v>0.467</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.461</v>
+        <v>0.467</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01284796573875804</v>
+        <v>-0.008565310492505361</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19983,10 +18523,10 @@
         <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.348</v>
+        <v>3.318</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01760563380281692</v>
+        <v>-0.02464788732394368</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20013,10 +18553,10 @@
         <v>10.32</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>10.16</v>
+        <v>10.13</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.01550387596899226</v>
+        <v>-0.01841085271317825</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20118,10 +18658,10 @@
         <v>0.094</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.105</v>
+        <v>0.097</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1170212765957446</v>
+        <v>0.04255319148936174</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20147,10 +18687,10 @@
         <v>4.5</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.4</v>
+        <v>4.28</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02222222222222214</v>
+        <v>-0.03777777777777776</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20176,10 +18716,10 @@
         <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>49.3</v>
+        <v>51.5</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.00817995910020447</v>
+        <v>0.01226993865030678</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20205,10 +18745,10 @@
         <v>9.279999999999999</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>9.24</v>
+        <v>9.4</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.004310344827586115</v>
+        <v>0.01077586206896567</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20295,7 +18835,7 @@
         <v>1.005</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.00701402805611212</v>
+        <v>0.002004008016032066</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20321,10 +18861,10 @@
         <v>122</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>121</v>
+        <v>121.5</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.00819672131147541</v>
+        <v>-0.004098360655737705</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -20379,10 +18919,10 @@
         <v>2.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>2.12</v>
+        <v>2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>0.009433962264150952</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -20476,10 +19016,10 @@
         <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.26</v>
+        <v>48.82</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.02137566137566133</v>
+        <v>0.0280423280423281</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -20534,10 +19074,10 @@
         <v>24.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>24.55</v>
+        <v>24.7</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0</v>
+        <v>0.002036659877800436</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -20563,10 +19103,10 @@
         <v>35.46</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>35.34</v>
+        <v>35.14</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.003384094754653058</v>
+        <v>-0.007050197405527355</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -20592,7 +19132,7 @@
         <v>165.8</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>166.9</v>
+        <v>167</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -20621,10 +19161,10 @@
         <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>164.1</v>
+        <v>166.5</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.03500473036896867</v>
+        <v>0.04541154210028375</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -20650,10 +19190,10 @@
         <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.82</v>
+        <v>24.88</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.005672609400324173</v>
+        <v>0.01134521880064835</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -20679,10 +19219,10 @@
         <v>1.87</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.87</v>
+        <v>1.864</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>-0.005347593582887705</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -20708,10 +19248,10 @@
         <v>226</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>228.5</v>
+        <v>225</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.01106194690265487</v>
+        <v>0.008849557522123894</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20737,10 +19277,10 @@
         <v>112.1</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>113.85</v>
+        <v>113.65</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01561106155218555</v>
+        <v>0.01427297056199829</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21664,275 +20204,275 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="28" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="28" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="34" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="28" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="28" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="31" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="32" dxfId="0" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F30:F39">
+    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="34" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="36" dxfId="0" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="18" dxfId="28" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="28" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="28" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="28" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="19">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="0">
       <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21960,7 +20500,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="52" t="n">
-        <v>46335</v>
+        <v>46276</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -21999,7 +20539,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 10:09</t>
+          <t>02/10/2026 10:52</t>
         </is>
       </c>
     </row>
@@ -22056,10 +20596,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.54</v>
+        <v>16.43</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1093226022803487</v>
+        <v>0.1113346747149564</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22086,10 +20626,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.3</v>
+        <v>74.26000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05674749270026658</v>
+        <v>-0.05725530024120847</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22116,10 +20656,10 @@
         <v>140</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>144</v>
+        <v>142.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02857142857142857</v>
+        <v>0.01785714285714286</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22146,7 +20686,7 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.3</v>
+        <v>125.4</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>0.007234726688102825</v>
@@ -22206,10 +20746,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35</v>
+        <v>35.12</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0266963292547275</v>
+        <v>-0.02391546162402668</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22236,10 +20776,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>209.6</v>
+        <v>208.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03052728954671598</v>
+        <v>-0.03422756706752996</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22296,10 +20836,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.05</v>
+        <v>20.2</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.1108647450110865</v>
+        <v>-0.1042128603104213</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -22398,7 +20938,7 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.063</v>
+        <v>0.062</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>-0.1249999999999999</v>
@@ -22428,10 +20968,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.48</v>
+        <v>3.495</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07076923076923076</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -22458,10 +20998,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.502</v>
+        <v>4.524</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.2271244635193134</v>
+        <v>-0.2223175965665236</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22488,10 +21028,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.248</v>
+        <v>2.208</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3837719298245614</v>
+        <v>-0.3903508771929824</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22518,7 +21058,7 @@
         <v>7.45</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.7</v>
+        <v>6.67</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>-0.1006711409395973</v>
@@ -22548,10 +21088,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.9</v>
+        <v>22.32</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1176470588235295</v>
+        <v>-0.09750201450443198</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22578,10 +21118,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>74.44</v>
+        <v>74.73999999999999</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05289957567185283</v>
+        <v>0.05742574257425746</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22608,10 +21148,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.16</v>
+        <v>7.23</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.105</v>
+        <v>-0.09624999999999995</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22638,10 +21178,10 @@
         <v>8.140000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.53</v>
+        <v>7.59</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.07493857493857498</v>
+        <v>-0.06142506142506153</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22668,10 +21208,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.8</v>
+        <v>22.84</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.04779411764705878</v>
+        <v>0.04963235294117639</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22773,10 +21313,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.855</v>
+        <v>5.898</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1346899224806202</v>
+        <v>0.1507751937984495</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22802,10 +21342,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.105</v>
+        <v>0.097</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.2804878048780487</v>
+        <v>0.1951219512195122</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22831,10 +21371,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.645</v>
+        <v>4.51</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2073378839590445</v>
+        <v>-0.2235494880546076</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22863,7 +21403,7 @@
         <v>1.005</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04739336492891</v>
+        <v>-0.05213270142180089</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22889,10 +21429,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.4</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.09302325581395357</v>
+        <v>0.08023255813953482</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22947,10 +21487,10 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.255</v>
+        <v>0.243</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.08928571428571436</v>
+        <v>-0.1321428571428573</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23131,10 +21671,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.9</v>
+        <v>6.96</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.1031175059952039</v>
+        <v>0.1047162270183853</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23160,10 +21700,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.1</v>
+        <v>5.104</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.02298850574712646</v>
+        <v>-0.02413793103448265</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23218,10 +21758,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.05</v>
+        <v>20.2</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1108647450110865</v>
+        <v>-0.1042128603104213</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23276,10 +21816,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.348</v>
+        <v>3.318</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1642536195706441</v>
+        <v>-0.1702446330504244</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -23305,10 +21845,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.06084070796460177</v>
+        <v>-0.05420353982300891</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -23334,10 +21874,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.549</v>
+        <v>1.565</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1729845168179392</v>
+        <v>-0.1703150026695141</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -23392,10 +21932,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>228.5</v>
+        <v>225</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02927927927927928</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24319,275 +22859,275 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="27" dxfId="28" stopIfTrue="1">
+      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="26" dxfId="28" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="25" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="29" dxfId="28" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="30" dxfId="28" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="28" dxfId="28" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
-      <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
+      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
+      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
       <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
-      <formula>IF($U242="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="60" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="60" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="61" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="61" dxfId="28" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="62" dxfId="28" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="63" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="63" dxfId="28" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
       <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="64" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="64" dxfId="28" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="65" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="65" dxfId="28" stopIfTrue="1">
+      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="2">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="22">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
+    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="22">
+    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="2">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="21" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
       <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="20" stopIfTrue="1">
-      <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="19">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
       <formula>$H81</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 11:36
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17911,7 +17911,7 @@
         <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>166.5</v>
+        <v>166.2</v>
       </c>
       <c r="G2" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -17941,7 +17941,7 @@
         <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.82</v>
+        <v>48.745</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -17971,7 +17971,7 @@
         <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.88</v>
+        <v>24.86</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -18001,7 +18001,7 @@
         <v>59.2</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>55.6</v>
+        <v>55.4</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>-0.05743243243243253</v>
@@ -18031,7 +18031,7 @@
         <v>112.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>113.65</v>
+        <v>113.55</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>0.01427297056199829</v>
@@ -18091,7 +18091,7 @@
         <v>226</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>0.008849557522123894</v>
@@ -18283,7 +18283,7 @@
         <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.208</v>
+        <v>2.216</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>-0.01155555555555547</v>
@@ -18313,7 +18313,7 @@
         <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>17.88</v>
+        <v>18</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>-0.01771871539313401</v>
@@ -18343,7 +18343,7 @@
         <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.524</v>
+        <v>4.516</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.008010680907877276</v>
@@ -18373,7 +18373,7 @@
         <v>23.18</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.84</v>
+        <v>22.88</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>-0.01466781708369283</v>
@@ -18403,7 +18403,7 @@
         <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.578</v>
+        <v>0.574</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>-0.001718213058419246</v>
@@ -18433,7 +18433,7 @@
         <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.766</v>
+        <v>10.77</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>0.007462686567164185</v>
@@ -18463,7 +18463,7 @@
         <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>374.75</v>
+        <v>374.55</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0.01116341627437788</v>
@@ -18523,7 +18523,7 @@
         <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.318</v>
+        <v>3.32</v>
       </c>
       <c r="G24" s="13" t="n">
         <v>-0.02464788732394368</v>
@@ -18716,7 +18716,7 @@
         <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>51.5</v>
+        <v>51.1</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.01226993865030678</v>
@@ -19016,7 +19016,7 @@
         <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.82</v>
+        <v>48.745</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -19103,7 +19103,7 @@
         <v>35.46</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>35.14</v>
+        <v>35.12</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>-0.007050197405527355</v>
@@ -19161,7 +19161,7 @@
         <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>166.5</v>
+        <v>166.2</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -19190,7 +19190,7 @@
         <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.88</v>
+        <v>24.86</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -19248,7 +19248,7 @@
         <v>226</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="G51" s="13" t="n">
         <v>0.008849557522123894</v>
@@ -19277,7 +19277,7 @@
         <v>112.1</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>113.65</v>
+        <v>113.55</v>
       </c>
       <c r="G52" s="13" t="n">
         <v>0.01427297056199829</v>
@@ -20626,7 +20626,7 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.26000000000001</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>-0.05725530024120847</v>
@@ -20746,7 +20746,7 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.12</v>
+        <v>35.14</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>-0.02391546162402668</v>
@@ -20776,7 +20776,7 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>208.8</v>
+        <v>209.4</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>-0.03422756706752996</v>
@@ -20968,7 +20968,7 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.495</v>
+        <v>3.5</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>0.07692307692307693</v>
@@ -20998,7 +20998,7 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.524</v>
+        <v>4.516</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>-0.2223175965665236</v>
@@ -21028,7 +21028,7 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.208</v>
+        <v>2.216</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>-0.3903508771929824</v>
@@ -21088,7 +21088,7 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.32</v>
+        <v>22.28</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>-0.09750201450443198</v>
@@ -21118,7 +21118,7 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>74.73999999999999</v>
+        <v>74.76000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0.05742574257425746</v>
@@ -21148,7 +21148,7 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.23</v>
+        <v>7.21</v>
       </c>
       <c r="G23" s="13" t="n">
         <v>-0.09624999999999995</v>
@@ -21208,7 +21208,7 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.84</v>
+        <v>22.88</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>0.04963235294117639</v>
@@ -21313,7 +21313,7 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.898</v>
+        <v>5.899</v>
       </c>
       <c r="G30" s="13" t="n">
         <v>0.1507751937984495</v>
@@ -21371,7 +21371,7 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.51</v>
+        <v>4.46</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>-0.2235494880546076</v>
@@ -21429,7 +21429,7 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.369999999999999</v>
+        <v>9.35</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0.08023255813953482</v>
@@ -21671,7 +21671,7 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.96</v>
+        <v>6.995</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.1047162270183853</v>
@@ -21700,7 +21700,7 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.104</v>
+        <v>5.112</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>-0.02413793103448265</v>
@@ -21816,7 +21816,7 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.318</v>
+        <v>3.32</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>-0.1702446330504244</v>
@@ -21845,7 +21845,7 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>84.7</v>
+        <v>84.65000000000001</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>-0.05420353982300891</v>
@@ -21874,7 +21874,7 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.565</v>
+        <v>1.566</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>-0.1703150026695141</v>
@@ -21932,7 +21932,7 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>225</v>
+        <v>225.5</v>
       </c>
       <c r="G52" s="13" t="n">
         <v>0.02702702702702703</v>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 11:56
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17884,7 +17884,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 10:52</t>
+          <t>02/10/2026 11:56</t>
         </is>
       </c>
     </row>
@@ -17911,7 +17911,7 @@
         <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>166.2</v>
+        <v>164.35</v>
       </c>
       <c r="G2" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -17941,7 +17941,7 @@
         <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.745</v>
+        <v>48.72</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -17971,7 +17971,7 @@
         <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.86</v>
+        <v>24.8</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -18001,7 +18001,7 @@
         <v>59.2</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>55.4</v>
+        <v>55.8</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>-0.05743243243243253</v>
@@ -18031,7 +18031,7 @@
         <v>112.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>113.55</v>
+        <v>112.55</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>0.01427297056199829</v>
@@ -18121,7 +18121,7 @@
         <v>165.8</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>167</v>
+        <v>166.6</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -18283,7 +18283,7 @@
         <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.216</v>
+        <v>2.184</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>-0.01155555555555547</v>
@@ -18313,7 +18313,7 @@
         <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>18</v>
+        <v>17.98</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>-0.01771871539313401</v>
@@ -18343,7 +18343,7 @@
         <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.516</v>
+        <v>4.51</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.008010680907877276</v>
@@ -18373,7 +18373,7 @@
         <v>23.18</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.88</v>
+        <v>22.82</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>-0.01466781708369283</v>
@@ -18403,7 +18403,7 @@
         <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.574</v>
+        <v>0.571</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>-0.001718213058419246</v>
@@ -18433,7 +18433,7 @@
         <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.77</v>
+        <v>10.708</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>0.007462686567164185</v>
@@ -18463,7 +18463,7 @@
         <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>374.55</v>
+        <v>373.9</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0.01116341627437788</v>
@@ -18493,7 +18493,7 @@
         <v>0.467</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.467</v>
+        <v>0.468</v>
       </c>
       <c r="G23" s="13" t="n">
         <v>-0.008565310492505361</v>
@@ -18523,7 +18523,7 @@
         <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.32</v>
+        <v>3.296</v>
       </c>
       <c r="G24" s="13" t="n">
         <v>-0.02464788732394368</v>
@@ -18553,7 +18553,7 @@
         <v>10.32</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>10.13</v>
+        <v>10.09</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>-0.01841085271317825</v>
@@ -18658,7 +18658,7 @@
         <v>0.094</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.097</v>
+        <v>0.094</v>
       </c>
       <c r="G30" s="13" t="n">
         <v>0.04255319148936174</v>
@@ -18687,7 +18687,7 @@
         <v>4.5</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="G31" s="13" t="n">
         <v>-0.03777777777777776</v>
@@ -18716,7 +18716,7 @@
         <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>51.1</v>
+        <v>51.5</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.01226993865030678</v>
@@ -18832,7 +18832,7 @@
         <v>0.998</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.005</v>
+        <v>1.015</v>
       </c>
       <c r="G36" s="13" t="n">
         <v>0.002004008016032066</v>
@@ -18919,7 +18919,7 @@
         <v>2.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>2</v>
+        <v>1.92</v>
       </c>
       <c r="G39" s="13" t="n">
         <v>0.009433962264150952</v>
@@ -19016,7 +19016,7 @@
         <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.745</v>
+        <v>48.72</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -19103,7 +19103,7 @@
         <v>35.46</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>35.12</v>
+        <v>35.18</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>-0.007050197405527355</v>
@@ -19132,7 +19132,7 @@
         <v>165.8</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>167</v>
+        <v>166.6</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -19161,7 +19161,7 @@
         <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>166.2</v>
+        <v>164.35</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -19190,7 +19190,7 @@
         <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.86</v>
+        <v>24.8</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -19277,7 +19277,7 @@
         <v>112.1</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>113.55</v>
+        <v>112.55</v>
       </c>
       <c r="G52" s="13" t="n">
         <v>0.01427297056199829</v>
@@ -20539,7 +20539,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 10:52</t>
+          <t>02/10/2026 11:56</t>
         </is>
       </c>
     </row>
@@ -20596,7 +20596,7 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.43</v>
+        <v>16.45</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0.1113346747149564</v>
@@ -20626,7 +20626,7 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.09999999999999</v>
+        <v>74.03</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>-0.05725530024120847</v>
@@ -20686,7 +20686,7 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.4</v>
+        <v>125.3</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>0.007234726688102825</v>
@@ -20746,7 +20746,7 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.14</v>
+        <v>35.16</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>-0.02391546162402668</v>
@@ -20776,7 +20776,7 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>209.4</v>
+        <v>209.2</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>-0.03422756706752996</v>
@@ -20836,7 +20836,7 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="G11" s="13" t="n">
         <v>-0.1042128603104213</v>
@@ -20998,7 +20998,7 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.516</v>
+        <v>4.51</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>-0.2223175965665236</v>
@@ -21028,7 +21028,7 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.216</v>
+        <v>2.184</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>-0.3903508771929824</v>
@@ -21088,7 +21088,7 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.28</v>
+        <v>22.2</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>-0.09750201450443198</v>
@@ -21118,7 +21118,7 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>74.76000000000001</v>
+        <v>74.54000000000001</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0.05742574257425746</v>
@@ -21208,7 +21208,7 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.88</v>
+        <v>22.82</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>0.04963235294117639</v>
@@ -21313,7 +21313,7 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.899</v>
+        <v>5.88</v>
       </c>
       <c r="G30" s="13" t="n">
         <v>0.1507751937984495</v>
@@ -21342,7 +21342,7 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.097</v>
+        <v>0.094</v>
       </c>
       <c r="G31" s="13" t="n">
         <v>0.1951219512195122</v>
@@ -21371,7 +21371,7 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.46</v>
+        <v>4.435</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>-0.2235494880546076</v>
@@ -21400,7 +21400,7 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.005</v>
+        <v>1.015</v>
       </c>
       <c r="G33" s="13" t="n">
         <v>-0.05213270142180089</v>
@@ -21429,7 +21429,7 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.35</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0.08023255813953482</v>
@@ -21671,7 +21671,7 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.995</v>
+        <v>6.95</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.1047162270183853</v>
@@ -21700,7 +21700,7 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.112</v>
+        <v>5.06</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>-0.02413793103448265</v>
@@ -21758,7 +21758,7 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.2</v>
+        <v>20.1</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>-0.1042128603104213</v>
@@ -21787,7 +21787,7 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.8</v>
+        <v>19.88</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>-0.08333333333333336</v>
@@ -21816,7 +21816,7 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.32</v>
+        <v>3.296</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>-0.1702446330504244</v>
@@ -21845,7 +21845,7 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>84.65000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>-0.05420353982300891</v>
@@ -21874,7 +21874,7 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.566</v>
+        <v>1.558</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>-0.1703150026695141</v>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 12:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -17884,7 +17884,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 11:56</t>
+          <t>02/10/2026 12:05</t>
         </is>
       </c>
     </row>
@@ -17911,7 +17911,7 @@
         <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>164.35</v>
+        <v>164.7</v>
       </c>
       <c r="G2" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -17941,7 +17941,7 @@
         <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.72</v>
+        <v>48.83</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -17971,7 +17971,7 @@
         <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.8</v>
+        <v>24.84</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -18061,7 +18061,7 @@
         <v>24.55</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>24.7</v>
+        <v>24.65</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>0.002036659877800436</v>
@@ -18121,7 +18121,7 @@
         <v>165.8</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>166.6</v>
+        <v>166.95</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -18151,7 +18151,7 @@
         <v>34.8</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>34.8</v>
+        <v>34.6</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>0</v>
@@ -18283,7 +18283,7 @@
         <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.184</v>
+        <v>2.178</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>-0.01155555555555547</v>
@@ -18313,7 +18313,7 @@
         <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>17.98</v>
+        <v>17.94</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>-0.01771871539313401</v>
@@ -18343,7 +18343,7 @@
         <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.51</v>
+        <v>4.522</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0.008010680907877276</v>
@@ -18403,7 +18403,7 @@
         <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.571</v>
+        <v>0.548</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>-0.001718213058419246</v>
@@ -18433,7 +18433,7 @@
         <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.708</v>
+        <v>10.704</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>0.007462686567164185</v>
@@ -18463,7 +18463,7 @@
         <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>373.9</v>
+        <v>373.15</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0.01116341627437788</v>
@@ -18523,7 +18523,7 @@
         <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.296</v>
+        <v>3.302</v>
       </c>
       <c r="G24" s="13" t="n">
         <v>-0.02464788732394368</v>
@@ -18553,7 +18553,7 @@
         <v>10.32</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>10.09</v>
+        <v>10.07</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>-0.01841085271317825</v>
@@ -18716,7 +18716,7 @@
         <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>51.5</v>
+        <v>51.3</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0.01226993865030678</v>
@@ -18861,7 +18861,7 @@
         <v>122</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>121.5</v>
+        <v>120.5</v>
       </c>
       <c r="G37" s="13" t="n">
         <v>-0.004098360655737705</v>
@@ -19016,7 +19016,7 @@
         <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.72</v>
+        <v>48.83</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.0280423280423281</v>
@@ -19045,7 +19045,7 @@
         <v>34.8</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>34.8</v>
+        <v>34.6</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>0</v>
@@ -19074,7 +19074,7 @@
         <v>24.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>24.7</v>
+        <v>24.65</v>
       </c>
       <c r="G45" s="13" t="n">
         <v>0.002036659877800436</v>
@@ -19132,7 +19132,7 @@
         <v>165.8</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>166.6</v>
+        <v>166.95</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>0.006634499396863657</v>
@@ -19161,7 +19161,7 @@
         <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>164.35</v>
+        <v>164.7</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>0.04541154210028375</v>
@@ -19190,7 +19190,7 @@
         <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.8</v>
+        <v>24.84</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>0.01134521880064835</v>
@@ -20539,7 +20539,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 11:56</t>
+          <t>02/10/2026 12:05</t>
         </is>
       </c>
     </row>
@@ -20596,7 +20596,7 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.45</v>
+        <v>16.49</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0.1113346747149564</v>
@@ -20626,7 +20626,7 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.03</v>
+        <v>74</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>-0.05725530024120847</v>
@@ -20776,7 +20776,7 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>209.2</v>
+        <v>209.8</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>-0.03422756706752996</v>
@@ -20836,7 +20836,7 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.1</v>
+        <v>20.05</v>
       </c>
       <c r="G11" s="13" t="n">
         <v>-0.1042128603104213</v>
@@ -20938,7 +20938,7 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.062</v>
+        <v>0.065</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>-0.1249999999999999</v>
@@ -20968,7 +20968,7 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.5</v>
+        <v>3.44</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>0.07692307692307693</v>
@@ -20998,7 +20998,7 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.51</v>
+        <v>4.522</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>-0.2223175965665236</v>
@@ -21028,7 +21028,7 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.184</v>
+        <v>2.178</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>-0.3903508771929824</v>
@@ -21088,7 +21088,7 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.2</v>
+        <v>22.16</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>-0.09750201450443198</v>
@@ -21148,7 +21148,7 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.21</v>
+        <v>7.22</v>
       </c>
       <c r="G23" s="13" t="n">
         <v>-0.09624999999999995</v>
@@ -21313,7 +21313,7 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.88</v>
+        <v>5.865</v>
       </c>
       <c r="G30" s="13" t="n">
         <v>0.1507751937984495</v>
@@ -21371,7 +21371,7 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.435</v>
+        <v>4.43</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>-0.2235494880546076</v>
@@ -21429,7 +21429,7 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.449999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0.08023255813953482</v>
@@ -21487,7 +21487,7 @@
         <v>0.28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.243</v>
+        <v>0.247</v>
       </c>
       <c r="G36" s="13" t="n">
         <v>-0.1321428571428573</v>
@@ -21671,7 +21671,7 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.95</v>
+        <v>6.96</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0.1047162270183853</v>
@@ -21700,7 +21700,7 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.06</v>
+        <v>5.05</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>-0.02413793103448265</v>
@@ -21758,7 +21758,7 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.1</v>
+        <v>20.05</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>-0.1042128603104213</v>
@@ -21787,7 +21787,7 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.88</v>
+        <v>19.78</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>-0.08333333333333336</v>
@@ -21816,7 +21816,7 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.296</v>
+        <v>3.302</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>-0.1702446330504244</v>
@@ -21874,7 +21874,7 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.558</v>
+        <v>1.56</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>-0.1703150026695141</v>
@@ -21903,7 +21903,7 @@
         <v>35.2</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>34.8</v>
+        <v>34.6</v>
       </c>
       <c r="G51" s="13" t="n">
         <v>-0.01136363636363658</v>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -16,16 +16,17 @@
   <definedNames>
     <definedName name="cours">[1]Cours!$A$2:$H$3000</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="000000"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -332,10 +333,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -463,14 +464,744 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
     <cellStyle name="Normal 4" xfId="2"/>
   </cellStyles>
-  <dxfs count="178">
+  <dxfs count="267">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -17844,8 +18575,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="53" t="n">
-        <v>46296</v>
+      <c r="A1" s="54" t="n">
+        <v>46063</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -17884,7 +18615,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 12:05</t>
+          <t>02/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -17911,10 +18642,10 @@
         <v>158.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>164.7</v>
+        <v>164.6</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.04541154210028375</v>
+        <v>0</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -17941,10 +18672,10 @@
         <v>47.25</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.83</v>
+        <v>48.74</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.0280423280423281</v>
+        <v>0</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -17971,10 +18702,10 @@
         <v>24.68</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.84</v>
+        <v>24.74</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01134521880064835</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18004,7 +18735,7 @@
         <v>55.8</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.05743243243243253</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18031,10 +18762,10 @@
         <v>112.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>112.55</v>
+        <v>112.1</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01427297056199829</v>
+        <v>0</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18064,7 +18795,7 @@
         <v>24.65</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.002036659877800436</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18091,10 +18822,10 @@
         <v>226</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.008849557522123894</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18121,10 +18852,10 @@
         <v>165.8</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>166.95</v>
+        <v>166.1</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.006634499396863657</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18283,10 +19014,10 @@
         <v>2.25</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.178</v>
+        <v>2.19</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01155555555555547</v>
+        <v>0</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18313,10 +19044,10 @@
         <v>18.06</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>17.94</v>
+        <v>17.9</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01771871539313401</v>
+        <v>0</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -18343,10 +19074,10 @@
         <v>4.494</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.522</v>
+        <v>4.55</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.008010680907877276</v>
+        <v>0</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -18373,10 +19104,10 @@
         <v>23.18</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.82</v>
+        <v>22.84</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01466781708369283</v>
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -18403,10 +19134,10 @@
         <v>0.582</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.548</v>
+        <v>0.551</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.001718213058419246</v>
+        <v>0</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -18433,10 +19164,10 @@
         <v>10.72</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.704</v>
+        <v>10.792</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.007462686567164185</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -18463,10 +19194,10 @@
         <v>371.75</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>373.15</v>
+        <v>374.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.01116341627437788</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -18496,7 +19227,7 @@
         <v>0.468</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.008565310492505361</v>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -18523,10 +19254,10 @@
         <v>3.408</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.302</v>
+        <v>3.328</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.02464788732394368</v>
+        <v>0</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -18553,10 +19284,10 @@
         <v>10.32</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>10.07</v>
+        <v>10.15</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.01841085271317825</v>
+        <v>0</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -18658,10 +19389,10 @@
         <v>0.094</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.094</v>
+        <v>0.09</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.04255319148936174</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -18687,10 +19418,10 @@
         <v>4.5</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.29</v>
+        <v>4.21</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03777777777777776</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -18716,10 +19447,10 @@
         <v>48.9</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>51.3</v>
+        <v>50.8</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.01226993865030678</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -18745,10 +19476,10 @@
         <v>9.279999999999999</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>9.4</v>
+        <v>9.42</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.01077586206896567</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -18777,7 +19508,7 @@
         <v>0.158</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.02469135802469138</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -18806,7 +19537,7 @@
         <v>3.47</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.002873563218390743</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -18832,10 +19563,10 @@
         <v>0.998</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.015</v>
+        <v>1.025</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.002004008016032066</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -18861,10 +19592,10 @@
         <v>122</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>120.5</v>
+        <v>120</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.004098360655737705</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -18919,10 +19650,10 @@
         <v>2.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.009433962264150952</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19016,10 +19747,10 @@
         <v>47.25</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.83</v>
+        <v>48.74</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0280423280423281</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19077,7 +19808,7 @@
         <v>24.65</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.002036659877800436</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19103,10 +19834,10 @@
         <v>35.46</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>35.18</v>
+        <v>35.14</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.007050197405527355</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19132,10 +19863,10 @@
         <v>165.8</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>166.95</v>
+        <v>166.1</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.006634499396863657</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19161,10 +19892,10 @@
         <v>158.55</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>164.7</v>
+        <v>164.6</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.04541154210028375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19190,10 +19921,10 @@
         <v>24.68</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.84</v>
+        <v>24.74</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01134521880064835</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19222,7 +19953,7 @@
         <v>1.864</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.005347593582887705</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19248,10 +19979,10 @@
         <v>226</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.008849557522123894</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19277,10 +20008,10 @@
         <v>112.1</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>112.55</v>
+        <v>112.1</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01427297056199829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -19356,11 +20087,27 @@
       <c r="A56" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="n"/>
-      <c r="C56" s="30" t="n"/>
-      <c r="D56" s="36" t="n"/>
-      <c r="E56" s="18" t="n"/>
-      <c r="F56" s="12" t="n"/>
+      <c r="B56" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D56" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="n">
+        <v>47.25</v>
+      </c>
+      <c r="F56" s="12" t="n">
+        <v>48.74</v>
+      </c>
       <c r="G56" s="37" t="n">
         <v>0</v>
       </c>
@@ -19370,11 +20117,27 @@
       <c r="A57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="n"/>
-      <c r="C57" s="30" t="n"/>
-      <c r="D57" s="36" t="n"/>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="12" t="n"/>
+      <c r="B57" s="36" t="inlineStr">
+        <is>
+          <t>ATE</t>
+        </is>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D57" s="36" t="inlineStr">
+        <is>
+          <t>ALTEN</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>81.25</v>
+      </c>
+      <c r="F57" s="12" t="n">
+        <v>80.25</v>
+      </c>
       <c r="G57" s="37" t="n">
         <v>0</v>
       </c>
@@ -19384,11 +20147,27 @@
       <c r="A58" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="36" t="n"/>
-      <c r="C58" s="30" t="n"/>
-      <c r="D58" s="36" t="n"/>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="12" t="n"/>
+      <c r="B58" s="36" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D58" s="36" t="inlineStr">
+        <is>
+          <t>CAP GEMINI</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="F58" s="12" t="n">
+        <v>112.1</v>
+      </c>
       <c r="G58" s="37" t="n">
         <v>0</v>
       </c>
@@ -19398,11 +20177,27 @@
       <c r="A59" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B59" s="36" t="n"/>
-      <c r="C59" s="30" t="n"/>
-      <c r="D59" s="36" t="n"/>
-      <c r="E59" s="18" t="n"/>
-      <c r="F59" s="12" t="n"/>
+      <c r="B59" s="36" t="inlineStr">
+        <is>
+          <t>SAVE</t>
+        </is>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D59" s="36" t="inlineStr">
+        <is>
+          <t>SAVENCIA</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="F59" s="12" t="n">
+        <v>55.8</v>
+      </c>
       <c r="G59" s="37" t="n">
         <v>0</v>
       </c>
@@ -19412,11 +20207,27 @@
       <c r="A60" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B60" s="36" t="n"/>
-      <c r="C60" s="30" t="n"/>
-      <c r="D60" s="36" t="n"/>
-      <c r="E60" s="18" t="n"/>
-      <c r="F60" s="12" t="n"/>
+      <c r="B60" s="36" t="inlineStr">
+        <is>
+          <t>TEP</t>
+        </is>
+      </c>
+      <c r="C60" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D60" s="36" t="inlineStr">
+        <is>
+          <t>TÉLÉPERFORMANCE</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="n">
+        <v>71.06</v>
+      </c>
+      <c r="F60" s="12" t="n">
+        <v>70.90000000000001</v>
+      </c>
       <c r="G60" s="37" t="n">
         <v>0</v>
       </c>
@@ -19426,11 +20237,27 @@
       <c r="A61" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B61" s="36" t="n"/>
-      <c r="C61" s="30" t="n"/>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="18" t="n"/>
-      <c r="F61" s="12" t="n"/>
+      <c r="B61" s="36" t="inlineStr">
+        <is>
+          <t>QDT</t>
+        </is>
+      </c>
+      <c r="C61" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D61" s="36" t="inlineStr">
+        <is>
+          <t>QUADIENT</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="F61" s="12" t="n">
+        <v>13.72</v>
+      </c>
       <c r="G61" s="37" t="n">
         <v>0</v>
       </c>
@@ -19440,11 +20267,27 @@
       <c r="A62" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B62" s="36" t="n"/>
-      <c r="C62" s="30" t="n"/>
-      <c r="D62" s="36" t="n"/>
-      <c r="E62" s="18" t="n"/>
-      <c r="F62" s="12" t="n"/>
+      <c r="B62" s="36" t="inlineStr">
+        <is>
+          <t>SOP</t>
+        </is>
+      </c>
+      <c r="C62" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D62" s="36" t="inlineStr">
+        <is>
+          <t>SOPRA STERIA GROUP</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="n">
+        <v>165.8</v>
+      </c>
+      <c r="F62" s="12" t="n">
+        <v>166.1</v>
+      </c>
       <c r="G62" s="37" t="n">
         <v>0</v>
       </c>
@@ -19454,11 +20297,27 @@
       <c r="A63" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B63" s="36" t="n"/>
-      <c r="C63" s="30" t="n"/>
-      <c r="D63" s="36" t="n"/>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="12" t="n"/>
+      <c r="B63" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C63" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D63" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>41.18</v>
+      </c>
+      <c r="F63" s="12" t="n">
+        <v>42.48</v>
+      </c>
       <c r="G63" s="37" t="n">
         <v>0</v>
       </c>
@@ -19565,11 +20424,27 @@
       <c r="A69" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="36" t="n"/>
-      <c r="C69" s="30" t="n"/>
-      <c r="D69" s="36" t="n"/>
-      <c r="E69" s="18" t="n"/>
-      <c r="F69" s="12" t="n"/>
+      <c r="B69" s="36" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D69" s="36" t="inlineStr">
+        <is>
+          <t>LINEDATA</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="F69" s="12" t="n">
+        <v>54.2</v>
+      </c>
       <c r="G69" s="37" t="n">
         <v>0</v>
       </c>
@@ -19579,11 +20454,27 @@
       <c r="A70" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B70" s="36" t="n"/>
-      <c r="C70" s="30" t="n"/>
-      <c r="D70" s="36" t="n"/>
-      <c r="E70" s="18" t="n"/>
-      <c r="F70" s="12" t="n"/>
+      <c r="B70" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D70" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="n">
+        <v>47.25</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <v>48.74</v>
+      </c>
       <c r="G70" s="37" t="n">
         <v>0</v>
       </c>
@@ -19593,11 +20484,27 @@
       <c r="A71" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B71" s="36" t="n"/>
-      <c r="C71" s="30" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="12" t="n"/>
+      <c r="B71" s="36" t="inlineStr">
+        <is>
+          <t>ATE</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D71" s="36" t="inlineStr">
+        <is>
+          <t>ALTEN</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>81.25</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <v>80.25</v>
+      </c>
       <c r="G71" s="37" t="n">
         <v>0</v>
       </c>
@@ -19607,11 +20514,27 @@
       <c r="A72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="36" t="n"/>
-      <c r="C72" s="30" t="n"/>
-      <c r="D72" s="36" t="n"/>
-      <c r="E72" s="18" t="n"/>
-      <c r="F72" s="12" t="n"/>
+      <c r="B72" s="36" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D72" s="36" t="inlineStr">
+        <is>
+          <t>CAP GEMINI</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>112.1</v>
+      </c>
       <c r="G72" s="37" t="n">
         <v>0</v>
       </c>
@@ -19621,11 +20544,27 @@
       <c r="A73" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="36" t="n"/>
-      <c r="C73" s="30" t="n"/>
-      <c r="D73" s="36" t="n"/>
-      <c r="E73" s="18" t="n"/>
-      <c r="F73" s="12" t="n"/>
+      <c r="B73" s="36" t="inlineStr">
+        <is>
+          <t>SAVE</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D73" s="36" t="inlineStr">
+        <is>
+          <t>SAVENCIA</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>55.8</v>
+      </c>
       <c r="G73" s="37" t="n">
         <v>0</v>
       </c>
@@ -19635,11 +20574,27 @@
       <c r="A74" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B74" s="36" t="n"/>
-      <c r="C74" s="30" t="n"/>
-      <c r="D74" s="36" t="n"/>
-      <c r="E74" s="18" t="n"/>
-      <c r="F74" s="12" t="n"/>
+      <c r="B74" s="36" t="inlineStr">
+        <is>
+          <t>TEP</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D74" s="36" t="inlineStr">
+        <is>
+          <t>TÉLÉPERFORMANCE</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="n">
+        <v>71.06</v>
+      </c>
+      <c r="F74" s="12" t="n">
+        <v>70.90000000000001</v>
+      </c>
       <c r="G74" s="37" t="n">
         <v>0</v>
       </c>
@@ -19649,11 +20604,27 @@
       <c r="A75" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B75" s="36" t="n"/>
-      <c r="C75" s="30" t="n"/>
-      <c r="D75" s="36" t="n"/>
-      <c r="E75" s="18" t="n"/>
-      <c r="F75" s="12" t="n"/>
+      <c r="B75" s="36" t="inlineStr">
+        <is>
+          <t>QDT</t>
+        </is>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D75" s="36" t="inlineStr">
+        <is>
+          <t>QUADIENT</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="F75" s="12" t="n">
+        <v>13.72</v>
+      </c>
       <c r="G75" s="37" t="n">
         <v>0</v>
       </c>
@@ -19663,11 +20634,27 @@
       <c r="A76" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="36" t="n"/>
-      <c r="C76" s="30" t="n"/>
-      <c r="D76" s="36" t="n"/>
-      <c r="E76" s="18" t="n"/>
-      <c r="F76" s="12" t="n"/>
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>SOP</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D76" s="36" t="inlineStr">
+        <is>
+          <t>SOPRA STERIA GROUP</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="n">
+        <v>165.8</v>
+      </c>
+      <c r="F76" s="12" t="n">
+        <v>166.1</v>
+      </c>
       <c r="G76" s="37" t="n">
         <v>0</v>
       </c>
@@ -19677,11 +20664,27 @@
       <c r="A77" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B77" s="36" t="n"/>
-      <c r="C77" s="30" t="n"/>
-      <c r="D77" s="36" t="n"/>
-      <c r="E77" s="18" t="n"/>
-      <c r="F77" s="12" t="n"/>
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D77" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>41.18</v>
+      </c>
+      <c r="F77" s="12" t="n">
+        <v>42.48</v>
+      </c>
       <c r="G77" s="37" t="n">
         <v>0</v>
       </c>
@@ -20204,275 +21207,275 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="36" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="0" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="35" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="34" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="34" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="33" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="32" dxfId="28" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="31" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
-      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
-      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="18" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="17" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="15" dxfId="28" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="28" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="13" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
-      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
-      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
-      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
-      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
-      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="25">
       <formula>$H81</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F67">
+    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
+      <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
+      <formula>IF($T265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
+      <formula>IF($U265="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82">
+    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
+      <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
+      <formula>IF($T278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F30:F39">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -20500,7 +21503,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="52" t="n">
-        <v>46276</v>
+        <v>46335</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -20539,7 +21542,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 12:05</t>
+          <t>02/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20566,10 +21569,10 @@
         <v>0.351</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.306</v>
+        <v>0.304</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1282051282051282</v>
+        <v>-0.113960113960114</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20596,10 +21599,10 @@
         <v>14.91</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.49</v>
+        <v>16.38</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1113346747149564</v>
+        <v>0.1073105298457413</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20626,10 +21629,10 @@
         <v>78.77</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74</v>
+        <v>74.31</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05725530024120847</v>
+        <v>-0.05408150311032112</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20659,7 +21662,7 @@
         <v>142.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01428571428571423</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20686,10 +21689,10 @@
         <v>124.4</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.3</v>
+        <v>125.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.007234726688102825</v>
+        <v>0.007234726688102766</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20719,7 +21722,7 @@
         <v>54.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1410526315789474</v>
+        <v>0.1368421052631579</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20746,10 +21749,10 @@
         <v>35.96</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.16</v>
+        <v>35.12</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02391546162402668</v>
+        <v>-0.02947719688542827</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20776,10 +21779,10 @@
         <v>216.2</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>209.8</v>
+        <v>210</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03422756706752996</v>
+        <v>-0.03145235892691944</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20806,10 +21809,10 @@
         <v>0.016</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.3125000000000001</v>
+        <v>-0.3125</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20836,10 +21839,10 @@
         <v>22.55</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.05</v>
+        <v>20.1</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.1042128603104213</v>
+        <v>-0.1219512195121951</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20938,10 +21941,10 @@
         <v>0.07199999999999999</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.065</v>
+        <v>0.062</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.111111111111111</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20968,10 +21971,10 @@
         <v>3.25</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.44</v>
+        <v>3.42</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.06461538461538452</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20998,10 +22001,10 @@
         <v>5.825</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.522</v>
+        <v>4.55</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.2223175965665236</v>
+        <v>-0.2284978540772533</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21028,10 +22031,10 @@
         <v>3.648</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.178</v>
+        <v>2.19</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3903508771929824</v>
+        <v>-0.3832236842105263</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21061,7 +22064,7 @@
         <v>6.67</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1006711409395973</v>
+        <v>-0.09932885906040267</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21088,10 +22091,10 @@
         <v>24.82</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.16</v>
+        <v>22.24</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.09750201450443198</v>
+        <v>-0.1023368251410153</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21118,10 +22121,10 @@
         <v>70.7</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>74.54000000000001</v>
+        <v>75.22</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05742574257425746</v>
+        <v>0.05431400282885446</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21148,10 +22151,10 @@
         <v>8</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.22</v>
+        <v>7.24</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.09624999999999995</v>
+        <v>-0.1025</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21181,7 +22184,7 @@
         <v>7.59</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.06142506142506153</v>
+        <v>-0.09090909090909094</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21208,10 +22211,10 @@
         <v>21.76</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.82</v>
+        <v>22.84</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.04963235294117639</v>
+        <v>0.06525735294117641</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -21313,10 +22316,10 @@
         <v>5.16</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.865</v>
+        <v>5.864</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1507751937984495</v>
+        <v>0.1081395348837209</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -21342,10 +22345,10 @@
         <v>0.082</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.094</v>
+        <v>0.09</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.1951219512195122</v>
+        <v>0.1463414634146341</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -21371,10 +22374,10 @@
         <v>5.86</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.43</v>
+        <v>4.4</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2235494880546076</v>
+        <v>-0.2218430034129694</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -21400,10 +22403,10 @@
         <v>1.055</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.015</v>
+        <v>1.025</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05213270142180089</v>
+        <v>-0.05402843601895724</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -21429,10 +22432,10 @@
         <v>8.6</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.6</v>
+        <v>9.44</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.08023255813953482</v>
+        <v>0.06860465116279069</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -21461,7 +22464,7 @@
         <v>25.1</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2364532019704434</v>
+        <v>0.2364532019704433</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -21490,7 +22493,7 @@
         <v>0.247</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1321428571428573</v>
+        <v>-0.1071428571428572</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21519,7 +22522,7 @@
         <v>1.22</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.04687500000000004</v>
+        <v>-0.09375000000000011</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21548,7 +22551,7 @@
         <v>0.139</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.13125</v>
+        <v>-0.1375</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21577,7 +22580,7 @@
         <v>19.45</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.02015113350125955</v>
+        <v>-0.02015113350125952</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21671,10 +22674,10 @@
         <v>6.255</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.96</v>
+        <v>6.945</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.1047162270183853</v>
+        <v>0.08153477218225413</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -21700,10 +22703,10 @@
         <v>5.22</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.05</v>
+        <v>5.04</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.02413793103448265</v>
+        <v>-0.01417624521072791</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -21758,10 +22761,10 @@
         <v>22.55</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.05</v>
+        <v>20.1</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1042128603104213</v>
+        <v>-0.1219512195121951</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -21787,10 +22790,10 @@
         <v>21.6</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.78</v>
+        <v>19.8</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.08333333333333336</v>
+        <v>-0.09351851851851867</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -21816,10 +22819,10 @@
         <v>4.006</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.302</v>
+        <v>3.328</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1702446330504244</v>
+        <v>-0.1492760858711932</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -21845,10 +22848,10 @@
         <v>90.40000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>84.8</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.05420353982300891</v>
+        <v>-0.05199115044247793</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -21874,10 +22877,10 @@
         <v>1.873</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.56</v>
+        <v>1.569</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1703150026695141</v>
+        <v>-0.183128670581954</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -21932,10 +22935,10 @@
         <v>222</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>225.5</v>
+        <v>226</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.01801801801801806</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22859,274 +23862,274 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="27" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="29" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="30" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="28" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
       <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="75" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="74" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
       <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="72" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
       <formula>IF($T230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="71" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="73" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="76" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
       <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
-    <cfRule type="expression" priority="79" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="77" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="81" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="82" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="80" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
       <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="78" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="12" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
       <formula>IF($U255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
       <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
       <formula>IF($U255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
       <formula>IF($T255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
       <formula>IF($T255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F67">
-    <cfRule type="expression" priority="83" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="83" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="84" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="84" dxfId="0" stopIfTrue="1">
       <formula>IF($AK39="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="85" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="85" dxfId="0" stopIfTrue="1">
       <formula>IF($T265="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="86" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="86" dxfId="0" stopIfTrue="1">
       <formula>IF($U265="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="2" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
       <formula>IF($T268="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
       <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
       <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
       <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="1" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
       <formula>IF($T268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="89" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
       <formula>IF($U278="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="87" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
       <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="88" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
       <formula>IF($T278="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="60" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="60" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="61" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="61" dxfId="0" stopIfTrue="1">
       <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="62" dxfId="0" stopIfTrue="1">
       <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="63" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="63" dxfId="0" stopIfTrue="1">
       <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="70" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
       <formula>IF($U291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="68" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
       <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
       <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="64" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="64" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="66" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
       <formula>IF($T293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="67" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
       <formula>IF($U293="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="65" dxfId="28" stopIfTrue="1">
+    <cfRule type="expression" priority="65" dxfId="0" stopIfTrue="1">
       <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="2">
+    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="28">
       <formula>#REF!</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="1" stopIfTrue="1">
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="27" stopIfTrue="1">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="25">
       <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-02 19:45
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Donnees" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,11 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="000000"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="166" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -333,10 +332,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -464,15 +463,14 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1"/>
     <cellStyle name="Normal 4" xfId="2"/>
   </cellStyles>
-  <dxfs count="267">
+  <dxfs count="356">
     <dxf>
       <font>
         <b val="1"/>
@@ -1204,6 +1202,206 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -1214,6 +1412,14 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -1248,14 +1454,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -1282,8 +1480,9 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <color indexed="10"/>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
         <extend val="0"/>
       </font>
     </dxf>
@@ -1308,9 +1507,8 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
+        <condense val="0"/>
+        <color indexed="10"/>
         <extend val="0"/>
       </font>
     </dxf>
@@ -1343,6 +1541,21 @@
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <condense val="0"/>
         <color rgb="FF006100"/>
         <extend val="0"/>
@@ -1355,13 +1568,6 @@
     </dxf>
     <dxf>
       <font>
-        <condense val="0"/>
-        <color indexed="10"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b val="1"/>
         <condense val="0"/>
         <color auto="1"/>
@@ -1396,14 +1602,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
-        <condense val="0"/>
-        <color auto="1"/>
-        <extend val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <condense val="0"/>
         <color indexed="10"/>
         <extend val="0"/>
@@ -1440,6 +1638,535 @@
       <font>
         <condense val="0"/>
         <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="12"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color indexed="18"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color rgb="FF006100"/>
+        <extend val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <condense val="0"/>
+        <color indexed="10"/>
+        <extend val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <condense val="0"/>
+        <color auto="1"/>
         <extend val="0"/>
       </font>
     </dxf>
@@ -18575,8 +19302,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="54" t="n">
-        <v>46063</v>
+      <c r="A1" s="53" t="n">
+        <v>46297</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -18615,7 +19342,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 13:00</t>
+          <t>02/10/2026 19:45</t>
         </is>
       </c>
     </row>
@@ -18639,10 +19366,10 @@
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>158.55</v>
+        <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>164.6</v>
+        <v>169.05</v>
       </c>
       <c r="G2" s="13" t="n">
         <v>0</v>
@@ -18669,10 +19396,10 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>47.25</v>
+        <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>48.74</v>
+        <v>50.19</v>
       </c>
       <c r="G3" s="13" t="n">
         <v>0</v>
@@ -18685,7 +19412,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>MRN</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -18695,14 +19422,14 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>JCDECAUX</t>
+          <t>MERSEN</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>24.68</v>
+        <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.74</v>
+        <v>42.66</v>
       </c>
       <c r="G4" s="13" t="n">
         <v>0</v>
@@ -18715,7 +19442,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>SAVE</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -18725,14 +19452,14 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>SAVENCIA</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>59.2</v>
+        <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>55.8</v>
+        <v>6.965</v>
       </c>
       <c r="G5" s="13" t="n">
         <v>0</v>
@@ -18745,24 +19472,24 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>CAP GEMINI</t>
+          <t>LINEDATA</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>112.1</v>
+        <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>112.1</v>
+        <v>54.2</v>
       </c>
       <c r="G6" s="13" t="n">
         <v>0</v>
@@ -18775,7 +19502,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>PLNW</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -18785,14 +19512,14 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>PLANISWARE</t>
+          <t>SCHNEIDER ELECTRIC</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>24.55</v>
+        <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>24.65</v>
+        <v>301.85</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>0</v>
@@ -18805,24 +19532,24 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>EXEL INDUSTRIES</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>226</v>
+        <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>226</v>
+        <v>17.4</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>0</v>
@@ -18835,7 +19562,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>SOP</t>
+          <t>LR</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -18845,14 +19572,14 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>SOPRA STERIA GROUP</t>
+          <t>LEGRAND SA</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>165.8</v>
+        <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>166.1</v>
+        <v>144.25</v>
       </c>
       <c r="G9" s="13" t="n">
         <v>0</v>
@@ -18865,24 +19592,24 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>CASINO GUICHARD</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>34.8</v>
+        <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>34.6</v>
+        <v>0.186</v>
       </c>
       <c r="G10" s="13" t="n">
         <v>0</v>
@@ -18895,24 +19622,24 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>FNAC</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>FNAC DARTY</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>34.5</v>
+        <v>227</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.5</v>
+        <v>227</v>
       </c>
       <c r="G11" s="13" t="n">
         <v>0</v>
@@ -18997,24 +19724,24 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>ADOC</t>
+          <t>SIGHT</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>ADOCIA</t>
+          <t>GENSIGHT BIOLO</t>
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>2.25</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.19</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G16" s="13" t="n">
         <v>0</v>
@@ -19027,7 +19754,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>FDE</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -19037,14 +19764,14 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>FRANCAISE ENER</t>
+          <t>AB SCIENCE</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>18.06</v>
+        <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>17.9</v>
+        <v>0.544</v>
       </c>
       <c r="G17" s="13" t="n">
         <v>0</v>
@@ -19057,7 +19784,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>NXI</t>
+          <t>OSE</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -19067,14 +19794,14 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>NEXITY</t>
+          <t>OSE IMMUNO</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>4.494</v>
+        <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.55</v>
+        <v>2.108</v>
       </c>
       <c r="G18" s="13" t="n">
         <v>0</v>
@@ -19087,7 +19814,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>MEDCL</t>
+          <t>NXI</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -19097,14 +19824,14 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>MEDINCELL</t>
+          <t>NEXITY</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>23.18</v>
+        <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.84</v>
+        <v>4.364</v>
       </c>
       <c r="G19" s="13" t="n">
         <v>0</v>
@@ -19117,7 +19844,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>AB</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -19127,14 +19854,14 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>AB SCIENCE</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>0.582</v>
+        <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.551</v>
+        <v>17.6</v>
       </c>
       <c r="G20" s="13" t="n">
         <v>0</v>
@@ -19147,24 +19874,24 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>WLN</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>WORLDLINE</t>
+          <t>CA PARIS IDF</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>10.72</v>
+        <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>10.792</v>
+        <v>85</v>
       </c>
       <c r="G21" s="13" t="n">
         <v>0</v>
@@ -19177,7 +19904,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>OR</t>
+          <t>FGA</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -19187,14 +19914,14 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>L'OREAL</t>
+          <t>FIGEAC AERO</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>371.75</v>
+        <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>374.4</v>
+        <v>11.18</v>
       </c>
       <c r="G22" s="13" t="n">
         <v>0</v>
@@ -19207,24 +19934,24 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>WLN</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>SOLUTIONS 30</t>
+          <t>WORLDLINE</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.467</v>
+        <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.468</v>
+        <v>10.57</v>
       </c>
       <c r="G23" s="13" t="n">
         <v>0</v>
@@ -19251,10 +19978,10 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>3.408</v>
+        <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.328</v>
+        <v>3.208</v>
       </c>
       <c r="G24" s="13" t="n">
         <v>0</v>
@@ -19267,24 +19994,24 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>EMEIS</t>
+          <t>LNA</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>EMEIS</t>
+          <t>LNA SANTE</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>10.32</v>
+        <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>10.15</v>
+        <v>25.2</v>
       </c>
       <c r="G25" s="13" t="n">
         <v>0</v>
@@ -19372,7 +20099,7 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>ALDBT</t>
+          <t>ALCPB</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -19382,14 +20109,14 @@
       </c>
       <c r="D30" s="51" t="inlineStr">
         <is>
-          <t>DBT</t>
+          <t>CAPITAL B</t>
         </is>
       </c>
       <c r="E30" s="18" t="n">
-        <v>0.094</v>
+        <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.09</v>
+        <v>5.799</v>
       </c>
       <c r="G30" s="13" t="n">
         <v>0</v>
@@ -19415,10 +20142,10 @@
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>4.5</v>
+        <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.21</v>
+        <v>4.52</v>
       </c>
       <c r="G31" s="13" t="n">
         <v>0</v>
@@ -19430,7 +20157,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>ALSEM</t>
+          <t>ALRIB</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -19440,14 +20167,14 @@
       </c>
       <c r="D32" s="51" t="inlineStr">
         <is>
-          <t>SEMCO TECHNOLOGIES</t>
+          <t>RIBER</t>
         </is>
       </c>
       <c r="E32" s="18" t="n">
-        <v>48.9</v>
+        <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>50.8</v>
+        <v>9.42</v>
       </c>
       <c r="G32" s="13" t="n">
         <v>0</v>
@@ -19459,7 +20186,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>ALICA</t>
+          <t>ALSEM</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -19469,14 +20196,14 @@
       </c>
       <c r="D33" s="51" t="inlineStr">
         <is>
-          <t>ICAP HOLDING</t>
+          <t>SEMCO TECHNOLOGIES</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>9.279999999999999</v>
+        <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>9.42</v>
+        <v>50.9</v>
       </c>
       <c r="G33" s="13" t="n">
         <v>0</v>
@@ -19488,7 +20215,7 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>ALIMP</t>
+          <t>ALICA</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -19498,14 +20225,14 @@
       </c>
       <c r="D34" s="51" t="inlineStr">
         <is>
-          <t>IMPLANET</t>
+          <t>ICAP HOLDING</t>
         </is>
       </c>
       <c r="E34" s="18" t="n">
-        <v>0.162</v>
+        <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.158</v>
+        <v>9.48</v>
       </c>
       <c r="G34" s="13" t="n">
         <v>0</v>
@@ -19517,7 +20244,7 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ALCWE</t>
+          <t>ALNMG</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -19527,14 +20254,14 @@
       </c>
       <c r="D35" s="51" t="inlineStr">
         <is>
-          <t>CHARWOOD ENERGY</t>
+          <t>NETMEDIA</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>3.48</v>
+        <v>0.419</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>3.47</v>
+        <v>0.419</v>
       </c>
       <c r="G35" s="13" t="n">
         <v>0</v>
@@ -19560,10 +20287,10 @@
         </is>
       </c>
       <c r="E36" s="18" t="n">
-        <v>0.998</v>
+        <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.025</v>
+        <v>1.035</v>
       </c>
       <c r="G36" s="13" t="n">
         <v>0</v>
@@ -19575,24 +20302,24 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>FMONC</t>
+          <t>ALCBI</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D37" s="51" t="inlineStr">
         <is>
-          <t>FINANCIERE MONCEY</t>
+          <t>CBI</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>122</v>
+        <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>120</v>
+        <v>0.141</v>
       </c>
       <c r="G37" s="13" t="n">
         <v>0</v>
@@ -19604,24 +20331,24 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>ALNLF</t>
+          <t>DPT</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D38" s="51" t="inlineStr">
         <is>
-          <t>NEOLIFE</t>
+          <t>ST DUPONT</t>
         </is>
       </c>
       <c r="E38" s="18" t="n">
-        <v>0.062</v>
+        <v>0.089</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.062</v>
+        <v>0.089</v>
       </c>
       <c r="G38" s="13" t="n">
         <v>0</v>
@@ -19633,7 +20360,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>ALECO</t>
+          <t>ALMCE</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -19643,14 +20370,14 @@
       </c>
       <c r="D39" s="51" t="inlineStr">
         <is>
-          <t>ECOMIAM</t>
+          <t>MON COURTIER ENERGIE</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>2.12</v>
+        <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>2</v>
+        <v>5.7</v>
       </c>
       <c r="G39" s="13" t="n">
         <v>0</v>
@@ -19730,7 +20457,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>STMPA</t>
+          <t>VIRP</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -19740,14 +20467,14 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>STMICROELECTRONICS</t>
+          <t>VIRBAC</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>47.25</v>
+        <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>48.74</v>
+        <v>309</v>
       </c>
       <c r="G43" s="13" t="n">
         <v>0</v>
@@ -19759,24 +20486,24 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>34.8</v>
+        <v>227</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>34.6</v>
+        <v>227</v>
       </c>
       <c r="G44" s="13" t="n">
         <v>0</v>
@@ -19788,24 +20515,24 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>PLNW</t>
+          <t>FNAC</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>PLANISWARE</t>
+          <t>FNAC DARTY</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
-        <v>24.55</v>
+        <v>34.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>24.65</v>
+        <v>34.55</v>
       </c>
       <c r="G45" s="13" t="n">
         <v>0</v>
@@ -19817,24 +20544,24 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>IPS</t>
+          <t>SELER</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>IPSOS</t>
+          <t>SELECTIRENTE</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>35.46</v>
+        <v>87</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>35.14</v>
+        <v>87</v>
       </c>
       <c r="G46" s="13" t="n">
         <v>0</v>
@@ -19846,7 +20573,7 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>SOP</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -19856,14 +20583,14 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>SOPRA STERIA GROUP</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>165.8</v>
+        <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>166.1</v>
+        <v>6.965</v>
       </c>
       <c r="G47" s="13" t="n">
         <v>0</v>
@@ -19875,7 +20602,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>SOI</t>
+          <t>ENX</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -19885,14 +20612,14 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOITEC </t>
+          <t>EURONEXT</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>158.55</v>
+        <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>164.6</v>
+        <v>160.6</v>
       </c>
       <c r="G48" s="13" t="n">
         <v>0</v>
@@ -19904,24 +20631,24 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>GPE</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>JCDECAUX</t>
+          <t>GPE PIZZORNO ENVI</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>24.68</v>
+        <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>24.74</v>
+        <v>62.25</v>
       </c>
       <c r="G49" s="13" t="n">
         <v>0</v>
@@ -19933,7 +20660,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>VAC</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -19943,14 +20670,14 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>PIERRE &amp; VACANCES</t>
+          <t>AIR LIQUIDE</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
-        <v>1.87</v>
+        <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.864</v>
+        <v>170.4</v>
       </c>
       <c r="G50" s="13" t="n">
         <v>0</v>
@@ -19962,7 +20689,7 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>NEX</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
@@ -19972,14 +20699,14 @@
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>NEXANS</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>226</v>
+        <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>226</v>
+        <v>136</v>
       </c>
       <c r="G51" s="13" t="n">
         <v>0</v>
@@ -19991,7 +20718,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
@@ -20001,14 +20728,14 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>CAP GEMINI</t>
+          <t>SCHNEIDER ELECTRIC</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>112.1</v>
+        <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>112.1</v>
+        <v>301.85</v>
       </c>
       <c r="G52" s="13" t="n">
         <v>0</v>
@@ -20087,27 +20814,11 @@
       <c r="A56" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="inlineStr">
-        <is>
-          <t>STMPA</t>
-        </is>
-      </c>
-      <c r="C56" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D56" s="36" t="inlineStr">
-        <is>
-          <t>STMICROELECTRONICS</t>
-        </is>
-      </c>
-      <c r="E56" s="18" t="n">
-        <v>47.25</v>
-      </c>
-      <c r="F56" s="12" t="n">
-        <v>48.74</v>
-      </c>
+      <c r="B56" s="36" t="n"/>
+      <c r="C56" s="30" t="n"/>
+      <c r="D56" s="36" t="n"/>
+      <c r="E56" s="18" t="n"/>
+      <c r="F56" s="12" t="n"/>
       <c r="G56" s="37" t="n">
         <v>0</v>
       </c>
@@ -20117,27 +20828,11 @@
       <c r="A57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="inlineStr">
-        <is>
-          <t>ATE</t>
-        </is>
-      </c>
-      <c r="C57" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D57" s="36" t="inlineStr">
-        <is>
-          <t>ALTEN</t>
-        </is>
-      </c>
-      <c r="E57" s="18" t="n">
-        <v>81.25</v>
-      </c>
-      <c r="F57" s="12" t="n">
-        <v>80.25</v>
-      </c>
+      <c r="B57" s="36" t="n"/>
+      <c r="C57" s="30" t="n"/>
+      <c r="D57" s="36" t="n"/>
+      <c r="E57" s="18" t="n"/>
+      <c r="F57" s="12" t="n"/>
       <c r="G57" s="37" t="n">
         <v>0</v>
       </c>
@@ -20147,27 +20842,11 @@
       <c r="A58" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="36" t="inlineStr">
-        <is>
-          <t>CAP</t>
-        </is>
-      </c>
-      <c r="C58" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D58" s="36" t="inlineStr">
-        <is>
-          <t>CAP GEMINI</t>
-        </is>
-      </c>
-      <c r="E58" s="18" t="n">
-        <v>112.1</v>
-      </c>
-      <c r="F58" s="12" t="n">
-        <v>112.1</v>
-      </c>
+      <c r="B58" s="36" t="n"/>
+      <c r="C58" s="30" t="n"/>
+      <c r="D58" s="36" t="n"/>
+      <c r="E58" s="18" t="n"/>
+      <c r="F58" s="12" t="n"/>
       <c r="G58" s="37" t="n">
         <v>0</v>
       </c>
@@ -20177,27 +20856,11 @@
       <c r="A59" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B59" s="36" t="inlineStr">
-        <is>
-          <t>SAVE</t>
-        </is>
-      </c>
-      <c r="C59" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D59" s="36" t="inlineStr">
-        <is>
-          <t>SAVENCIA</t>
-        </is>
-      </c>
-      <c r="E59" s="18" t="n">
-        <v>59.2</v>
-      </c>
-      <c r="F59" s="12" t="n">
-        <v>55.8</v>
-      </c>
+      <c r="B59" s="36" t="n"/>
+      <c r="C59" s="30" t="n"/>
+      <c r="D59" s="36" t="n"/>
+      <c r="E59" s="18" t="n"/>
+      <c r="F59" s="12" t="n"/>
       <c r="G59" s="37" t="n">
         <v>0</v>
       </c>
@@ -20207,29 +20870,13 @@
       <c r="A60" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B60" s="36" t="inlineStr">
-        <is>
-          <t>TEP</t>
-        </is>
-      </c>
-      <c r="C60" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D60" s="36" t="inlineStr">
-        <is>
-          <t>TÉLÉPERFORMANCE</t>
-        </is>
-      </c>
-      <c r="E60" s="18" t="n">
-        <v>71.06</v>
-      </c>
-      <c r="F60" s="12" t="n">
-        <v>70.90000000000001</v>
-      </c>
-      <c r="G60" s="37" t="n">
-        <v>0</v>
+      <c r="B60" s="36" t="n"/>
+      <c r="C60" s="30" t="n"/>
+      <c r="D60" s="36" t="n"/>
+      <c r="E60" s="18" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -20237,29 +20884,13 @@
       <c r="A61" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B61" s="36" t="inlineStr">
-        <is>
-          <t>QDT</t>
-        </is>
-      </c>
-      <c r="C61" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D61" s="36" t="inlineStr">
-        <is>
-          <t>QUADIENT</t>
-        </is>
-      </c>
-      <c r="E61" s="18" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="F61" s="12" t="n">
-        <v>13.72</v>
-      </c>
-      <c r="G61" s="37" t="n">
-        <v>0</v>
+      <c r="B61" s="36" t="n"/>
+      <c r="C61" s="30" t="n"/>
+      <c r="D61" s="36" t="n"/>
+      <c r="E61" s="18" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -20267,29 +20898,13 @@
       <c r="A62" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B62" s="36" t="inlineStr">
-        <is>
-          <t>SOP</t>
-        </is>
-      </c>
-      <c r="C62" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D62" s="36" t="inlineStr">
-        <is>
-          <t>SOPRA STERIA GROUP</t>
-        </is>
-      </c>
-      <c r="E62" s="18" t="n">
-        <v>165.8</v>
-      </c>
-      <c r="F62" s="12" t="n">
-        <v>166.1</v>
-      </c>
-      <c r="G62" s="37" t="n">
-        <v>0</v>
+      <c r="B62" s="36" t="n"/>
+      <c r="C62" s="30" t="n"/>
+      <c r="D62" s="36" t="n"/>
+      <c r="E62" s="18" t="n"/>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -20297,29 +20912,13 @@
       <c r="A63" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B63" s="36" t="inlineStr">
-        <is>
-          <t>MRN</t>
-        </is>
-      </c>
-      <c r="C63" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D63" s="36" t="inlineStr">
-        <is>
-          <t>MERSEN</t>
-        </is>
-      </c>
-      <c r="E63" s="18" t="n">
-        <v>41.18</v>
-      </c>
-      <c r="F63" s="12" t="n">
-        <v>42.48</v>
-      </c>
-      <c r="G63" s="37" t="n">
-        <v>0</v>
+      <c r="B63" s="36" t="n"/>
+      <c r="C63" s="30" t="n"/>
+      <c r="D63" s="36" t="n"/>
+      <c r="E63" s="18" t="n"/>
+      <c r="F63" s="12" t="n"/>
+      <c r="G63" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -20424,27 +21023,11 @@
       <c r="A69" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="36" t="inlineStr">
-        <is>
-          <t>LIN</t>
-        </is>
-      </c>
-      <c r="C69" s="30" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D69" s="36" t="inlineStr">
-        <is>
-          <t>LINEDATA</t>
-        </is>
-      </c>
-      <c r="E69" s="18" t="n">
-        <v>54</v>
-      </c>
-      <c r="F69" s="12" t="n">
-        <v>54.2</v>
-      </c>
+      <c r="B69" s="36" t="n"/>
+      <c r="C69" s="30" t="n"/>
+      <c r="D69" s="36" t="n"/>
+      <c r="E69" s="18" t="n"/>
+      <c r="F69" s="12" t="n"/>
       <c r="G69" s="37" t="n">
         <v>0</v>
       </c>
@@ -20454,27 +21037,11 @@
       <c r="A70" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B70" s="36" t="inlineStr">
-        <is>
-          <t>STMPA</t>
-        </is>
-      </c>
-      <c r="C70" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D70" s="36" t="inlineStr">
-        <is>
-          <t>STMICROELECTRONICS</t>
-        </is>
-      </c>
-      <c r="E70" s="18" t="n">
-        <v>47.25</v>
-      </c>
-      <c r="F70" s="12" t="n">
-        <v>48.74</v>
-      </c>
+      <c r="B70" s="36" t="n"/>
+      <c r="C70" s="30" t="n"/>
+      <c r="D70" s="36" t="n"/>
+      <c r="E70" s="18" t="n"/>
+      <c r="F70" s="12" t="n"/>
       <c r="G70" s="37" t="n">
         <v>0</v>
       </c>
@@ -20484,27 +21051,11 @@
       <c r="A71" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B71" s="36" t="inlineStr">
-        <is>
-          <t>ATE</t>
-        </is>
-      </c>
-      <c r="C71" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D71" s="36" t="inlineStr">
-        <is>
-          <t>ALTEN</t>
-        </is>
-      </c>
-      <c r="E71" s="18" t="n">
-        <v>81.25</v>
-      </c>
-      <c r="F71" s="12" t="n">
-        <v>80.25</v>
-      </c>
+      <c r="B71" s="36" t="n"/>
+      <c r="C71" s="30" t="n"/>
+      <c r="D71" s="36" t="n"/>
+      <c r="E71" s="18" t="n"/>
+      <c r="F71" s="12" t="n"/>
       <c r="G71" s="37" t="n">
         <v>0</v>
       </c>
@@ -20514,27 +21065,11 @@
       <c r="A72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="36" t="inlineStr">
-        <is>
-          <t>CAP</t>
-        </is>
-      </c>
-      <c r="C72" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D72" s="36" t="inlineStr">
-        <is>
-          <t>CAP GEMINI</t>
-        </is>
-      </c>
-      <c r="E72" s="18" t="n">
-        <v>112.1</v>
-      </c>
-      <c r="F72" s="12" t="n">
-        <v>112.1</v>
-      </c>
+      <c r="B72" s="36" t="n"/>
+      <c r="C72" s="30" t="n"/>
+      <c r="D72" s="36" t="n"/>
+      <c r="E72" s="18" t="n"/>
+      <c r="F72" s="12" t="n"/>
       <c r="G72" s="37" t="n">
         <v>0</v>
       </c>
@@ -20544,27 +21079,11 @@
       <c r="A73" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="36" t="inlineStr">
-        <is>
-          <t>SAVE</t>
-        </is>
-      </c>
-      <c r="C73" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D73" s="36" t="inlineStr">
-        <is>
-          <t>SAVENCIA</t>
-        </is>
-      </c>
-      <c r="E73" s="18" t="n">
-        <v>59.2</v>
-      </c>
-      <c r="F73" s="12" t="n">
-        <v>55.8</v>
-      </c>
+      <c r="B73" s="36" t="n"/>
+      <c r="C73" s="30" t="n"/>
+      <c r="D73" s="36" t="n"/>
+      <c r="E73" s="18" t="n"/>
+      <c r="F73" s="12" t="n"/>
       <c r="G73" s="37" t="n">
         <v>0</v>
       </c>
@@ -20574,29 +21093,13 @@
       <c r="A74" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B74" s="36" t="inlineStr">
-        <is>
-          <t>TEP</t>
-        </is>
-      </c>
-      <c r="C74" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D74" s="36" t="inlineStr">
-        <is>
-          <t>TÉLÉPERFORMANCE</t>
-        </is>
-      </c>
-      <c r="E74" s="18" t="n">
-        <v>71.06</v>
-      </c>
-      <c r="F74" s="12" t="n">
-        <v>70.90000000000001</v>
-      </c>
-      <c r="G74" s="37" t="n">
-        <v>0</v>
+      <c r="B74" s="36" t="n"/>
+      <c r="C74" s="30" t="n"/>
+      <c r="D74" s="36" t="n"/>
+      <c r="E74" s="18" t="n"/>
+      <c r="F74" s="12" t="n"/>
+      <c r="G74" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -20604,29 +21107,13 @@
       <c r="A75" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B75" s="36" t="inlineStr">
-        <is>
-          <t>QDT</t>
-        </is>
-      </c>
-      <c r="C75" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D75" s="36" t="inlineStr">
-        <is>
-          <t>QUADIENT</t>
-        </is>
-      </c>
-      <c r="E75" s="18" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="F75" s="12" t="n">
-        <v>13.72</v>
-      </c>
-      <c r="G75" s="37" t="n">
-        <v>0</v>
+      <c r="B75" s="36" t="n"/>
+      <c r="C75" s="30" t="n"/>
+      <c r="D75" s="36" t="n"/>
+      <c r="E75" s="18" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -20634,29 +21121,13 @@
       <c r="A76" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="36" t="inlineStr">
-        <is>
-          <t>SOP</t>
-        </is>
-      </c>
-      <c r="C76" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D76" s="36" t="inlineStr">
-        <is>
-          <t>SOPRA STERIA GROUP</t>
-        </is>
-      </c>
-      <c r="E76" s="18" t="n">
-        <v>165.8</v>
-      </c>
-      <c r="F76" s="12" t="n">
-        <v>166.1</v>
-      </c>
-      <c r="G76" s="37" t="n">
-        <v>0</v>
+      <c r="B76" s="36" t="n"/>
+      <c r="C76" s="30" t="n"/>
+      <c r="D76" s="36" t="n"/>
+      <c r="E76" s="18" t="n"/>
+      <c r="F76" s="12" t="n"/>
+      <c r="G76" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -20664,29 +21135,13 @@
       <c r="A77" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B77" s="36" t="inlineStr">
-        <is>
-          <t>MRN</t>
-        </is>
-      </c>
-      <c r="C77" s="30" t="inlineStr">
-        <is>
-          <t>SRD</t>
-        </is>
-      </c>
-      <c r="D77" s="36" t="inlineStr">
-        <is>
-          <t>MERSEN</t>
-        </is>
-      </c>
-      <c r="E77" s="18" t="n">
-        <v>41.18</v>
-      </c>
-      <c r="F77" s="12" t="n">
-        <v>42.48</v>
-      </c>
-      <c r="G77" s="37" t="n">
-        <v>0</v>
+      <c r="B77" s="36" t="n"/>
+      <c r="C77" s="30" t="n"/>
+      <c r="D77" s="36" t="n"/>
+      <c r="E77" s="18" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="37" t="e">
+        <v>#VALUE!</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21502,8 +21957,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
-      <c r="A1" s="52" t="n">
-        <v>46335</v>
+      <c r="A1" s="53" t="n">
+        <v>46063</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -21542,7 +21997,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>02/10/2026 13:00</t>
+          <t>02/10/2026 19:45</t>
         </is>
       </c>
     </row>
@@ -21552,27 +22007,27 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>VMX</t>
+          <t>SOI</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>VERIMATRIX</t>
+          <t xml:space="preserve">SOITEC </t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>0.351</v>
+        <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>0.304</v>
+        <v>169.05</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.113960113960114</v>
+        <v>0</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21582,27 +22037,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>OVH</t>
+          <t>STMPA</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>OVH GROUPE</t>
+          <t>STMICROELECTRONICS</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>14.91</v>
+        <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>16.38</v>
+        <v>50.19</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1073105298457413</v>
+        <v>0</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21612,7 +22067,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>MRN</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -21622,17 +22077,17 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>TOTALENERGIES</t>
+          <t>MERSEN</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>78.77</v>
+        <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>74.31</v>
+        <v>42.66</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05408150311032112</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21642,7 +22097,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -21652,17 +22107,17 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>140</v>
+        <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>142.5</v>
+        <v>6.965</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01428571428571423</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21672,27 +22127,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>EXA</t>
+          <t>LIN</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>EXAIL TECH</t>
+          <t>LINEDATA</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>124.4</v>
+        <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>125.5</v>
+        <v>54.2</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.007234726688102766</v>
+        <v>0</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21702,27 +22157,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>LINEDATA</t>
+          <t>SCHNEIDER ELECTRIC</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>47.5</v>
+        <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>54.2</v>
+        <v>301.85</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.1368421052631579</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21732,27 +22187,27 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>RUI</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>RUBIS</t>
+          <t>EXEL INDUSTRIES</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>35.96</v>
+        <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>35.12</v>
+        <v>17.4</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.02947719688542827</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21762,7 +22217,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>LR</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -21772,17 +22227,17 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>GAZTRANS TECHN</t>
+          <t>LEGRAND SA</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>216.2</v>
+        <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>210</v>
+        <v>144.25</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03145235892691944</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21792,27 +22247,27 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>LAT</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>LATECOERE</t>
+          <t>CASINO GUICHARD</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>0.016</v>
+        <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.01</v>
+        <v>0.186</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.3125</v>
+        <v>0</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21822,7 +22277,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>MTU</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -21832,17 +22287,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>MANITOU</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>22.55</v>
+        <v>227</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>20.1</v>
+        <v>227</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.1219512195121951</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21858,7 +22313,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>-0.03977493163122617</v>
+        <v>0</v>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
@@ -21924,27 +22379,27 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>NACON</t>
+          <t>SIGHT</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>NACON</t>
+          <t>GENSIGHT BIOLO</t>
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.062</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.111111111111111</v>
+        <v>0</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21954,7 +22409,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>ARAMI</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -21964,17 +22419,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>ARAMIS</t>
+          <t>AB SCIENCE</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>3.25</v>
+        <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>3.42</v>
+        <v>0.544</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.06461538461538452</v>
+        <v>0</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21984,7 +22439,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>NXI</t>
+          <t>OSE</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -21994,17 +22449,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>NEXITY</t>
+          <t>OSE IMMUNO</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>5.825</v>
+        <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.55</v>
+        <v>2.108</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.2284978540772533</v>
+        <v>0</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -22014,7 +22469,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ADOC</t>
+          <t>NXI</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -22024,17 +22479,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>ADOCIA</t>
+          <t>NEXITY</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>3.648</v>
+        <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>2.19</v>
+        <v>4.364</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.3832236842105263</v>
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -22044,7 +22499,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>GBT</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -22054,17 +22509,17 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>GUERBET</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>7.45</v>
+        <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.67</v>
+        <v>17.6</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.09932885906040267</v>
+        <v>0</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -22074,27 +22529,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>ATO</t>
+          <t>CAF</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>CA PARIS IDF</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>24.82</v>
+        <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.24</v>
+        <v>85</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1023368251410153</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -22104,7 +22559,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>ERF</t>
+          <t>FGA</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -22114,17 +22569,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>EUROFINS SCIENTIFIC</t>
+          <t>FIGEAC AERO</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>70.7</v>
+        <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>75.22</v>
+        <v>11.18</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05431400282885446</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -22134,27 +22589,27 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>ANTIN</t>
+          <t>WLN</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>ANTIN INFRA</t>
+          <t>WORLDLINE</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>8</v>
+        <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>7.24</v>
+        <v>10.57</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.1025</v>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22164,7 +22619,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>CRI</t>
+          <t>CLARI</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -22174,17 +22629,17 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>CHARGEURS</t>
+          <t>CLARIANE</t>
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>8.140000000000001</v>
+        <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>7.59</v>
+        <v>3.208</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.09090909090909094</v>
+        <v>0</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22194,27 +22649,27 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>MEDCL</t>
+          <t>LNA</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>MEDINCELL</t>
+          <t>LNA SANTE</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>21.76</v>
+        <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>22.84</v>
+        <v>25.2</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.06525735294117641</v>
+        <v>0</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22230,7 +22685,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.09337206841239842</v>
+        <v>0</v>
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
@@ -22297,290 +22752,290 @@
       <c r="A30" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>ALCPB</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
+      <c r="D30" s="51" t="inlineStr">
         <is>
           <t>CAPITAL B</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>5.16</v>
+      <c r="E30" s="18" t="n">
+        <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.864</v>
+        <v>5.799</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.1081395348837209</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
       <c r="A31" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>ALDBT</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>ALWIT</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D31" s="10" t="inlineStr">
-        <is>
-          <t>DBT</t>
-        </is>
-      </c>
-      <c r="E31" s="11" t="n">
-        <v>0.082</v>
+      <c r="D31" s="51" t="inlineStr">
+        <is>
+          <t>WITBE</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.09</v>
+        <v>4.52</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.1463414634146341</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
       <c r="A32" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>ALKAL</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>ALRIB</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
-        <is>
-          <t>KALRAY</t>
-        </is>
-      </c>
-      <c r="E32" s="11" t="n">
-        <v>5.86</v>
+      <c r="D32" s="51" t="inlineStr">
+        <is>
+          <t>RIBER</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="n">
+        <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>4.4</v>
+        <v>9.42</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.2218430034129694</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
       <c r="A33" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>ALNTG</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>ALSEM</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D33" s="10" t="inlineStr">
-        <is>
-          <t>NETGEM</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="n">
-        <v>1.055</v>
+      <c r="D33" s="51" t="inlineStr">
+        <is>
+          <t>SEMCO TECHNOLOGIES</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.025</v>
+        <v>50.9</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05402843601895724</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
       <c r="A34" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>ALRIB</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>ALICA</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
-        <is>
-          <t>RIBER</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="n">
-        <v>8.6</v>
+      <c r="D34" s="51" t="inlineStr">
+        <is>
+          <t>ICAP HOLDING</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="n">
+        <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.44</v>
+        <v>9.48</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.06860465116279069</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
       <c r="A35" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>ALERS</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>ALNMG</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>EUROBIO SCIENT</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>20.3</v>
+      <c r="D35" s="51" t="inlineStr">
+        <is>
+          <t>NETMEDIA</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>0.419</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>25.1</v>
+        <v>0.419</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0.2364532019704433</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
       <c r="A36" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>ALJXR</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>ALNTG</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHOS          </t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>0.28</v>
+      <c r="D36" s="51" t="inlineStr">
+        <is>
+          <t>NETGEM</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="n">
+        <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.247</v>
+        <v>1.035</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.1071428571428572</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
       <c r="A37" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>ALNN6</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>ALCBI</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>ENENSYS TECHNO</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="n">
-        <v>1.28</v>
+      <c r="D37" s="51" t="inlineStr">
+        <is>
+          <t>CBI</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="n">
+        <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.22</v>
+        <v>0.141</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.09375000000000011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
       <c r="A38" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>ALKLH</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
-        <is>
-          <t>EG</t>
-        </is>
-      </c>
-      <c r="D38" s="10" t="inlineStr">
-        <is>
-          <t>KLEA HOLDING</t>
-        </is>
-      </c>
-      <c r="E38" s="11" t="n">
-        <v>0.16</v>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>DPT</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D38" s="51" t="inlineStr">
+        <is>
+          <t>ST DUPONT</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="n">
+        <v>0.089</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.139</v>
+        <v>0.089</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1375</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
       <c r="A39" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>ALDNX</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>ALMCE</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>EG</t>
         </is>
       </c>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>DNXCORP</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="n">
-        <v>19.85</v>
+      <c r="D39" s="51" t="inlineStr">
+        <is>
+          <t>MON COURTIER ENERGIE</t>
+        </is>
+      </c>
+      <c r="E39" s="18" t="n">
+        <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>19.45</v>
+        <v>5.7</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.02015113350125952</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22594,7 +23049,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.007487657864445452</v>
+        <v>0</v>
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
@@ -22657,7 +23112,7 @@
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>XFAB</t>
+          <t>VIRP</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
@@ -22667,17 +23122,17 @@
       </c>
       <c r="D43" s="10" t="inlineStr">
         <is>
-          <t>X-FAB SILICON</t>
+          <t>VIRBAC</t>
         </is>
       </c>
       <c r="E43" s="11" t="n">
-        <v>6.255</v>
+        <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>6.945</v>
+        <v>309</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.08153477218225413</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22686,7 +23141,7 @@
       </c>
       <c r="B44" s="9" t="inlineStr">
         <is>
-          <t>UBI</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
@@ -22696,17 +23151,17 @@
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>UBISOFT</t>
+          <t>TOTAL GABON</t>
         </is>
       </c>
       <c r="E44" s="11" t="n">
-        <v>5.22</v>
+        <v>227</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>5.04</v>
+        <v>227</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01417624521072791</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22715,7 +23170,7 @@
       </c>
       <c r="B45" s="9" t="inlineStr">
         <is>
-          <t>SELER</t>
+          <t>FNAC</t>
         </is>
       </c>
       <c r="C45" s="9" t="inlineStr">
@@ -22725,17 +23180,17 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>SELECTIRENTE</t>
+          <t>FNAC DARTY</t>
         </is>
       </c>
       <c r="E45" s="11" t="n">
-        <v>85.5</v>
+        <v>34.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>86.5</v>
+        <v>34.55</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.01169590643274865</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22744,27 +23199,27 @@
       </c>
       <c r="B46" s="9" t="inlineStr">
         <is>
-          <t>MTU</t>
+          <t>SELER</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>MANITOU</t>
+          <t>SELECTIRENTE</t>
         </is>
       </c>
       <c r="E46" s="11" t="n">
-        <v>22.55</v>
+        <v>87</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>20.1</v>
+        <v>87</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1219512195121951</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22773,7 +23228,7 @@
       </c>
       <c r="B47" s="9" t="inlineStr">
         <is>
-          <t>JCQ</t>
+          <t>XFAB</t>
         </is>
       </c>
       <c r="C47" s="9" t="inlineStr">
@@ -22783,17 +23238,17 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>JACQUET METAL</t>
+          <t>X-FAB SILICON</t>
         </is>
       </c>
       <c r="E47" s="11" t="n">
-        <v>21.6</v>
+        <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.8</v>
+        <v>6.965</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.09351851851851867</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22802,7 +23257,7 @@
       </c>
       <c r="B48" s="9" t="inlineStr">
         <is>
-          <t>CLARI</t>
+          <t>ENX</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
@@ -22812,17 +23267,17 @@
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>CLARIANE</t>
+          <t>EURONEXT</t>
         </is>
       </c>
       <c r="E48" s="11" t="n">
-        <v>4.006</v>
+        <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>3.328</v>
+        <v>160.6</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1492760858711932</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22831,7 +23286,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>VIRI</t>
+          <t>GPE</t>
         </is>
       </c>
       <c r="C49" s="9" t="inlineStr">
@@ -22841,17 +23296,17 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>VIRIDIEN</t>
+          <t>GPE PIZZORNO ENVI</t>
         </is>
       </c>
       <c r="E49" s="11" t="n">
-        <v>90.40000000000001</v>
+        <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>85.09999999999999</v>
+        <v>62.25</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.05199115044247793</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22860,7 +23315,7 @@
       </c>
       <c r="B50" s="9" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -22870,17 +23325,17 @@
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>EUTELSAT COMMUNICATION</t>
+          <t>AIR LIQUIDE</t>
         </is>
       </c>
       <c r="E50" s="11" t="n">
-        <v>1.873</v>
+        <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.569</v>
+        <v>170.4</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.183128670581954</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22889,27 +23344,27 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>NEX</t>
         </is>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>FREY</t>
+          <t>NEXANS</t>
         </is>
       </c>
       <c r="E51" s="11" t="n">
-        <v>35.2</v>
+        <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>34.6</v>
+        <v>136</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01136363636363658</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22918,7 +23373,7 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
@@ -22928,17 +23383,17 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>SCHNEIDER ELECTRIC</t>
         </is>
       </c>
       <c r="E52" s="11" t="n">
-        <v>222</v>
+        <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>226</v>
+        <v>301.85</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01801801801801806</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22952,7 +23407,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>-0.05141568298676826</v>
+        <v>0</v>
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>
@@ -23014,13 +23469,29 @@
       <c r="A56" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="n"/>
-      <c r="C56" s="30" t="n"/>
-      <c r="D56" s="36" t="n"/>
-      <c r="E56" s="18" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B56" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D56" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="n">
+        <v>50.34</v>
+      </c>
+      <c r="F56" s="12" t="n">
+        <v>50.19</v>
+      </c>
+      <c r="G56" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -23028,13 +23499,29 @@
       <c r="A57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="n"/>
-      <c r="C57" s="30" t="n"/>
-      <c r="D57" s="36" t="n"/>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="12" t="n"/>
-      <c r="G57" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B57" s="36" t="inlineStr">
+        <is>
+          <t>QDT</t>
+        </is>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D57" s="36" t="inlineStr">
+        <is>
+          <t>QUADIENT</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>13.86</v>
+      </c>
+      <c r="F57" s="12" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="G57" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -23042,13 +23529,29 @@
       <c r="A58" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="36" t="n"/>
-      <c r="C58" s="30" t="n"/>
-      <c r="D58" s="36" t="n"/>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B58" s="36" t="inlineStr">
+        <is>
+          <t>XFAB</t>
+        </is>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D58" s="36" t="inlineStr">
+        <is>
+          <t>X-FAB SILICON</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="n">
+        <v>6.995</v>
+      </c>
+      <c r="F58" s="12" t="n">
+        <v>6.965</v>
+      </c>
+      <c r="G58" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -23056,13 +23559,29 @@
       <c r="A59" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B59" s="36" t="n"/>
-      <c r="C59" s="30" t="n"/>
-      <c r="D59" s="36" t="n"/>
-      <c r="E59" s="18" t="n"/>
-      <c r="F59" s="12" t="n"/>
-      <c r="G59" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B59" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D59" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="F59" s="12" t="n">
+        <v>42.66</v>
+      </c>
+      <c r="G59" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -23223,13 +23742,29 @@
       <c r="A69" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="36" t="n"/>
-      <c r="C69" s="30" t="n"/>
-      <c r="D69" s="36" t="n"/>
-      <c r="E69" s="18" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B69" s="36" t="inlineStr">
+        <is>
+          <t>QDT</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D69" s="36" t="inlineStr">
+        <is>
+          <t>QUADIENT</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="n">
+        <v>13.86</v>
+      </c>
+      <c r="F69" s="12" t="n">
+        <v>13.98</v>
+      </c>
+      <c r="G69" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -23237,13 +23772,29 @@
       <c r="A70" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B70" s="36" t="n"/>
-      <c r="C70" s="30" t="n"/>
-      <c r="D70" s="36" t="n"/>
-      <c r="E70" s="18" t="n"/>
-      <c r="F70" s="12" t="n"/>
-      <c r="G70" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B70" s="36" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D70" s="36" t="inlineStr">
+        <is>
+          <t>LINEDATA</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="G70" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -23251,13 +23802,29 @@
       <c r="A71" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B71" s="36" t="n"/>
-      <c r="C71" s="30" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="12" t="n"/>
-      <c r="G71" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B71" s="36" t="inlineStr">
+        <is>
+          <t>XFAB</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D71" s="36" t="inlineStr">
+        <is>
+          <t>X-FAB SILICON</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>6.995</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <v>6.965</v>
+      </c>
+      <c r="G71" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -23265,13 +23832,29 @@
       <c r="A72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="36" t="n"/>
-      <c r="C72" s="30" t="n"/>
-      <c r="D72" s="36" t="n"/>
-      <c r="E72" s="18" t="n"/>
-      <c r="F72" s="12" t="n"/>
-      <c r="G72" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B72" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D72" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="n">
+        <v>50.34</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>50.19</v>
+      </c>
+      <c r="G72" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -23279,13 +23862,29 @@
       <c r="A73" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="36" t="n"/>
-      <c r="C73" s="30" t="n"/>
-      <c r="D73" s="36" t="n"/>
-      <c r="E73" s="18" t="n"/>
-      <c r="F73" s="12" t="n"/>
-      <c r="G73" s="37" t="e">
-        <v>#VALUE!</v>
+      <c r="B73" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D73" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="n">
+        <v>42.6</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>42.66</v>
+      </c>
+      <c r="G73" s="37" t="n">
+        <v>0</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -23797,116 +24396,102 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B56:B65">
-    <cfRule type="expression" priority="16" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="22" dxfId="76" stopIfTrue="1">
       <formula>IF(AO56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69:B78">
-    <cfRule type="expression" priority="14" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="20" dxfId="76" stopIfTrue="1">
       <formula>IF(AO69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B81">
-    <cfRule type="expression" priority="56" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="62" dxfId="76" stopIfTrue="1">
       <formula>IF(AN62&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B82:B91">
-    <cfRule type="expression" priority="20" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="26" dxfId="76" stopIfTrue="1">
       <formula>IF(AL82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="expression" priority="52" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="58" dxfId="76" stopIfTrue="1">
       <formula>IF(AL91&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="expression" priority="55" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="61" dxfId="76" stopIfTrue="1">
       <formula>IF(AN75&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96:B105">
-    <cfRule type="expression" priority="18" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="24" dxfId="76" stopIfTrue="1">
       <formula>IF(AO96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B106">
-    <cfRule type="expression" priority="53" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="59" dxfId="76" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="expression" priority="54" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="60" dxfId="76" stopIfTrue="1">
       <formula>IF(AN104&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D56:D65">
-    <cfRule type="expression" priority="15" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="21" dxfId="76" stopIfTrue="1">
       <formula>IF(AQ56&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D69:D78">
-    <cfRule type="expression" priority="13" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="19" dxfId="76" stopIfTrue="1">
       <formula>IF(AQ69&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D82:D91">
-    <cfRule type="expression" priority="19" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="25" dxfId="76" stopIfTrue="1">
       <formula>IF(AN82&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D96:D105">
-    <cfRule type="expression" priority="17" dxfId="76" stopIfTrue="1">
+    <cfRule type="expression" priority="23" dxfId="76" stopIfTrue="1">
       <formula>IF(AQ96&gt;0,TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F11 F16:F25">
-    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="32" dxfId="0" stopIfTrue="1">
+      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="34" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
       <formula>IF($T200="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
-      <formula>IF($T200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="36" dxfId="0" stopIfTrue="1">
       <formula>IF($U200="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="28" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN1048554="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F30:F39">
-    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN5="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
-      <formula>IF($T230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
-      <formula>IF($U230="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F43:F52">
+    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
+      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+    </cfRule>
     <cfRule type="expression" priority="79" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="77" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="81" dxfId="0" stopIfTrue="1">
       <formula>IF($T242="AAA",TRUE,FALSE)</formula>
@@ -23914,31 +24499,152 @@
     <cfRule type="expression" priority="82" dxfId="0" stopIfTrue="1">
       <formula>IF($U242="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="80" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN17="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="78" dxfId="0" stopIfTrue="1">
-      <formula>IF($T242="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F82:F91">
+    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F56:F65">
-    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+  <conditionalFormatting sqref="F83:F91">
+    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
+      <formula>IF($T279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
+      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F96:F97">
+    <cfRule type="expression" priority="74" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="75" dxfId="0" stopIfTrue="1">
+      <formula>IF($T291="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+    <cfRule type="expression" priority="76" dxfId="0" stopIfTrue="1">
+      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F96:F106">
+    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F98:F106">
+    <cfRule type="expression" priority="71" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="72" dxfId="0" stopIfTrue="1">
+      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="73" dxfId="0" stopIfTrue="1">
+      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
+    <cfRule type="cellIs" priority="64" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="65" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="63" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12 G16:G28">
+    <cfRule type="cellIs" priority="37" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G43:G54">
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="45" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G53:G54">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="29" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="30" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G56:G67">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="56" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="57" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G69:G80">
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="41" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G82:G92">
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="53" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G96:G106">
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="28">
+      <formula>#REF!</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="27" stopIfTrue="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="49" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
+      <formula>#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H81">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="25">
+      <formula>$H81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F67">
@@ -23955,182 +24661,75 @@
       <formula>IF($U265="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F69:F78">
-    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
-      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F82">
-    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
-      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
-    </cfRule>
     <cfRule type="expression" priority="87" dxfId="0" stopIfTrue="1">
       <formula>IF($AJ53="AAA",TRUE,FALSE)</formula>
     </cfRule>
     <cfRule type="expression" priority="88" dxfId="0" stopIfTrue="1">
       <formula>IF($T278="AAA",TRUE,FALSE)</formula>
     </cfRule>
+    <cfRule type="expression" priority="89" dxfId="0" stopIfTrue="1">
+      <formula>IF($U278="AAA",TRUE,FALSE)</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F82:F91">
-    <cfRule type="expression" priority="60" dxfId="0" stopIfTrue="1">
+  <conditionalFormatting sqref="F56:F65">
+    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F83:F91">
-    <cfRule type="expression" priority="61" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN55="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="14" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="62" dxfId="0" stopIfTrue="1">
-      <formula>IF($T279="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="63" dxfId="0" stopIfTrue="1">
-      <formula>IF($U279="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="16" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN30="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
+      <formula>IF($T255="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
+      <formula>IF($U255="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F96:F97">
-    <cfRule type="expression" priority="70" dxfId="0" stopIfTrue="1">
-      <formula>IF($U291="AAA",TRUE,FALSE)</formula>
+  <conditionalFormatting sqref="F69:F78">
+    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
+      <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="68" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN65="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="8" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="69" dxfId="0" stopIfTrue="1">
-      <formula>IF($T291="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN43="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
+      <formula>IF($T268="AAA",TRUE,FALSE)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="0" stopIfTrue="1">
+      <formula>IF($U268="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F96:F106">
-    <cfRule type="expression" priority="64" dxfId="0" stopIfTrue="1">
+  <conditionalFormatting sqref="F30:F39">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>IF(#REF!="AAA",TRUE,FALSE)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F98:F106">
-    <cfRule type="expression" priority="66" dxfId="0" stopIfTrue="1">
-      <formula>IF($T293="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="67" dxfId="0" stopIfTrue="1">
-      <formula>IF($U293="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="expression" priority="65" dxfId="0" stopIfTrue="1">
-      <formula>IF($AN68="AAA",TRUE,FALSE)</formula>
+    <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
+      <formula>IF($AN6="AAA",TRUE,FALSE)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G12 G16:G26 G30:G41">
-    <cfRule type="cellIs" priority="58" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
+    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
+      <formula>IF($T228="AAA",TRUE,FALSE)</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="59" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="57" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G12 G16:G28">
-    <cfRule type="cellIs" priority="31" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30:G41 G43:G54 G56:G67">
-    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43:G54">
-    <cfRule type="cellIs" priority="39" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G53:G54">
-    <cfRule type="cellIs" priority="24" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="23" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G56:G67">
-    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="51" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G69:G80">
-    <cfRule type="cellIs" priority="35" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G82:G92">
-    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="47" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G96:G106">
-    <cfRule type="cellIs" priority="43" operator="greaterThanOrEqual" dxfId="26" stopIfTrue="1">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="28">
-      <formula>#REF!</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="27" stopIfTrue="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H81">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="25">
-      <formula>$H81</formula>
+    <cfRule type="expression" priority="6" dxfId="0" stopIfTrue="1">
+      <formula>IF($U228="AAA",TRUE,FALSE)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-05 16:51
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 16:23</t>
+          <t>05/10/2026 16:51</t>
         </is>
       </c>
     </row>
@@ -18585,11 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>166.9</v>
-      </c>
-      <c r="G2" s="13">
-        <f>(F2/E2-1)</f>
-        <v/>
+        <v>165.5</v>
+      </c>
+      <c r="G2" s="13" t="n">
+        <v>-0.03046280023432917</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18616,11 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="G3" s="13">
-        <f>(F3/E3-1)</f>
-        <v/>
+        <v>50.91</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>0.0113230035756852</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18647,11 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>42.44</v>
-      </c>
-      <c r="G4" s="13">
-        <f>(F4/E4-1)</f>
-        <v/>
+        <v>42.66</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>0.001408450704225239</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18678,11 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.85</v>
-      </c>
-      <c r="G5" s="13">
-        <f>(F5/E5-1)</f>
-        <v/>
+        <v>6.885</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>-0.01572551822730526</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18709,11 +18705,10 @@
         <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="G6" s="13">
-        <f>(F6/E6-1)</f>
-        <v/>
+        <v>54</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>-0.003690036900369056</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18740,11 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>271</v>
-      </c>
-      <c r="G7" s="13">
-        <f>(F7/E7-1)</f>
-        <v/>
+        <v>273.3</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>-0.09801980198019798</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18771,11 +18765,10 @@
         <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>17.1</v>
-      </c>
-      <c r="G8" s="13">
-        <f>(F8/E8-1)</f>
-        <v/>
+        <v>17.2</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>-0.01149425287356318</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18802,11 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>142.35</v>
-      </c>
-      <c r="G9" s="13">
-        <f>(F9/E9-1)</f>
-        <v/>
+        <v>142.95</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>-0.01106883431338653</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,11 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.177</v>
-      </c>
-      <c r="G10" s="13">
-        <f>(F10/E10-1)</f>
-        <v/>
+        <v>0.176</v>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>-0.0537634408602151</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18866,9 +18857,8 @@
       <c r="F11" s="12" t="n">
         <v>226</v>
       </c>
-      <c r="G11" s="13">
-        <f>(F11/E11-1)</f>
-        <v/>
+      <c r="G11" s="13" t="n">
+        <v>-0.004405286343612335</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18977,9 +18967,8 @@
       <c r="F16" s="12" t="n">
         <v>0.081</v>
       </c>
-      <c r="G16" s="13">
-        <f>(F16/E16-1)</f>
-        <v/>
+      <c r="G16" s="13" t="n">
+        <v>-0.03571428571428575</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19008,9 +18997,8 @@
       <c r="F17" s="12" t="n">
         <v>0.547</v>
       </c>
-      <c r="G17" s="13">
-        <f>(F17/E17-1)</f>
-        <v/>
+      <c r="G17" s="13" t="n">
+        <v>0.005514705882352946</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19037,11 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.132</v>
-      </c>
-      <c r="G18" s="13">
-        <f>(F18/E18-1)</f>
-        <v/>
+        <v>2.108</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>-0.002838221381267637</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19068,11 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.374</v>
-      </c>
-      <c r="G19" s="13">
-        <f>(F19/E19-1)</f>
-        <v/>
+        <v>4.412</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>0.00136177939173859</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19099,11 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.58</v>
-      </c>
-      <c r="G20" s="13">
-        <f>(F20/E20-1)</f>
-        <v/>
+        <v>17.68</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>-0.004504504504504609</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19130,11 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>84.06</v>
-      </c>
-      <c r="G21" s="13">
-        <f>(F21/E21-1)</f>
-        <v/>
+        <v>84.06999999999999</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>-0.01094117647058832</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19161,11 +19145,10 @@
         <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>11.18</v>
-      </c>
-      <c r="G22" s="13">
-        <f>(F22/E22-1)</f>
-        <v/>
+        <v>11.2</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>0.009009009009008978</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19192,11 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.38</v>
-      </c>
-      <c r="G23" s="13">
-        <f>(F23/E23-1)</f>
-        <v/>
+        <v>10.4</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>-0.00687547746371268</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19223,11 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.284</v>
-      </c>
-      <c r="G24" s="13">
-        <f>(F24/E24-1)</f>
-        <v/>
+        <v>3.304</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.02672467371037907</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19254,11 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="G25" s="13">
-        <f>(F25/E25-1)</f>
-        <v/>
+        <v>24</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>-0.02834008097165989</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19368,11 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.832</v>
-      </c>
-      <c r="G30" s="13">
-        <f>(F30/E30-1)</f>
-        <v/>
+        <v>5.807</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>0.006063756063756088</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19398,11 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="G31" s="13">
-        <f>(F31/E31-1)</f>
-        <v/>
+        <v>4.34</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>-0.03982300884955747</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19428,11 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.91</v>
-      </c>
-      <c r="G32" s="13">
-        <f>(F32/E32-1)</f>
-        <v/>
+        <v>9.93</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>0.04746835443037967</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19458,11 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>48.05</v>
-      </c>
-      <c r="G33" s="13">
-        <f>(F33/E33-1)</f>
-        <v/>
+        <v>48.25</v>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>-0.04832347140039453</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19490,9 +19466,8 @@
       <c r="F34" s="12" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="G34" s="13">
-        <f>(F34/E34-1)</f>
-        <v/>
+      <c r="G34" s="13" t="n">
+        <v>-0.01473684210526322</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19520,9 +19495,8 @@
       <c r="F35" s="12" t="n">
         <v>0.419</v>
       </c>
-      <c r="G35" s="13">
-        <f>(F35/E35-1)</f>
-        <v/>
+      <c r="G35" s="13" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19550,9 +19524,8 @@
       <c r="F36" s="12" t="n">
         <v>1.03</v>
       </c>
-      <c r="G36" s="13">
-        <f>(F36/E36-1)</f>
-        <v/>
+      <c r="G36" s="13" t="n">
+        <v>-0.004830917874396033</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19578,11 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.143</v>
-      </c>
-      <c r="G37" s="13">
-        <f>(F37/E37-1)</f>
-        <v/>
+        <v>0.138</v>
+      </c>
+      <c r="G37" s="13" t="n">
+        <v>-0.02127659574468067</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19638,11 +19610,10 @@
         <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="G39" s="13">
-        <f>(F39/E39-1)</f>
-        <v/>
+        <v>5.75</v>
+      </c>
+      <c r="G39" s="13" t="n">
+        <v>0.008771929824561372</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19741,9 +19712,8 @@
       <c r="F43" s="12" t="n">
         <v>310</v>
       </c>
-      <c r="G43" s="13">
-        <f>(F43/E43-1)</f>
-        <v/>
+      <c r="G43" s="13" t="n">
+        <v>0.006493506493506494</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19771,9 +19741,8 @@
       <c r="F44" s="12" t="n">
         <v>226</v>
       </c>
-      <c r="G44" s="13">
-        <f>(F44/E44-1)</f>
-        <v/>
+      <c r="G44" s="13" t="n">
+        <v>-0.004405286343612335</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19801,9 +19770,8 @@
       <c r="F45" s="12" t="n">
         <v>34.65</v>
       </c>
-      <c r="G45" s="13">
-        <f>(F45/E45-1)</f>
-        <v/>
+      <c r="G45" s="13" t="n">
+        <v>0.002894356005788753</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19829,11 +19797,10 @@
         <v>87</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>87</v>
-      </c>
-      <c r="G46" s="13">
-        <f>(F46/E46-1)</f>
-        <v/>
+        <v>86.5</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <v>-0.005747126436781609</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19859,11 +19826,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.85</v>
-      </c>
-      <c r="G47" s="13">
-        <f>(F47/E47-1)</f>
-        <v/>
+        <v>6.885</v>
+      </c>
+      <c r="G47" s="13" t="n">
+        <v>-0.01572551822730526</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19889,11 +19855,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>161.2</v>
-      </c>
-      <c r="G48" s="13">
-        <f>(F48/E48-1)</f>
-        <v/>
+        <v>162.2</v>
+      </c>
+      <c r="G48" s="13" t="n">
+        <v>0.01059190031152641</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19921,9 +19886,8 @@
       <c r="F49" s="12" t="n">
         <v>62.1</v>
       </c>
-      <c r="G49" s="13">
-        <f>(F49/E49-1)</f>
-        <v/>
+      <c r="G49" s="13" t="n">
+        <v>-0.002409638554216845</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19949,11 +19913,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>171.38</v>
-      </c>
-      <c r="G50" s="13">
-        <f>(F50/E50-1)</f>
-        <v/>
+        <v>170.98</v>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>0.004818993888105273</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19979,11 +19942,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>133.3</v>
-      </c>
-      <c r="G51" s="13">
-        <f>(F51/E51-1)</f>
-        <v/>
+        <v>134.1</v>
+      </c>
+      <c r="G51" s="13" t="n">
+        <v>-0.01686217008797662</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -20009,11 +19971,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>271</v>
-      </c>
-      <c r="G52" s="13">
-        <f>(F52/E52-1)</f>
-        <v/>
+        <v>273.3</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>-0.09801980198019798</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21343,7 +21304,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 16:23</t>
+          <t>05/10/2026 16:51</t>
         </is>
       </c>
     </row>
@@ -21370,11 +21331,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.66</v>
-      </c>
-      <c r="G2" s="13">
-        <f>(F2/E2-1)</f>
-        <v/>
+        <v>15.74</v>
+      </c>
+      <c r="G2" s="13" t="n">
+        <v>-0.1000571755288736</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21401,11 +21361,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.36</v>
-      </c>
-      <c r="G3" s="13">
-        <f>(F3/E3-1)</f>
-        <v/>
+        <v>24.34</v>
+      </c>
+      <c r="G3" s="13" t="n">
+        <v>-0.03642121931908162</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21432,11 +21391,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="G4" s="13">
-        <f>(F4/E4-1)</f>
-        <v/>
+        <v>12.1</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>-0.02024291497975709</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21463,11 +21421,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.855</v>
-      </c>
-      <c r="G5" s="13">
-        <f>(F5/E5-1)</f>
-        <v/>
+        <v>7.87</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>-0.04836759371221275</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21494,11 +21451,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>60.65</v>
-      </c>
-      <c r="G6" s="13">
-        <f>(F6/E6-1)</f>
-        <v/>
+        <v>60.75</v>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>0.00164880461665295</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21525,11 +21481,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.735</v>
-      </c>
-      <c r="G7" s="13">
-        <f>(F7/E7-1)</f>
-        <v/>
+        <v>1.72</v>
+      </c>
+      <c r="G7" s="13" t="n">
+        <v>-0.1018276762402089</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21556,11 +21511,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="G8" s="13">
-        <f>(F8/E8-1)</f>
-        <v/>
+        <v>54</v>
+      </c>
+      <c r="G8" s="13" t="n">
+        <v>0.115702479338843</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21587,11 +21541,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="G9" s="13">
-        <f>(F9/E9-1)</f>
-        <v/>
+        <v>3.33</v>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>-0.08767123287671229</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21620,9 +21573,8 @@
       <c r="F10" s="12" t="n">
         <v>101</v>
       </c>
-      <c r="G10" s="13">
-        <f>(F10/E10-1)</f>
-        <v/>
+      <c r="G10" s="13" t="n">
+        <v>-0.01941747572815534</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21651,9 +21603,8 @@
       <c r="F11" s="12" t="n">
         <v>34.65</v>
       </c>
-      <c r="G11" s="13">
-        <f>(F11/E11-1)</f>
-        <v/>
+      <c r="G11" s="13" t="n">
+        <v>0.00434782608695648</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21760,11 +21711,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.67</v>
-      </c>
-      <c r="G16" s="13">
-        <f>(F16/E16-1)</f>
-        <v/>
+        <v>4.68</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>0.008620689655172422</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21791,11 +21741,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.374</v>
-      </c>
-      <c r="G17" s="13">
-        <f>(F17/E17-1)</f>
-        <v/>
+        <v>4.412</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>-0.160418648905804</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21824,9 +21773,8 @@
       <c r="F18" s="12" t="n">
         <v>4.005</v>
       </c>
-      <c r="G18" s="13">
-        <f>(F18/E18-1)</f>
-        <v/>
+      <c r="G18" s="13" t="n">
+        <v>-0.0462014765420338</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21853,11 +21801,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.34</v>
-      </c>
-      <c r="G19" s="13">
-        <f>(F19/E19-1)</f>
-        <v/>
+        <v>21.3</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>-0.1072925398155909</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21884,11 +21831,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.58</v>
-      </c>
-      <c r="G20" s="13">
-        <f>(F20/E20-1)</f>
-        <v/>
+        <v>17.68</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>-0.1580952380952381</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21915,11 +21861,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.457</v>
-      </c>
-      <c r="G21" s="13">
-        <f>(F21/E21-1)</f>
-        <v/>
+        <v>0.46</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>-0.1033138401559454</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21946,11 +21891,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.17</v>
-      </c>
-      <c r="G22" s="13">
-        <f>(F22/E22-1)</f>
-        <v/>
+        <v>7.21</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>-0.019047619047619</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21977,11 +21921,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.15</v>
-      </c>
-      <c r="G23" s="13">
-        <f>(F23/E23-1)</f>
-        <v/>
+        <v>29.35</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>0.01381692573402425</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -22008,11 +21951,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="G24" s="13">
-        <f>(F24/E24-1)</f>
-        <v/>
+        <v>51.9</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.02366863905325435</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22041,9 +21983,8 @@
       <c r="F25" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="G25" s="13">
-        <f>(F25/E25-1)</f>
-        <v/>
+      <c r="G25" s="13" t="n">
+        <v>-0.1304347826086958</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22153,11 +22094,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.832</v>
-      </c>
-      <c r="G30" s="13">
-        <f>(F30/E30-1)</f>
-        <v/>
+        <v>5.807</v>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>0.02056239015817223</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22183,11 +22123,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.109</v>
-      </c>
-      <c r="G31" s="13">
-        <f>(F31/E31-1)</f>
-        <v/>
+        <v>0.11</v>
+      </c>
+      <c r="G31" s="13" t="n">
+        <v>-0.03508771929824565</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22243,11 +22182,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.44</v>
-      </c>
-      <c r="G33" s="13">
-        <f>(F33/E33-1)</f>
-        <v/>
+        <v>4.34</v>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>0.1071428571428571</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22273,11 +22211,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>18.85</v>
-      </c>
-      <c r="G34" s="13">
-        <f>(F34/E34-1)</f>
-        <v/>
+        <v>19</v>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>-0.1284403669724771</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22305,9 +22242,8 @@
       <c r="F35" s="12" t="n">
         <v>0.858</v>
       </c>
-      <c r="G35" s="13">
-        <f>(F35/E35-1)</f>
-        <v/>
+      <c r="G35" s="13" t="n">
+        <v>-0.2473684210526315</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22333,11 +22269,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="G36" s="13">
-        <f>(F36/E36-1)</f>
-        <v/>
+        <v>4.7</v>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>-0.03688524590163929</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22363,11 +22298,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.65</v>
-      </c>
-      <c r="G37" s="13">
-        <f>(F37/E37-1)</f>
-        <v/>
+        <v>2.63</v>
+      </c>
+      <c r="G37" s="13" t="n">
+        <v>-0.1174496644295302</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22393,11 +22327,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.865</v>
-      </c>
-      <c r="G38" s="13">
-        <f>(F38/E38-1)</f>
-        <v/>
+        <v>4.89</v>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>-0.04492187500000008</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22423,11 +22356,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.143</v>
-      </c>
-      <c r="G39" s="13">
-        <f>(F39/E39-1)</f>
-        <v/>
+        <v>0.138</v>
+      </c>
+      <c r="G39" s="13" t="n">
+        <v>0.02222222222222224</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22524,11 +22456,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.855</v>
-      </c>
-      <c r="G43" s="13">
-        <f>(F43/E43-1)</f>
-        <v/>
+        <v>7.87</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>-0.04836759371221275</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22554,11 +22485,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="G44" s="13">
-        <f>(F44/E44-1)</f>
-        <v/>
+        <v>54</v>
+      </c>
+      <c r="G44" s="13" t="n">
+        <v>0.115702479338843</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22584,11 +22514,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="G45" s="13">
-        <f>(F45/E45-1)</f>
-        <v/>
+        <v>12.1</v>
+      </c>
+      <c r="G45" s="13" t="n">
+        <v>-0.02024291497975709</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22614,11 +22543,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>93.84</v>
-      </c>
-      <c r="G46" s="13">
-        <f>(F46/E46-1)</f>
-        <v/>
+        <v>94.09999999999999</v>
+      </c>
+      <c r="G46" s="13" t="n">
+        <v>-0.03506972928630026</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22646,9 +22574,8 @@
       <c r="F47" s="12" t="n">
         <v>101</v>
       </c>
-      <c r="G47" s="13">
-        <f>(F47/E47-1)</f>
-        <v/>
+      <c r="G47" s="13" t="n">
+        <v>-0.01941747572815534</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22676,9 +22603,8 @@
       <c r="F48" s="12" t="n">
         <v>8.869999999999999</v>
       </c>
-      <c r="G48" s="13">
-        <f>(F48/E48-1)</f>
-        <v/>
+      <c r="G48" s="13" t="n">
+        <v>-0.03376906318082794</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22704,11 +22630,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.65</v>
-      </c>
-      <c r="G49" s="13">
-        <f>(F49/E49-1)</f>
-        <v/>
+        <v>60.75</v>
+      </c>
+      <c r="G49" s="13" t="n">
+        <v>0.00164880461665295</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22734,11 +22659,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.735</v>
-      </c>
-      <c r="G50" s="13">
-        <f>(F50/E50-1)</f>
-        <v/>
+        <v>1.72</v>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>-0.1018276762402089</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22764,11 +22688,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="G51" s="13">
-        <f>(F51/E51-1)</f>
-        <v/>
+        <v>3.33</v>
+      </c>
+      <c r="G51" s="13" t="n">
+        <v>-0.08767123287671229</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22794,11 +22717,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.36</v>
-      </c>
-      <c r="G52" s="13">
-        <f>(F52/E52-1)</f>
-        <v/>
+        <v>24.34</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>-0.03642121931908162</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-05 19:50
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 16:51</t>
+          <t>05/10/2026 19:50</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>165.5</v>
+        <v>168.25</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.03046280023432917</v>
+        <v>-0.01435266549502044</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>50.91</v>
+        <v>50.92</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.0113230035756852</v>
+        <v>0.01152165276122365</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>42.66</v>
+        <v>42.6</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.001408450704225239</v>
+        <v>0</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.885</v>
+        <v>6.92</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01572551822730526</v>
+        <v>-0.01072194424588995</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>273.3</v>
+        <v>273.5</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.09801980198019798</v>
+        <v>-0.09735973597359736</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>142.95</v>
+        <v>143.15</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01106883431338653</v>
+        <v>-0.009685230024213114</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.176</v>
+        <v>0.174</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.0537634408602151</v>
+        <v>-0.06451612903225812</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.081</v>
+        <v>0.08</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.03571428571428575</v>
+        <v>-0.04761904761904766</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.547</v>
+        <v>0.54</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.005514705882352946</v>
+        <v>-0.007352941176470594</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.108</v>
+        <v>2.088</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.002838221381267637</v>
+        <v>-0.01229895931882678</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.412</v>
+        <v>4.482</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.00136177939173859</v>
+        <v>0.01724920562868827</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.68</v>
+        <v>17.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.004504504504504609</v>
+        <v>-0.01463963963963973</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>84.06999999999999</v>
+        <v>84.39</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.01094117647058832</v>
+        <v>-0.007176470588235288</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.4</v>
+        <v>10.386</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.00687547746371268</v>
+        <v>-0.008212375859434712</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.304</v>
+        <v>3.308</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02672467371037907</v>
+        <v>0.02796768178993159</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>24</v>
+        <v>23.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.02834008097165989</v>
+        <v>-0.03643724696356269</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.807</v>
+        <v>5.767</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.006063756063756088</v>
+        <v>-0.0008662508662508478</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.34</v>
+        <v>4.4</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03982300884955747</v>
+        <v>-0.02654867256637151</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.93</v>
+        <v>9.85</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.04746835443037967</v>
+        <v>0.03902953586497882</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>48.25</v>
+        <v>48.3</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04832347140039453</v>
+        <v>-0.04733727810650899</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.03</v>
+        <v>1.025</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.004830917874396033</v>
+        <v>-0.00966183574879228</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02127659574468067</v>
+        <v>-0.007092198581560094</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19580,11 +19580,10 @@
         <v>0.089</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="G38" s="13">
-        <f>(F38/E38-1)</f>
-        <v/>
+        <v>0.083</v>
+      </c>
+      <c r="G38" s="13" t="n">
+        <v>-0.06741573033707855</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19710,10 +19709,10 @@
         <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.006493506493506494</v>
+        <v>0.003246753246753247</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19768,10 +19767,10 @@
         <v>34.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>34.65</v>
+        <v>34.75</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.002894356005788753</v>
+        <v>0.005788712011577507</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19826,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.885</v>
+        <v>6.92</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01572551822730526</v>
+        <v>-0.01072194424588995</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19855,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>162.2</v>
+        <v>162</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.01059190031152641</v>
+        <v>0.009345794392523364</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19913,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>170.98</v>
+        <v>171.32</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.004818993888105273</v>
+        <v>0.006817113305124568</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19942,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>134.1</v>
+        <v>134.3</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01686217008797662</v>
+        <v>-0.01539589442815245</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19971,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>273.3</v>
+        <v>273.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.09801980198019798</v>
+        <v>-0.09735973597359736</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21304,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 16:51</t>
+          <t>05/10/2026 19:50</t>
         </is>
       </c>
     </row>
@@ -21331,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.74</v>
+        <v>15.7</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1000571755288736</v>
+        <v>-0.1023441966838193</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21391,10 +21390,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.02024291497975709</v>
+        <v>-0.02834008097165989</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21421,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.87</v>
+        <v>7.905</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.04836759371221275</v>
+        <v>-0.04413542926239412</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21451,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>60.75</v>
+        <v>61.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.00164880461665295</v>
+        <v>0.01236603462489695</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21541,10 +21540,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.33</v>
+        <v>3.35</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.08767123287671229</v>
+        <v>-0.08219178082191776</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21571,10 +21570,10 @@
         <v>103</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01941747572815534</v>
+        <v>-0.009708737864077669</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21601,10 +21600,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.65</v>
+        <v>34.75</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.00434782608695648</v>
+        <v>0.007246376811594203</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21711,10 +21710,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.68</v>
+        <v>4.73</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.008620689655172422</v>
+        <v>0.01939655172413809</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21741,10 +21740,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.412</v>
+        <v>4.482</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.160418648905804</v>
+        <v>-0.1470980019029495</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21771,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.005</v>
+        <v>3.973</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0462014765420338</v>
+        <v>-0.05382233865206001</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21801,10 +21800,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.3</v>
+        <v>21.36</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1072925398155909</v>
+        <v>-0.104777870913663</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21831,10 +21830,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.68</v>
+        <v>17.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1580952380952381</v>
+        <v>-0.1666666666666667</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21861,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.46</v>
+        <v>0.458</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1033138401559454</v>
+        <v>-0.1072124756335282</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21891,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.21</v>
+        <v>7.18</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.019047619047619</v>
+        <v>-0.02312925170068026</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21921,10 +21920,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.35</v>
+        <v>29.1</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01381692573402425</v>
+        <v>0.005181347150259141</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21951,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>51.9</v>
+        <v>51.6</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02366863905325435</v>
+        <v>0.0177514792899408</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21981,10 +21980,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.06</v>
+        <v>0.057</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1304347826086958</v>
+        <v>-0.1739130434782609</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22094,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.807</v>
+        <v>5.767</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.02056239015817223</v>
+        <v>0.01353251318101932</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22123,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.11</v>
+        <v>0.109</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03508771929824565</v>
+        <v>-0.04385964912280706</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22152,11 +22151,10 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.089</v>
-      </c>
-      <c r="G32" s="13">
-        <f>(F32/E32-1)</f>
-        <v/>
+        <v>0.083</v>
+      </c>
+      <c r="G32" s="13" t="n">
+        <v>-0.05681818181818171</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22182,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.34</v>
+        <v>4.4</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1224489795918368</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22211,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>19</v>
+        <v>18.8</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1284403669724771</v>
+        <v>-0.1376146788990826</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22240,10 +22238,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.858</v>
+        <v>0.866</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.2473684210526315</v>
+        <v>-0.2403508771929824</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22298,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.63</v>
+        <v>2.55</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1174496644295302</v>
+        <v>-0.1442953020134229</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22327,10 +22325,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.89</v>
+        <v>4.87</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.04492187500000008</v>
+        <v>-0.048828125</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22356,10 +22354,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.02222222222222224</v>
+        <v>0.03703703703703707</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22456,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.87</v>
+        <v>7.905</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.04836759371221275</v>
+        <v>-0.04413542926239412</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22514,10 +22512,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12.1</v>
+        <v>12</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.02024291497975709</v>
+        <v>-0.02834008097165989</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22543,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>94.09999999999999</v>
+        <v>93.95999999999999</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.03506972928630026</v>
+        <v>-0.03650533223954063</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22572,10 +22570,10 @@
         <v>103</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01941747572815534</v>
+        <v>-0.009708737864077669</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22630,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>60.75</v>
+        <v>61.4</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.00164880461665295</v>
+        <v>0.01236603462489695</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22688,10 +22686,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.33</v>
+        <v>3.35</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.08767123287671229</v>
+        <v>-0.08219178082191776</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-06 14:01
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 19:50</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>168.25</v>
+        <v>167.6</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01435266549502044</v>
+        <v>-0.01816051552431163</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>50.92</v>
+        <v>52.01</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01152165276122365</v>
+        <v>0.03317441398490256</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>42.6</v>
+        <v>43.68</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0</v>
+        <v>0.0253521126760563</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.92</v>
+        <v>6.925</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01072194424588995</v>
+        <v>-0.01000714796283063</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54</v>
+        <v>54.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.003690036900369056</v>
+        <v>0.003690036900368925</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>273.5</v>
+        <v>263.85</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.09735973597359736</v>
+        <v>-0.1292079207920791</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>143.15</v>
+        <v>146.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.009685230024213114</v>
+        <v>0.01556554825319958</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.174</v>
+        <v>0.178</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.06451612903225812</v>
+        <v>-0.04301075268817208</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>227</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>226</v>
+        <v>225.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.004405286343612335</v>
+        <v>-0.006607929515418502</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.08</v>
+        <v>0.083</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04761904761904766</v>
+        <v>-0.01190476190476191</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.54</v>
+        <v>0.556</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.007352941176470594</v>
+        <v>0.02205882352941178</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.088</v>
+        <v>2.188</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.01229895931882678</v>
+        <v>0.03500473036896892</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01463963963963973</v>
+        <v>-0.02027027027027044</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>84.39</v>
+        <v>87.33</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.007176470588235288</v>
+        <v>0.02741176470588233</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.386</v>
+        <v>10.902</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.008212375859434712</v>
+        <v>0.04106187929717339</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.308</v>
+        <v>3.368</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02796768178993159</v>
+        <v>0.04661280298321936</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.8</v>
+        <v>23.6</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.03643724696356269</v>
+        <v>-0.0445344129554655</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.767</v>
+        <v>5.857</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.0008662508662508478</v>
+        <v>0.01472626472626472</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.4</v>
+        <v>4.28</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02654867256637151</v>
+        <v>-0.05309734513274322</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.85</v>
+        <v>10</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.03902953586497882</v>
+        <v>0.05485232067510544</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>48.3</v>
+        <v>50.8</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04733727810650899</v>
+        <v>0.001972386587771091</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19464,10 +19464,10 @@
         <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.359999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.01473684210526322</v>
+        <v>0.04210526315789478</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.025</v>
+        <v>1.02</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.00966183574879228</v>
+        <v>-0.01449275362318831</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.14</v>
+        <v>0.139</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.007092198581560094</v>
+        <v>-0.01418439716312038</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19609,10 +19609,10 @@
         <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.75</v>
+        <v>5.65</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.008771929824561372</v>
+        <v>-0.008771929824561372</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19709,10 +19709,10 @@
         <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>309</v>
+        <v>314.5</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.003246753246753247</v>
+        <v>0.0211038961038961</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19738,10 +19738,10 @@
         <v>227</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>226</v>
+        <v>225.5</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.004405286343612335</v>
+        <v>-0.006607929515418502</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19767,10 +19767,10 @@
         <v>34.55</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>34.75</v>
+        <v>34.6</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.005788712011577507</v>
+        <v>0.001447178002894479</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19825,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.92</v>
+        <v>6.925</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01072194424588995</v>
+        <v>-0.01000714796283063</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19854,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>162</v>
+        <v>162.6</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.009345794392523364</v>
+        <v>0.01308411214953267</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19883,10 +19883,10 @@
         <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>62.1</v>
+        <v>62.35</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.002409638554216845</v>
+        <v>0.001606425702811268</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19912,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>171.32</v>
+        <v>169.44</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.006817113305124568</v>
+        <v>-0.004231311706629048</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19941,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>134.3</v>
+        <v>134.1</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01539589442815245</v>
+        <v>-0.01686217008797662</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19970,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>273.5</v>
+        <v>263.85</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.09735973597359736</v>
+        <v>-0.1292079207920791</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>05/10/2026 19:50</t>
+          <t>06/10/2026 14:01</t>
         </is>
       </c>
     </row>
@@ -21330,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.7</v>
+        <v>15.88</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1023441966838193</v>
+        <v>-0.09205260148656362</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21360,10 +21360,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.34</v>
+        <v>24.58</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03642121931908162</v>
+        <v>-0.02692003167062562</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21390,10 +21390,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.02834008097165989</v>
+        <v>-0.0445344129554655</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21420,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.905</v>
+        <v>7.59</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.04413542926239412</v>
+        <v>-0.08222490931076176</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21450,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>61.4</v>
+        <v>59.4</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01236603462489695</v>
+        <v>-0.02061005770816158</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21480,10 +21480,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.72</v>
+        <v>1.795</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.1018276762402089</v>
+        <v>-0.06266318537859013</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21510,10 +21510,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>54</v>
+        <v>54.4</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.115702479338843</v>
+        <v>0.1239669421487603</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21540,10 +21540,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.35</v>
+        <v>3.425</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.08219178082191776</v>
+        <v>-0.06164383561643838</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21570,10 +21570,10 @@
         <v>103</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.009708737864077669</v>
+        <v>-0.01941747572815534</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21600,10 +21600,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.75</v>
+        <v>34.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.007246376811594203</v>
+        <v>0.002898550724637722</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21710,10 +21710,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.73</v>
+        <v>4.86</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.01939655172413809</v>
+        <v>0.04741379310344842</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21770,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.973</v>
+        <v>4.095</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.05382233865206001</v>
+        <v>-0.02476780185758516</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21800,10 +21800,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.36</v>
+        <v>21.8</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.104777870913663</v>
+        <v>-0.0863369656328583</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21830,10 +21830,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1666666666666667</v>
+        <v>-0.1714285714285715</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21860,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.458</v>
+        <v>0.475</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1072124756335282</v>
+        <v>-0.07407407407407414</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21890,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.18</v>
+        <v>7.27</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02312925170068026</v>
+        <v>-0.01088435374149661</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21920,10 +21920,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.1</v>
+        <v>29.6</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.005181347150259141</v>
+        <v>0.02245250431778937</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21950,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>51.6</v>
+        <v>52.6</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.0177514792899408</v>
+        <v>0.03747534516765283</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21980,10 +21980,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.057</v>
+        <v>0.06</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1739130434782609</v>
+        <v>-0.1304347826086958</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22093,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.767</v>
+        <v>5.857</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01353251318101932</v>
+        <v>0.02934973637961332</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22122,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.109</v>
+        <v>0.113</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.04385964912280706</v>
+        <v>-0.008771929824561412</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22180,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.4</v>
+        <v>4.28</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.1224489795918368</v>
+        <v>0.09183673469387764</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22209,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>18.8</v>
+        <v>18.1</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1376146788990826</v>
+        <v>-0.1697247706422018</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22238,10 +22238,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.866</v>
+        <v>0.874</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.2403508771929824</v>
+        <v>-0.2333333333333333</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22267,10 +22267,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.7</v>
+        <v>4.79</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03688524590163929</v>
+        <v>-0.01844262295081964</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22296,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.55</v>
+        <v>2.6</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1442953020134229</v>
+        <v>-0.1275167785234899</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22325,10 +22325,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.87</v>
+        <v>4.92</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.048828125</v>
+        <v>-0.03906250000000003</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22354,10 +22354,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.14</v>
+        <v>0.139</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.03703703703703707</v>
+        <v>0.02962962962962966</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22454,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.905</v>
+        <v>7.59</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.04413542926239412</v>
+        <v>-0.08222490931076176</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22483,10 +22483,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>54</v>
+        <v>54.4</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.115702479338843</v>
+        <v>0.1239669421487603</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22512,10 +22512,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>12</v>
+        <v>11.8</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.02834008097165989</v>
+        <v>-0.0445344129554655</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22541,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>93.95999999999999</v>
+        <v>94.95999999999999</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.03650533223954063</v>
+        <v>-0.02625102543068091</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22570,10 +22570,10 @@
         <v>103</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.009708737864077669</v>
+        <v>-0.01941747572815534</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22599,10 +22599,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.869999999999999</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03376906318082794</v>
+        <v>-0.03267973856209139</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22628,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>61.4</v>
+        <v>59.4</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01236603462489695</v>
+        <v>-0.02061005770816158</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22657,10 +22657,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.72</v>
+        <v>1.795</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1018276762402089</v>
+        <v>-0.06266318537859013</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22686,10 +22686,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.35</v>
+        <v>3.425</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.08219178082191776</v>
+        <v>-0.06164383561643838</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22715,10 +22715,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.34</v>
+        <v>24.58</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03642121931908162</v>
+        <v>-0.02692003167062562</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-06 14:34
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>06/10/2026 14:34</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>167.6</v>
+        <v>167.2</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01816051552431163</v>
+        <v>-0.02050380785002929</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>52.01</v>
+        <v>51.76</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.03317441398490256</v>
+        <v>0.02820818434644407</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>43.68</v>
+        <v>43.72</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.0253521126760563</v>
+        <v>0.02629107981220651</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.925</v>
+        <v>6.92</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01000714796283063</v>
+        <v>-0.01072194424588995</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>263.85</v>
+        <v>262.8</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.1292079207920791</v>
+        <v>-0.1326732673267326</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>146.8</v>
+        <v>146.5</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01556554825319958</v>
+        <v>0.01349014181943956</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.178</v>
+        <v>0.179</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.04301075268817208</v>
+        <v>-0.03763440860215057</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.188</v>
+        <v>2.196</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.03500473036896892</v>
+        <v>0.03878902554399257</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.482</v>
+        <v>4.488</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01724920562868827</v>
+        <v>0.01861098502042686</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>87.33</v>
+        <v>87.27</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.02741176470588233</v>
+        <v>0.02670588235294113</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.902</v>
+        <v>10.892</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.04106187929717339</v>
+        <v>0.04010695187165775</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.368</v>
+        <v>3.382</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.04661280298321936</v>
+        <v>0.05096333126165325</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.6</v>
+        <v>23.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0445344129554655</v>
+        <v>-0.03643724696356269</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.857</v>
+        <v>5.889</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.01472626472626472</v>
+        <v>0.02027027027027027</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.28</v>
+        <v>4.3</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.05309734513274322</v>
+        <v>-0.04867256637168137</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>10</v>
+        <v>10.04</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.05485232067510544</v>
+        <v>0.05907172995780577</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>50.8</v>
+        <v>51</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.001972386587771091</v>
+        <v>0.005917159763313553</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.139</v>
+        <v>0.137</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01418439716312038</v>
+        <v>-0.02836879432624097</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19825,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.925</v>
+        <v>6.92</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01000714796283063</v>
+        <v>-0.01072194424588995</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19854,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>162.6</v>
+        <v>162.9</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.01308411214953267</v>
+        <v>0.01495327102803742</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19883,10 +19883,10 @@
         <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>62.35</v>
+        <v>62.25</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.001606425702811268</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19912,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>169.44</v>
+        <v>169.62</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.004231311706629048</v>
+        <v>-0.003173483779971745</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19941,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>134.1</v>
+        <v>133.3</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.01686217008797662</v>
+        <v>-0.02272727272727269</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19970,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>263.85</v>
+        <v>262.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.1292079207920791</v>
+        <v>-0.1326732673267326</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 14:01</t>
+          <t>06/10/2026 14:34</t>
         </is>
       </c>
     </row>
@@ -21330,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.88</v>
+        <v>15.82</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.09205260148656362</v>
+        <v>-0.09548313321898218</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21420,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.59</v>
+        <v>7.57</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.08222490931076176</v>
+        <v>-0.08464328899637234</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21450,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>59.4</v>
+        <v>58.9</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.02061005770816158</v>
+        <v>-0.02885408079142622</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21740,10 +21740,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.482</v>
+        <v>4.488</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1470980019029495</v>
+        <v>-0.1459562321598477</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21770,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.095</v>
+        <v>4.068</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02476780185758516</v>
+        <v>-0.0311979042629198</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21860,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.475</v>
+        <v>0.476</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.07407407407407414</v>
+        <v>-0.07212475633528272</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21890,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.27</v>
+        <v>7.28</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01088435374149661</v>
+        <v>-0.009523809523809441</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21950,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52.6</v>
+        <v>52.7</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03747534516765283</v>
+        <v>0.03944773175542406</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22093,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.857</v>
+        <v>5.889</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.02934973637961332</v>
+        <v>0.03497363796133564</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22122,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.113</v>
+        <v>0.114</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.008771929824561412</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22180,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.28</v>
+        <v>4.3</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.09183673469387764</v>
+        <v>0.09693877551020405</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22209,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>18.1</v>
+        <v>18.4</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1697247706422018</v>
+        <v>-0.1559633027522937</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22267,10 +22267,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.79</v>
+        <v>4.72</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.01844262295081964</v>
+        <v>-0.03278688524590167</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22296,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.6</v>
+        <v>2.445</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1275167785234899</v>
+        <v>-0.1795302013422819</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22354,10 +22354,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.139</v>
+        <v>0.137</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.02962962962962966</v>
+        <v>0.01481481481481483</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22454,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.59</v>
+        <v>7.57</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.08222490931076176</v>
+        <v>-0.08464328899637234</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22541,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>94.95999999999999</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02625102543068091</v>
+        <v>-0.02481542247744054</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22628,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>59.4</v>
+        <v>58.9</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.02061005770816158</v>
+        <v>-0.02885408079142622</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-06 19:06
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 14:34</t>
+          <t>06/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>167.2</v>
+        <v>167.45</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02050380785002929</v>
+        <v>-0.01903925014645577</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>51.76</v>
+        <v>52.14</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.02820818434644407</v>
+        <v>0.03575685339690102</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>43.72</v>
+        <v>43.36</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02629107981220651</v>
+        <v>0.01784037558685441</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.92</v>
+        <v>6.845</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.01072194424588995</v>
+        <v>-0.02144388849177989</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>262.8</v>
+        <v>262.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.1326732673267326</v>
+        <v>-0.1339933993399341</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>17.2</v>
+        <v>17.15</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01149425287356318</v>
+        <v>-0.01436781609195402</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>146.5</v>
+        <v>148.1</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01349014181943956</v>
+        <v>0.02455897613282589</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.179</v>
+        <v>0.183</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.03763440860215057</v>
+        <v>-0.01612903225806453</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.083</v>
+        <v>0.08</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01190476190476191</v>
+        <v>-0.04761904761904766</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.556</v>
+        <v>0.546</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02205882352941178</v>
+        <v>0.003676470588235297</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.196</v>
+        <v>2.14</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.03878902554399257</v>
+        <v>0.01229895931882699</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.488</v>
+        <v>4.518</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01861098502042686</v>
+        <v>0.02541988197911941</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02027027027027044</v>
+        <v>-0.009009009009009016</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>87.27</v>
+        <v>86.14</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.02670588235294113</v>
+        <v>0.01341176470588236</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>11.2</v>
+        <v>11.02</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.009009009009008978</v>
+        <v>-0.007207207207207214</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.892</v>
+        <v>10.64</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.04010695187165775</v>
+        <v>0.0160427807486632</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.382</v>
+        <v>3.344</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.05096333126165325</v>
+        <v>0.03915475450590426</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.8</v>
+        <v>23.7</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.03643724696356269</v>
+        <v>-0.04048582995951417</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.889</v>
+        <v>5.836</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.02027027027027027</v>
+        <v>0.0110880110880111</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.04867256637168137</v>
+        <v>-0.02654867256637151</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>10.04</v>
+        <v>9.83</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.05907172995780577</v>
+        <v>0.03691983122362865</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>51</v>
+        <v>49.9</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.005917159763313553</v>
+        <v>-0.01577909270216971</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19464,10 +19464,10 @@
         <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.9</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.04210526315789478</v>
+        <v>0.0210526315789473</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.02</v>
+        <v>1.025</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.01449275362318831</v>
+        <v>-0.00966183574879228</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.137</v>
+        <v>0.139</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02836879432624097</v>
+        <v>-0.01418439716312038</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19580,10 +19580,10 @@
         <v>0.089</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.083</v>
+        <v>0.089</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.06741573033707855</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19609,10 +19609,10 @@
         <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.65</v>
+        <v>5.5</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.008771929824561372</v>
+        <v>-0.03508771929824565</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19709,10 +19709,10 @@
         <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>314.5</v>
+        <v>310</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0211038961038961</v>
+        <v>0.006493506493506494</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19825,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.92</v>
+        <v>6.845</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01072194424588995</v>
+        <v>-0.02144388849177989</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19854,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>162.9</v>
+        <v>164.4</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.01495327102803742</v>
+        <v>0.02429906542056078</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19912,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>169.62</v>
+        <v>169.58</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.003173483779971745</v>
+        <v>-0.003408556652562201</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19941,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>133.3</v>
+        <v>133</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02272727272727269</v>
+        <v>-0.02492668621700884</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19970,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>262.8</v>
+        <v>262.4</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.1326732673267326</v>
+        <v>-0.1339933993399341</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 14:34</t>
+          <t>06/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -21330,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.82</v>
+        <v>15.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.09548313321898218</v>
+        <v>-0.096626643796455</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21360,10 +21360,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.58</v>
+        <v>24.4</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02692003167062562</v>
+        <v>-0.03404592240696765</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21390,10 +21390,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.0445344129554655</v>
+        <v>-0.03643724696356269</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21420,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.57</v>
+        <v>7.685</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.08464328899637234</v>
+        <v>-0.07073760580411124</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21450,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>58.9</v>
+        <v>56.85</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.02885408079142622</v>
+        <v>-0.06265457543281117</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21540,10 +21540,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.425</v>
+        <v>3.44</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.06164383561643838</v>
+        <v>-0.05753424657534246</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21710,10 +21710,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.86</v>
+        <v>4.87</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.04741379310344842</v>
+        <v>0.04956896551724147</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21740,10 +21740,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.488</v>
+        <v>4.518</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1459562321598477</v>
+        <v>-0.1402473834443387</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21770,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.068</v>
+        <v>4.074</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0311979042629198</v>
+        <v>-0.02976899261728983</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21800,10 +21800,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.8</v>
+        <v>21.74</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.0863369656328583</v>
+        <v>-0.0888516345347863</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21830,10 +21830,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.4</v>
+        <v>17.6</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1714285714285715</v>
+        <v>-0.1619047619047618</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21860,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.476</v>
+        <v>0.468</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.07212475633528272</v>
+        <v>-0.087719298245614</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21890,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.28</v>
+        <v>7.26</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.009523809523809441</v>
+        <v>-0.01224489795918366</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21920,10 +21920,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.6</v>
+        <v>29.65</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02245250431778937</v>
+        <v>0.02417962003454229</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21950,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52.7</v>
+        <v>52.5</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03944773175542406</v>
+        <v>0.0355029585798816</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21980,10 +21980,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.06</v>
+        <v>0.056</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1304347826086958</v>
+        <v>-0.1884057971014493</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22093,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.889</v>
+        <v>5.836</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.03497363796133564</v>
+        <v>0.02565905096660807</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22122,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.114</v>
+        <v>0.124</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>0.08771929824561399</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22151,10 +22151,10 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.083</v>
+        <v>0.089</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.05681818181818171</v>
+        <v>0.01136363636363637</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22180,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.09693877551020405</v>
+        <v>0.1224489795918368</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22209,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>18.4</v>
+        <v>17.7</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1559633027522937</v>
+        <v>-0.1880733944954129</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22296,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.445</v>
+        <v>2.405</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1795302013422819</v>
+        <v>-0.1929530201342282</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22325,10 +22325,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.92</v>
+        <v>4.935</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03906250000000003</v>
+        <v>-0.0361328125000001</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22354,10 +22354,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.137</v>
+        <v>0.139</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.01481481481481483</v>
+        <v>0.02962962962962966</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22454,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.57</v>
+        <v>7.685</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.08464328899637234</v>
+        <v>-0.07073760580411124</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22512,10 +22512,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>11.8</v>
+        <v>11.9</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.0445344129554655</v>
+        <v>-0.03643724696356269</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22541,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.09999999999999</v>
+        <v>94.76000000000001</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02481542247744054</v>
+        <v>-0.02830188679245274</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22599,10 +22599,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.880000000000001</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03267973856209139</v>
+        <v>-0.0348583877995643</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22628,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>58.9</v>
+        <v>56.85</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.02885408079142622</v>
+        <v>-0.06265457543281117</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22686,10 +22686,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.425</v>
+        <v>3.44</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.06164383561643838</v>
+        <v>-0.05753424657534246</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22715,10 +22715,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.58</v>
+        <v>24.4</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02692003167062562</v>
+        <v>-0.03404592240696765</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-06 20:47
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 19:06</t>
+          <t>06/10/2026 20:47</t>
         </is>
       </c>
     </row>
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 19:06</t>
+          <t>06/10/2026 20:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-07 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 20:47</t>
+          <t>07/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>167.45</v>
+        <v>161.05</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01903925014645577</v>
+        <v>-0.05653192735793777</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>52.14</v>
+        <v>50.11</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.03575685339690102</v>
+        <v>-0.004568931267381882</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>43.36</v>
+        <v>41.98</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01784037558685441</v>
+        <v>-0.01455399061032875</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.845</v>
+        <v>6.46</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02144388849177989</v>
+        <v>-0.07648320228734813</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.4</v>
+        <v>54.2</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.003690036900368925</v>
+        <v>0</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>262.4</v>
+        <v>258.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.1339933993399341</v>
+        <v>-0.1478547854785479</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>17.15</v>
+        <v>17.2</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01436781609195402</v>
+        <v>-0.01149425287356318</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>148.1</v>
+        <v>144.4</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02455897613282589</v>
+        <v>-0.001037703216880012</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.183</v>
+        <v>0.184</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01612903225806453</v>
+        <v>-0.01075268817204302</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>227</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>225.5</v>
+        <v>227</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.006607929515418502</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.08</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.04761904761904766</v>
+        <v>0.01190476190476191</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.546</v>
+        <v>0.534</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.003676470588235297</v>
+        <v>-0.01838235294117649</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.14</v>
+        <v>2.148</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01229895931882699</v>
+        <v>0.01608325449385064</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.518</v>
+        <v>4.644</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.02541988197911941</v>
+        <v>0.05401724920562879</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.6</v>
+        <v>14.8</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.009009009009009016</v>
+        <v>-0.1666666666666667</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>86.14</v>
+        <v>87.18000000000001</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01341176470588236</v>
+        <v>0.02564705882352949</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>11.02</v>
+        <v>10.78</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.007207207207207214</v>
+        <v>-0.02882882882882886</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.64</v>
+        <v>10.374</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.0160427807486632</v>
+        <v>-0.009358288770053378</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.344</v>
+        <v>3.33</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03915475450590426</v>
+        <v>0.03480422622747051</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.7</v>
+        <v>23.5</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.04048582995951417</v>
+        <v>-0.04858299595141698</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.836</v>
+        <v>5.421</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.0110880110880111</v>
+        <v>-0.06081081081081081</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.4</v>
+        <v>4.19</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02654867256637151</v>
+        <v>-0.07300884955752195</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.83</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.03691983122362865</v>
+        <v>0.007383966244725768</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>49.9</v>
+        <v>48.55</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01577909270216971</v>
+        <v>-0.04240631163708098</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19464,10 +19464,10 @@
         <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.699999999999999</v>
+        <v>9.66</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.0210526315789473</v>
+        <v>0.01684210526315791</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19493,10 +19493,10 @@
         <v>0.419</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.419</v>
+        <v>0.418</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>-0.002386634844868737</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.035</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.025</v>
+        <v>1.015</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.00966183574879228</v>
+        <v>-0.01932367149758456</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>0.141</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.139</v>
+        <v>0.125</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01418439716312038</v>
+        <v>-0.1134751773049645</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19609,10 +19609,10 @@
         <v>5.7</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.03508771929824565</v>
+        <v>-0.0175438596491229</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19709,10 +19709,10 @@
         <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.006493506493506494</v>
+        <v>0.01948051948051948</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19738,10 +19738,10 @@
         <v>227</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>225.5</v>
+        <v>227</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.006607929515418502</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19825,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.845</v>
+        <v>6.46</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.02144388849177989</v>
+        <v>-0.07648320228734813</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19854,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>164.4</v>
+        <v>162.1</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.02429906542056078</v>
+        <v>0.009968847352024886</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19883,10 +19883,10 @@
         <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>62.25</v>
+        <v>62.35</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0</v>
+        <v>0.001606425702811268</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19912,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>169.58</v>
+        <v>168.7</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.003408556652562201</v>
+        <v>-0.008580159849553409</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19941,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>133</v>
+        <v>130.2</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.02492668621700884</v>
+        <v>-0.04545454545454558</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19970,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>262.4</v>
+        <v>258.2</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.1339933993399341</v>
+        <v>-0.1478547854785479</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>06/10/2026 20:47</t>
+          <t>07/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21330,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.8</v>
+        <v>15.62</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.096626643796455</v>
+        <v>-0.1069182389937107</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21360,10 +21360,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.4</v>
+        <v>24.52</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03404592240696765</v>
+        <v>-0.02929532858273958</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21390,10 +21390,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>11.9</v>
+        <v>11.65</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.03643724696356269</v>
+        <v>-0.05668016194331978</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21420,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.685</v>
+        <v>7.91</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.07073760580411124</v>
+        <v>-0.04353083434099147</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21450,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.85</v>
+        <v>57.15</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.06265457543281117</v>
+        <v>-0.05770816158285243</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21480,10 +21480,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.795</v>
+        <v>1.81</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.06266318537859013</v>
+        <v>-0.05483028720626631</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21510,10 +21510,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>54.4</v>
+        <v>54.2</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.1239669421487603</v>
+        <v>0.1198347107438017</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21540,10 +21540,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.44</v>
+        <v>3.455</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.05753424657534246</v>
+        <v>-0.05342465753424654</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21570,10 +21570,10 @@
         <v>103</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01941747572815534</v>
+        <v>-0.009708737864077669</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21710,10 +21710,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.87</v>
+        <v>4.785</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.04956896551724147</v>
+        <v>0.0312500000000001</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21740,10 +21740,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.518</v>
+        <v>4.644</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1402473834443387</v>
+        <v>-0.1162702188392007</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21770,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.074</v>
+        <v>4.095</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02976899261728983</v>
+        <v>-0.02476780185758516</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21800,10 +21800,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.74</v>
+        <v>22.14</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.0888516345347863</v>
+        <v>-0.07208717518860012</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21830,10 +21830,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>17.6</v>
+        <v>14.8</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1619047619047618</v>
+        <v>-0.2952380952380952</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21860,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.468</v>
+        <v>0.463</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.087719298245614</v>
+        <v>-0.09746588693957113</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21890,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.26</v>
+        <v>7.37</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01224489795918366</v>
+        <v>0.002721088435374213</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21920,10 +21920,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.65</v>
+        <v>29.2</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02417962003454229</v>
+        <v>0.008635578583765112</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21950,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52.5</v>
+        <v>52</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.0355029585798816</v>
+        <v>0.02564102564102558</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22093,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.836</v>
+        <v>5.421</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.02565905096660807</v>
+        <v>-0.04727592267135327</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22122,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.124</v>
+        <v>0.128</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.08771929824561399</v>
+        <v>0.1228070175438596</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22180,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.4</v>
+        <v>4.19</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.1224489795918368</v>
+        <v>0.06887755102040828</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22209,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>17.7</v>
+        <v>17.8</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1880733944954129</v>
+        <v>-0.1834862385321101</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22238,10 +22238,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.874</v>
+        <v>0.9</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.2333333333333333</v>
+        <v>-0.2105263157894736</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22267,10 +22267,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.72</v>
+        <v>4.82</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03278688524590167</v>
+        <v>-0.01229508196721303</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22296,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.405</v>
+        <v>2.565</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1929530201342282</v>
+        <v>-0.139261744966443</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22325,10 +22325,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.935</v>
+        <v>4.985</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.0361328125000001</v>
+        <v>-0.02636718749999996</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22354,10 +22354,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.139</v>
+        <v>0.125</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.02962962962962966</v>
+        <v>-0.07407407407407414</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22454,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.685</v>
+        <v>7.91</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.07073760580411124</v>
+        <v>-0.04353083434099147</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22483,10 +22483,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>54.4</v>
+        <v>54.2</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.1239669421487603</v>
+        <v>0.1198347107438017</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22512,10 +22512,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>11.9</v>
+        <v>11.65</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.03643724696356269</v>
+        <v>-0.05668016194331978</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22541,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>94.76000000000001</v>
+        <v>94.94</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02830188679245274</v>
+        <v>-0.02645611156685806</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22570,10 +22570,10 @@
         <v>103</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01941747572815534</v>
+        <v>-0.009708737864077669</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22599,10 +22599,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.859999999999999</v>
+        <v>8.84</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.0348583877995643</v>
+        <v>-0.03703703703703702</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22628,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>56.85</v>
+        <v>57.15</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.06265457543281117</v>
+        <v>-0.05770816158285243</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22657,10 +22657,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.795</v>
+        <v>1.81</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.06266318537859013</v>
+        <v>-0.05483028720626631</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22686,10 +22686,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.44</v>
+        <v>3.455</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.05753424657534246</v>
+        <v>-0.05342465753424654</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22715,10 +22715,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.4</v>
+        <v>24.52</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03404592240696765</v>
+        <v>-0.02929532858273958</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-07 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>07/10/2026 13:00</t>
+          <t>07/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>170.7</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>161.05</v>
+        <v>159.9</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.05653192735793777</v>
+        <v>-0.063268892794376</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>50.34</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>50.11</v>
+        <v>49.85</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.004568931267381882</v>
+        <v>-0.009733810091378664</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>42.6</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>41.98</v>
+        <v>40.18</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01455399061032875</v>
+        <v>-0.05680751173708924</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>6.995</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>6.46</v>
+        <v>6.515</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.07648320228734813</v>
+        <v>-0.06862044317369556</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>54.2</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.2</v>
+        <v>50.8</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0</v>
+        <v>-0.06273062730627317</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>303</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>258.2</v>
+        <v>252</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.1478547854785479</v>
+        <v>-0.1683168316831683</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>17.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>17.2</v>
+        <v>17</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01149425287356318</v>
+        <v>-0.02298850574712636</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>144.55</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>144.4</v>
+        <v>141.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.001037703216880012</v>
+        <v>-0.02040816326530624</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>0.186</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.184</v>
+        <v>0.175</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01075268817204302</v>
+        <v>-0.05913978494623661</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>227</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>227</v>
+        <v>225.5</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>-0.006607929515418502</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>0.08400000000000001</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.01190476190476191</v>
+        <v>-0.01190476190476191</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>0.544</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.534</v>
+        <v>0.528</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01838235294117649</v>
+        <v>-0.02941176470588238</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>2.114</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.148</v>
+        <v>2.138</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01608325449385064</v>
+        <v>0.01135288552507097</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>4.406</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>4.644</v>
+        <v>4.742</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.05401724920562879</v>
+        <v>0.07625964593735822</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>17.76</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.1666666666666667</v>
+        <v>-0.1835585585585586</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>85</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>87.18000000000001</v>
+        <v>86.34999999999999</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.02564705882352949</v>
+        <v>0.0158823529411764</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>11.1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.78</v>
+        <v>10.54</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02882882882882886</v>
+        <v>-0.0504504504504505</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>10.472</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>10.374</v>
+        <v>10.378</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.009358288770053378</v>
+        <v>-0.008976317799847157</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>3.218</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>3.33</v>
+        <v>3.274</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03480422622747051</v>
+        <v>0.01740211311373525</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>24.7</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>23.5</v>
+        <v>22.9</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.04858299595141698</v>
+        <v>-0.07287449392712554</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>5.772</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.421</v>
+        <v>5.37</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06081081081081081</v>
+        <v>-0.06964656964656966</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>4.52</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>4.19</v>
+        <v>4.15</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.07300884955752195</v>
+        <v>-0.08185840707964585</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>9.48</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>9.550000000000001</v>
+        <v>9.57</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.007383966244725768</v>
+        <v>0.009493670886075934</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>50.7</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>48.55</v>
+        <v>47.5</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04240631163708098</v>
+        <v>-0.06311637080867856</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19464,10 +19464,10 @@
         <v>9.5</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>9.66</v>
+        <v>9.6</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.01684210526315791</v>
+        <v>0.01052631578947365</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19709,10 +19709,10 @@
         <v>308</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.01948051948051948</v>
+        <v>0.02922077922077922</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19738,10 +19738,10 @@
         <v>227</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>227</v>
+        <v>225.5</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0</v>
+        <v>-0.006607929515418502</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19825,10 +19825,10 @@
         <v>6.995</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>6.46</v>
+        <v>6.515</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.07648320228734813</v>
+        <v>-0.06862044317369556</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19854,10 +19854,10 @@
         <v>160.5</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>162.1</v>
+        <v>162.9</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.009968847352024886</v>
+        <v>0.01495327102803742</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19883,10 +19883,10 @@
         <v>62.25</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>62.35</v>
+        <v>62.25</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.001606425702811268</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19912,10 +19912,10 @@
         <v>170.16</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>168.7</v>
+        <v>168.72</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.008580159849553409</v>
+        <v>-0.008462623413258097</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19941,10 +19941,10 @@
         <v>136.4</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>130.2</v>
+        <v>128.1</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.04545454545454558</v>
+        <v>-0.06085043988269803</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19970,10 +19970,10 @@
         <v>303</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>258.2</v>
+        <v>252</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.1478547854785479</v>
+        <v>-0.1683168316831683</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21303,7 +21303,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>07/10/2026 13:00</t>
+          <t>07/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -21330,10 +21330,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.62</v>
+        <v>15.61</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1069182389937107</v>
+        <v>-0.1074899942824471</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21360,10 +21360,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.52</v>
+        <v>24.22</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02929532858273958</v>
+        <v>-0.04117181314330969</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21420,10 +21420,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>7.91</v>
+        <v>7.845</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.04353083434099147</v>
+        <v>-0.0513905683192261</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21450,10 +21450,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>57.15</v>
+        <v>56</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.05770816158285243</v>
+        <v>-0.07666941467436107</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21480,10 +21480,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.81</v>
+        <v>1.76</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.05483028720626631</v>
+        <v>-0.08093994778067887</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21510,10 +21510,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>54.2</v>
+        <v>50.8</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.1198347107438017</v>
+        <v>0.04958677685950411</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21540,10 +21540,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.455</v>
+        <v>3.365</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.05342465753424654</v>
+        <v>-0.07808219178082183</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21710,10 +21710,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.785</v>
+        <v>4.745</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.0312500000000001</v>
+        <v>0.02262931034482768</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21740,10 +21740,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.644</v>
+        <v>4.742</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1162702188392007</v>
+        <v>-0.09762131303520455</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21770,10 +21770,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.095</v>
+        <v>4.117</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02476780185758516</v>
+        <v>-0.01952845915694209</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21800,10 +21800,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.14</v>
+        <v>21.9</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.07208717518860012</v>
+        <v>-0.08214585079631186</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21830,10 +21830,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.2952380952380952</v>
+        <v>-0.3095238095238095</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21860,10 +21860,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.463</v>
+        <v>0.458</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.09746588693957113</v>
+        <v>-0.1072124756335282</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21890,10 +21890,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.37</v>
+        <v>7.23</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.002721088435374213</v>
+        <v>-0.01632653061224479</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21920,10 +21920,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.2</v>
+        <v>29.05</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.008635578583765112</v>
+        <v>0.003454231433506094</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21950,10 +21950,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52</v>
+        <v>52.3</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02564102564102558</v>
+        <v>0.03155818540433913</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21980,10 +21980,10 @@
         <v>0.06900000000000001</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>0.056</v>
+        <v>0.059</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1884057971014493</v>
+        <v>-0.1449275362318842</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22093,10 +22093,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.421</v>
+        <v>5.37</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.04727592267135327</v>
+        <v>-0.05623901581722324</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22122,10 +22122,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.128</v>
+        <v>0.123</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.1228070175438596</v>
+        <v>0.07894736842105257</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22180,10 +22180,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.19</v>
+        <v>4.15</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.06887755102040828</v>
+        <v>0.05867346938775521</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22209,10 +22209,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>17.8</v>
+        <v>17.9</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1834862385321101</v>
+        <v>-0.1788990825688074</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22267,10 +22267,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.82</v>
+        <v>4.77</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.01229508196721303</v>
+        <v>-0.02254098360655744</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22296,10 +22296,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.565</v>
+        <v>2.525</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.139261744966443</v>
+        <v>-0.1526845637583893</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22325,10 +22325,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.985</v>
+        <v>4.93</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.02636718749999996</v>
+        <v>-0.03710937500000008</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22454,10 +22454,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>7.91</v>
+        <v>7.845</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.04353083434099147</v>
+        <v>-0.0513905683192261</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22483,10 +22483,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>54.2</v>
+        <v>50.8</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.1198347107438017</v>
+        <v>0.04958677685950411</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22541,10 +22541,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>94.94</v>
+        <v>95.22</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02645611156685806</v>
+        <v>-0.02358490566037733</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22599,10 +22599,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.84</v>
+        <v>8.66</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03703703703703702</v>
+        <v>-0.0566448801742919</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22628,10 +22628,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>57.15</v>
+        <v>56</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.05770816158285243</v>
+        <v>-0.07666941467436107</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22657,10 +22657,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.81</v>
+        <v>1.76</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05483028720626631</v>
+        <v>-0.08093994778067887</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22686,10 +22686,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.455</v>
+        <v>3.365</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.05342465753424654</v>
+        <v>-0.07808219178082183</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22715,10 +22715,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.52</v>
+        <v>24.22</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.02929532858273958</v>
+        <v>-0.04117181314330969</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-08 19:06
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>08/10/2026 13:00</t>
+          <t>08/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>14.9</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.84</v>
+        <v>14.86</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.004026845637583926</v>
+        <v>-0.002684563758389324</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>148</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>148</v>
+        <v>149.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0</v>
+        <v>0.01013513513513514</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>28.13</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>27.71</v>
+        <v>27.7</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01493067899040164</v>
+        <v>-0.01528617134731602</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>14.84</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.42</v>
+        <v>14.38</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02830188679245283</v>
+        <v>-0.03099730458221018</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>318</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>315</v>
+        <v>317.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.009433962264150943</v>
+        <v>-0.001572327044025157</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>166.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>166.5</v>
+        <v>165.6</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>-0.00540540540540544</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>21.61</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>21.69</v>
+        <v>21.58</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.003701989819528082</v>
+        <v>-0.001388246182323051</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>34.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>34.65</v>
+        <v>34.6</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>-0.001443001443001361</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>36.06</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>36.02</v>
+        <v>35.88</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.001109262340543515</v>
+        <v>-0.004991680532445916</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>15.955</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>15.935</v>
+        <v>16.09</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.001253525540582863</v>
+        <v>0.008461297398934489</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18957,10 +18957,10 @@
         <v>14.48</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>13.54</v>
+        <v>14.54</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.06491712707182329</v>
+        <v>0.00414364640883969</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19017,10 +19017,10 @@
         <v>10.64</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>10.54</v>
+        <v>10.68</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.009398496240601637</v>
+        <v>0.003759398496240521</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19047,10 +19047,10 @@
         <v>1.538</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.508</v>
+        <v>1.482</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01950585175552667</v>
+        <v>-0.03641092327698313</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19077,10 +19077,10 @@
         <v>22.9</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>22.2</v>
+        <v>23.3</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03056768558951962</v>
+        <v>0.01746724890829704</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19107,10 +19107,10 @@
         <v>31.65</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>31.8</v>
+        <v>32</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.004739336492891062</v>
+        <v>0.0110584518167457</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19137,10 +19137,10 @@
         <v>10.374</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.314</v>
+        <v>10.15</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.005783689994216358</v>
+        <v>-0.02159244264507424</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19167,10 +19167,10 @@
         <v>0.454</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.46</v>
+        <v>0.445</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01321585903083702</v>
+        <v>-0.01982378854625552</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19197,10 +19197,10 @@
         <v>74.09999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>72.90000000000001</v>
+        <v>73</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01619433198380552</v>
+        <v>-0.01484480431848845</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19361,10 +19361,10 @@
         <v>9.859999999999999</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.720000000000001</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.01419878296146032</v>
+        <v>-0.02231237322515202</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19390,10 +19390,10 @@
         <v>0.252</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.254</v>
+        <v>0.235</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.007936507936507943</v>
+        <v>-0.06746031746031753</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19448,10 +19448,10 @@
         <v>0.276</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.264</v>
+        <v>0.262</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.04347826086956525</v>
+        <v>-0.05072463768115946</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19564,10 +19564,10 @@
         <v>2.32</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>2.32</v>
+        <v>2.14</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0</v>
+        <v>-0.0775862068965516</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19691,10 +19691,10 @@
         <v>110.9</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>114.4</v>
+        <v>110.5</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.03155996393146979</v>
+        <v>-0.003606853020739456</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19720,10 +19720,10 @@
         <v>166.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>166.5</v>
+        <v>165.6</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0</v>
+        <v>-0.00540540540540544</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19749,10 +19749,10 @@
         <v>80.75</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>80.40000000000001</v>
+        <v>81.05</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.004334365325077329</v>
+        <v>0.003715170278637736</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19778,10 +19778,10 @@
         <v>15.955</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>15.935</v>
+        <v>16.09</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.001253525540582863</v>
+        <v>0.008461297398934489</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19807,10 +19807,10 @@
         <v>28.13</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>27.71</v>
+        <v>27.7</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01493067899040164</v>
+        <v>-0.01528617134731602</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19836,10 +19836,10 @@
         <v>95.26000000000001</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>95.94</v>
+        <v>95.48</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.00713835817761907</v>
+        <v>0.002309468822170889</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19865,10 +19865,10 @@
         <v>21.61</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>21.69</v>
+        <v>21.58</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.003701989819528082</v>
+        <v>-0.001388246182323051</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19894,10 +19894,10 @@
         <v>34.65</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>34.65</v>
+        <v>34.6</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0</v>
+        <v>-0.001443001443001361</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19923,10 +19923,10 @@
         <v>318</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>315</v>
+        <v>317.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.009433962264150943</v>
+        <v>-0.001572327044025157</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19952,10 +19952,10 @@
         <v>36.06</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>36.02</v>
+        <v>35.88</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.001109262340543515</v>
+        <v>-0.004991680532445916</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21233,7 +21233,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>08/10/2026 13:00</t>
+          <t>08/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -21260,10 +21260,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.37</v>
+        <v>15.48</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1212121212121212</v>
+        <v>-0.1149228130360205</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21290,10 +21290,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.08</v>
+        <v>23.94</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.04671417260490907</v>
+        <v>-0.05225653206650832</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21320,10 +21320,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>11.3</v>
+        <v>11.15</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.08502024291497967</v>
+        <v>-0.09716599190283395</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21350,10 +21350,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8</v>
+        <v>8.09</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.0326481257557436</v>
+        <v>-0.02176541717049573</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21380,10 +21380,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.55</v>
+        <v>54.75</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.1005770816158286</v>
+        <v>-0.09727947238252264</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21410,10 +21410,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.73</v>
+        <v>1.725</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.0966057441253264</v>
+        <v>-0.09921671018276759</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21470,10 +21470,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.25</v>
+        <v>3.215</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.1095890410958904</v>
+        <v>-0.1191780821917808</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21530,10 +21530,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.65</v>
+        <v>34.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.00434782608695648</v>
+        <v>0.002898550724637722</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21632,10 +21632,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.615</v>
+        <v>4.495</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.005387931034482644</v>
+        <v>-0.03124999999999991</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21662,10 +21662,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.72</v>
+        <v>4.692</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1018078020932446</v>
+        <v>-0.1071360608943863</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21692,10 +21692,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.958</v>
+        <v>3.987</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.05739461776613471</v>
+        <v>-0.0504882114789235</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21722,10 +21722,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>22.06</v>
+        <v>21.04</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.07544006705783741</v>
+        <v>-0.1181894383906119</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21752,10 +21752,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>13.54</v>
+        <v>14.54</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.3552380952380953</v>
+        <v>-0.3076190476190477</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21782,10 +21782,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.46</v>
+        <v>0.445</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1033138401559454</v>
+        <v>-0.1325536062378168</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21812,10 +21812,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.16</v>
+        <v>7.23</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02585034013605435</v>
+        <v>-0.01632653061224479</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21842,10 +21842,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>29.2</v>
+        <v>28.85</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.008635578583765112</v>
+        <v>-0.003454231433505971</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21872,10 +21872,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>51.8</v>
+        <v>52.3</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02169625246548312</v>
+        <v>0.03155818540433913</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22007,10 +22007,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.327</v>
+        <v>5.326</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06379613356766264</v>
+        <v>-0.06397188049209152</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22067,9 +22067,8 @@
       <c r="F32" s="12" t="n">
         <v>0.089</v>
       </c>
-      <c r="G32" s="13">
-        <f>(F32/E32-1)</f>
-        <v/>
+      <c r="G32" s="13" t="n">
+        <v>0.01136363636363637</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22095,10 +22094,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.07</v>
+        <v>4.11</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.03826530612244907</v>
+        <v>0.04846938775510214</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22124,10 +22123,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>17.8</v>
+        <v>17.75</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1834862385321101</v>
+        <v>-0.1857798165137615</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22153,10 +22152,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.958</v>
+        <v>0.9</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.1596491228070175</v>
+        <v>-0.2105263157894736</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22182,10 +22181,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.7</v>
+        <v>4.71</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03688524590163929</v>
+        <v>-0.03483606557377047</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22211,10 +22210,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.485</v>
+        <v>2.41</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1661073825503356</v>
+        <v>-0.1912751677852348</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22240,10 +22239,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.765</v>
+        <v>4.585</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.06933593750000008</v>
+        <v>-0.1044921875</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22269,10 +22268,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.123</v>
+        <v>0.119</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.08888888888888896</v>
+        <v>-0.1185185185185186</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22366,10 +22365,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>8</v>
+        <v>8.09</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.0326481257557436</v>
+        <v>-0.02176541717049573</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22424,10 +22423,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>11.3</v>
+        <v>11.15</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.08502024291497967</v>
+        <v>-0.09716599190283395</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22453,10 +22452,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.94</v>
+        <v>95.48</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.01620180475799834</v>
+        <v>-0.02091878589007375</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22511,10 +22510,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.76</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.0457516339869281</v>
+        <v>-0.04357298474945537</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22540,10 +22539,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>54.55</v>
+        <v>54.75</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.1005770816158286</v>
+        <v>-0.09727947238252264</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22569,10 +22568,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.73</v>
+        <v>1.725</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0966057441253264</v>
+        <v>-0.09921671018276759</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22598,10 +22597,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.25</v>
+        <v>3.215</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1095890410958904</v>
+        <v>-0.1191780821917808</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22627,10 +22626,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.08</v>
+        <v>23.94</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.04671417260490907</v>
+        <v>-0.05225653206650832</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22725,10 +22724,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>77.05</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.02861825516893591</v>
+        <v>-0.02244074634392319</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -22755,10 +22754,10 @@
         <v>76.44</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>76.04000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.005232862375719407</v>
+        <v>-0.007064364207221246</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -22785,10 +22784,10 @@
         <v>17.49</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>15.37</v>
+        <v>15.48</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.1212121212121212</v>
+        <v>-0.1149228130360205</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -22815,10 +22814,10 @@
         <v>8.27</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>8</v>
+        <v>8.09</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>-0.0326481257557436</v>
+        <v>-0.02176541717049573</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -22998,10 +22997,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>77.05</v>
+        <v>77.54000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.02861825516893591</v>
+        <v>-0.02244074634392319</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -23028,10 +23027,10 @@
         <v>8.27</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>8</v>
+        <v>8.09</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.0326481257557436</v>
+        <v>-0.02176541717049573</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -23058,10 +23057,10 @@
         <v>76.44</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>76.04000000000001</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.005232862375719407</v>
+        <v>-0.007064364207221246</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -23088,10 +23087,10 @@
         <v>17.49</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>15.37</v>
+        <v>15.48</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.1212121212121212</v>
+        <v>-0.1149228130360205</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-09 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>08/10/2026 19:06</t>
+          <t>09/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>14.9</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.86</v>
+        <v>15.22</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.002684563758389324</v>
+        <v>0.02147651006711411</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>148</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>149.5</v>
+        <v>151.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.01013513513513514</v>
+        <v>0.02364864864864865</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>28.13</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>27.7</v>
+        <v>28.22</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01528617134731602</v>
+        <v>0.003199431212228932</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>14.84</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.38</v>
+        <v>14.51</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.03099730458221018</v>
+        <v>-0.02223719676549866</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>318</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>317.5</v>
+        <v>318.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.001572327044025157</v>
+        <v>0.001572327044025157</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>166.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>165.6</v>
+        <v>170.1</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.00540540540540544</v>
+        <v>0.02162162162162159</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>21.61</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>21.58</v>
+        <v>21.89</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.001388246182323051</v>
+        <v>0.01295696436834804</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18795,10 +18795,10 @@
         <v>34.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>34.6</v>
+        <v>34.55</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.001443001443001361</v>
+        <v>-0.002886002886002927</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>36.06</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>35.88</v>
+        <v>36.74</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.004991680532445916</v>
+        <v>0.01885745978924015</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>15.955</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>16.09</v>
+        <v>15.965</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.008461297398934489</v>
+        <v>0.0006267627702914313</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18957,10 +18957,10 @@
         <v>14.48</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>14.54</v>
+        <v>14.76</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.00414364640883969</v>
+        <v>0.01933701657458559</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19017,10 +19017,10 @@
         <v>10.64</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>10.68</v>
+        <v>10.8</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.003759398496240521</v>
+        <v>0.01503759398496242</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19077,10 +19077,10 @@
         <v>22.9</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>23.3</v>
+        <v>23.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.01746724890829704</v>
+        <v>0.02620087336244548</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19107,10 +19107,10 @@
         <v>31.65</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.0110584518167457</v>
+        <v>0.02685624012638235</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19137,10 +19137,10 @@
         <v>10.374</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.15</v>
+        <v>10.6</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.02159244264507424</v>
+        <v>0.02178523231154801</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19167,10 +19167,10 @@
         <v>0.454</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.445</v>
+        <v>0.456</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01982378854625552</v>
+        <v>0.004405286343612339</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19197,10 +19197,10 @@
         <v>74.09999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>73</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01484480431848845</v>
+        <v>-0.01349527665317139</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19227,10 +19227,10 @@
         <v>12.74</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>12.8</v>
+        <v>12.62</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.004709576138147605</v>
+        <v>-0.009419152276295211</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19332,10 +19332,10 @@
         <v>0.13</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.122</v>
+        <v>0.12</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06153846153846159</v>
+        <v>-0.07692307692307698</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19361,10 +19361,10 @@
         <v>9.859999999999999</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.640000000000001</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02231237322515202</v>
+        <v>0.002028397565923058</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19390,10 +19390,10 @@
         <v>0.252</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.235</v>
+        <v>0.259</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.06746031746031753</v>
+        <v>0.0277777777777778</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19448,10 +19448,10 @@
         <v>0.276</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.262</v>
+        <v>0.264</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.05072463768115946</v>
+        <v>-0.04347826086956525</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19477,10 +19477,10 @@
         <v>1.36</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.02205882352941178</v>
+        <v>-0.007352941176470594</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19535,10 +19535,10 @@
         <v>2.76</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.75</v>
+        <v>2.71</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.003623188405797024</v>
+        <v>-0.01811594202898545</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19691,10 +19691,10 @@
         <v>110.9</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>110.5</v>
+        <v>114.85</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.003606853020739456</v>
+        <v>0.03561767357980152</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19720,10 +19720,10 @@
         <v>166.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>165.6</v>
+        <v>170.1</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.00540540540540544</v>
+        <v>0.02162162162162159</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19749,10 +19749,10 @@
         <v>80.75</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>81.05</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.003715170278637736</v>
+        <v>0.02291021671826618</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19778,10 +19778,10 @@
         <v>15.955</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>16.09</v>
+        <v>15.965</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.008461297398934489</v>
+        <v>0.0006267627702914313</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19807,10 +19807,10 @@
         <v>28.13</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>27.7</v>
+        <v>28.22</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01528617134731602</v>
+        <v>0.003199431212228932</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19836,10 +19836,10 @@
         <v>95.26000000000001</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>95.48</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.002309468822170889</v>
+        <v>0.02015536426621879</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19865,10 +19865,10 @@
         <v>21.61</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>21.58</v>
+        <v>21.89</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.001388246182323051</v>
+        <v>0.01295696436834804</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19894,10 +19894,10 @@
         <v>34.65</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>34.6</v>
+        <v>34.55</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.001443001443001361</v>
+        <v>-0.002886002886002927</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19923,10 +19923,10 @@
         <v>318</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>317.5</v>
+        <v>318.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.001572327044025157</v>
+        <v>0.001572327044025157</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19952,10 +19952,10 @@
         <v>36.06</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>35.88</v>
+        <v>36.74</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.004991680532445916</v>
+        <v>0.01885745978924015</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21233,7 +21233,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>08/10/2026 19:06</t>
+          <t>09/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21260,10 +21260,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.48</v>
+        <v>15.54</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1149228130360205</v>
+        <v>-0.111492281303602</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21290,10 +21290,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>23.94</v>
+        <v>24.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.05225653206650832</v>
+        <v>-0.03008709422011091</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21320,10 +21320,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>11.15</v>
+        <v>11.4</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.09716599190283395</v>
+        <v>-0.07692307692307687</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21350,10 +21350,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8.09</v>
+        <v>8.08</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02176541717049573</v>
+        <v>-0.02297460701330103</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21380,10 +21380,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>54.75</v>
+        <v>56.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.09727947238252264</v>
+        <v>-0.06842539159109644</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21410,10 +21410,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.725</v>
+        <v>1.74</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.09921671018276759</v>
+        <v>-0.09138381201044389</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21440,10 +21440,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>49.6</v>
+        <v>50</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.02479338842975213</v>
+        <v>0.03305785123966945</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21470,10 +21470,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.215</v>
+        <v>3.24</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.1191780821917808</v>
+        <v>-0.1123287671232876</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21530,10 +21530,10 @@
         <v>34.5</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>34.6</v>
+        <v>34.55</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.002898550724637722</v>
+        <v>0.001449275362318758</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21632,10 +21632,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.495</v>
+        <v>4.555</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.03124999999999991</v>
+        <v>-0.01831896551724137</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21662,10 +21662,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.692</v>
+        <v>4.596</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1071360608943863</v>
+        <v>-0.1254043767840152</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21692,10 +21692,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.987</v>
+        <v>4.053</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0504882114789235</v>
+        <v>-0.0347701833769945</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21722,10 +21722,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.04</v>
+        <v>21.96</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1181894383906119</v>
+        <v>-0.07963118189438385</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21752,10 +21752,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>14.54</v>
+        <v>14.76</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.3076190476190477</v>
+        <v>-0.2971428571428572</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21782,10 +21782,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.445</v>
+        <v>0.456</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1325536062378168</v>
+        <v>-0.1111111111111111</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21812,10 +21812,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.23</v>
+        <v>7.3</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01632653061224479</v>
+        <v>-0.00680272108843535</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21842,10 +21842,10 @@
         <v>28.95</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>28.85</v>
+        <v>29.75</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.003454231433505971</v>
+        <v>0.02763385146804839</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21872,10 +21872,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>52.3</v>
+        <v>53.2</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03155818540433913</v>
+        <v>0.04930966469428007</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22007,10 +22007,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.326</v>
+        <v>5.422</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06397188049209152</v>
+        <v>-0.04710017574692454</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22036,10 +22036,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.122</v>
+        <v>0.12</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.07017543859649117</v>
+        <v>0.05263157894736834</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22094,10 +22094,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.11</v>
+        <v>4.07</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.04846938775510214</v>
+        <v>0.03826530612244907</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22123,10 +22123,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>17.75</v>
+        <v>17.65</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1857798165137615</v>
+        <v>-0.1903669724770643</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22152,10 +22152,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.9</v>
+        <v>0.954</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.2105263157894736</v>
+        <v>-0.1631578947368421</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22181,10 +22181,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.71</v>
+        <v>4.72</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03483606557377047</v>
+        <v>-0.03278688524590167</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22210,10 +22210,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.41</v>
+        <v>2.465</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1912751677852348</v>
+        <v>-0.1728187919463088</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22239,10 +22239,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.585</v>
+        <v>4.73</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.1044921875</v>
+        <v>-0.07617187499999993</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22268,10 +22268,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.119</v>
+        <v>0.125</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.1185185185185186</v>
+        <v>-0.07407407407407414</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22365,10 +22365,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>8.09</v>
+        <v>8.08</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.02176541717049573</v>
+        <v>-0.02297460701330103</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22394,10 +22394,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>49.6</v>
+        <v>50</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.02479338842975213</v>
+        <v>0.03305785123966945</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22423,10 +22423,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>11.15</v>
+        <v>11.4</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.09716599190283395</v>
+        <v>-0.07692307692307687</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22452,10 +22452,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>95.48</v>
+        <v>97.18000000000001</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02091878589007375</v>
+        <v>-0.003486464315012195</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22510,10 +22510,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.779999999999999</v>
+        <v>8.76</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04357298474945537</v>
+        <v>-0.0457516339869281</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22539,10 +22539,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>54.75</v>
+        <v>56.5</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.09727947238252264</v>
+        <v>-0.06842539159109644</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22568,10 +22568,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.725</v>
+        <v>1.74</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.09921671018276759</v>
+        <v>-0.09138381201044389</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22597,10 +22597,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.215</v>
+        <v>3.24</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1191780821917808</v>
+        <v>-0.1123287671232876</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22626,10 +22626,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>23.94</v>
+        <v>24.5</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.05225653206650832</v>
+        <v>-0.03008709422011091</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22724,10 +22724,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>77.54000000000001</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.02244074634392319</v>
+        <v>-0.02597075138678755</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -22754,10 +22754,10 @@
         <v>76.44</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>75.90000000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.007064364207221246</v>
+        <v>-0.003401360544217568</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -22784,10 +22784,10 @@
         <v>17.49</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>15.48</v>
+        <v>15.54</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.1149228130360205</v>
+        <v>-0.111492281303602</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -22814,10 +22814,10 @@
         <v>8.27</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>8.09</v>
+        <v>8.08</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>-0.02176541717049573</v>
+        <v>-0.02297460701330103</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>77.54000000000001</v>
+        <v>77.26000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.02244074634392319</v>
+        <v>-0.02597075138678755</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>8.27</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>8.09</v>
+        <v>8.08</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.02176541717049573</v>
+        <v>-0.02297460701330103</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>76.44</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>75.90000000000001</v>
+        <v>76.18000000000001</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.007064364207221246</v>
+        <v>-0.003401360544217568</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -23087,10 +23087,10 @@
         <v>17.49</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>15.48</v>
+        <v>15.54</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.1149228130360205</v>
+        <v>-0.111492281303602</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-09 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18558,7 +18558,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>09/10/2026 13:00</t>
+          <t>09/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -18585,10 +18585,10 @@
         <v>14.9</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.22</v>
+        <v>15.32</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.02147651006711411</v>
+        <v>0.02818791946308724</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18615,10 +18615,10 @@
         <v>148</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>151.5</v>
+        <v>150</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.02364864864864865</v>
+        <v>0.01351351351351351</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18645,10 +18645,10 @@
         <v>28.13</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>28.22</v>
+        <v>28.17</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.003199431212228932</v>
+        <v>0.001421969427657401</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18675,10 +18675,10 @@
         <v>14.84</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>14.51</v>
+        <v>14.48</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02223719676549866</v>
+        <v>-0.02425876010781667</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18705,10 +18705,10 @@
         <v>318</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>318.5</v>
+        <v>316</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.001572327044025157</v>
+        <v>-0.006289308176100629</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18735,10 +18735,10 @@
         <v>166.5</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>170.1</v>
+        <v>169</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02162162162162159</v>
+        <v>0.01501501501501501</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18765,10 +18765,10 @@
         <v>21.61</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>21.89</v>
+        <v>21.76</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.01295696436834804</v>
+        <v>0.006941230911615092</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18825,10 +18825,10 @@
         <v>36.06</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>36.74</v>
+        <v>36.1</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01885745978924015</v>
+        <v>0.001109262340543515</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18855,10 +18855,10 @@
         <v>15.955</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>15.965</v>
+        <v>15.93</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.0006267627702914313</v>
+        <v>-0.001566906925728634</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18957,10 +18957,10 @@
         <v>14.48</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>14.76</v>
+        <v>14.92</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.01933701657458559</v>
+        <v>0.03038674033149168</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19017,10 +19017,10 @@
         <v>10.64</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>10.8</v>
+        <v>10.78</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01503759398496242</v>
+        <v>0.01315789473684199</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19047,10 +19047,10 @@
         <v>1.538</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.482</v>
+        <v>1.51</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.03641092327698313</v>
+        <v>-0.01820546163849156</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19137,10 +19137,10 @@
         <v>10.374</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>10.6</v>
+        <v>10.58</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.02178523231154801</v>
+        <v>0.01985733564680928</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19167,10 +19167,10 @@
         <v>0.454</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.456</v>
+        <v>0.444</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.004405286343612339</v>
+        <v>-0.02202643171806169</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19197,10 +19197,10 @@
         <v>74.09999999999999</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>73.09999999999999</v>
+        <v>72.8</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01349527665317139</v>
+        <v>-0.01754385964912277</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19227,10 +19227,10 @@
         <v>12.74</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>12.62</v>
+        <v>12.6</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.009419152276295211</v>
+        <v>-0.01098901098901103</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19332,10 +19332,10 @@
         <v>0.13</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.12</v>
+        <v>0.117</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.07692307692307698</v>
+        <v>-0.09999999999999998</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19390,10 +19390,10 @@
         <v>0.252</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.259</v>
+        <v>0.241</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.0277777777777778</v>
+        <v>-0.04365079365079369</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19448,10 +19448,10 @@
         <v>0.276</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.264</v>
+        <v>0.262</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.04347826086956525</v>
+        <v>-0.05072463768115946</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19477,10 +19477,10 @@
         <v>1.36</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.007352941176470594</v>
+        <v>-0.02205882352941178</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19506,10 +19506,10 @@
         <v>3.46</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>3.46</v>
+        <v>3.47</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>0.002890173410404691</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19535,10 +19535,10 @@
         <v>2.76</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.71</v>
+        <v>2.81</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01811594202898545</v>
+        <v>0.01811594202898561</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19564,10 +19564,10 @@
         <v>2.32</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>2.14</v>
+        <v>2</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.0775862068965516</v>
+        <v>-0.1379310344827586</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19691,10 +19691,10 @@
         <v>110.9</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>114.85</v>
+        <v>115.35</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.03561767357980152</v>
+        <v>0.04012623985572578</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19720,10 +19720,10 @@
         <v>166.5</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>170.1</v>
+        <v>169</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.02162162162162159</v>
+        <v>0.01501501501501501</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19749,10 +19749,10 @@
         <v>80.75</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>82.59999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.02291021671826618</v>
+        <v>0.03034055727554183</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19778,10 +19778,10 @@
         <v>15.955</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>15.965</v>
+        <v>15.93</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.0006267627702914313</v>
+        <v>-0.001566906925728634</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19807,10 +19807,10 @@
         <v>28.13</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>28.22</v>
+        <v>28.17</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.003199431212228932</v>
+        <v>0.001421969427657401</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19836,10 +19836,10 @@
         <v>95.26000000000001</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>97.18000000000001</v>
+        <v>97.62</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.02015536426621879</v>
+        <v>0.02477430191056056</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19865,10 +19865,10 @@
         <v>21.61</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>21.89</v>
+        <v>21.76</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01295696436834804</v>
+        <v>0.006941230911615092</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19923,10 +19923,10 @@
         <v>318</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>318.5</v>
+        <v>316</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.001572327044025157</v>
+        <v>-0.006289308176100629</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19952,10 +19952,10 @@
         <v>36.06</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>36.74</v>
+        <v>36.1</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01885745978924015</v>
+        <v>0.001109262340543515</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21233,7 +21233,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>09/10/2026 13:00</t>
+          <t>09/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -21260,10 +21260,10 @@
         <v>17.49</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.54</v>
+        <v>15.69</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.111492281303602</v>
+        <v>-0.1029159519725557</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21290,10 +21290,10 @@
         <v>25.26</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03008709422011091</v>
+        <v>-0.02612826603325416</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21320,10 +21320,10 @@
         <v>12.35</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>11.4</v>
+        <v>11.35</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.07692307692307687</v>
+        <v>-0.08097165991902834</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21350,10 +21350,10 @@
         <v>8.27</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>8.08</v>
+        <v>8.18</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.02297460701330103</v>
+        <v>-0.01088270858524787</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21380,10 +21380,10 @@
         <v>60.65</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.5</v>
+        <v>58.55</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.06842539159109644</v>
+        <v>-0.03462489694971149</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21410,10 +21410,10 @@
         <v>1.915</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>1.74</v>
+        <v>1.735</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.09138381201044389</v>
+        <v>-0.09399477806788509</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21440,10 +21440,10 @@
         <v>48.4</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>50</v>
+        <v>50.8</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.03305785123966945</v>
+        <v>0.04958677685950411</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21470,10 +21470,10 @@
         <v>3.65</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>3.24</v>
+        <v>3.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.1123287671232876</v>
+        <v>-0.09589041095890413</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21500,10 +21500,10 @@
         <v>103</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.009708737864077669</v>
+        <v>-0.01941747572815534</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21632,10 +21632,10 @@
         <v>4.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>4.555</v>
+        <v>4.545</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01831896551724137</v>
+        <v>-0.02047413793103443</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21662,10 +21662,10 @@
         <v>5.255</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>4.596</v>
+        <v>4.6</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.1254043767840152</v>
+        <v>-0.1246431969552807</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21692,10 +21692,10 @@
         <v>4.199</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>4.053</v>
+        <v>4.014</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0347701833769945</v>
+        <v>-0.04405810907358886</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21722,10 +21722,10 @@
         <v>23.86</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>21.96</v>
+        <v>21.08</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.07963118189438385</v>
+        <v>-0.1165129924559933</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21752,10 +21752,10 @@
         <v>21</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>14.76</v>
+        <v>14.92</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.2971428571428572</v>
+        <v>-0.2895238095238095</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21782,10 +21782,10 @@
         <v>0.513</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>0.456</v>
+        <v>0.444</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.1111111111111111</v>
+        <v>-0.1345029239766082</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21812,10 +21812,10 @@
         <v>7.35</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>7.3</v>
+        <v>7.42</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.00680272108843535</v>
+        <v>0.009523809523809563</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21872,10 +21872,10 @@
         <v>50.7</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>53.2</v>
+        <v>53</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.04930966469428007</v>
+        <v>0.04536489151873761</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -22007,10 +22007,10 @@
         <v>5.69</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>5.422</v>
+        <v>5.606</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.04710017574692454</v>
+        <v>-0.01476274165202118</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22036,10 +22036,10 @@
         <v>0.114</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.12</v>
+        <v>0.117</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.05263157894736834</v>
+        <v>0.02631578947368423</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22065,10 +22065,10 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.089</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.01136363636363637</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22094,10 +22094,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>4.07</v>
+        <v>4.12</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.03826530612244907</v>
+        <v>0.05102040816326536</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22123,10 +22123,10 @@
         <v>21.8</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>17.65</v>
+        <v>17.8</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1903669724770643</v>
+        <v>-0.1834862385321101</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22152,10 +22152,10 @@
         <v>1.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>0.954</v>
+        <v>0.848</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.1631578947368421</v>
+        <v>-0.2561403508771929</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22181,10 +22181,10 @@
         <v>4.88</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>4.72</v>
+        <v>4.79</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03278688524590167</v>
+        <v>-0.01844262295081964</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22210,10 +22210,10 @@
         <v>2.98</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>2.465</v>
+        <v>2.62</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.1728187919463088</v>
+        <v>-0.1208053691275167</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22239,10 +22239,10 @@
         <v>5.12</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>4.73</v>
+        <v>4.78</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.07617187499999993</v>
+        <v>-0.06640624999999997</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22268,10 +22268,10 @@
         <v>0.135</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>0.125</v>
+        <v>0.124</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.07407407407407414</v>
+        <v>-0.08148148148148154</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22365,10 +22365,10 @@
         <v>8.27</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>8.08</v>
+        <v>8.18</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>-0.02297460701330103</v>
+        <v>-0.01088270858524787</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -22394,10 +22394,10 @@
         <v>48.4</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>50</v>
+        <v>50.8</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.03305785123966945</v>
+        <v>0.04958677685950411</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -22423,10 +22423,10 @@
         <v>12.35</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>11.4</v>
+        <v>11.35</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.07692307692307687</v>
+        <v>-0.08097165991902834</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -22452,10 +22452,10 @@
         <v>97.52</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>97.18000000000001</v>
+        <v>97.62</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.003486464315012195</v>
+        <v>0.00102543068088606</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -22481,10 +22481,10 @@
         <v>103</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.009708737864077669</v>
+        <v>-0.01941747572815534</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -22510,10 +22510,10 @@
         <v>9.18</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>8.76</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.0457516339869281</v>
+        <v>-0.02396514161220031</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -22539,10 +22539,10 @@
         <v>60.65</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>56.5</v>
+        <v>58.55</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.06842539159109644</v>
+        <v>-0.03462489694971149</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -22568,10 +22568,10 @@
         <v>1.915</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>1.74</v>
+        <v>1.735</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.09138381201044389</v>
+        <v>-0.09399477806788509</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -22597,10 +22597,10 @@
         <v>3.65</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>3.24</v>
+        <v>3.3</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.1123287671232876</v>
+        <v>-0.09589041095890413</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -22626,10 +22626,10 @@
         <v>25.26</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>-0.03008709422011091</v>
+        <v>-0.02612826603325416</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -22724,10 +22724,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>77.26000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.02597075138678755</v>
+        <v>-0.0105900151285929</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -22754,10 +22754,10 @@
         <v>76.44</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>76.18000000000001</v>
+        <v>76.88</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.003401360544217568</v>
+        <v>0.005756148613291441</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -22784,10 +22784,10 @@
         <v>17.49</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>15.54</v>
+        <v>15.69</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.111492281303602</v>
+        <v>-0.1029159519725557</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -22814,10 +22814,10 @@
         <v>8.27</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>8.08</v>
+        <v>8.18</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>-0.02297460701330103</v>
+        <v>-0.01088270858524787</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>79.31999999999999</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>77.26000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.02597075138678755</v>
+        <v>-0.0105900151285929</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>8.27</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>8.08</v>
+        <v>8.18</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.02297460701330103</v>
+        <v>-0.01088270858524787</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>76.44</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>76.18000000000001</v>
+        <v>76.88</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.003401360544217568</v>
+        <v>0.005756148613291441</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -23087,10 +23087,10 @@
         <v>17.49</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>15.54</v>
+        <v>15.69</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.111492281303602</v>
+        <v>-0.1029159519725557</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-12 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>12/10/2026 15:37</t>
+          <t>12/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.14</v>
+        <v>14.86</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.003947368421052548</v>
+        <v>-0.02236842105263157</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.18</v>
+        <v>8.145</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0</v>
+        <v>-0.004278728606356985</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>28.02</v>
+        <v>28.21</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.008141592920353997</v>
+        <v>-0.001415929203539793</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20136,10 +20136,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.4</v>
+        <v>24.72</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-0.008130081300813123</v>
+        <v>0.004878048780487701</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20166,10 +20166,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>81.05</v>
+        <v>80.95</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.006832298136645928</v>
+        <v>0.005590062111801277</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20196,10 +20196,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>78.95</v>
+        <v>79</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.005348274544759986</v>
+        <v>0.005984973895326613</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20226,10 +20226,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.004291845493562232</v>
+        <v>0.0128755364806867</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20256,10 +20256,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.475</v>
+        <v>1.465</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01444291609353517</v>
+        <v>0.007565337001375599</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20286,10 +20286,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.001574803149606299</v>
+        <v>-0.001574803149606299</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20316,10 +20316,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>216.6</v>
+        <v>215.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.0009242144177448642</v>
+        <v>-0.00369685767097972</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20418,10 +20418,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125</v>
+        <v>124.8</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.001602564102564125</v>
+        <v>0</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20448,10 +20448,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.494999999999999</v>
+        <v>9.41</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.02365038560411315</v>
+        <v>-0.0323907455012853</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20478,10 +20478,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.126</v>
+        <v>2.13</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.003748828491096536</v>
+        <v>-0.001874414245548268</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20508,10 +20508,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.426</v>
+        <v>1.4</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03333333333333337</v>
+        <v>0.01449275362318842</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20538,10 +20538,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21</v>
+        <v>21.9</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.00756143667296787</v>
+        <v>0.0349716446124763</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20568,10 +20568,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>12.64</v>
+        <v>12.6</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.003174603174603248</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20598,10 +20598,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>54.2</v>
+        <v>54.45</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01722574796010872</v>
+        <v>-0.01269265639165904</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20628,10 +20628,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.458</v>
+        <v>0.456</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.03854875283446715</v>
+        <v>0.0340136054421769</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20658,10 +20658,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>30.6</v>
+        <v>30.72</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.001308900523560298</v>
+        <v>0.005235602094240842</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20793,10 +20793,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1125000000000001</v>
+        <v>-0.1249999999999999</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20822,10 +20822,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.859999999999999</v>
+        <v>9.84</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.004040404040404133</v>
+        <v>-0.006060606060606111</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20851,10 +20851,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.153</v>
+        <v>0.161</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03164556962025319</v>
+        <v>0.01898734177215192</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20880,10 +20880,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.39</v>
+        <v>1.32</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.06923076923076912</v>
+        <v>0.0153846153846154</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20909,10 +20909,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.23</v>
+        <v>0.229</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.04564315352697088</v>
+        <v>-0.04979253112033188</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20938,10 +20938,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>10.02</v>
+        <v>9.93</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01183431952662732</v>
+        <v>-0.02071005917159771</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20996,10 +20996,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.57</v>
+        <v>3.78</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.0484581497797357</v>
+        <v>0.1101321585903084</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21054,10 +21054,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.02</v>
+        <v>4.04</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.15850144092219</v>
+        <v>0.1642651296829971</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21579,10 +21579,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>215.4</v>
+        <v>213.2</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.01221804511278193</v>
+        <v>0.001879699248120194</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21609,10 +21609,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>15.14</v>
+        <v>14.86</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.003947368421052548</v>
+        <v>-0.02236842105263157</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21639,10 +21639,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50.6</v>
+        <v>50</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.003937007874015665</v>
+        <v>-0.01574803149606294</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21699,10 +21699,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.004291845493562232</v>
+        <v>0.0128755364806867</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21729,10 +21729,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>30.6</v>
+        <v>30.72</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.001308900523560298</v>
+        <v>0.005235602094240842</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21759,10 +21759,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>76.2</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.01804123711340195</v>
+        <v>-0.03221649484536083</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21789,10 +21789,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>25.35</v>
+        <v>25.3</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.01197604790419165</v>
+        <v>0.009980039920159681</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21819,10 +21819,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>78.95</v>
+        <v>79</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.005348274544759986</v>
+        <v>0.005984973895326613</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21849,10 +21849,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>116.2</v>
+        <v>115.55</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.009995654063450723</v>
+        <v>0.00434593654932638</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22696,7 +22696,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>12/10/2026 15:37</t>
+          <t>12/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22723,10 +22723,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>46.355</v>
+        <v>45.535</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.02771311384547168</v>
+        <v>0.009533311162842251</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22753,10 +22753,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>83.84999999999999</v>
+        <v>84.05</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.07915057915057903</v>
+        <v>0.08172458172458165</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22783,10 +22783,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.4</v>
+        <v>24.72</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.02243589743589753</v>
+        <v>-0.009615384615384694</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22843,10 +22843,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>81.05</v>
+        <v>80.95</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06295081967213111</v>
+        <v>0.06163934426229512</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22873,10 +22873,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>58.4</v>
+        <v>58</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.0626003210272873</v>
+        <v>-0.06902086677367572</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22903,10 +22903,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>6.03</v>
+        <v>5.985</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.07938931297709917</v>
+        <v>-0.08625954198473275</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22933,10 +22933,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>54.75</v>
+        <v>54.85</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.04533565823888407</v>
+        <v>-0.04359197907585004</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22963,10 +22963,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.03311258278145696</v>
+        <v>0.04194260485651214</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22993,10 +22993,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.83</v>
+        <v>18.96</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>0.006903876792352766</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23095,10 +23095,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.054</v>
+        <v>2.062</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.2160305343511451</v>
+        <v>-0.2129770992366413</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23125,10 +23125,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.0288659793814433</v>
+        <v>0.02783505154639175</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23155,10 +23155,10 @@
         <v>0.012</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>0.011</v>
+        <v>0.012</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.08333333333333341</v>
+        <v>0</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -23185,10 +23185,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.458</v>
+        <v>0.456</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.05761316872427977</v>
+        <v>-0.06172839506172834</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23215,10 +23215,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.5</v>
+        <v>4.455</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.004464285714285619</v>
+        <v>-0.005580357142857222</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23245,10 +23245,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21</v>
+        <v>21.9</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.06082289803220033</v>
+        <v>-0.02057245080500898</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23275,10 +23275,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.272</v>
+        <v>1.282</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1178918169209431</v>
+        <v>-0.1109570041608876</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23335,10 +23335,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.554</v>
+        <v>0.544</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1900584795321637</v>
+        <v>-0.2046783625730994</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23499,10 +23499,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>45.95</v>
+        <v>46.15</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.03161222339304531</v>
+        <v>-0.02739726027397269</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23828,10 +23828,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>169.2</v>
+        <v>169</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.02359346642468226</v>
+        <v>0.02238354506957041</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23857,10 +23857,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.35</v>
+        <v>25.3</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.04752066115702488</v>
+        <v>0.04545454545454551</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23886,10 +23886,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.88</v>
+        <v>1.878</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.0107526881720429</v>
+        <v>0.009677419354838599</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23915,10 +23915,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.83</v>
+        <v>18.96</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0</v>
+        <v>0.006903876792352766</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23944,10 +23944,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.4</v>
+        <v>24.72</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.02243589743589753</v>
+        <v>-0.009615384615384694</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23973,10 +23973,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>46.355</v>
+        <v>45.535</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.02771311384547168</v>
+        <v>0.009533311162842251</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24002,10 +24002,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>98.38</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.005313713468219865</v>
+        <v>0.01267116288575511</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24031,10 +24031,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>103</v>
+        <v>103.2</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.07039711191335737</v>
+        <v>-0.0685920577617328</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24060,10 +24060,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>58.4</v>
+        <v>58</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.0626003210272873</v>
+        <v>-0.06902086677367572</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24089,10 +24089,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>83.84999999999999</v>
+        <v>84.05</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.07915057915057903</v>
+        <v>0.08172458172458165</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-13 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>12/10/2026 19:05</t>
+          <t>13/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.86</v>
+        <v>14.78</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02236842105263157</v>
+        <v>-0.02763157894736842</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.145</v>
+        <v>8.195</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.004278728606356985</v>
+        <v>0.001833740831295913</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>28.21</v>
+        <v>28.47</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.001415929203539793</v>
+        <v>0.007787610619468986</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20136,10 +20136,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.72</v>
+        <v>25.02</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.004878048780487701</v>
+        <v>0.01707317073170724</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20166,10 +20166,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>80.95</v>
+        <v>82</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.005590062111801277</v>
+        <v>0.01863354037267081</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20196,10 +20196,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79</v>
+        <v>79.22</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.005984973895326613</v>
+        <v>0.008786451037819913</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20226,10 +20226,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.0128755364806867</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20256,10 +20256,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.465</v>
+        <v>1.476</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.007565337001375599</v>
+        <v>0.01513067400275105</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20286,10 +20286,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>317</v>
+        <v>326.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.001574803149606299</v>
+        <v>0.02834645669291339</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20316,10 +20316,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>215.6</v>
+        <v>216.4</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.00369685767097972</v>
+        <v>0</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20418,10 +20418,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>124.8</v>
+        <v>125.1</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0</v>
+        <v>0.002403846153846131</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20448,10 +20448,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.41</v>
+        <v>9.6</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.0323907455012853</v>
+        <v>-0.012853470437018</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20478,10 +20478,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.13</v>
+        <v>2.114</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.001874414245548268</v>
+        <v>-0.009372071227741339</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20508,10 +20508,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.4</v>
+        <v>1.407</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01449275362318842</v>
+        <v>0.01956521739130445</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20538,10 +20538,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21.9</v>
+        <v>21.76</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.0349716446124763</v>
+        <v>0.02835538752362956</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20568,10 +20568,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>12.6</v>
+        <v>12.66</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0</v>
+        <v>0.004761904761904801</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20598,10 +20598,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>54.45</v>
+        <v>54.95</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01269265639165904</v>
+        <v>-0.003626473254759669</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20628,10 +20628,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.456</v>
+        <v>0.434</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.0340136054421769</v>
+        <v>-0.01587301587301589</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20658,10 +20658,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>30.72</v>
+        <v>31.28</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.005235602094240842</v>
+        <v>0.02356020942408385</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20688,10 +20688,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.36</v>
+        <v>14.57</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.00897170462387859</v>
+        <v>0.005521048999309873</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20793,10 +20793,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1249999999999999</v>
+        <v>-0.1375</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20822,10 +20822,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.84</v>
+        <v>9.9</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.006060606060606111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20851,10 +20851,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.161</v>
+        <v>0.163</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.01898734177215192</v>
+        <v>0.03164556962025319</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20880,10 +20880,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.32</v>
+        <v>1.37</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.0153846153846154</v>
+        <v>0.05384615384615389</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20909,10 +20909,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.229</v>
+        <v>0.245</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.04979253112033188</v>
+        <v>0.016597510373444</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20938,10 +20938,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.93</v>
+        <v>9.84</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.02071005917159771</v>
+        <v>-0.02958579881656812</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20967,10 +20967,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>19.75</v>
+        <v>18.55</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.002538071065989884</v>
+        <v>-0.05837563451776643</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20996,10 +20996,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.78</v>
+        <v>3.865</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.1101321585903084</v>
+        <v>0.1350954478707784</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21025,10 +21025,10 @@
         <v>0.013</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.076923076923077</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21054,10 +21054,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.04</v>
+        <v>4.03</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1642651296829971</v>
+        <v>0.1613832853025937</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21579,10 +21579,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>213.2</v>
+        <v>214.6</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.001879699248120194</v>
+        <v>0.008458646616541273</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21609,10 +21609,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>14.86</v>
+        <v>14.78</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.02236842105263157</v>
+        <v>-0.02763157894736842</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21639,10 +21639,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50</v>
+        <v>50.6</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.01574803149606294</v>
+        <v>-0.003937007874015665</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21669,10 +21669,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>150.5</v>
+        <v>145.5</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.009868421052631578</v>
+        <v>-0.04276315789473684</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21699,10 +21699,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.0128755364806867</v>
+        <v>0</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21729,10 +21729,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>30.72</v>
+        <v>31.28</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.005235602094240842</v>
+        <v>0.02356020942408385</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21759,10 +21759,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>75.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.03221649484536083</v>
+        <v>-0.01804123711340195</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21789,10 +21789,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>25.3</v>
+        <v>25.25</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.009980039920159681</v>
+        <v>0.007984031936127716</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21819,10 +21819,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>79</v>
+        <v>79.22</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.005984973895326613</v>
+        <v>0.008786451037819913</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21849,10 +21849,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>115.55</v>
+        <v>116.35</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.00434593654932638</v>
+        <v>0.01129943502824856</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22696,7 +22696,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>12/10/2026 19:05</t>
+          <t>13/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22723,10 +22723,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>45.535</v>
+        <v>44.49</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.009533311162842251</v>
+        <v>-0.01363485201197195</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22753,10 +22753,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>84.05</v>
+        <v>85</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.08172458172458165</v>
+        <v>0.09395109395109391</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22783,10 +22783,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.72</v>
+        <v>25.02</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.009615384615384694</v>
+        <v>0.002403846153846102</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22813,10 +22813,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>150.5</v>
+        <v>145.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.04513888888888889</v>
+        <v>0.01041666666666667</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22843,10 +22843,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>80.95</v>
+        <v>82</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06163934426229512</v>
+        <v>0.07540983606557378</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22873,10 +22873,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>58</v>
+        <v>57.55</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.06902086677367572</v>
+        <v>-0.07624398073836276</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22903,10 +22903,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.985</v>
+        <v>5.825</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.08625954198473275</v>
+        <v>-0.1106870229007633</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22933,10 +22933,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>54.85</v>
+        <v>55.35</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.04359197907585004</v>
+        <v>-0.03487358326068003</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22963,10 +22963,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.04194260485651214</v>
+        <v>0.02869757174392936</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22993,10 +22993,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>18.96</v>
+        <v>19.04</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.006903876792352766</v>
+        <v>0.01115241635687737</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23095,10 +23095,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.062</v>
+        <v>2.1</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.2129770992366413</v>
+        <v>-0.1984732824427481</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23125,10 +23125,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02783505154639175</v>
+        <v>0.02577319587628866</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23185,10 +23185,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.456</v>
+        <v>0.434</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.06172839506172834</v>
+        <v>-0.1069958847736625</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23215,10 +23215,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.455</v>
+        <v>4.515</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.005580357142857222</v>
+        <v>0.007812499999999833</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23245,10 +23245,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.9</v>
+        <v>21.76</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02057245080500898</v>
+        <v>-0.02683363148479418</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23275,10 +23275,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.282</v>
+        <v>1.278</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1109570041608876</v>
+        <v>-0.1137309292649098</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23305,10 +23305,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.076</v>
+        <v>0.077</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.02564102564102566</v>
+        <v>-0.01282051282051283</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23335,10 +23335,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.544</v>
+        <v>0.599</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.2046783625730994</v>
+        <v>-0.1242690058479533</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23365,10 +23365,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>36</v>
+        <v>35.7</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0136986301369863</v>
+        <v>-0.02191780821917801</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23470,10 +23470,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.837</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3195121951219512</v>
+        <v>-0.3357723577235773</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23499,10 +23499,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>46.15</v>
+        <v>44.5</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.02739726027397269</v>
+        <v>-0.0621707060063225</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23528,10 +23528,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.005</v>
+        <v>1.03</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.02551020408163256</v>
+        <v>0.05102040816326536</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23557,10 +23557,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.86</v>
+        <v>3.88</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05392156862745102</v>
+        <v>-0.0490196078431373</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23586,10 +23586,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.86</v>
+        <v>4.85</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.05813953488372089</v>
+        <v>-0.06007751937984505</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23644,10 +23644,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>30</v>
+        <v>29.8</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.04458598726114645</v>
+        <v>-0.05095541401273879</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23731,10 +23731,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2134831460674158</v>
+        <v>-0.199438202247191</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23828,10 +23828,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>169</v>
+        <v>169.5</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.02238354506957041</v>
+        <v>0.0254083484573502</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23857,10 +23857,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.3</v>
+        <v>25.25</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.04545454545454551</v>
+        <v>0.04338842975206614</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23886,10 +23886,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.878</v>
+        <v>1.874</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.009677419354838599</v>
+        <v>0.007526881720430114</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23915,10 +23915,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>18.96</v>
+        <v>19.04</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.006903876792352766</v>
+        <v>0.01115241635687737</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23944,10 +23944,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.72</v>
+        <v>25.02</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.009615384615384694</v>
+        <v>0.002403846153846102</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23973,10 +23973,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>45.535</v>
+        <v>44.49</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.009533311162842251</v>
+        <v>-0.01363485201197195</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24002,10 +24002,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>99.09999999999999</v>
+        <v>99.48</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01267116288575511</v>
+        <v>0.01655426118945437</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24031,10 +24031,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>103.2</v>
+        <v>105.1</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0685920577617328</v>
+        <v>-0.05144404332129967</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24060,10 +24060,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>58</v>
+        <v>57.55</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.06902086677367572</v>
+        <v>-0.07624398073836276</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24089,10 +24089,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>84.05</v>
+        <v>85</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.08172458172458165</v>
+        <v>0.09395109395109391</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-13 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>13/10/2026 13:00</t>
+          <t>13/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.78</v>
+        <v>14.76</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02763157894736842</v>
+        <v>-0.0289473684210526</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.195</v>
+        <v>8.255000000000001</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.001833740831295913</v>
+        <v>0.009168704156479348</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>28.47</v>
+        <v>29.22</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.007787610619468986</v>
+        <v>0.03433628318584066</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20136,10 +20136,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.02</v>
+        <v>24.94</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01707317073170724</v>
+        <v>0.01382113821138211</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20166,10 +20166,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>82</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01863354037267081</v>
+        <v>0.03540372670807446</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20196,10 +20196,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79.22</v>
+        <v>79.87</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.008786451037819913</v>
+        <v>0.0170635425951866</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20256,10 +20256,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.476</v>
+        <v>1.512</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01513067400275105</v>
+        <v>0.03988995873452549</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20286,10 +20286,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>326.5</v>
+        <v>325</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02834645669291339</v>
+        <v>0.02362204724409449</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20418,10 +20418,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125.1</v>
+        <v>125.2</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.002403846153846131</v>
+        <v>0.003205128205128251</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20448,10 +20448,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.6</v>
+        <v>9.57</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.012853470437018</v>
+        <v>-0.01593830334190225</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20478,10 +20478,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.114</v>
+        <v>2.044</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.009372071227741339</v>
+        <v>-0.04217432052483593</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20508,10 +20508,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.407</v>
+        <v>1.355</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01956521739130445</v>
+        <v>-0.01811594202898545</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20538,10 +20538,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21.76</v>
+        <v>21.5</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.02835538752362956</v>
+        <v>0.0160680529300567</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20568,10 +20568,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>12.66</v>
+        <v>13.18</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.004761904761904801</v>
+        <v>0.04603174603174604</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20628,10 +20628,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.434</v>
+        <v>0.438</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01587301587301589</v>
+        <v>-0.00680272108843538</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20658,10 +20658,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>31.28</v>
+        <v>31.4</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.02356020942408385</v>
+        <v>0.0274869109947644</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20688,10 +20688,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.57</v>
+        <v>14.62</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.005521048999309873</v>
+        <v>0.008971704623878468</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20793,10 +20793,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.074</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1375</v>
+        <v>-0.07500000000000007</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20822,10 +20822,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.9</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.004040404040404133</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20851,10 +20851,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.163</v>
+        <v>0.186</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.03164556962025319</v>
+        <v>0.1772151898734177</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20880,10 +20880,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.37</v>
+        <v>1.28</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.05384615384615389</v>
+        <v>-0.0153846153846154</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20909,10 +20909,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.245</v>
+        <v>0.248</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.016597510373444</v>
+        <v>0.029045643153527</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20996,10 +20996,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.865</v>
+        <v>3.97</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.1350954478707784</v>
+        <v>0.1659324522760647</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21025,10 +21025,10 @@
         <v>0.013</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0</v>
+        <v>0.076923076923077</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21054,10 +21054,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.03</v>
+        <v>4.02</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1613832853025937</v>
+        <v>0.15850144092219</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21579,10 +21579,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>214.6</v>
+        <v>214.4</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.008458646616541273</v>
+        <v>0.007518796992481176</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21609,10 +21609,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>14.78</v>
+        <v>14.76</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.02763157894736842</v>
+        <v>-0.0289473684210526</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21669,10 +21669,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>145.5</v>
+        <v>148</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.04276315789473684</v>
+        <v>-0.02631578947368421</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21729,10 +21729,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>31.28</v>
+        <v>31.4</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.02356020942408385</v>
+        <v>0.0274869109947644</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21759,10 +21759,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>76.2</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.01804123711340195</v>
+        <v>-0.02190721649484522</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21789,10 +21789,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>25.25</v>
+        <v>26</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.007984031936127716</v>
+        <v>0.03792415169660675</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21819,10 +21819,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>79.22</v>
+        <v>79.87</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.008786451037819913</v>
+        <v>0.0170635425951866</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21849,10 +21849,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>116.35</v>
+        <v>119.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.01129943502824856</v>
+        <v>0.03867883528900481</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22696,7 +22696,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>13/10/2026 13:00</t>
+          <t>13/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22723,10 +22723,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>44.49</v>
+        <v>43.785</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01363485201197195</v>
+        <v>-0.0292650482208181</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22753,10 +22753,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>85</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.09395109395109391</v>
+        <v>0.09909909909909913</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22783,10 +22783,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.02</v>
+        <v>24.94</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.002403846153846102</v>
+        <v>-0.0008012820512820341</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22813,10 +22813,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>145.5</v>
+        <v>148</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01041666666666667</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22843,10 +22843,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>82</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.07540983606557378</v>
+        <v>0.09311475409836058</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22873,10 +22873,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>57.55</v>
+        <v>56.9</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.07624398073836276</v>
+        <v>-0.08667736757624396</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22903,10 +22903,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.825</v>
+        <v>5.785</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1106870229007633</v>
+        <v>-0.1167938931297709</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22933,10 +22933,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.35</v>
+        <v>55.15</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03487358326068003</v>
+        <v>-0.03836094158674809</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22993,10 +22993,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.04</v>
+        <v>19.09</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01115241635687737</v>
+        <v>0.01380775358470534</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23095,10 +23095,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.1</v>
+        <v>2.032</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1984732824427481</v>
+        <v>-0.2244274809160305</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23125,10 +23125,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>995</v>
+        <v>1002</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02577319587628866</v>
+        <v>0.03298969072164949</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23185,10 +23185,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.434</v>
+        <v>0.438</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1069958847736625</v>
+        <v>-0.09876543209876541</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23215,10 +23215,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.515</v>
+        <v>4.55</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.007812499999999833</v>
+        <v>0.01562499999999986</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23245,10 +23245,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.76</v>
+        <v>21.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02683363148479418</v>
+        <v>-0.03846153846153844</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23275,10 +23275,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.278</v>
+        <v>1.272</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1137309292649098</v>
+        <v>-0.1178918169209431</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23335,10 +23335,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.599</v>
+        <v>0.58</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1242690058479533</v>
+        <v>-0.1520467836257311</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23365,10 +23365,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>35.7</v>
+        <v>34.9</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.02191780821917801</v>
+        <v>-0.04383561643835621</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23470,10 +23470,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3357723577235773</v>
+        <v>-0.3398373983739837</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23499,10 +23499,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>44.5</v>
+        <v>43.75</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.0621707060063225</v>
+        <v>-0.07797681770284516</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23528,10 +23528,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.03</v>
+        <v>1.02</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.05102040816326536</v>
+        <v>0.04081632653061228</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23557,10 +23557,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.88</v>
+        <v>3.71</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0490196078431373</v>
+        <v>-0.09068627450980395</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23586,10 +23586,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.85</v>
+        <v>4.74</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.06007751937984505</v>
+        <v>-0.08139534883720928</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23615,10 +23615,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.58</v>
+        <v>4.62</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.08399999999999999</v>
+        <v>-0.07599999999999998</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23644,10 +23644,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>29.8</v>
+        <v>30.3</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05095541401273879</v>
+        <v>-0.0350318471337579</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23673,10 +23673,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.29</v>
+        <v>1.28</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.007692307692307699</v>
+        <v>-0.0153846153846154</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23828,10 +23828,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>169.5</v>
+        <v>174.2</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0254083484573502</v>
+        <v>0.05384150030248019</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23857,10 +23857,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.25</v>
+        <v>26</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.04338842975206614</v>
+        <v>0.07438016528925623</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23886,10 +23886,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.874</v>
+        <v>1.878</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.007526881720430114</v>
+        <v>0.009677419354838599</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23915,10 +23915,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.04</v>
+        <v>19.09</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01115241635687737</v>
+        <v>0.01380775358470534</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23944,10 +23944,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>25.02</v>
+        <v>24.94</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.002403846153846102</v>
+        <v>-0.0008012820512820341</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23973,10 +23973,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>44.49</v>
+        <v>43.785</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01363485201197195</v>
+        <v>-0.0292650482208181</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24002,10 +24002,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>99.48</v>
+        <v>100.95</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.01655426118945437</v>
+        <v>0.03157572041692217</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24060,10 +24060,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>57.55</v>
+        <v>56.9</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.07624398073836276</v>
+        <v>-0.08667736757624396</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24089,10 +24089,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>85</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.09395109395109391</v>
+        <v>0.09909909909909913</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-14 09:11
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -19980,7 +19980,7 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1" thickBot="1">
       <c r="A1" s="54" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>13/10/2026 19:05</t>
+          <t>14/10/2026 09:11</t>
         </is>
       </c>
     </row>
@@ -20029,7 +20029,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>QDT</t>
+          <t>RCO</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -20039,17 +20039,17 @@
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>QUADIENT</t>
+          <t>REMY COINTREAU</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>15.2</v>
+        <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.76</v>
+        <v>45.5</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.0289473684210526</v>
+        <v>-0.003067484662576699</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20059,7 +20059,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>MAU</t>
+          <t>BAIN</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -20069,17 +20069,17 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>MAUREL ET PROM</t>
+          <t>BAINS MER MONACO</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>8.18</v>
+        <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.255000000000001</v>
+        <v>148</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.009168704156479348</v>
+        <v>-0.01986754966887417</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20089,7 +20089,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>EDEN</t>
+          <t>DEC</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -20099,17 +20099,17 @@
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>EDENRED</t>
+          <t>JCDECAUX</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>28.25</v>
+        <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>29.22</v>
+        <v>24.94</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.03433628318584066</v>
+        <v>-0.003993610223642087</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20119,7 +20119,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>DEC</t>
+          <t>EKI</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -20129,17 +20129,18 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>JCDECAUX</t>
+          <t>EKINOPS</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>24.6</v>
+        <v>2.5</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.94</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>0.01382113821138211</v>
+        <v>2.5</v>
+      </c>
+      <c r="G5" s="13">
+        <f>(F5/E5-1)</f>
+        <v/>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -20163,13 +20164,13 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>80.5</v>
+        <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
         <v>83.34999999999999</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.03540372670807446</v>
+        <v>0.0006002400960383813</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20179,7 +20180,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>PUB</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -20189,17 +20190,17 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>TOTALENERGIES</t>
+          <t>PUBLICIS GRP</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>78.53</v>
+        <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>79.87</v>
+        <v>100.95</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0170635425951866</v>
+        <v>0</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20209,7 +20210,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>ENX</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
@@ -20219,14 +20220,14 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>EURONEXT</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
-        <v>233</v>
+        <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>233</v>
+        <v>166</v>
       </c>
       <c r="G8" s="13" t="n">
         <v>0</v>
@@ -20239,7 +20240,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>VIV</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -20249,17 +20250,17 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIVENDI </t>
+          <t>SODEXO</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>1.454</v>
+        <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.512</v>
+        <v>55.15</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.03988995873452549</v>
+        <v>0</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20269,7 +20270,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>VIRP</t>
+          <t>EDEN</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -20279,17 +20280,17 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>VIRBAC</t>
+          <t>EDENRED</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>317.5</v>
+        <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>325</v>
+        <v>29.22</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02362204724409449</v>
+        <v>0.0006849315068493004</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20299,7 +20300,7 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>GTT</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
@@ -20309,17 +20310,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>GAZTRANS TECHN</t>
+          <t>TOTALENERGIES</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>216.4</v>
+        <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>216.4</v>
+        <v>79.87</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0</v>
+        <v>-0.0002503442233069974</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20401,7 +20402,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>EXA</t>
+          <t>ATO</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -20411,17 +20412,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>EXAIL TECH</t>
+          <t>ATOS</t>
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>124.8</v>
+        <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125.2</v>
+        <v>21.5</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.003205128205128251</v>
+        <v>-0.006469500924214444</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20431,7 +20432,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>OPM</t>
+          <t>FDE</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -20441,17 +20442,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>OPMOBILITY</t>
+          <t>FRANCAISE ENER</t>
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>9.725</v>
+        <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.57</v>
+        <v>14.96</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01593830334190225</v>
+        <v>0.002680965147453145</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20461,7 +20462,7 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>OSE</t>
+          <t>ABVX</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
@@ -20471,17 +20472,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>OSE IMMUNO</t>
+          <t>ABIVAX</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>2.134</v>
+        <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.044</v>
+        <v>76.5</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.04217432052483593</v>
+        <v>-0.005847953216374306</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20491,7 +20492,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>ETL</t>
+          <t>EQS</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -20501,17 +20502,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>EUTELSAT COMMUNICATION</t>
+          <t>EQUASENS</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>1.38</v>
+        <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.355</v>
+        <v>28.5</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.01811594202898545</v>
+        <v>0.003521126760563431</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20521,7 +20522,7 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>ATO</t>
+          <t>ETL</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -20531,17 +20532,17 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>EUTELSAT COMMUNICATION</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>21.16</v>
+        <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>21.5</v>
+        <v>1.355</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.0160680529300567</v>
+        <v>-0.01094890510948914</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20551,7 +20552,7 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>TFF</t>
+          <t>CRI</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -20561,17 +20562,17 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>TFF GROUP</t>
+          <t>CHARGEURS</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>12.6</v>
+        <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.18</v>
+        <v>7.35</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.04603174603174604</v>
+        <v>0</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20581,7 +20582,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>SK</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -20591,17 +20592,17 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>SEB</t>
+          <t>LVMH</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>55.15</v>
+        <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>54.95</v>
+        <v>384</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.003626473254759669</v>
+        <v>-0.0001301913813305855</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20611,27 +20612,27 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>ELEC</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>SRD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>SOLUTIONS 30</t>
+          <t>ELECTICITE DE STRASBOURG</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>0.441</v>
+        <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.438</v>
+        <v>154</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.00680272108843538</v>
+        <v>0</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20641,7 +20642,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>ITP</t>
+          <t>FGA</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -20651,17 +20652,17 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>INTER PARFUMS</t>
+          <t>FIGEAC AERO</t>
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>30.56</v>
+        <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>31.4</v>
+        <v>10.86</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.0274869109947644</v>
+        <v>-0.003669724770642287</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20671,7 +20672,7 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>ICAD</t>
+          <t>ASY</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -20681,17 +20682,17 @@
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>ICADE</t>
+          <t>ASSYSTEM</t>
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>14.49</v>
+        <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.62</v>
+        <v>32</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.008971704623878468</v>
+        <v>-0.001560062402496011</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20776,27 +20777,27 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>AVT</t>
+          <t>ALCWE</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D30" s="51" t="inlineStr">
         <is>
-          <t>AVENIR TELECOM</t>
+          <t>CHARWOOD ENERGY</t>
         </is>
       </c>
       <c r="E30" s="18" t="n">
-        <v>0.08</v>
+        <v>4.02</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.074</v>
+        <v>4.02</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.07500000000000007</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20805,7 +20806,7 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>ALICA</t>
+          <t>ALIMP</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -20815,17 +20816,17 @@
       </c>
       <c r="D31" s="51" t="inlineStr">
         <is>
-          <t>ICAP HOLDING</t>
+          <t>IMPLANET</t>
         </is>
       </c>
       <c r="E31" s="18" t="n">
-        <v>9.9</v>
+        <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.859999999999999</v>
+        <v>0.186</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.004040404040404133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20834,7 +20835,7 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>ALIMP</t>
+          <t>ALNTG</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -20844,17 +20845,17 @@
       </c>
       <c r="D32" s="51" t="inlineStr">
         <is>
-          <t>IMPLANET</t>
+          <t>NETGEM</t>
         </is>
       </c>
       <c r="E32" s="18" t="n">
-        <v>0.158</v>
+        <v>1.02</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.186</v>
+        <v>1.02</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.1772151898734177</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20863,27 +20864,27 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>ALINV</t>
+          <t>AVT</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D33" s="51" t="inlineStr">
         <is>
-          <t>INVIBES ADVERTISING</t>
+          <t>AVENIR TELECOM</t>
         </is>
       </c>
       <c r="E33" s="18" t="n">
-        <v>1.3</v>
+        <v>0.074</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.28</v>
+        <v>0.074</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0153846153846154</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20906,13 +20907,13 @@
         </is>
       </c>
       <c r="E34" s="18" t="n">
-        <v>0.241</v>
+        <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
         <v>0.248</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0.029045643153527</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20921,27 +20922,27 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>ALESE</t>
+          <t>ABLD</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>EG</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D35" s="51" t="inlineStr">
         <is>
-          <t>ENTECH</t>
+          <t>ABL DIAGNOSTICS</t>
         </is>
       </c>
       <c r="E35" s="18" t="n">
-        <v>10.14</v>
+        <v>2.58</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.84</v>
+        <v>2.58</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.02958579881656812</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20950,7 +20951,7 @@
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>ALDNX</t>
+          <t>ALESA</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -20960,17 +20961,17 @@
       </c>
       <c r="D36" s="51" t="inlineStr">
         <is>
-          <t>DNXCORP</t>
+          <t>ECOSLOPS</t>
         </is>
       </c>
       <c r="E36" s="18" t="n">
-        <v>19.7</v>
+        <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.55</v>
+        <v>0.95</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05837563451776643</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20979,7 +20980,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>ALMDT</t>
+          <t>ALNLF</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -20989,17 +20990,17 @@
       </c>
       <c r="D37" s="51" t="inlineStr">
         <is>
-          <t>MEDIAN TECHNOLOGIES</t>
+          <t>NEOLIFE</t>
         </is>
       </c>
       <c r="E37" s="18" t="n">
-        <v>3.405</v>
+        <v>0.058</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>3.97</v>
+        <v>0.058</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.1659324522760647</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21008,27 +21009,27 @@
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>ALCBX</t>
+          <t>ALMCE</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>EG</t>
         </is>
       </c>
       <c r="D38" s="51" t="inlineStr">
         <is>
-          <t>CIBOX INTERACTIVE</t>
+          <t>MON COURTIER ENERGIE</t>
         </is>
       </c>
       <c r="E38" s="18" t="n">
-        <v>0.013</v>
+        <v>5.7</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.014</v>
+        <v>5.7</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0.076923076923077</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21037,7 +21038,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>ALCWE</t>
+          <t>ALGLD</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -21047,17 +21048,17 @@
       </c>
       <c r="D39" s="51" t="inlineStr">
         <is>
-          <t>CHARWOOD ENERGY</t>
+          <t>GOLD BY GOLD</t>
         </is>
       </c>
       <c r="E39" s="18" t="n">
-        <v>3.47</v>
+        <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.02</v>
+        <v>4.77</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.15850144092219</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21562,7 +21563,7 @@
       </c>
       <c r="B69" s="36" t="inlineStr">
         <is>
-          <t>DIM</t>
+          <t>TTE</t>
         </is>
       </c>
       <c r="C69" s="30" t="inlineStr">
@@ -21572,17 +21573,17 @@
       </c>
       <c r="D69" s="36" t="inlineStr">
         <is>
-          <t>SARTORIUS STED</t>
+          <t>TOTALENERGIES</t>
         </is>
       </c>
       <c r="E69" s="18" t="n">
-        <v>212.8</v>
+        <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>214.4</v>
+        <v>79.87</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.007518796992481176</v>
+        <v>-0.0002503442233069974</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21592,7 +21593,7 @@
       </c>
       <c r="B70" s="36" t="inlineStr">
         <is>
-          <t>QDT</t>
+          <t>IPS</t>
         </is>
       </c>
       <c r="C70" s="30" t="inlineStr">
@@ -21602,17 +21603,17 @@
       </c>
       <c r="D70" s="36" t="inlineStr">
         <is>
-          <t>QUADIENT</t>
+          <t>IPSOS</t>
         </is>
       </c>
       <c r="E70" s="18" t="n">
-        <v>15.2</v>
+        <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>14.76</v>
+        <v>36.34</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.0289473684210526</v>
+        <v>0.00110192837465582</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21622,27 +21623,27 @@
       </c>
       <c r="B71" s="36" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>QDT</t>
         </is>
       </c>
       <c r="C71" s="30" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>SRD</t>
         </is>
       </c>
       <c r="D71" s="36" t="inlineStr">
         <is>
-          <t>LINEDATA</t>
+          <t>QUADIENT</t>
         </is>
       </c>
       <c r="E71" s="18" t="n">
-        <v>50.8</v>
+        <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50.6</v>
+        <v>14.76</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.003937007874015665</v>
+        <v>-0.001353179972936372</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21652,7 +21653,7 @@
       </c>
       <c r="B72" s="36" t="inlineStr">
         <is>
-          <t>BAIN</t>
+          <t>MAU</t>
         </is>
       </c>
       <c r="C72" s="30" t="inlineStr">
@@ -21662,17 +21663,17 @@
       </c>
       <c r="D72" s="36" t="inlineStr">
         <is>
-          <t>BAINS MER MONACO</t>
+          <t>MAUREL ET PROM</t>
         </is>
       </c>
       <c r="E72" s="18" t="n">
-        <v>152</v>
+        <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>148</v>
+        <v>8.255000000000001</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.02631578947368421</v>
+        <v>-0.001813784764207835</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21682,7 +21683,7 @@
       </c>
       <c r="B73" s="36" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>BAIN</t>
         </is>
       </c>
       <c r="C73" s="30" t="inlineStr">
@@ -21692,17 +21693,17 @@
       </c>
       <c r="D73" s="36" t="inlineStr">
         <is>
-          <t>TOTAL GABON</t>
+          <t>BAINS MER MONACO</t>
         </is>
       </c>
       <c r="E73" s="18" t="n">
-        <v>233</v>
+        <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>233</v>
+        <v>148</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0</v>
+        <v>-0.01986754966887417</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21712,7 +21713,7 @@
       </c>
       <c r="B74" s="36" t="inlineStr">
         <is>
-          <t>ITP</t>
+          <t>BIM</t>
         </is>
       </c>
       <c r="C74" s="30" t="inlineStr">
@@ -21722,17 +21723,17 @@
       </c>
       <c r="D74" s="36" t="inlineStr">
         <is>
-          <t>INTER PARFUMS</t>
+          <t>BIOMERIEUX</t>
         </is>
       </c>
       <c r="E74" s="18" t="n">
-        <v>30.56</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>31.4</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.0274869109947644</v>
+        <v>0</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21742,7 +21743,7 @@
       </c>
       <c r="B75" s="36" t="inlineStr">
         <is>
-          <t>VETO</t>
+          <t>DSY</t>
         </is>
       </c>
       <c r="C75" s="30" t="inlineStr">
@@ -21752,17 +21753,17 @@
       </c>
       <c r="D75" s="36" t="inlineStr">
         <is>
-          <t>VETOQUINOL</t>
+          <t>DASSAULT SYSTEMES</t>
         </is>
       </c>
       <c r="E75" s="18" t="n">
-        <v>77.59999999999999</v>
+        <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>75.90000000000001</v>
+        <v>22.61</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.02190721649484522</v>
+        <v>0.003105590062111814</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21772,7 +21773,7 @@
       </c>
       <c r="B76" s="36" t="inlineStr">
         <is>
-          <t>PLNW</t>
+          <t>EKI</t>
         </is>
       </c>
       <c r="C76" s="30" t="inlineStr">
@@ -21782,17 +21783,18 @@
       </c>
       <c r="D76" s="36" t="inlineStr">
         <is>
-          <t>PLANISWARE</t>
+          <t>EKINOPS</t>
         </is>
       </c>
       <c r="E76" s="18" t="n">
-        <v>25.05</v>
+        <v>2.5</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>26</v>
-      </c>
-      <c r="G76" s="37" t="n">
-        <v>0.03792415169660675</v>
+        <v>2.5</v>
+      </c>
+      <c r="G76" s="37">
+        <f>(F76/E76-1)</f>
+        <v/>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -21802,7 +21804,7 @@
       </c>
       <c r="B77" s="36" t="inlineStr">
         <is>
-          <t>TTE</t>
+          <t>ITP</t>
         </is>
       </c>
       <c r="C77" s="30" t="inlineStr">
@@ -21812,17 +21814,17 @@
       </c>
       <c r="D77" s="36" t="inlineStr">
         <is>
-          <t>TOTALENERGIES</t>
+          <t>INTER PARFUMS</t>
         </is>
       </c>
       <c r="E77" s="18" t="n">
-        <v>78.53</v>
+        <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>79.87</v>
+        <v>31.4</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.0170635425951866</v>
+        <v>-0.000636537237428489</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21832,7 +21834,7 @@
       </c>
       <c r="B78" s="36" t="inlineStr">
         <is>
-          <t>CAP</t>
+          <t>VIRP</t>
         </is>
       </c>
       <c r="C78" s="30" t="inlineStr">
@@ -21842,17 +21844,17 @@
       </c>
       <c r="D78" s="36" t="inlineStr">
         <is>
-          <t>CAP GEMINI</t>
+          <t>VIRBAC</t>
         </is>
       </c>
       <c r="E78" s="18" t="n">
-        <v>115.05</v>
+        <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>119.5</v>
+        <v>325</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.03867883528900481</v>
+        <v>0</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22696,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>13/10/2026 19:05</t>
+          <t>14/10/2026 09:11</t>
         </is>
       </c>
     </row>
@@ -23012,7 +23014,7 @@
         </is>
       </c>
       <c r="G12" s="20" t="n">
-        <v>0.005525740344178309</v>
+        <v>-0.0003299294548089748</v>
       </c>
       <c r="H12" s="46" t="inlineStr">
         <is>
@@ -23384,7 +23386,7 @@
         </is>
       </c>
       <c r="G26" s="24" t="n">
-        <v>-0.08065833317770481</v>
+        <v>-0.06483785123515742</v>
       </c>
       <c r="H26" s="46" t="inlineStr">
         <is>
@@ -23748,7 +23750,7 @@
         </is>
       </c>
       <c r="G40" s="29" t="n">
-        <v>-0.07795620060891631</v>
+        <v>-0.09408255955388364</v>
       </c>
       <c r="H40" s="46" t="inlineStr">
         <is>
@@ -24106,7 +24108,7 @@
         </is>
       </c>
       <c r="G53" s="34" t="n">
-        <v>0.001620501514687844</v>
+        <v>0.01198111400713893</v>
       </c>
       <c r="H53" s="46" t="inlineStr">
         <is>
@@ -24168,14 +24170,29 @@
       <c r="A56" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B56" s="36" t="n"/>
-      <c r="C56" s="30" t="n"/>
-      <c r="D56" s="36" t="n"/>
-      <c r="E56" s="18" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="37">
-        <f>(F56/E56-1)</f>
-        <v/>
+      <c r="B56" s="36" t="inlineStr">
+        <is>
+          <t>ABCA</t>
+        </is>
+      </c>
+      <c r="C56" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D56" s="36" t="inlineStr">
+        <is>
+          <t>ABC ARBITRAGE</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F56" s="12" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="G56" s="37" t="n">
+        <v>-0.02068965517241381</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24183,14 +24200,29 @@
       <c r="A57" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B57" s="36" t="n"/>
-      <c r="C57" s="30" t="n"/>
-      <c r="D57" s="36" t="n"/>
-      <c r="E57" s="18" t="n"/>
-      <c r="F57" s="12" t="n"/>
-      <c r="G57" s="37">
-        <f>(F57/E57-1)</f>
-        <v/>
+      <c r="B57" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C57" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D57" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E57" s="18" t="n">
+        <v>45.105</v>
+      </c>
+      <c r="F57" s="12" t="n">
+        <v>43.785</v>
+      </c>
+      <c r="G57" s="37" t="n">
+        <v>-0.0292650482208181</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24198,14 +24230,29 @@
       <c r="A58" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B58" s="36" t="n"/>
-      <c r="C58" s="30" t="n"/>
-      <c r="D58" s="36" t="n"/>
-      <c r="E58" s="18" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="37">
-        <f>(F58/E58-1)</f>
-        <v/>
+      <c r="B58" s="36" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="C58" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D58" s="36" t="inlineStr">
+        <is>
+          <t>TOTALENERGIES</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="F58" s="12" t="n">
+        <v>79.87</v>
+      </c>
+      <c r="G58" s="37" t="n">
+        <v>-0.001500187523440309</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24213,14 +24260,29 @@
       <c r="A59" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B59" s="36" t="n"/>
-      <c r="C59" s="30" t="n"/>
-      <c r="D59" s="36" t="n"/>
-      <c r="E59" s="18" t="n"/>
-      <c r="F59" s="12" t="n"/>
-      <c r="G59" s="37">
-        <f>(F59/E59-1)</f>
-        <v/>
+      <c r="B59" s="36" t="inlineStr">
+        <is>
+          <t>TEP</t>
+        </is>
+      </c>
+      <c r="C59" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D59" s="36" t="inlineStr">
+        <is>
+          <t>TÉLÉPERFORMANCE</t>
+        </is>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="F59" s="12" t="n">
+        <v>73.98</v>
+      </c>
+      <c r="G59" s="37" t="n">
+        <v>0.0223880597014926</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24228,14 +24290,29 @@
       <c r="A60" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B60" s="36" t="n"/>
-      <c r="C60" s="30" t="n"/>
-      <c r="D60" s="36" t="n"/>
-      <c r="E60" s="18" t="n"/>
-      <c r="F60" s="12" t="n"/>
-      <c r="G60" s="37">
-        <f>(F60/E60-1)</f>
-        <v/>
+      <c r="B60" s="36" t="inlineStr">
+        <is>
+          <t>ATE</t>
+        </is>
+      </c>
+      <c r="C60" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D60" s="36" t="inlineStr">
+        <is>
+          <t>ALTEN</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="n">
+        <v>76.25</v>
+      </c>
+      <c r="F60" s="12" t="n">
+        <v>83.34999999999999</v>
+      </c>
+      <c r="G60" s="37" t="n">
+        <v>0.09311475409836058</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24243,14 +24320,29 @@
       <c r="A61" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B61" s="36" t="n"/>
-      <c r="C61" s="30" t="n"/>
-      <c r="D61" s="36" t="n"/>
-      <c r="E61" s="18" t="n"/>
-      <c r="F61" s="12" t="n"/>
-      <c r="G61" s="37">
-        <f>(F61/E61-1)</f>
-        <v/>
+      <c r="B61" s="36" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C61" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D61" s="36" t="inlineStr">
+        <is>
+          <t>VALEO</t>
+        </is>
+      </c>
+      <c r="E61" s="18" t="n">
+        <v>14.855</v>
+      </c>
+      <c r="F61" s="12" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="G61" s="37" t="n">
+        <v>-0.08246381689666776</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24258,14 +24350,29 @@
       <c r="A62" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B62" s="36" t="n"/>
-      <c r="C62" s="30" t="n"/>
-      <c r="D62" s="36" t="n"/>
-      <c r="E62" s="18" t="n"/>
-      <c r="F62" s="12" t="n"/>
-      <c r="G62" s="37">
-        <f>(F62/E62-1)</f>
-        <v/>
+      <c r="B62" s="36" t="inlineStr">
+        <is>
+          <t>STF</t>
+        </is>
+      </c>
+      <c r="C62" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D62" s="36" t="inlineStr">
+        <is>
+          <t>STEF</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="n">
+        <v>126.4</v>
+      </c>
+      <c r="F62" s="12" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="G62" s="37" t="n">
+        <v>-0.02848101265822791</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24273,14 +24380,29 @@
       <c r="A63" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B63" s="36" t="n"/>
-      <c r="C63" s="30" t="n"/>
-      <c r="D63" s="36" t="n"/>
-      <c r="E63" s="18" t="n"/>
-      <c r="F63" s="12" t="n"/>
-      <c r="G63" s="37">
-        <f>(F63/E63-1)</f>
-        <v/>
+      <c r="B63" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C63" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D63" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="F63" s="12" t="n">
+        <v>40.56</v>
+      </c>
+      <c r="G63" s="37" t="n">
+        <v>-0.0112140419307655</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24288,14 +24410,29 @@
       <c r="A64" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B64" s="36" t="n"/>
-      <c r="C64" s="30" t="n"/>
-      <c r="D64" s="36" t="n"/>
-      <c r="E64" s="18" t="n"/>
-      <c r="F64" s="12" t="n"/>
-      <c r="G64" s="37">
-        <f>(F64/E64-1)</f>
-        <v/>
+      <c r="B64" s="36" t="inlineStr">
+        <is>
+          <t>INF</t>
+        </is>
+      </c>
+      <c r="C64" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D64" s="36" t="inlineStr">
+        <is>
+          <t>INFOTEL</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="F64" s="12" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="G64" s="37" t="n">
+        <v>-0.04114713216957602</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24386,14 +24523,29 @@
       <c r="A69" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B69" s="36" t="n"/>
-      <c r="C69" s="30" t="n"/>
-      <c r="D69" s="36" t="n"/>
-      <c r="E69" s="18" t="n"/>
-      <c r="F69" s="12" t="n"/>
-      <c r="G69" s="37">
-        <f>(F69/E69-1)</f>
-        <v/>
+      <c r="B69" s="36" t="inlineStr">
+        <is>
+          <t>ABCA</t>
+        </is>
+      </c>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D69" s="36" t="inlineStr">
+        <is>
+          <t>ABC ARBITRAGE</t>
+        </is>
+      </c>
+      <c r="E69" s="18" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F69" s="12" t="n">
+        <v>5.68</v>
+      </c>
+      <c r="G69" s="37" t="n">
+        <v>-0.02068965517241381</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24401,14 +24553,29 @@
       <c r="A70" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B70" s="36" t="n"/>
-      <c r="C70" s="30" t="n"/>
-      <c r="D70" s="36" t="n"/>
-      <c r="E70" s="18" t="n"/>
-      <c r="F70" s="12" t="n"/>
-      <c r="G70" s="37">
-        <f>(F70/E70-1)</f>
-        <v/>
+      <c r="B70" s="36" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="C70" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D70" s="36" t="inlineStr">
+        <is>
+          <t>TOTALENERGIES</t>
+        </is>
+      </c>
+      <c r="E70" s="18" t="n">
+        <v>79.98999999999999</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <v>79.87</v>
+      </c>
+      <c r="G70" s="37" t="n">
+        <v>-0.001500187523440309</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24416,14 +24583,29 @@
       <c r="A71" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B71" s="36" t="n"/>
-      <c r="C71" s="30" t="n"/>
-      <c r="D71" s="36" t="n"/>
-      <c r="E71" s="18" t="n"/>
-      <c r="F71" s="12" t="n"/>
-      <c r="G71" s="37">
-        <f>(F71/E71-1)</f>
-        <v/>
+      <c r="B71" s="36" t="inlineStr">
+        <is>
+          <t>LIN</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D71" s="36" t="inlineStr">
+        <is>
+          <t>LINEDATA</t>
+        </is>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>54.2</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="G71" s="37" t="n">
+        <v>-0.06642066420664208</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24431,14 +24613,29 @@
       <c r="A72" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B72" s="36" t="n"/>
-      <c r="C72" s="30" t="n"/>
-      <c r="D72" s="36" t="n"/>
-      <c r="E72" s="18" t="n"/>
-      <c r="F72" s="12" t="n"/>
-      <c r="G72" s="37">
-        <f>(F72/E72-1)</f>
-        <v/>
+      <c r="B72" s="36" t="inlineStr">
+        <is>
+          <t>TEP</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D72" s="36" t="inlineStr">
+        <is>
+          <t>TÉLÉPERFORMANCE</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <v>73.98</v>
+      </c>
+      <c r="G72" s="37" t="n">
+        <v>0.0223880597014926</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24446,14 +24643,29 @@
       <c r="A73" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B73" s="36" t="n"/>
-      <c r="C73" s="30" t="n"/>
-      <c r="D73" s="36" t="n"/>
-      <c r="E73" s="18" t="n"/>
-      <c r="F73" s="12" t="n"/>
-      <c r="G73" s="37">
-        <f>(F73/E73-1)</f>
-        <v/>
+      <c r="B73" s="36" t="inlineStr">
+        <is>
+          <t>MRN</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D73" s="36" t="inlineStr">
+        <is>
+          <t>MERSEN</t>
+        </is>
+      </c>
+      <c r="E73" s="18" t="n">
+        <v>41.02</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <v>40.56</v>
+      </c>
+      <c r="G73" s="37" t="n">
+        <v>-0.0112140419307655</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24461,14 +24673,29 @@
       <c r="A74" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="B74" s="36" t="n"/>
-      <c r="C74" s="30" t="n"/>
-      <c r="D74" s="36" t="n"/>
-      <c r="E74" s="18" t="n"/>
-      <c r="F74" s="12" t="n"/>
-      <c r="G74" s="37">
-        <f>(F74/E74-1)</f>
-        <v/>
+      <c r="B74" s="36" t="inlineStr">
+        <is>
+          <t>STMPA</t>
+        </is>
+      </c>
+      <c r="C74" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D74" s="36" t="inlineStr">
+        <is>
+          <t>STMICROELECTRONICS</t>
+        </is>
+      </c>
+      <c r="E74" s="18" t="n">
+        <v>45.105</v>
+      </c>
+      <c r="F74" s="12" t="n">
+        <v>43.785</v>
+      </c>
+      <c r="G74" s="37" t="n">
+        <v>-0.0292650482208181</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24476,14 +24703,29 @@
       <c r="A75" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B75" s="36" t="n"/>
-      <c r="C75" s="30" t="n"/>
-      <c r="D75" s="36" t="n"/>
-      <c r="E75" s="18" t="n"/>
-      <c r="F75" s="12" t="n"/>
-      <c r="G75" s="37">
-        <f>(F75/E75-1)</f>
-        <v/>
+      <c r="B75" s="36" t="inlineStr">
+        <is>
+          <t>ATE</t>
+        </is>
+      </c>
+      <c r="C75" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D75" s="36" t="inlineStr">
+        <is>
+          <t>ALTEN</t>
+        </is>
+      </c>
+      <c r="E75" s="18" t="n">
+        <v>76.25</v>
+      </c>
+      <c r="F75" s="12" t="n">
+        <v>83.34999999999999</v>
+      </c>
+      <c r="G75" s="37" t="n">
+        <v>0.09311475409836058</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24491,14 +24733,29 @@
       <c r="A76" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="B76" s="36" t="n"/>
-      <c r="C76" s="30" t="n"/>
-      <c r="D76" s="36" t="n"/>
-      <c r="E76" s="18" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="37">
-        <f>(F76/E76-1)</f>
-        <v/>
+      <c r="B76" s="36" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D76" s="36" t="inlineStr">
+        <is>
+          <t>VALEO</t>
+        </is>
+      </c>
+      <c r="E76" s="18" t="n">
+        <v>14.855</v>
+      </c>
+      <c r="F76" s="12" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="G76" s="37" t="n">
+        <v>-0.08246381689666776</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24506,14 +24763,29 @@
       <c r="A77" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B77" s="36" t="n"/>
-      <c r="C77" s="30" t="n"/>
-      <c r="D77" s="36" t="n"/>
-      <c r="E77" s="18" t="n"/>
-      <c r="F77" s="12" t="n"/>
-      <c r="G77" s="37">
-        <f>(F77/E77-1)</f>
-        <v/>
+      <c r="B77" s="36" t="inlineStr">
+        <is>
+          <t>STF</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D77" s="36" t="inlineStr">
+        <is>
+          <t>STEF</t>
+        </is>
+      </c>
+      <c r="E77" s="18" t="n">
+        <v>126.4</v>
+      </c>
+      <c r="F77" s="12" t="n">
+        <v>122.8</v>
+      </c>
+      <c r="G77" s="37" t="n">
+        <v>-0.02848101265822791</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24521,14 +24793,29 @@
       <c r="A78" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="B78" s="36" t="n"/>
-      <c r="C78" s="30" t="n"/>
-      <c r="D78" s="36" t="n"/>
-      <c r="E78" s="18" t="n"/>
-      <c r="F78" s="12" t="n"/>
-      <c r="G78" s="37">
-        <f>(F78/E78-1)</f>
-        <v/>
+      <c r="B78" s="36" t="inlineStr">
+        <is>
+          <t>INF</t>
+        </is>
+      </c>
+      <c r="C78" s="30" t="inlineStr">
+        <is>
+          <t>SRD</t>
+        </is>
+      </c>
+      <c r="D78" s="36" t="inlineStr">
+        <is>
+          <t>INFOTEL</t>
+        </is>
+      </c>
+      <c r="E78" s="18" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="F78" s="12" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="G78" s="37" t="n">
+        <v>-0.04114713216957602</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -24540,7 +24827,7 @@
         </is>
       </c>
       <c r="G79" s="34" t="n">
-        <v>-0.02041189464377998</v>
+        <v>-0.01679331018207544</v>
       </c>
       <c r="H79" s="6" t="n"/>
     </row>
@@ -24587,7 +24874,7 @@
         </is>
       </c>
       <c r="H81" s="49" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" thickBot="1">

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-14 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 09:11</t>
+          <t>14/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>45.5</v>
+        <v>47.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.003067484662576699</v>
+        <v>0.04732690622261167</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.01986754966887417</v>
+        <v>0.006622516556291391</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.94</v>
+        <v>25.06</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.003993610223642087</v>
+        <v>0.0007987220447284176</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>83.34999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.0006002400960383813</v>
+        <v>0.01200480192076831</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>100.95</v>
+        <v>101.05</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0</v>
+        <v>0.0009905894006933562</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>166</v>
+        <v>165.4</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0</v>
+        <v>-0.003614457831325267</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.15</v>
+        <v>55.05</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0</v>
+        <v>-0.001813236627379899</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>29.22</v>
+        <v>28.87</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.0006849315068493004</v>
+        <v>-0.01130136986301364</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>79.87</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0002503442233069974</v>
+        <v>0.0005006884466141726</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>21.5</v>
+        <v>22.42</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.006469500924214444</v>
+        <v>0.03604436229205181</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14.96</v>
+        <v>14.76</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.002680965147453145</v>
+        <v>-0.01072386058981234</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>76.5</v>
+        <v>77.55</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.005847953216374306</v>
+        <v>0.007797270955165618</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.5</v>
+        <v>28.85</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.003521126760563431</v>
+        <v>0.01584507042253531</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.355</v>
+        <v>1.525</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01094890510948914</v>
+        <v>0.1131386861313867</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20569,10 +20569,10 @@
         <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7.35</v>
+        <v>7.3</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0</v>
+        <v>-0.00680272108843535</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>384</v>
+        <v>387.6</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.0001301913813305855</v>
+        <v>0.009243588074469499</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>154</v>
+        <v>157.2</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0</v>
+        <v>0.02077922077922071</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>10.86</v>
+        <v>11.04</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.003669724770642287</v>
+        <v>0.01284403669724759</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>32</v>
+        <v>32.1</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.001560062402496011</v>
+        <v>0.001560062402496233</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.186</v>
+        <v>0.156</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.1612903225806452</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20881,10 +20881,10 @@
         <v>0.074</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.074</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0</v>
+        <v>-0.05405405405405392</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20910,10 +20910,10 @@
         <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.248</v>
+        <v>0.239</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>0</v>
+        <v>-0.03629032258064519</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20939,10 +20939,10 @@
         <v>2.58</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2.58</v>
+        <v>2.54</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>0</v>
+        <v>-0.01550387596899226</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20968,10 +20968,10 @@
         <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.95</v>
+        <v>0.958</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0</v>
+        <v>0.008421052631578956</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21055,10 +21055,10 @@
         <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.77</v>
+        <v>4.73</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.00838574423480066</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.87</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.0002503442233069974</v>
+        <v>0.0005006884466141726</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>36.34</v>
+        <v>36.48</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.00110192837465582</v>
+        <v>0.004958677685950406</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21640,10 +21640,10 @@
         <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>14.76</v>
+        <v>14.68</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.001353179972936372</v>
+        <v>-0.006765899864681979</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.255000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.001813784764207835</v>
+        <v>0.01934703748488515</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01986754966887417</v>
+        <v>0.006622516556291391</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>85.40000000000001</v>
+        <v>86.05</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0</v>
+        <v>0.007611241217798495</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>22.61</v>
+        <v>22.32</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.003105590062111814</v>
+        <v>-0.009760425909494183</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>31.4</v>
+        <v>31.62</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.000636537237428489</v>
+        <v>0.006365372374283872</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21851,10 +21851,10 @@
         <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0</v>
+        <v>0.02769230769230769</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 09:11</t>
+          <t>14/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>43.785</v>
+        <v>44.165</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.0292650482208181</v>
+        <v>-0.02084026161179465</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>85.40000000000001</v>
+        <v>86.05</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.09909909909909913</v>
+        <v>0.1074646074646074</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.94</v>
+        <v>25.06</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.0008012820512820341</v>
+        <v>0.004006410256410171</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02777777777777778</v>
+        <v>0.05555555555555555</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>83.34999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.09311475409836058</v>
+        <v>0.1055737704918032</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22875,10 +22875,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>56.9</v>
+        <v>58.15</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.08667736757624396</v>
+        <v>-0.06661316211878007</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.785</v>
+        <v>5.825</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1167938931297709</v>
+        <v>-0.1106870229007633</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.15</v>
+        <v>55.05</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03836094158674809</v>
+        <v>-0.04010462074978211</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22965,10 +22965,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>233</v>
+        <v>232.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02869757174392936</v>
+        <v>0.02649006622516556</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.09</v>
+        <v>19.13</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01380775358470534</v>
+        <v>0.01593202336696764</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.032</v>
+        <v>2.07</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.2244274809160305</v>
+        <v>-0.2099236641221375</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23127,10 +23127,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1002</v>
+        <v>1000</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.03298969072164949</v>
+        <v>0.03092783505154639</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.55</v>
+        <v>4.54</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.01562499999999986</v>
+        <v>0.01339285714285705</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.5</v>
+        <v>22.42</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.03846153846153844</v>
+        <v>0.002683363148479529</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.272</v>
+        <v>1.262</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1178918169209431</v>
+        <v>-0.1248266296809986</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.58</v>
+        <v>0.572</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1520467836257311</v>
+        <v>-0.1637426900584797</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23367,10 +23367,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>34.9</v>
+        <v>35</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.04383561643835621</v>
+        <v>-0.0410958904109589</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.803</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3398373983739837</v>
+        <v>-0.3471544715447154</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>43.75</v>
+        <v>43.8</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.07797681770284516</v>
+        <v>-0.07692307692307704</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23559,10 +23559,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.71</v>
+        <v>3.74</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.09068627450980395</v>
+        <v>-0.0833333333333333</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.74</v>
+        <v>4.82</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.08139534883720928</v>
+        <v>-0.06589147286821702</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23646,10 +23646,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.0350318471337579</v>
+        <v>-0.04140127388535023</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23675,10 +23675,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.28</v>
+        <v>1.295</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.0153846153846154</v>
+        <v>-0.003846153846153935</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.7</v>
+        <v>5.12</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.199438202247191</v>
+        <v>-0.2808988764044944</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>174.2</v>
+        <v>172.7</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05384150030248019</v>
+        <v>0.04476709013914081</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>26</v>
+        <v>25.55</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.07438016528925623</v>
+        <v>0.05578512396694221</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.878</v>
+        <v>1.896</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.009677419354838599</v>
+        <v>0.01935483870967732</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.09</v>
+        <v>19.13</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01380775358470534</v>
+        <v>0.01593202336696764</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.94</v>
+        <v>25.06</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.0008012820512820341</v>
+        <v>0.004006410256410171</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>43.785</v>
+        <v>44.165</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.0292650482208181</v>
+        <v>-0.02084026161179465</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>100.95</v>
+        <v>101.05</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.03157572041692217</v>
+        <v>0.03259758839157979</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>105.1</v>
+        <v>106.7</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05144404332129967</v>
+        <v>-0.0370036101083032</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24062,10 +24062,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>56.9</v>
+        <v>58.15</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.08667736757624396</v>
+        <v>-0.06661316211878007</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>85.40000000000001</v>
+        <v>86.05</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.09909909909909913</v>
+        <v>0.1074646074646074</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24189,10 +24189,10 @@
         <v>5.8</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>5.68</v>
+        <v>5.73</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.02068965517241381</v>
+        <v>-0.01206896551724128</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>43.785</v>
+        <v>44.165</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.0292650482208181</v>
+        <v>-0.02084026161179465</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>79.87</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.001500187523440309</v>
+        <v>-0.0007500937617200659</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>73.98</v>
+        <v>73.94</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.0223880597014926</v>
+        <v>0.0218352681039248</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>83.34999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.09311475409836058</v>
+        <v>0.1055737704918032</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>13.63</v>
+        <v>13.94</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.08246381689666776</v>
+        <v>-0.06159542241669477</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24369,10 +24369,10 @@
         <v>126.4</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>122.8</v>
+        <v>121</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.02848101265822791</v>
+        <v>-0.04272151898734181</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>40.56</v>
+        <v>42.28</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>-0.0112140419307655</v>
+        <v>0.03071672354948801</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>38.45</v>
+        <v>39.1</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.04114713216957602</v>
+        <v>-0.02493765586034912</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24542,10 +24542,10 @@
         <v>5.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>5.68</v>
+        <v>5.73</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.02068965517241381</v>
+        <v>-0.01206896551724128</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>79.87</v>
+        <v>79.93000000000001</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.001500187523440309</v>
+        <v>-0.0007500937617200659</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50.6</v>
+        <v>50.2</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.06642066420664208</v>
+        <v>-0.07380073800738007</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>73.98</v>
+        <v>73.94</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.0223880597014926</v>
+        <v>0.0218352681039248</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>40.56</v>
+        <v>42.28</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.0112140419307655</v>
+        <v>0.03071672354948801</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>43.785</v>
+        <v>44.165</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.0292650482208181</v>
+        <v>-0.02084026161179465</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>83.34999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.09311475409836058</v>
+        <v>0.1055737704918032</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>13.63</v>
+        <v>13.94</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.08246381689666776</v>
+        <v>-0.06159542241669477</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24782,10 +24782,10 @@
         <v>126.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>122.8</v>
+        <v>121</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.02848101265822791</v>
+        <v>-0.04272151898734181</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>38.45</v>
+        <v>39.1</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.04114713216957602</v>
+        <v>-0.02493765586034912</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-14 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 13:00</t>
+          <t>14/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>47.8</v>
+        <v>47.4</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.04732690622261167</v>
+        <v>0.03856266432953545</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.006622516556291391</v>
+        <v>0</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.06</v>
+        <v>24.64</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.0007987220447284176</v>
+        <v>-0.01597444089456863</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.3</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01200480192076831</v>
+        <v>0.01920768307322939</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>101.05</v>
+        <v>99.94</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0009905894006933562</v>
+        <v>-0.01000495294700352</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>165.4</v>
+        <v>166.9</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.003614457831325267</v>
+        <v>0.005421686746987986</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.05</v>
+        <v>55.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.001813236627379899</v>
+        <v>0.002719854941069784</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>28.87</v>
+        <v>28.73</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01130136986301364</v>
+        <v>-0.01609589041095887</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>79.93000000000001</v>
+        <v>80.25</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.0005006884466141726</v>
+        <v>0.004506196019526842</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>22.42</v>
+        <v>22.1</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.03604436229205181</v>
+        <v>0.02125693160813313</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14.76</v>
+        <v>14.04</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01072386058981234</v>
+        <v>-0.05898123324396788</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>77.55</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.007797270955165618</v>
+        <v>0.03118908382066266</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.85</v>
+        <v>28.6</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.01584507042253531</v>
+        <v>0.007042253521126861</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.525</v>
+        <v>1.69</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1131386861313867</v>
+        <v>0.2335766423357663</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20569,10 +20569,10 @@
         <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7.3</v>
+        <v>7.26</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.00680272108843535</v>
+        <v>-0.01224489795918366</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>387.6</v>
+        <v>390.3</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.009243588074469499</v>
+        <v>0.01627392266631949</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>157.2</v>
+        <v>156.2</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02077922077922071</v>
+        <v>0.01428571428571421</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>11.04</v>
+        <v>11.06</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.01284403669724759</v>
+        <v>0.01467889908256882</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>32.1</v>
+        <v>31.7</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.001560062402496233</v>
+        <v>-0.01092043681747263</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.156</v>
+        <v>0.164</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1612903225806452</v>
+        <v>-0.1182795698924731</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20910,10 +20910,10 @@
         <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.239</v>
+        <v>0.234</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.03629032258064519</v>
+        <v>-0.05645161290322574</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20997,10 +20997,10 @@
         <v>0.058</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.058</v>
+        <v>0.061</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>0.05172413793103441</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21026,10 +21026,10 @@
         <v>5.7</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>5.7</v>
+        <v>5.65</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>0</v>
+        <v>-0.008771929824561372</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21055,10 +21055,10 @@
         <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.73</v>
+        <v>4.69</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.00838574423480066</v>
+        <v>-0.01677148846960151</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.93000000000001</v>
+        <v>80.25</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.0005006884466141726</v>
+        <v>0.004506196019526842</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>36.48</v>
+        <v>35.8</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.004958677685950406</v>
+        <v>-0.01377410468319559</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.43</v>
+        <v>8.315</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.01934703748488515</v>
+        <v>0.005441354292623934</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.006622516556291391</v>
+        <v>0</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>86.05</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.007611241217798495</v>
+        <v>0.005269320843091201</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>22.32</v>
+        <v>22.47</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.009760425909494183</v>
+        <v>-0.003105590062111814</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>31.62</v>
+        <v>32.04</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.006365372374283872</v>
+        <v>0.01973265436028</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21851,10 +21851,10 @@
         <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>334</v>
+        <v>335.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.02769230769230769</v>
+        <v>0.03230769230769231</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 13:00</t>
+          <t>14/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>44.165</v>
+        <v>43.05</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02084026161179465</v>
+        <v>-0.04556035916195544</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>86.05</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1074646074646074</v>
+        <v>0.1048906048906048</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.06</v>
+        <v>24.64</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.004006410256410171</v>
+        <v>-0.01282051282051283</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.05555555555555555</v>
+        <v>0.04861111111111111</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.3</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.1055737704918032</v>
+        <v>0.1134426229508197</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.825</v>
+        <v>5.725</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1106870229007633</v>
+        <v>-0.1259541984732825</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.05</v>
+        <v>55.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.04010462074978211</v>
+        <v>-0.03574542284219711</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22965,10 +22965,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>232.5</v>
+        <v>228.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02649006622516556</v>
+        <v>0.008830022075055188</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.13</v>
+        <v>19.02</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01593202336696764</v>
+        <v>0.01009028146574622</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.07</v>
+        <v>2.168</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.2099236641221375</v>
+        <v>-0.1725190839694656</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23187,10 +23187,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.438</v>
+        <v>0.412</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.09876543209876541</v>
+        <v>-0.1522633744855967</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.54</v>
+        <v>4.44</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.01339285714285705</v>
+        <v>-0.008928571428571435</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.42</v>
+        <v>22.1</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.002683363148479529</v>
+        <v>-0.0116279069767441</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.262</v>
+        <v>1.266</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1248266296809986</v>
+        <v>-0.1220527045769764</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23307,10 +23307,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.077</v>
+        <v>0.075</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>-0.0384615384615385</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.572</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1637426900584797</v>
+        <v>-0.1754385964912282</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.803</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3471544715447154</v>
+        <v>-0.3414634146341463</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>43.8</v>
+        <v>44.35</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.07692307692307704</v>
+        <v>-0.065331928345627</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.82</v>
+        <v>4.79</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.06589147286821702</v>
+        <v>-0.07170542635658916</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23646,10 +23646,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>30.1</v>
+        <v>29.8</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.04140127388535023</v>
+        <v>-0.05095541401273879</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23675,10 +23675,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.295</v>
+        <v>1.3</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.003846153846153935</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.12</v>
+        <v>5.48</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2808988764044944</v>
+        <v>-0.2303370786516853</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>172.7</v>
+        <v>172.9</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.04476709013914081</v>
+        <v>0.04597701149425284</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.55</v>
+        <v>25.65</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.05578512396694221</v>
+        <v>0.0599173553719008</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.896</v>
+        <v>1.884</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.01935483870967732</v>
+        <v>0.0129032258064515</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.13</v>
+        <v>19.02</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01593202336696764</v>
+        <v>0.01009028146574622</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>25.06</v>
+        <v>24.64</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.004006410256410171</v>
+        <v>-0.01282051282051283</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>44.165</v>
+        <v>43.05</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02084026161179465</v>
+        <v>-0.04556035916195544</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>101.05</v>
+        <v>99.94</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.03259758839157979</v>
+        <v>0.02125485387287961</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>106.7</v>
+        <v>105.1</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0370036101083032</v>
+        <v>-0.05144404332129967</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>86.05</v>
+        <v>85.84999999999999</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.1074646074646074</v>
+        <v>0.1048906048906048</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24189,10 +24189,10 @@
         <v>5.8</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>5.73</v>
+        <v>5.71</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.01206896551724128</v>
+        <v>-0.01551724137931032</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>44.165</v>
+        <v>43.05</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.02084026161179465</v>
+        <v>-0.04556035916195544</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>79.93000000000001</v>
+        <v>80.25</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.0007500937617200659</v>
+        <v>0.003250406300787663</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>73.94</v>
+        <v>73.78</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.0218352681039248</v>
+        <v>0.01962410171365398</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>84.3</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.1055737704918032</v>
+        <v>0.1134426229508197</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>13.94</v>
+        <v>13.67</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.06159542241669477</v>
+        <v>-0.07977112083473581</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24369,10 +24369,10 @@
         <v>126.4</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>121</v>
+        <v>121.8</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.04272151898734181</v>
+        <v>-0.03639240506329121</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>42.28</v>
+        <v>41.76</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.03071672354948801</v>
+        <v>0.01803998049731826</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>39.1</v>
+        <v>38.55</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.02493765586034912</v>
+        <v>-0.03865336658354125</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24542,10 +24542,10 @@
         <v>5.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>5.73</v>
+        <v>5.71</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.01206896551724128</v>
+        <v>-0.01551724137931032</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>79.93000000000001</v>
+        <v>80.25</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.0007500937617200659</v>
+        <v>0.003250406300787663</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50.2</v>
+        <v>50.8</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.07380073800738007</v>
+        <v>-0.06273062730627317</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>73.94</v>
+        <v>73.78</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.0218352681039248</v>
+        <v>0.01962410171365398</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>42.28</v>
+        <v>41.76</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.03071672354948801</v>
+        <v>0.01803998049731826</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>44.165</v>
+        <v>43.05</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.02084026161179465</v>
+        <v>-0.04556035916195544</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>84.3</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.1055737704918032</v>
+        <v>0.1134426229508197</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>13.94</v>
+        <v>13.67</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.06159542241669477</v>
+        <v>-0.07977112083473581</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24782,10 +24782,10 @@
         <v>126.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>121</v>
+        <v>121.8</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.04272151898734181</v>
+        <v>-0.03639240506329121</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>39.1</v>
+        <v>38.55</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.02493765586034912</v>
+        <v>-0.03865336658354125</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-15 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 19:05</t>
+          <t>15/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>47.4</v>
+        <v>48.06</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.03856266432953545</v>
+        <v>0.05302366345311135</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>151</v>
+        <v>151.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0</v>
+        <v>0.003311258278145695</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.64</v>
+        <v>25.28</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01597444089456863</v>
+        <v>0.009584664536741293</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01920768307322939</v>
+        <v>-0.003601440576230458</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>99.94</v>
+        <v>101.85</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.01000495294700352</v>
+        <v>0.008915304606240628</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>166.9</v>
+        <v>168.2</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.005421686746987986</v>
+        <v>0.0132530120481927</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.3</v>
+        <v>55.7</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.002719854941069784</v>
+        <v>0.00997280145058938</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>28.73</v>
+        <v>29.08</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01609589041095887</v>
+        <v>-0.004109589041095925</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>80.25</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.004506196019526842</v>
+        <v>0.01301789961196653</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>22.1</v>
+        <v>21.44</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.02125693160813313</v>
+        <v>-0.009242144177449136</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14.04</v>
+        <v>14</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.05898123324396788</v>
+        <v>-0.0616621983914209</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>79.34999999999999</v>
+        <v>78.25</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.03118908382066266</v>
+        <v>0.01689408706952563</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.6</v>
+        <v>28.35</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.007042253521126861</v>
+        <v>-0.00176056338028159</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.69</v>
+        <v>1.574</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.2335766423357663</v>
+        <v>0.1489051094890511</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>390.3</v>
+        <v>393.9</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.01627392266631949</v>
+        <v>0.02564770212211943</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>156.2</v>
+        <v>155</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01428571428571421</v>
+        <v>0.006493506493506494</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>11.06</v>
+        <v>10.7</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.01467889908256882</v>
+        <v>-0.01834862385321111</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>31.7</v>
+        <v>33.5</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.01092043681747263</v>
+        <v>0.04524180967238699</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20794,10 +20794,10 @@
         <v>4.02</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>4.02</v>
+        <v>4.03</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0</v>
+        <v>0.002487562189054895</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.164</v>
+        <v>0.16</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1182795698924731</v>
+        <v>-0.1397849462365591</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20852,10 +20852,10 @@
         <v>1.02</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.02</v>
+        <v>0.976</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0</v>
+        <v>-0.04313725490196082</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20881,10 +20881,10 @@
         <v>0.074</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.073</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05405405405405392</v>
+        <v>-0.01351351351351353</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20910,10 +20910,10 @@
         <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.234</v>
+        <v>0.237</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.05645161290322574</v>
+        <v>-0.04435483870967746</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20939,10 +20939,10 @@
         <v>2.58</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2.54</v>
+        <v>2.5</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01550387596899226</v>
+        <v>-0.03100775193798452</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20968,10 +20968,10 @@
         <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.958</v>
+        <v>0.96</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.008421052631578956</v>
+        <v>0.01052631578947369</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20997,10 +20997,10 @@
         <v>0.058</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.061</v>
+        <v>0.059</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.05172413793103441</v>
+        <v>0.01724137931034472</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21055,10 +21055,10 @@
         <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.69</v>
+        <v>4.28</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.01677148846960151</v>
+        <v>-0.1027253668763101</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>80.25</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.004506196019526842</v>
+        <v>0.01301789961196653</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>35.8</v>
+        <v>36.04</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.01377410468319559</v>
+        <v>-0.007162534435261654</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21640,10 +21640,10 @@
         <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>14.68</v>
+        <v>14.58</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.006765899864681979</v>
+        <v>-0.01353179972936396</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.315</v>
+        <v>8.06</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.005441354292623934</v>
+        <v>-0.02539298669891162</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>151</v>
+        <v>151.5</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0</v>
+        <v>0.003311258278145695</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>85.84999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.005269320843091201</v>
+        <v>0.008196721311475277</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>22.47</v>
+        <v>22.5</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.003105590062111814</v>
+        <v>-0.001774622892635277</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>32.04</v>
+        <v>31.94</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.01973265436028</v>
+        <v>0.01654996817313811</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21851,10 +21851,10 @@
         <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>335.5</v>
+        <v>333.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.03230769230769231</v>
+        <v>0.02615384615384615</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>14/10/2026 19:05</t>
+          <t>15/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>43.05</v>
+        <v>40.045</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.04556035916195544</v>
+        <v>-0.1121826848464692</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>85.84999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1048906048906048</v>
+        <v>0.108108108108108</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>24.64</v>
+        <v>25.28</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>0.01282051282051283</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>151</v>
+        <v>151.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.04861111111111111</v>
+        <v>0.05208333333333334</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.1134426229508197</v>
+        <v>0.08852459016393442</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22875,10 +22875,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>58.15</v>
+        <v>56.25</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.06661316211878007</v>
+        <v>-0.09711075441412516</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.725</v>
+        <v>5.445</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1259541984732825</v>
+        <v>-0.1687022900763358</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.3</v>
+        <v>55.7</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.03574542284219711</v>
+        <v>-0.028770706190061</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22965,10 +22965,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>228.5</v>
+        <v>229</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.008830022075055188</v>
+        <v>0.01103752759381899</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.02</v>
+        <v>19.19</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01009028146574622</v>
+        <v>0.01911842804036129</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.168</v>
+        <v>2.31</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1725190839694656</v>
+        <v>-0.1183206106870229</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23127,10 +23127,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.03092783505154639</v>
+        <v>0.02989690721649485</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23187,10 +23187,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.412</v>
+        <v>0.413</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1522633744855967</v>
+        <v>-0.1502057613168724</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.44</v>
+        <v>4.31</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.008928571428571435</v>
+        <v>-0.03794642857142875</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.1</v>
+        <v>21.44</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.0116279069767441</v>
+        <v>-0.0411449016100178</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.266</v>
+        <v>1.268</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1220527045769764</v>
+        <v>-0.1206657420249653</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23307,10 +23307,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.075</v>
+        <v>0.076</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.0384615384615385</v>
+        <v>-0.02564102564102566</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.57</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1754385964912282</v>
+        <v>-0.1666666666666668</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23367,10 +23367,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>35</v>
+        <v>35.5</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0410958904109589</v>
+        <v>-0.0273972602739726</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.789</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3414634146341463</v>
+        <v>-0.3585365853658536</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>44.35</v>
+        <v>40.85</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.065331928345627</v>
+        <v>-0.1390937829293994</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23530,10 +23530,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>1.02</v>
+        <v>0.976</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>0.04081632653061228</v>
+        <v>-0.004081632653061228</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.79</v>
+        <v>4.705</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.07170542635658916</v>
+        <v>-0.08817829457364343</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23617,10 +23617,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.62</v>
+        <v>4.72</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.07599999999999998</v>
+        <v>-0.05600000000000005</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23646,10 +23646,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>29.8</v>
+        <v>30</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05095541401273879</v>
+        <v>-0.04458598726114645</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23675,10 +23675,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.007692307692307699</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23704,10 +23704,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.145</v>
+        <v>1.13</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.08399999999999999</v>
+        <v>-0.09600000000000009</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.48</v>
+        <v>5.38</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2303370786516853</v>
+        <v>-0.2443820224719101</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>172.9</v>
+        <v>173.6</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.04597701149425284</v>
+        <v>0.05021173623714448</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.65</v>
+        <v>25.6</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.0599173553719008</v>
+        <v>0.05785123966942158</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.884</v>
+        <v>1.882</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.0129032258064515</v>
+        <v>0.0118279569892472</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.02</v>
+        <v>19.19</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01009028146574622</v>
+        <v>0.01911842804036129</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>24.64</v>
+        <v>25.28</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>-0.01282051282051283</v>
+        <v>0.01282051282051283</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>43.05</v>
+        <v>40.045</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04556035916195544</v>
+        <v>-0.1121826848464692</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>99.94</v>
+        <v>101.85</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.02125485387287961</v>
+        <v>0.04077253218884115</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>105.1</v>
+        <v>106.3</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05144404332129967</v>
+        <v>-0.04061371841155235</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24062,10 +24062,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>58.15</v>
+        <v>56.25</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.06661316211878007</v>
+        <v>-0.09711075441412516</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>85.84999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.1048906048906048</v>
+        <v>0.108108108108108</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24189,10 +24189,10 @@
         <v>5.8</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>5.71</v>
+        <v>5.67</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.01551724137931032</v>
+        <v>-0.02241379310344826</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>43.05</v>
+        <v>40.045</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.04556035916195544</v>
+        <v>-0.1121826848464692</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>80.25</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>0.003250406300787663</v>
+        <v>0.01175146893361685</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>73.78</v>
+        <v>74.44</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.01962410171365398</v>
+        <v>0.02874516307352126</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.1134426229508197</v>
+        <v>0.08852459016393442</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>13.67</v>
+        <v>13.405</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.07977112083473581</v>
+        <v>-0.09761023224503541</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24369,10 +24369,10 @@
         <v>126.4</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>121.8</v>
+        <v>122</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.03639240506329121</v>
+        <v>-0.03481012658227853</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>41.76</v>
+        <v>40.24</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>0.01803998049731826</v>
+        <v>-0.01901511457825454</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>38.55</v>
+        <v>38.35</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.03865336658354125</v>
+        <v>-0.04364089775561097</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24542,10 +24542,10 @@
         <v>5.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>5.71</v>
+        <v>5.67</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.01551724137931032</v>
+        <v>-0.02241379310344826</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>80.25</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.003250406300787663</v>
+        <v>0.01175146893361685</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>50.8</v>
+        <v>47.4</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.06273062730627317</v>
+        <v>-0.1254612546125462</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>73.78</v>
+        <v>74.44</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.01962410171365398</v>
+        <v>0.02874516307352126</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>41.76</v>
+        <v>40.24</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.01803998049731826</v>
+        <v>-0.01901511457825454</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>43.05</v>
+        <v>40.045</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.04556035916195544</v>
+        <v>-0.1121826848464692</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.1134426229508197</v>
+        <v>0.08852459016393442</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>13.67</v>
+        <v>13.405</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.07977112083473581</v>
+        <v>-0.09761023224503541</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24782,10 +24782,10 @@
         <v>126.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>121.8</v>
+        <v>122</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.03639240506329121</v>
+        <v>-0.03481012658227853</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>38.55</v>
+        <v>38.35</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.03865336658354125</v>
+        <v>-0.04364089775561097</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-15 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>15/10/2026 13:00</t>
+          <t>15/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>48.06</v>
+        <v>49.34</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.05302366345311135</v>
+        <v>0.08106923751095536</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>151.5</v>
+        <v>147.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.003311258278145695</v>
+        <v>-0.02317880794701987</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.28</v>
+        <v>25.66</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.009584664536741293</v>
+        <v>0.02476038338658151</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>83</v>
+        <v>84.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.003601440576230458</v>
+        <v>0.014405762304922</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>101.85</v>
+        <v>103.1</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.008915304606240628</v>
+        <v>0.02129767211490828</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>168.2</v>
+        <v>166.1</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.0132530120481927</v>
+        <v>0.0006024096385541827</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.7</v>
+        <v>55.85</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.00997280145058938</v>
+        <v>0.01269265639165916</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>29.08</v>
+        <v>29.38</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.004109589041095925</v>
+        <v>0.006164383561643826</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>80.93000000000001</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01301789961196653</v>
+        <v>0.005757917136062007</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>21.44</v>
+        <v>21.8</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.009242144177449136</v>
+        <v>0.007393715341959341</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14</v>
+        <v>14.74</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.0616621983914209</v>
+        <v>-0.01206434316353885</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>78.25</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01689408706952563</v>
+        <v>0.06692657569850541</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.35</v>
+        <v>28.5</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.00176056338028159</v>
+        <v>0.003521126760563431</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.574</v>
+        <v>1.536</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1489051094890511</v>
+        <v>0.1211678832116788</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20569,10 +20569,10 @@
         <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7.26</v>
+        <v>7.2</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.01224489795918366</v>
+        <v>-0.02040816326530605</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>393.9</v>
+        <v>396.6</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.02564770212211943</v>
+        <v>0.03267803671396956</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.006493506493506494</v>
+        <v>0.01948051948051948</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>10.7</v>
+        <v>10.72</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01834862385321111</v>
+        <v>-0.01651376146788988</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>33.5</v>
+        <v>34.35</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.04524180967238699</v>
+        <v>0.07176287051482073</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.16</v>
+        <v>0.158</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1397849462365591</v>
+        <v>-0.1505376344086021</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20852,10 +20852,10 @@
         <v>1.02</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.976</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.04313725490196082</v>
+        <v>-0.07647058823529418</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20881,10 +20881,10 @@
         <v>0.074</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.073</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01351351351351353</v>
+        <v>-0.02702702702702705</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20939,10 +20939,10 @@
         <v>2.58</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2.5</v>
+        <v>2.54</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.03100775193798452</v>
+        <v>-0.01550387596899226</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20968,10 +20968,10 @@
         <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.01052631578947369</v>
+        <v>-0.03157894736842096</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20997,10 +20997,10 @@
         <v>0.058</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.059</v>
+        <v>0.058</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.01724137931034472</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21026,10 +21026,10 @@
         <v>5.7</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>5.65</v>
+        <v>5.6</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.008771929824561372</v>
+        <v>-0.0175438596491229</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -21055,10 +21055,10 @@
         <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.28</v>
+        <v>4.17</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.1027253668763101</v>
+        <v>-0.1257861635220125</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>80.93000000000001</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.01301789961196653</v>
+        <v>0.005757917136062007</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>36.04</v>
+        <v>36.1</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.007162534435261654</v>
+        <v>-0.00550964187327812</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21640,10 +21640,10 @@
         <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>14.58</v>
+        <v>14.56</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.01353179972936396</v>
+        <v>-0.01488497970230033</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.06</v>
+        <v>8.01</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.02539298669891162</v>
+        <v>-0.03143893591293831</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>151.5</v>
+        <v>147.5</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.003311258278145695</v>
+        <v>-0.02317880794701987</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>86.09999999999999</v>
+        <v>87.45</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.008196721311475277</v>
+        <v>0.02400468384074938</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>22.5</v>
+        <v>23.04</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.001774622892635277</v>
+        <v>0.02218278615794144</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>31.94</v>
+        <v>32</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.01654996817313811</v>
+        <v>0.01845957988542324</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21851,10 +21851,10 @@
         <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>333.5</v>
+        <v>336.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.02615384615384615</v>
+        <v>0.03538461538461538</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>15/10/2026 13:00</t>
+          <t>15/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>40.045</v>
+        <v>41.32</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.1121826848464692</v>
+        <v>-0.08391530872408817</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>86.09999999999999</v>
+        <v>87.45</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.108108108108108</v>
+        <v>0.1254826254826255</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.28</v>
+        <v>25.66</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.01282051282051283</v>
+        <v>0.02804487179487176</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>151.5</v>
+        <v>147.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.05208333333333334</v>
+        <v>0.02430555555555556</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>83</v>
+        <v>84.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.08852459016393442</v>
+        <v>0.1081967213114754</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22875,10 +22875,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>56.25</v>
+        <v>57.45</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.09711075441412516</v>
+        <v>-0.07784911717495978</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.445</v>
+        <v>5.545</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1687022900763358</v>
+        <v>-0.1534351145038168</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.7</v>
+        <v>55.85</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.028770706190061</v>
+        <v>-0.02615518744551002</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22965,10 +22965,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>229</v>
+        <v>229.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01103752759381899</v>
+        <v>0.01324503311258278</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.19</v>
+        <v>19.14</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01911842804036129</v>
+        <v>0.01646309081253331</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.31</v>
+        <v>2.57</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.1183206106870229</v>
+        <v>-0.01908396946564896</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23127,10 +23127,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.02989690721649485</v>
+        <v>0.03092783505154639</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23187,10 +23187,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.413</v>
+        <v>0.43</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1502057613168724</v>
+        <v>-0.1152263374485597</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.31</v>
+        <v>4.305</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03794642857142875</v>
+        <v>-0.03906250000000015</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.44</v>
+        <v>21.8</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.0411449016100178</v>
+        <v>-0.02504472271914127</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.268</v>
+        <v>1.296</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1206657420249653</v>
+        <v>-0.1012482662968099</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23307,10 +23307,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.076</v>
+        <v>0.074</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.02564102564102566</v>
+        <v>-0.05128205128205133</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1666666666666668</v>
+        <v>-0.195906432748538</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23367,10 +23367,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>35.5</v>
+        <v>35.2</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0273972602739726</v>
+        <v>-0.03561643835616431</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.789</v>
+        <v>0.76</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3585365853658536</v>
+        <v>-0.3821138211382114</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>40.85</v>
+        <v>40.55</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1390937829293994</v>
+        <v>-0.1454162276080085</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23530,10 +23530,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.976</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.004081632653061228</v>
+        <v>-0.03877551020408167</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23559,10 +23559,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.74</v>
+        <v>3.71</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0833333333333333</v>
+        <v>-0.09068627450980395</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.705</v>
+        <v>4.665</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.08817829457364343</v>
+        <v>-0.09593023255813955</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23617,10 +23617,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.72</v>
+        <v>4.62</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.05600000000000005</v>
+        <v>-0.07599999999999998</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23646,10 +23646,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>30</v>
+        <v>29.8</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.04458598726114645</v>
+        <v>-0.05095541401273879</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23704,10 +23704,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.13</v>
+        <v>1.18</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.09600000000000009</v>
+        <v>-0.05600000000000005</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.38</v>
+        <v>5.56</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2443820224719101</v>
+        <v>-0.2191011235955057</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>173.6</v>
+        <v>178</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.05021173623714448</v>
+        <v>0.0768300060496067</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>25.6</v>
+        <v>26.4</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.05785123966942158</v>
+        <v>0.09090909090909088</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.882</v>
+        <v>1.884</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.0118279569892472</v>
+        <v>0.0129032258064515</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.19</v>
+        <v>19.14</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01911842804036129</v>
+        <v>0.01646309081253331</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>25.28</v>
+        <v>25.66</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.01282051282051283</v>
+        <v>0.02804487179487176</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>40.045</v>
+        <v>41.32</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.1121826848464692</v>
+        <v>-0.08391530872408817</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>101.85</v>
+        <v>103.1</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04077253218884115</v>
+        <v>0.05354588187206208</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>106.3</v>
+        <v>107.3</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.04061371841155235</v>
+        <v>-0.0315884476534296</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24062,10 +24062,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>56.25</v>
+        <v>57.45</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.09711075441412516</v>
+        <v>-0.07784911717495978</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>86.09999999999999</v>
+        <v>87.45</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.108108108108108</v>
+        <v>0.1254826254826255</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>40.045</v>
+        <v>41.32</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.1121826848464692</v>
+        <v>-0.08391530872408817</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>80.93000000000001</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>0.01175146893361685</v>
+        <v>0.004500562570321284</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>74.44</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.02874516307352126</v>
+        <v>0.05666113875069091</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>83</v>
+        <v>84.5</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.08852459016393442</v>
+        <v>0.1081967213114754</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>13.405</v>
+        <v>13.6</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.09761023224503541</v>
+        <v>-0.08448333894311684</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>40.24</v>
+        <v>40.08</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>-0.01901511457825454</v>
+        <v>-0.02291565090199914</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>38.35</v>
+        <v>38.45</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.04364089775561097</v>
+        <v>-0.04114713216957602</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>80.93000000000001</v>
+        <v>80.34999999999999</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.01175146893361685</v>
+        <v>0.004500562570321284</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>47.4</v>
+        <v>48</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.1254612546125462</v>
+        <v>-0.1143911439114392</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>74.44</v>
+        <v>76.45999999999999</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.02874516307352126</v>
+        <v>0.05666113875069091</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>40.24</v>
+        <v>40.08</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01901511457825454</v>
+        <v>-0.02291565090199914</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>40.045</v>
+        <v>41.32</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.1121826848464692</v>
+        <v>-0.08391530872408817</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>83</v>
+        <v>84.5</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.08852459016393442</v>
+        <v>0.1081967213114754</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>13.405</v>
+        <v>13.6</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.09761023224503541</v>
+        <v>-0.08448333894311684</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>38.35</v>
+        <v>38.45</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.04364089775561097</v>
+        <v>-0.04114713216957602</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-16 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>15/10/2026 19:05</t>
+          <t>16/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>49.34</v>
+        <v>50.4</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.08106923751095536</v>
+        <v>0.1042944785276073</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>147.5</v>
+        <v>148.5</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02317880794701987</v>
+        <v>-0.01655629139072848</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.66</v>
+        <v>25.92</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02476038338658151</v>
+        <v>0.03514376996805122</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.5</v>
+        <v>87.05</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.014405762304922</v>
+        <v>0.04501800720288116</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>103.1</v>
+        <v>105</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02129767211490828</v>
+        <v>0.04011887072808318</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>166.1</v>
+        <v>166.3</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.0006024096385541827</v>
+        <v>0.001807228915662719</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.85</v>
+        <v>56.45</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.01269265639165916</v>
+        <v>0.02357207615593843</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>29.38</v>
+        <v>30.33</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.006164383561643826</v>
+        <v>0.03869863013698627</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>80.34999999999999</v>
+        <v>79.83</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.005757917136062007</v>
+        <v>-0.00075103266992117</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>21.8</v>
+        <v>22.7</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.007393715341959341</v>
+        <v>0.04898336414048053</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14.74</v>
+        <v>14.8</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01206434316353885</v>
+        <v>-0.008042895442359197</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>82.09999999999999</v>
+        <v>81.34999999999999</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.06692657569850541</v>
+        <v>0.05717998700454829</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.5</v>
+        <v>28.9</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.003521126760563431</v>
+        <v>0.0176056338028169</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.536</v>
+        <v>1.743</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1211678832116788</v>
+        <v>0.2722627737226277</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20569,10 +20569,10 @@
         <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7.2</v>
+        <v>7.41</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02040816326530605</v>
+        <v>0.008163265306122517</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>396.6</v>
+        <v>399.05</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.03267803671396956</v>
+        <v>0.03905741439916677</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>157</v>
+        <v>157.4</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01948051948051948</v>
+        <v>0.02207792207792212</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>10.72</v>
+        <v>10.78</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.01651376146788988</v>
+        <v>-0.0110091743119267</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>34.35</v>
+        <v>33.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.07176287051482073</v>
+        <v>0.0546021840873635</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20794,10 +20794,10 @@
         <v>4.02</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>4.03</v>
+        <v>4.02</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>0.002487562189054895</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.158</v>
+        <v>0.157</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1505376344086021</v>
+        <v>-0.1559139784946237</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20852,10 +20852,10 @@
         <v>1.02</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.07647058823529418</v>
+        <v>-0.07843137254901968</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20910,10 +20910,10 @@
         <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.237</v>
+        <v>0.225</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.04435483870967746</v>
+        <v>-0.09274193548387094</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20939,10 +20939,10 @@
         <v>2.58</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2.54</v>
+        <v>2.52</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01550387596899226</v>
+        <v>-0.02325581395348839</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -20968,10 +20968,10 @@
         <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.92</v>
+        <v>0.89</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03157894736842096</v>
+        <v>-0.06315789473684205</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>80.34999999999999</v>
+        <v>79.83</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.005757917136062007</v>
+        <v>-0.00075103266992117</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>36.1</v>
+        <v>37.48</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.00550964187327812</v>
+        <v>0.03250688705234159</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21640,10 +21640,10 @@
         <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>14.56</v>
+        <v>15.24</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.01488497970230033</v>
+        <v>0.03112313937753727</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.01</v>
+        <v>8.145</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03143893591293831</v>
+        <v>-0.01511487303506651</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>147.5</v>
+        <v>148.5</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.02317880794701987</v>
+        <v>-0.01655629139072848</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>87.45</v>
+        <v>87.8</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.02400468384074938</v>
+        <v>0.02810304449648702</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>23.04</v>
+        <v>23.48</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.02218278615794144</v>
+        <v>0.04170363797692996</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>32</v>
+        <v>32.46</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.01845957988542324</v>
+        <v>0.03309993634627623</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>15/10/2026 19:05</t>
+          <t>16/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>41.32</v>
+        <v>41.36</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.08391530872408817</v>
+        <v>-0.08302848908103309</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>87.45</v>
+        <v>87.8</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1254826254826255</v>
+        <v>0.1299871299871299</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.66</v>
+        <v>25.92</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02804487179487176</v>
+        <v>0.03846153846153849</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>147.5</v>
+        <v>148.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02430555555555556</v>
+        <v>0.03125</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.5</v>
+        <v>87.05</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.1081967213114754</v>
+        <v>0.141639344262295</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22875,10 +22875,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>57.45</v>
+        <v>58.85</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.07784911717495978</v>
+        <v>-0.05537720706260026</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.545</v>
+        <v>5.56</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.1534351145038168</v>
+        <v>-0.151145038167939</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>55.85</v>
+        <v>56.45</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.02615518744551002</v>
+        <v>-0.01569311246730599</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.14</v>
+        <v>19.19</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01646309081253331</v>
+        <v>0.01911842804036129</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.57</v>
+        <v>2.38</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01908396946564896</v>
+        <v>-0.09160305343511459</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23127,10 +23127,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1000</v>
+        <v>1012</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.03092783505154639</v>
+        <v>0.04329896907216495</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23187,10 +23187,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.43</v>
+        <v>0.444</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.1152263374485597</v>
+        <v>-0.08641975308641972</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.305</v>
+        <v>4.43</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03906250000000015</v>
+        <v>-0.01116071428571444</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>21.8</v>
+        <v>22.7</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.02504472271914127</v>
+        <v>0.01520572450805008</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.296</v>
+        <v>1.306</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.1012482662968099</v>
+        <v>-0.09431345353675444</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23307,10 +23307,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.074</v>
+        <v>0.076</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.05128205128205133</v>
+        <v>-0.02564102564102566</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.55</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.195906432748538</v>
+        <v>-0.1842105263157895</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23367,10 +23367,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>35.2</v>
+        <v>35.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.03561643835616431</v>
+        <v>-0.0191780821917809</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.76</v>
+        <v>0.714</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.3821138211382114</v>
+        <v>-0.4195121951219513</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>40.55</v>
+        <v>40.3</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1454162276080085</v>
+        <v>-0.1506849315068494</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23530,10 +23530,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03877551020408167</v>
+        <v>-0.04081632653061228</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23559,10 +23559,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.71</v>
+        <v>3.78</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.09068627450980395</v>
+        <v>-0.07352941176470594</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.665</v>
+        <v>4.52</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.09593023255813955</v>
+        <v>-0.1240310077519381</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23675,10 +23675,10 @@
         <v>1.3</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>1.29</v>
+        <v>1.295</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.007692307692307699</v>
+        <v>-0.003846153846153935</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -23704,10 +23704,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.18</v>
+        <v>1.17</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.05600000000000005</v>
+        <v>-0.06400000000000006</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.56</v>
+        <v>5.5</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2191011235955057</v>
+        <v>-0.2275280898876405</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>178</v>
+        <v>182.2</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.0768300060496067</v>
+        <v>0.1022383545069569</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>26.4</v>
+        <v>26.6</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.09090909090909088</v>
+        <v>0.09917355371900835</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.884</v>
+        <v>1.882</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.0129032258064515</v>
+        <v>0.0118279569892472</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.14</v>
+        <v>19.19</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01646309081253331</v>
+        <v>0.01911842804036129</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>25.66</v>
+        <v>25.92</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.02804487179487176</v>
+        <v>0.03846153846153849</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>41.32</v>
+        <v>41.36</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.08391530872408817</v>
+        <v>-0.08302848908103309</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>103.1</v>
+        <v>105</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05354588187206208</v>
+        <v>0.07296137339055794</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>107.3</v>
+        <v>108.2</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.0315884476534296</v>
+        <v>-0.02346570397111908</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24062,10 +24062,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>57.45</v>
+        <v>58.85</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.07784911717495978</v>
+        <v>-0.05537720706260026</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>87.45</v>
+        <v>87.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.1254826254826255</v>
+        <v>0.1299871299871299</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24189,10 +24189,10 @@
         <v>5.8</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>5.67</v>
+        <v>5.72</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.02241379310344826</v>
+        <v>-0.01379310344827587</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>41.32</v>
+        <v>41.36</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.08391530872408817</v>
+        <v>-0.08302848908103309</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>80.34999999999999</v>
+        <v>79.83</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>0.004500562570321284</v>
+        <v>-0.002000250031253864</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>76.45999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.05666113875069091</v>
+        <v>0.0558319513543395</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>84.5</v>
+        <v>87.05</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.1081967213114754</v>
+        <v>0.141639344262295</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>13.6</v>
+        <v>14.515</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.08448333894311684</v>
+        <v>-0.02288791652642207</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24369,10 +24369,10 @@
         <v>126.4</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>122</v>
+        <v>121.4</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.03481012658227853</v>
+        <v>-0.03955696202531645</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>40.08</v>
+        <v>40.7</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>-0.02291565090199914</v>
+        <v>-0.007801072647489036</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>38.45</v>
+        <v>38.5</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.04114713216957602</v>
+        <v>-0.03990024937655864</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24542,10 +24542,10 @@
         <v>5.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>5.67</v>
+        <v>5.72</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.02241379310344826</v>
+        <v>-0.01379310344827587</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>80.34999999999999</v>
+        <v>79.83</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.004500562570321284</v>
+        <v>-0.002000250031253864</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>48</v>
+        <v>48.6</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.1143911439114392</v>
+        <v>-0.1033210332103321</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>76.45999999999999</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.05666113875069091</v>
+        <v>0.0558319513543395</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>40.08</v>
+        <v>40.7</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.02291565090199914</v>
+        <v>-0.007801072647489036</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>41.32</v>
+        <v>41.36</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.08391530872408817</v>
+        <v>-0.08302848908103309</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>84.5</v>
+        <v>87.05</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.1081967213114754</v>
+        <v>0.141639344262295</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>13.6</v>
+        <v>14.515</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.08448333894311684</v>
+        <v>-0.02288791652642207</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24782,10 +24782,10 @@
         <v>126.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>122</v>
+        <v>121.4</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.03481012658227853</v>
+        <v>-0.03955696202531645</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>38.45</v>
+        <v>38.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.04114713216957602</v>
+        <v>-0.03990024937655864</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-16 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -20019,7 +20019,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/10/2026 13:00</t>
+          <t>16/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -20046,10 +20046,10 @@
         <v>45.64</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>50.4</v>
+        <v>51.05</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.1042944785276073</v>
+        <v>0.1185363716038562</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -20076,10 +20076,10 @@
         <v>151</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>148.5</v>
+        <v>148</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.01655629139072848</v>
+        <v>-0.01986754966887417</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -20106,10 +20106,10 @@
         <v>25.04</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.92</v>
+        <v>25.84</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.03514376996805122</v>
+        <v>0.03194888178913741</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -20167,10 +20167,10 @@
         <v>83.3</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>87.05</v>
+        <v>83.75</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.04501800720288116</v>
+        <v>0.005402160864345773</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -20197,10 +20197,10 @@
         <v>100.95</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>105</v>
+        <v>102.55</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.04011887072808318</v>
+        <v>0.01584943041109454</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -20227,10 +20227,10 @@
         <v>166</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>166.3</v>
+        <v>167.3</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.001807228915662719</v>
+        <v>0.007831325301204888</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -20257,10 +20257,10 @@
         <v>55.15</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>56.45</v>
+        <v>56.35</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02357207615593843</v>
+        <v>0.02175883952855853</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -20287,10 +20287,10 @@
         <v>29.2</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>30.33</v>
+        <v>30.05</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.03869863013698627</v>
+        <v>0.02910958904109594</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -20317,10 +20317,10 @@
         <v>79.89</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>79.83</v>
+        <v>80.45</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.00075103266992117</v>
+        <v>0.00700963825259735</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -20419,10 +20419,10 @@
         <v>21.64</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>22.7</v>
+        <v>22.48</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.04898336414048053</v>
+        <v>0.0388170055452865</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -20449,10 +20449,10 @@
         <v>14.92</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.008042895442359197</v>
+        <v>-0.02815013404825737</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -20479,10 +20479,10 @@
         <v>76.95</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>81.34999999999999</v>
+        <v>78.5</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.05717998700454829</v>
+        <v>0.02014294996751133</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -20509,10 +20509,10 @@
         <v>28.4</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>28.9</v>
+        <v>28.7</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.0176056338028169</v>
+        <v>0.01056338028169017</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -20539,10 +20539,10 @@
         <v>1.37</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1.743</v>
+        <v>1.775</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.2722627737226277</v>
+        <v>0.2956204379562042</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -20569,10 +20569,10 @@
         <v>7.35</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>7.41</v>
+        <v>7.24</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.008163265306122517</v>
+        <v>-0.01496598639455775</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -20599,10 +20599,10 @@
         <v>384.05</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>399.05</v>
+        <v>397.9</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.03905741439916677</v>
+        <v>0.0360630126285639</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -20629,10 +20629,10 @@
         <v>154</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>157.4</v>
+        <v>157.2</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02207792207792212</v>
+        <v>0.02077922077922071</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -20659,10 +20659,10 @@
         <v>10.9</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>10.78</v>
+        <v>10.76</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.0110091743119267</v>
+        <v>-0.01284403669724776</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -20689,10 +20689,10 @@
         <v>32.05</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>33.8</v>
+        <v>34</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0546021840873635</v>
+        <v>0.06084243369734799</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -20823,10 +20823,10 @@
         <v>0.186</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.157</v>
+        <v>0.154</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1559139784946237</v>
+        <v>-0.1720430107526882</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -20852,10 +20852,10 @@
         <v>1.02</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.07843137254901968</v>
+        <v>-0.0490196078431373</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -20881,10 +20881,10 @@
         <v>0.074</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02702702702702705</v>
+        <v>-0.06756756756756745</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -20910,10 +20910,10 @@
         <v>0.248</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.225</v>
+        <v>0.224</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.09274193548387094</v>
+        <v>-0.09677419354838707</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -20968,10 +20968,10 @@
         <v>0.95</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>0.89</v>
+        <v>0.92</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06315789473684205</v>
+        <v>-0.03157894736842096</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -20997,10 +20997,10 @@
         <v>0.058</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>0.058</v>
+        <v>0.054</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0</v>
+        <v>-0.06896551724137936</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -21055,10 +21055,10 @@
         <v>4.77</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.17</v>
+        <v>4.13</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.1257861635220125</v>
+        <v>-0.1341719077568134</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -21580,10 +21580,10 @@
         <v>79.89</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>79.83</v>
+        <v>80.45</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.00075103266992117</v>
+        <v>0.00700963825259735</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -21610,10 +21610,10 @@
         <v>36.3</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>37.48</v>
+        <v>36.86</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.03250688705234159</v>
+        <v>0.01542699724517913</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -21640,10 +21640,10 @@
         <v>14.78</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>15.24</v>
+        <v>14.96</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.03112313937753727</v>
+        <v>0.01217861975642771</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -21670,10 +21670,10 @@
         <v>8.27</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>8.145</v>
+        <v>8.137</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.01511487303506651</v>
+        <v>-0.01608222490931066</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -21700,10 +21700,10 @@
         <v>151</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>148.5</v>
+        <v>148</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01655629139072848</v>
+        <v>-0.01986754966887417</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -21730,10 +21730,10 @@
         <v>85.40000000000001</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>87.8</v>
+        <v>87.3</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.02810304449648702</v>
+        <v>0.02224824355971887</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -21760,10 +21760,10 @@
         <v>22.54</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>23.48</v>
+        <v>23</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.04170363797692996</v>
+        <v>0.02040816326530616</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -21821,10 +21821,10 @@
         <v>31.42</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>32.46</v>
+        <v>32.38</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.03309993634627623</v>
+        <v>0.03055378739656273</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -21851,10 +21851,10 @@
         <v>325</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>336.5</v>
+        <v>337.5</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.03538461538461538</v>
+        <v>0.03846153846153846</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>16/10/2026 13:00</t>
+          <t>16/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -22725,10 +22725,10 @@
         <v>45.105</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>41.36</v>
+        <v>41.095</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.08302848908103309</v>
+        <v>-0.0889036692162731</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -22755,10 +22755,10 @@
         <v>77.7</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>87.8</v>
+        <v>87.3</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.1299871299871299</v>
+        <v>0.1235521235521235</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -22785,10 +22785,10 @@
         <v>24.96</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>25.92</v>
+        <v>25.84</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.03846153846153849</v>
+        <v>0.03525641025641021</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -22815,10 +22815,10 @@
         <v>144</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>148.5</v>
+        <v>148</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.03125</v>
+        <v>0.02777777777777778</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -22845,10 +22845,10 @@
         <v>76.25</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>87.05</v>
+        <v>83.75</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.141639344262295</v>
+        <v>0.09836065573770492</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -22875,10 +22875,10 @@
         <v>62.3</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>58.85</v>
+        <v>59</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.05537720706260026</v>
+        <v>-0.05296950240770461</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -22905,10 +22905,10 @@
         <v>6.55</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.56</v>
+        <v>5.525</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.151145038167939</v>
+        <v>-0.1564885496183205</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -22935,10 +22935,10 @@
         <v>57.35</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>56.45</v>
+        <v>56.35</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01569311246730599</v>
+        <v>-0.01743679163034002</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -22965,10 +22965,10 @@
         <v>226.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>229.5</v>
+        <v>228.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01324503311258278</v>
+        <v>0.008830022075055188</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -22995,10 +22995,10 @@
         <v>18.83</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>19.19</v>
+        <v>19.13</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.01911842804036129</v>
+        <v>0.01593202336696764</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -23097,10 +23097,10 @@
         <v>2.62</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>2.38</v>
+        <v>2.288</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.09160305343511459</v>
+        <v>-0.1267175572519085</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -23127,10 +23127,10 @@
         <v>970</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1012</v>
+        <v>1000</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.04329896907216495</v>
+        <v>0.03092783505154639</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -23187,10 +23187,10 @@
         <v>0.486</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.444</v>
+        <v>0.431</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>-0.08641975308641972</v>
+        <v>-0.1131687242798354</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -23217,10 +23217,10 @@
         <v>4.48</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>4.43</v>
+        <v>4.345</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01116071428571444</v>
+        <v>-0.03013392857142872</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -23247,10 +23247,10 @@
         <v>22.36</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>22.7</v>
+        <v>22.48</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01520572450805008</v>
+        <v>0.0053667262969589</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -23277,10 +23277,10 @@
         <v>1.442</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1.306</v>
+        <v>1.302</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.09431345353675444</v>
+        <v>-0.09708737864077663</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -23307,10 +23307,10 @@
         <v>0.078</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.076</v>
+        <v>0.082</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.02564102564102566</v>
+        <v>0.05128205128205133</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -23337,10 +23337,10 @@
         <v>0.6840000000000001</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.543</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>-0.1842105263157895</v>
+        <v>-0.206140350877193</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -23367,10 +23367,10 @@
         <v>36.5</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>35.8</v>
+        <v>36.8</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0191780821917809</v>
+        <v>0.008219178082191704</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -23472,10 +23472,10 @@
         <v>1.23</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.714</v>
+        <v>0.72</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.4195121951219513</v>
+        <v>-0.4146341463414634</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -23501,10 +23501,10 @@
         <v>47.45</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>40.3</v>
+        <v>39.6</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.1506849315068494</v>
+        <v>-0.1654373024236038</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -23530,10 +23530,10 @@
         <v>0.98</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.04081632653061228</v>
+        <v>-0.01020408163265307</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -23559,10 +23559,10 @@
         <v>4.08</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.78</v>
+        <v>3.92</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07352941176470594</v>
+        <v>-0.03921568627450984</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -23588,10 +23588,10 @@
         <v>5.16</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>4.52</v>
+        <v>4.595</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1240310077519381</v>
+        <v>-0.1094961240310078</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -23617,10 +23617,10 @@
         <v>5</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>4.62</v>
+        <v>4.64</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.07599999999999998</v>
+        <v>-0.07200000000000006</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -23646,10 +23646,10 @@
         <v>31.4</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>29.8</v>
+        <v>30.4</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05095541401273879</v>
+        <v>-0.03184713375796178</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -23704,10 +23704,10 @@
         <v>1.25</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>1.17</v>
+        <v>1.13</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.06400000000000006</v>
+        <v>-0.09600000000000009</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -23733,10 +23733,10 @@
         <v>7.12</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>5.5</v>
+        <v>5.44</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.2275280898876405</v>
+        <v>-0.2359550561797752</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -23830,10 +23830,10 @@
         <v>165.3</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>182.2</v>
+        <v>175.5</v>
       </c>
       <c r="G43" s="13" t="n">
-        <v>0.1022383545069569</v>
+        <v>0.06170598911070773</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -23859,10 +23859,10 @@
         <v>24.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>26.6</v>
+        <v>25.9</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>0.09917355371900835</v>
+        <v>0.07024793388429749</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -23888,10 +23888,10 @@
         <v>1.86</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>1.882</v>
+        <v>1.89</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>0.0118279569892472</v>
+        <v>0.01612903225806441</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -23917,10 +23917,10 @@
         <v>18.83</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>19.19</v>
+        <v>19.13</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01911842804036129</v>
+        <v>0.01593202336696764</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -23946,10 +23946,10 @@
         <v>24.96</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>25.92</v>
+        <v>25.84</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.03846153846153849</v>
+        <v>0.03525641025641021</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -23975,10 +23975,10 @@
         <v>45.105</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>41.36</v>
+        <v>41.095</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.08302848908103309</v>
+        <v>-0.0889036692162731</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -24004,10 +24004,10 @@
         <v>97.86</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>105</v>
+        <v>102.55</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.07296137339055794</v>
+        <v>0.0479256080114449</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -24033,10 +24033,10 @@
         <v>110.8</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>108.2</v>
+        <v>108.6</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02346570397111908</v>
+        <v>-0.01985559566787006</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -24062,10 +24062,10 @@
         <v>62.3</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>58.85</v>
+        <v>59</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.05537720706260026</v>
+        <v>-0.05296950240770461</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -24091,10 +24091,10 @@
         <v>77.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>87.8</v>
+        <v>87.3</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.1299871299871299</v>
+        <v>0.1235521235521235</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -24189,10 +24189,10 @@
         <v>5.8</v>
       </c>
       <c r="F56" s="12" t="n">
-        <v>5.72</v>
+        <v>5.66</v>
       </c>
       <c r="G56" s="37" t="n">
-        <v>-0.01379310344827587</v>
+        <v>-0.0241379310344827</v>
       </c>
       <c r="H56" s="6" t="n"/>
     </row>
@@ -24219,10 +24219,10 @@
         <v>45.105</v>
       </c>
       <c r="F57" s="12" t="n">
-        <v>41.36</v>
+        <v>41.095</v>
       </c>
       <c r="G57" s="37" t="n">
-        <v>-0.08302848908103309</v>
+        <v>-0.0889036692162731</v>
       </c>
       <c r="H57" s="6" t="n"/>
     </row>
@@ -24249,10 +24249,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F58" s="12" t="n">
-        <v>79.83</v>
+        <v>80.45</v>
       </c>
       <c r="G58" s="37" t="n">
-        <v>-0.002000250031253864</v>
+        <v>0.005750718839855081</v>
       </c>
       <c r="H58" s="6" t="n"/>
     </row>
@@ -24279,10 +24279,10 @@
         <v>72.36</v>
       </c>
       <c r="F59" s="12" t="n">
-        <v>76.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="G59" s="37" t="n">
-        <v>0.0558319513543395</v>
+        <v>0.02681039248203424</v>
       </c>
       <c r="H59" s="6" t="n"/>
     </row>
@@ -24309,10 +24309,10 @@
         <v>76.25</v>
       </c>
       <c r="F60" s="12" t="n">
-        <v>87.05</v>
+        <v>83.75</v>
       </c>
       <c r="G60" s="37" t="n">
-        <v>0.141639344262295</v>
+        <v>0.09836065573770492</v>
       </c>
       <c r="H60" s="6" t="n"/>
     </row>
@@ -24339,10 +24339,10 @@
         <v>14.855</v>
       </c>
       <c r="F61" s="12" t="n">
-        <v>14.515</v>
+        <v>13.925</v>
       </c>
       <c r="G61" s="37" t="n">
-        <v>-0.02288791652642207</v>
+        <v>-0.06260518343991919</v>
       </c>
       <c r="H61" s="6" t="n"/>
     </row>
@@ -24369,10 +24369,10 @@
         <v>126.4</v>
       </c>
       <c r="F62" s="12" t="n">
-        <v>121.4</v>
+        <v>121</v>
       </c>
       <c r="G62" s="37" t="n">
-        <v>-0.03955696202531645</v>
+        <v>-0.04272151898734181</v>
       </c>
       <c r="H62" s="6" t="n"/>
     </row>
@@ -24399,10 +24399,10 @@
         <v>41.02</v>
       </c>
       <c r="F63" s="12" t="n">
-        <v>40.7</v>
+        <v>40.28</v>
       </c>
       <c r="G63" s="37" t="n">
-        <v>-0.007801072647489036</v>
+        <v>-0.01803998049731843</v>
       </c>
       <c r="H63" s="6" t="n"/>
     </row>
@@ -24429,10 +24429,10 @@
         <v>40.1</v>
       </c>
       <c r="F64" s="12" t="n">
-        <v>38.5</v>
+        <v>38.8</v>
       </c>
       <c r="G64" s="37" t="n">
-        <v>-0.03990024937655864</v>
+        <v>-0.03241895261845397</v>
       </c>
       <c r="H64" s="6" t="n"/>
     </row>
@@ -24542,10 +24542,10 @@
         <v>5.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>5.72</v>
+        <v>5.66</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.01379310344827587</v>
+        <v>-0.0241379310344827</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -24572,10 +24572,10 @@
         <v>79.98999999999999</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>79.83</v>
+        <v>80.45</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.002000250031253864</v>
+        <v>0.005750718839855081</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -24602,10 +24602,10 @@
         <v>54.2</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>48.6</v>
+        <v>48</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.1033210332103321</v>
+        <v>-0.1143911439114392</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -24632,10 +24632,10 @@
         <v>72.36</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>76.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>0.0558319513543395</v>
+        <v>0.02681039248203424</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -24662,10 +24662,10 @@
         <v>41.02</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>40.7</v>
+        <v>40.28</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.007801072647489036</v>
+        <v>-0.01803998049731843</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -24692,10 +24692,10 @@
         <v>45.105</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>41.36</v>
+        <v>41.095</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.08302848908103309</v>
+        <v>-0.0889036692162731</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -24722,10 +24722,10 @@
         <v>76.25</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>87.05</v>
+        <v>83.75</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.141639344262295</v>
+        <v>0.09836065573770492</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -24752,10 +24752,10 @@
         <v>14.855</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>14.515</v>
+        <v>13.925</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.02288791652642207</v>
+        <v>-0.06260518343991919</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -24782,10 +24782,10 @@
         <v>126.4</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>121.4</v>
+        <v>121</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.03955696202531645</v>
+        <v>-0.04272151898734181</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -24812,10 +24812,10 @@
         <v>40.1</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>38.5</v>
+        <v>38.8</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.03990024937655864</v>
+        <v>-0.03241895261845397</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour auto - 2026-10-16 20:04
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bourse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9399DB9F-69C1-4F57-846F-47F33913793E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536B8F27-6AC2-41B2-88D2-38F2E1D8923E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Donnees" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="178">
   <si>
     <t>Code</t>
   </si>
@@ -510,6 +510,72 @@
   <si>
     <t>VETOQUINOL</t>
   </si>
+  <si>
+    <t>FNAC</t>
+  </si>
+  <si>
+    <t>FNAC DARTY</t>
+  </si>
+  <si>
+    <t>BB</t>
+  </si>
+  <si>
+    <t>BIC</t>
+  </si>
+  <si>
+    <t>AMUN</t>
+  </si>
+  <si>
+    <t>AMUNDI GROUP</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>GETLINK SE</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>VALEO</t>
+  </si>
+  <si>
+    <t>ABCA</t>
+  </si>
+  <si>
+    <t>ABC ARBITRAGE</t>
+  </si>
+  <si>
+    <t>IPN</t>
+  </si>
+  <si>
+    <t>IPSEN</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <t>DASSAULT AVIATION</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THALES </t>
+  </si>
+  <si>
+    <t>TEP</t>
+  </si>
+  <si>
+    <t>TÉLÉPERFORMANCE</t>
+  </si>
+  <si>
+    <t>AIR</t>
+  </si>
+  <si>
+    <t>AIRBUS GROUP</t>
+  </si>
 </sst>
 </file>
 
@@ -963,7 +1029,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 4" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="357">
+  <dxfs count="358">
     <dxf>
       <font>
         <b/>
@@ -2607,6 +2673,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2614,6 +2681,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2660,6 +2729,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2667,6 +2737,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2693,6 +2765,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2701,6 +2775,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2709,6 +2784,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2716,6 +2792,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2747,6 +2825,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2755,6 +2835,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2763,6 +2844,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2789,6 +2871,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2822,6 +2906,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -2830,6 +2916,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -2838,6 +2925,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2846,6 +2934,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2854,6 +2943,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2862,6 +2952,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2870,6 +2961,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2878,6 +2970,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2886,6 +2979,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2894,6 +2988,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2902,6 +2997,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2910,6 +3006,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2918,6 +3015,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2926,6 +3024,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2934,6 +3033,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2942,6 +3042,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2950,6 +3051,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2958,6 +3060,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2966,6 +3069,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2974,6 +3078,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2982,6 +3087,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2990,6 +3096,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -2998,6 +3105,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3006,6 +3114,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3014,6 +3123,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3022,6 +3132,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3030,6 +3141,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3038,6 +3150,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3046,6 +3159,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3054,6 +3168,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3062,6 +3177,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3070,6 +3186,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3078,6 +3195,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3086,6 +3204,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3094,6 +3213,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3102,6 +3222,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3110,6 +3231,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3118,6 +3240,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3126,6 +3249,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3134,6 +3258,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3142,6 +3267,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3150,6 +3276,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3158,6 +3285,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3166,6 +3294,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3174,6 +3303,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3182,6 +3312,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3190,6 +3321,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3198,6 +3330,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3206,6 +3339,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3214,6 +3348,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3222,6 +3357,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3230,6 +3366,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3238,6 +3375,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3246,6 +3384,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3254,6 +3393,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3262,6 +3402,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3270,6 +3411,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3278,6 +3420,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3286,6 +3429,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3294,6 +3438,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3302,6 +3447,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3310,6 +3456,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3318,6 +3465,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3336,6 +3484,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3343,6 +3492,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3389,6 +3540,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3396,6 +3548,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3422,6 +3576,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3430,6 +3586,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3438,6 +3595,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3445,6 +3603,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3476,6 +3636,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3484,6 +3646,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3492,6 +3655,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3518,6 +3682,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3551,6 +3717,8 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="10"/>
@@ -3559,6 +3727,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color auto="1"/>
@@ -3567,6 +3736,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3575,6 +3745,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3583,6 +3754,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3591,6 +3763,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3599,6 +3772,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3607,6 +3781,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3615,6 +3790,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3623,6 +3799,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3631,6 +3808,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3639,6 +3817,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3647,6 +3826,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3655,6 +3835,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3663,6 +3844,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3671,6 +3853,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3679,6 +3862,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3687,6 +3871,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3695,6 +3880,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3703,6 +3889,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3711,6 +3898,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3719,6 +3907,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3727,6 +3916,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3735,6 +3925,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3743,6 +3934,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3751,6 +3943,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3759,6 +3952,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3767,6 +3961,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3775,6 +3970,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3783,6 +3979,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3791,6 +3988,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3799,6 +3997,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3807,6 +4006,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3815,6 +4015,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3823,6 +4024,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3831,6 +4033,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3839,6 +4042,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3847,6 +4051,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3855,6 +4060,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3863,6 +4069,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3871,6 +4078,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3879,6 +4087,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3887,6 +4096,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3895,6 +4105,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3903,6 +4114,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3911,6 +4123,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3919,6 +4132,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3927,6 +4141,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3935,6 +4150,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3943,6 +4159,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="12"/>
@@ -3951,6 +4168,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3959,6 +4177,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3967,6 +4186,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3975,14 +4195,24 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
       </font>
     </dxf>
     <dxf>
-      <font>
-        <b/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFD966"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3991,6 +4221,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -3999,6 +4230,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4007,6 +4239,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4015,6 +4248,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4023,6 +4257,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4031,6 +4266,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4039,6 +4275,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -4047,6 +4284,7 @@
     <dxf>
       <font>
         <b/>
+        <i val="0"/>
         <condense val="0"/>
         <extend val="0"/>
         <color indexed="18"/>
@@ -21594,140 +21832,240 @@
       <c r="A43" s="8">
         <v>1</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9"/>
-      <c r="D43" s="10"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="12"/>
-      <c r="G43" s="13" t="e">
+      <c r="B43" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E43" s="11">
+        <v>34.6</v>
+      </c>
+      <c r="F43" s="12">
+        <v>34.6</v>
+      </c>
+      <c r="G43" s="13">
         <f>(F43/E43-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A44" s="15">
         <v>2</v>
       </c>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="12"/>
-      <c r="G44" s="13" t="e">
+      <c r="B44" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E44" s="11">
+        <v>67.2</v>
+      </c>
+      <c r="F44" s="12">
+        <v>67.2</v>
+      </c>
+      <c r="G44" s="13">
         <f>(F44/E44-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A45" s="8">
         <v>3</v>
       </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="12"/>
-      <c r="G45" s="13" t="e">
+      <c r="B45" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E45" s="11">
+        <v>89</v>
+      </c>
+      <c r="F45" s="12">
+        <v>89</v>
+      </c>
+      <c r="G45" s="13">
         <f>(F45/E45-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A46" s="15">
         <v>4</v>
       </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="12"/>
-      <c r="G46" s="13" t="e">
+      <c r="B46" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E46" s="11">
+        <v>30.05</v>
+      </c>
+      <c r="F46" s="12">
+        <v>30.05</v>
+      </c>
+      <c r="G46" s="13">
         <f>(F46/E46-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A47" s="8">
         <v>5</v>
       </c>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="12"/>
-      <c r="G47" s="13" t="e">
+      <c r="B47" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E47" s="11">
+        <v>19.190000000000001</v>
+      </c>
+      <c r="F47" s="12">
+        <v>19.190000000000001</v>
+      </c>
+      <c r="G47" s="13">
         <f>(F47/E47-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A48" s="15">
         <v>6</v>
       </c>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="12"/>
-      <c r="G48" s="13" t="e">
+      <c r="B48" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E48" s="11">
+        <v>15.39</v>
+      </c>
+      <c r="F48" s="12">
+        <v>15.39</v>
+      </c>
+      <c r="G48" s="13">
         <f>(F48/E48-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A49" s="8">
         <v>7</v>
       </c>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="12"/>
-      <c r="G49" s="13" t="e">
+      <c r="B49" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E49" s="11">
+        <v>32.46</v>
+      </c>
+      <c r="F49" s="12">
+        <v>32.46</v>
+      </c>
+      <c r="G49" s="13">
         <f>(F49/E49-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A50" s="15">
         <v>8</v>
       </c>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="12"/>
-      <c r="G50" s="13" t="e">
+      <c r="B50" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E50" s="11">
+        <v>13.95</v>
+      </c>
+      <c r="F50" s="12">
+        <v>13.95</v>
+      </c>
+      <c r="G50" s="13">
         <f>(F50/E50-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A51" s="8">
         <v>9</v>
       </c>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="12"/>
-      <c r="G51" s="13" t="e">
+      <c r="B51" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E51" s="11">
+        <v>5.7</v>
+      </c>
+      <c r="F51" s="12">
+        <v>5.7</v>
+      </c>
+      <c r="G51" s="13">
         <f>(F51/E51-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A52" s="15">
         <v>10</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="12"/>
-      <c r="G52" s="13" t="e">
+      <c r="B52" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="E52" s="11">
+        <v>149</v>
+      </c>
+      <c r="F52" s="12">
+        <v>149</v>
+      </c>
+      <c r="G52" s="13">
         <f>(F52/E52-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="15.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
@@ -21783,14 +22121,24 @@
       <c r="A56" s="8">
         <v>1</v>
       </c>
-      <c r="B56" s="36"/>
-      <c r="C56" s="30"/>
-      <c r="D56" s="36"/>
-      <c r="E56" s="18"/>
-      <c r="F56" s="12"/>
-      <c r="G56" s="37" t="e">
+      <c r="B56" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="C56" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D56" s="36" t="s">
+        <v>121</v>
+      </c>
+      <c r="E56" s="18">
+        <v>57.8</v>
+      </c>
+      <c r="F56" s="12">
+        <v>57.8</v>
+      </c>
+      <c r="G56" s="37">
         <f>(F56/E56-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H56" s="6"/>
     </row>
@@ -21798,14 +22146,24 @@
       <c r="A57" s="15">
         <v>2</v>
       </c>
-      <c r="B57" s="36"/>
-      <c r="C57" s="30"/>
-      <c r="D57" s="36"/>
-      <c r="E57" s="18"/>
-      <c r="F57" s="12"/>
-      <c r="G57" s="37" t="e">
+      <c r="B57" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D57" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="E57" s="18">
+        <v>31.4</v>
+      </c>
+      <c r="F57" s="12">
+        <v>31.4</v>
+      </c>
+      <c r="G57" s="37">
         <f>(F57/E57-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H57" s="6"/>
     </row>
@@ -21813,14 +22171,24 @@
       <c r="A58" s="8">
         <v>3</v>
       </c>
-      <c r="B58" s="36"/>
-      <c r="C58" s="30"/>
-      <c r="D58" s="36"/>
-      <c r="E58" s="18"/>
-      <c r="F58" s="12"/>
-      <c r="G58" s="37" t="e">
+      <c r="B58" s="36" t="s">
+        <v>82</v>
+      </c>
+      <c r="C58" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" s="36" t="s">
+        <v>83</v>
+      </c>
+      <c r="E58" s="18">
+        <v>32.4</v>
+      </c>
+      <c r="F58" s="12">
+        <v>32.4</v>
+      </c>
+      <c r="G58" s="37">
         <f>(F58/E58-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H58" s="6"/>
     </row>
@@ -21828,14 +22196,24 @@
       <c r="A59" s="15">
         <v>4</v>
       </c>
-      <c r="B59" s="36"/>
-      <c r="C59" s="30"/>
-      <c r="D59" s="36"/>
-      <c r="E59" s="18"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="37" t="e">
+      <c r="B59" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="C59" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D59" s="36" t="s">
+        <v>54</v>
+      </c>
+      <c r="E59" s="18">
+        <v>36.619999999999997</v>
+      </c>
+      <c r="F59" s="12">
+        <v>36.619999999999997</v>
+      </c>
+      <c r="G59" s="37">
         <f>(F59/E59-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H59" s="6"/>
     </row>
@@ -21843,14 +22221,24 @@
       <c r="A60" s="8">
         <v>5</v>
       </c>
-      <c r="B60" s="36"/>
-      <c r="C60" s="30"/>
-      <c r="D60" s="36"/>
-      <c r="E60" s="18"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="37" t="e">
+      <c r="B60" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C60" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D60" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="E60" s="18">
+        <v>80.709999999999994</v>
+      </c>
+      <c r="F60" s="12">
+        <v>80.709999999999994</v>
+      </c>
+      <c r="G60" s="37">
         <f>(F60/E60-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H60" s="6"/>
     </row>
@@ -21858,14 +22246,24 @@
       <c r="A61" s="15">
         <v>6</v>
       </c>
-      <c r="B61" s="36"/>
-      <c r="C61" s="30"/>
-      <c r="D61" s="36"/>
-      <c r="E61" s="18"/>
-      <c r="F61" s="12"/>
-      <c r="G61" s="37" t="e">
+      <c r="B61" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="C61" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D61" s="36" t="s">
+        <v>123</v>
+      </c>
+      <c r="E61" s="18">
+        <v>121.35</v>
+      </c>
+      <c r="F61" s="12">
+        <v>121.35</v>
+      </c>
+      <c r="G61" s="37">
         <f>(F61/E61-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H61" s="6"/>
     </row>
@@ -21873,14 +22271,24 @@
       <c r="A62" s="8">
         <v>7</v>
       </c>
-      <c r="B62" s="36"/>
-      <c r="C62" s="30"/>
-      <c r="D62" s="36"/>
-      <c r="E62" s="18"/>
-      <c r="F62" s="12"/>
-      <c r="G62" s="37" t="e">
+      <c r="B62" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="C62" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62" s="36" t="s">
+        <v>171</v>
+      </c>
+      <c r="E62" s="18">
+        <v>303.8</v>
+      </c>
+      <c r="F62" s="12">
+        <v>303.8</v>
+      </c>
+      <c r="G62" s="37">
         <f>(F62/E62-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H62" s="6"/>
     </row>
@@ -21888,14 +22296,24 @@
       <c r="A63" s="15">
         <v>8</v>
       </c>
-      <c r="B63" s="36"/>
-      <c r="C63" s="30"/>
-      <c r="D63" s="36"/>
-      <c r="E63" s="18"/>
-      <c r="F63" s="12"/>
-      <c r="G63" s="37" t="e">
+      <c r="B63" s="36" t="s">
+        <v>172</v>
+      </c>
+      <c r="C63" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D63" s="36" t="s">
+        <v>173</v>
+      </c>
+      <c r="E63" s="18">
+        <v>234</v>
+      </c>
+      <c r="F63" s="12">
+        <v>234</v>
+      </c>
+      <c r="G63" s="37">
         <f>(F63/E63-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H63" s="6"/>
     </row>
@@ -21903,14 +22321,24 @@
       <c r="A64" s="8">
         <v>9</v>
       </c>
-      <c r="B64" s="36"/>
-      <c r="C64" s="30"/>
-      <c r="D64" s="36"/>
-      <c r="E64" s="18"/>
-      <c r="F64" s="12"/>
-      <c r="G64" s="37" t="e">
+      <c r="B64" s="36" t="s">
+        <v>174</v>
+      </c>
+      <c r="C64" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D64" s="36" t="s">
+        <v>175</v>
+      </c>
+      <c r="E64" s="18">
+        <v>74.680000000000007</v>
+      </c>
+      <c r="F64" s="12">
+        <v>74.680000000000007</v>
+      </c>
+      <c r="G64" s="37">
         <f>(F64/E64-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H64" s="6"/>
     </row>
@@ -21918,14 +22346,24 @@
       <c r="A65" s="15">
         <v>10</v>
       </c>
-      <c r="B65" s="36"/>
-      <c r="C65" s="30"/>
-      <c r="D65" s="36"/>
-      <c r="E65" s="18"/>
-      <c r="F65" s="12"/>
-      <c r="G65" s="37" t="e">
+      <c r="B65" s="36" t="s">
+        <v>176</v>
+      </c>
+      <c r="C65" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" s="36" t="s">
+        <v>177</v>
+      </c>
+      <c r="E65" s="18">
+        <v>198.82</v>
+      </c>
+      <c r="F65" s="12">
+        <v>198.82</v>
+      </c>
+      <c r="G65" s="37">
         <f>(F65/E65-1)</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="H65" s="6"/>
     </row>
@@ -22989,7 +23427,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="52">
-        <v>46213</v>
+        <v>46304</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-21 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>20/10/2026 19:05</t>
+          <t>21/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>49.84</v>
+        <v>50</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.0331716779825411</v>
+        <v>-0.03006789524733263</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.2</v>
+        <v>25.34</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02552204176334107</v>
+        <v>-0.02010827532869295</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.694</v>
+        <v>1.85</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.04077010192525485</v>
+        <v>0.04756511891279733</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.8</v>
+        <v>32.2</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.04458598726114645</v>
+        <v>0.02547770700636956</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.95</v>
+        <v>57.1</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01064773735581192</v>
+        <v>0.01330967169476486</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>169.1</v>
+        <v>171.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0113636363636364</v>
+        <v>0.02511961722488049</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>80.05</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.008177425350018544</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>32</v>
+        <v>31.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01234567901234563</v>
+        <v>-0.01851851851851846</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,10 +18833,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.077</v>
+        <v>0.083</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.06097560975609762</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.8</v>
+        <v>2.84</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0277777777777778</v>
+        <v>-0.0138888888888889</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>14.2</v>
+        <v>13.7</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.02203856749311297</v>
+        <v>-0.05647382920110195</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.004629629629629695</v>
+        <v>-0.009259259259259391</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>421.8</v>
+        <v>422.2</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02631578947368416</v>
+        <v>-0.02539242843951985</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.618</v>
+        <v>1.628</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.04657179818887455</v>
+        <v>0.05304010349288477</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.9</v>
+        <v>5.86</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.03594771241830061</v>
+        <v>-0.04248366013071892</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>28.75</v>
+        <v>29</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.007005253940455316</v>
+        <v>0.01576182136602449</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.8</v>
+        <v>59</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.003389830508474624</v>
+        <v>0</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>125.6</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>125.4</v>
+        <v>125.3</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.001592356687897999</v>
+        <v>-0.002388535031847111</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>9.09</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.08214285714285709</v>
+        <v>0.07738095238095243</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.505</v>
+        <v>5.46</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.04260869565217393</v>
+        <v>-0.05043478260869566</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19340,10 +19340,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.978</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.05507246376811589</v>
+        <v>-0.09178743961352655</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19369,10 +19369,10 @@
         <v>15.8</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>15.8</v>
+        <v>15.5</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.01898734177215194</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>24.3</v>
+        <v>24</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.02016129032258064</v>
+        <v>-0.03225806451612906</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.88</v>
+        <v>3.9</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01020408163265307</v>
+        <v>-0.005102040816326535</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19486,10 +19486,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2</v>
+        <v>1.92</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01960784313725492</v>
+        <v>-0.05882352941176475</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19515,10 +19515,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>27</v>
+        <v>26.4</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03571428571428571</v>
+        <v>-0.0571428571428572</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19544,10 +19544,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22</v>
+        <v>22.75</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03719912472647709</v>
+        <v>-0.004376367614879712</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19602,10 +19602,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>24.5</v>
+        <v>24.15</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.006085192697768705</v>
+        <v>-0.02028397565922921</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>66.09999999999999</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01636904761904774</v>
+        <v>-0.01562499999999996</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>87.95</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01179775280898873</v>
+        <v>-0.006741573033707801</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>29.38</v>
+        <v>27.86</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.02229617304492518</v>
+        <v>-0.07287853577371052</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.26</v>
+        <v>19.29</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.003647733194372083</v>
+        <v>0.005211047420531415</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>15.14</v>
+        <v>14.79</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.01624431448992852</v>
+        <v>-0.03898635477582855</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>32.38</v>
+        <v>34</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>-0.002464571780653059</v>
+        <v>0.04744300677757237</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>13.61</v>
+        <v>13.495</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.02437275985663082</v>
+        <v>-0.03261648745519714</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.7</v>
+        <v>5.74</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0</v>
+        <v>0.007017543859649129</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>151.9</v>
+        <v>153</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01946308724832219</v>
+        <v>0.02684563758389262</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>20/10/2026 19:05</t>
+          <t>21/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.06</v>
+        <v>8.24</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.01466992665036665</v>
+        <v>0.007334963325183435</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>29.38</v>
+        <v>27.86</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.03999999999999997</v>
+        <v>-0.01380530973451329</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.2</v>
+        <v>25.34</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02439024390243894</v>
+        <v>0.03008130081300807</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21394,10 +21394,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>84.3</v>
+        <v>86.8</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.04720496894409934</v>
+        <v>0.07826086956521736</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>80.05</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.01935566025722649</v>
+        <v>0.02776009168470639</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0128755364806867</v>
+        <v>-0.008583690987124463</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.558</v>
+        <v>1.556</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.07152682255845949</v>
+        <v>0.07015130674002758</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21514,10 +21514,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>343.5</v>
+        <v>347.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.08188976377952756</v>
+        <v>0.09448818897637795</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>202.8</v>
+        <v>203.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.06284658040665432</v>
+        <v>-0.05822550831792973</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21646,10 +21646,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125.4</v>
+        <v>125.3</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.004807692307692376</v>
+        <v>0.004006410256410257</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21706,10 +21706,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.09</v>
+        <v>2.078</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02061855670103095</v>
+        <v>-0.02624179943767575</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.694</v>
+        <v>1.85</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.227536231884058</v>
+        <v>0.3405797101449277</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>22.84</v>
+        <v>25.88</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.07939508506616255</v>
+        <v>0.2230623818525519</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.98</v>
+        <v>13.92</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.1095238095238096</v>
+        <v>0.1047619047619048</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>57.95</v>
+        <v>58.1</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05077062556663652</v>
+        <v>0.05349048050770631</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.438</v>
+        <v>0.445</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.00680272108843538</v>
+        <v>0.009070294784580506</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>32.38</v>
+        <v>34</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.05955497382198965</v>
+        <v>0.1125654450261781</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.48</v>
+        <v>14.76</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.0006901311249137189</v>
+        <v>0.01863354037267078</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22021,10 +22021,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.066</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.175</v>
+        <v>-0.1375</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.48</v>
+        <v>9.4</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.04242424242424241</v>
+        <v>-0.0505050505050505</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22079,10 +22079,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.153</v>
+        <v>0.154</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03164556962025319</v>
+        <v>-0.02531645569620256</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22108,10 +22108,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.05384615384615389</v>
+        <v>-0.04615384615384619</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22137,10 +22137,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.207</v>
+        <v>0.209</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1410788381742739</v>
+        <v>-0.1327800829875519</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.539999999999999</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.05917159763313623</v>
+        <v>-0.06706114398422088</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22195,10 +22195,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.3</v>
+        <v>18.75</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.07106598984771567</v>
+        <v>-0.04822335025380707</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.16</v>
+        <v>4.17</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.221732745961821</v>
+        <v>0.2246696035242291</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>214.4</v>
+        <v>214.2</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.007518796992481176</v>
+        <v>0.006578947368420946</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22847,10 +22847,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>46.8</v>
+        <v>46.2</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.07874015748031496</v>
+        <v>-0.0905511811023621</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22877,10 +22877,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.04605263157894737</v>
+        <v>-0.03947368421052631</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.0128755364806867</v>
+        <v>-0.008583690987124463</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>32.38</v>
+        <v>34</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.05955497382198965</v>
+        <v>0.1125654450261781</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>79.8</v>
+        <v>80</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.02835051546391756</v>
+        <v>0.03092783505154647</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>26.8</v>
+        <v>27.5</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.06986027944111776</v>
+        <v>0.09780439121756485</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>80.05</v>
+        <v>80.70999999999999</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.01935566025722649</v>
+        <v>0.02776009168470639</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>123.5</v>
+        <v>125.6</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.07344632768361585</v>
+        <v>0.0916992611907866</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-21 19:06
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/10/2026 13:00</t>
+          <t>21/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>50</v>
+        <v>50.3</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.03006789524733263</v>
+        <v>-0.02424830261881668</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.34</v>
+        <v>25.16</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02010827532869295</v>
+        <v>-0.0270688321732405</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.85</v>
+        <v>1.885</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.04756511891279733</v>
+        <v>0.06738391845979615</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.2</v>
+        <v>32.4</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02547770700636956</v>
+        <v>0.03184713375796178</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>57.1</v>
+        <v>56.7</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.01330967169476486</v>
+        <v>0.006211180124223627</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>171.4</v>
+        <v>173.8</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02511961722488049</v>
+        <v>0.03947368421052645</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>80.70999999999999</v>
+        <v>80.77</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0</v>
+        <v>0.0007434023045471723</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>31.8</v>
+        <v>32.05</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01851851851851846</v>
+        <v>-0.01080246913580251</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.84</v>
+        <v>2.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0138888888888889</v>
+        <v>-0.0277777777777778</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>21.4</v>
+        <v>20.9</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.009259259259259391</v>
+        <v>-0.03240740740740754</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>422.2</v>
+        <v>423.4</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02539242843951985</v>
+        <v>-0.0226223453370268</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.628</v>
+        <v>1.63</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.05304010349288477</v>
+        <v>0.05433376455368684</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.86</v>
+        <v>5.81</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.04248366013071892</v>
+        <v>-0.05065359477124191</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>29</v>
+        <v>28.95</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01576182136602449</v>
+        <v>0.01401050788091063</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>9.050000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.07738095238095243</v>
+        <v>0.1047619047619046</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.46</v>
+        <v>5.43</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.05043478260869566</v>
+        <v>-0.05565217391304353</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19340,10 +19340,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.978</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.09178743961352655</v>
+        <v>-0.05507246376811589</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19369,10 +19369,10 @@
         <v>15.8</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>15.5</v>
+        <v>15.7</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.01898734177215194</v>
+        <v>-0.006329113924050722</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>24</v>
+        <v>24.4</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03225806451612906</v>
+        <v>-0.0161290322580646</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.9</v>
+        <v>3.89</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.005102040816326535</v>
+        <v>-0.007653061224489746</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19486,10 +19486,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.05882352941176475</v>
+        <v>-0.01960784313725492</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19515,10 +19515,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>26.4</v>
+        <v>26.2</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.0571428571428572</v>
+        <v>-0.06428571428571431</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19544,10 +19544,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22.75</v>
+        <v>22.7</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.004376367614879712</v>
+        <v>-0.006564551422319567</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19573,10 +19573,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.259</v>
+        <v>0.256</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.02264150943396228</v>
+        <v>-0.03396226415094342</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19602,10 +19602,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>24.15</v>
+        <v>23.2</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.02028397565922921</v>
+        <v>-0.05882352941176468</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>66.15000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01562499999999996</v>
+        <v>-0.01190476190476186</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>88.40000000000001</v>
+        <v>88.8</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.006741573033707801</v>
+        <v>-0.002247191011235987</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>27.86</v>
+        <v>26.62</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.07287853577371052</v>
+        <v>-0.1141430948419301</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.29</v>
+        <v>19.37</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.005211047420531415</v>
+        <v>0.009379885356956733</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>14.79</v>
+        <v>14.87</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03898635477582855</v>
+        <v>-0.03378817413905142</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>34</v>
+        <v>34.88</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.04744300677757237</v>
+        <v>0.07455329636475667</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>13.495</v>
+        <v>13.475</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.03261648745519714</v>
+        <v>-0.03405017921146951</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.74</v>
+        <v>5.71</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.007017543859649129</v>
+        <v>0.001754385964912243</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>153</v>
+        <v>152.3</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02684563758389262</v>
+        <v>0.02214765100671149</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/10/2026 13:00</t>
+          <t>21/10/2026 19:06</t>
         </is>
       </c>
     </row>
@@ -21274,10 +21274,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15</v>
+        <v>15.08</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01315789473684206</v>
+        <v>-0.007894736842105211</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.24</v>
+        <v>8.164999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.007334963325183435</v>
+        <v>-0.001833740831295913</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>27.86</v>
+        <v>26.62</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01380530973451329</v>
+        <v>-0.05769911504424775</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.34</v>
+        <v>25.16</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.03008130081300807</v>
+        <v>0.02276422764227637</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21394,10 +21394,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>86.8</v>
+        <v>87.25</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.07826086956521736</v>
+        <v>0.08385093167701864</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>80.70999999999999</v>
+        <v>80.77</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02776009168470639</v>
+        <v>0.02852413090538641</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.008583690987124463</v>
+        <v>-0.0128755364806867</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.556</v>
+        <v>1.566</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.07015130674002758</v>
+        <v>0.07702888583218714</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21514,10 +21514,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>347.5</v>
+        <v>345</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.09448818897637795</v>
+        <v>0.08661417322834646</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>203.8</v>
+        <v>204.2</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05822550831792973</v>
+        <v>-0.05637707948244</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21676,10 +21676,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.59</v>
+        <v>9.525</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.01388174807197941</v>
+        <v>-0.02056555269922872</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21706,10 +21706,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.078</v>
+        <v>2.072</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02624179943767575</v>
+        <v>-0.02905342080599805</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.85</v>
+        <v>1.885</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.3405797101449277</v>
+        <v>0.3659420289855074</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>25.88</v>
+        <v>26.1</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.2230623818525519</v>
+        <v>0.2334593572778829</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.92</v>
+        <v>14</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.1047619047619048</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.1</v>
+        <v>57.95</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05349048050770631</v>
+        <v>0.05077062556663652</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.445</v>
+        <v>0.453</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.009070294784580506</v>
+        <v>0.02721088435374152</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>34</v>
+        <v>34.88</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1125654450261781</v>
+        <v>0.1413612565445027</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.76</v>
+        <v>14.5</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.01863354037267078</v>
+        <v>0.0006901311249137189</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.0505050505050505</v>
+        <v>-0.06060606060606057</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22079,10 +22079,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.154</v>
+        <v>0.153</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.02531645569620256</v>
+        <v>-0.03164556962025319</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22137,10 +22137,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.209</v>
+        <v>0.208</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1327800829875519</v>
+        <v>-0.1369294605809129</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.460000000000001</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.06706114398422088</v>
+        <v>-0.0749506903353057</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22195,10 +22195,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.75</v>
+        <v>18.4</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.04822335025380707</v>
+        <v>-0.06598984771573609</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.17</v>
+        <v>4.25</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.2246696035242291</v>
+        <v>0.2481644640234949</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22282,10 +22282,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.03</v>
+        <v>4.02</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1613832853025937</v>
+        <v>0.15850144092219</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>214.2</v>
+        <v>214.8</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.006578947368420946</v>
+        <v>0.009398496240601503</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22817,10 +22817,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>15</v>
+        <v>15.08</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.01315789473684206</v>
+        <v>-0.007894736842105211</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22847,10 +22847,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>46.2</v>
+        <v>44.8</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.0905511811023621</v>
+        <v>-0.1181102362204725</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22877,10 +22877,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>146</v>
+        <v>146.5</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03947368421052631</v>
+        <v>-0.03618421052631579</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.008583690987124463</v>
+        <v>-0.0128755364806867</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>34</v>
+        <v>34.88</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.1125654450261781</v>
+        <v>0.1413612565445027</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>80</v>
+        <v>79.7</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.03092783505154647</v>
+        <v>0.0270618556701032</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>27.5</v>
+        <v>27.65</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.09780439121756485</v>
+        <v>0.1037924151696606</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>80.70999999999999</v>
+        <v>80.77</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.02776009168470639</v>
+        <v>0.02852413090538641</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>125.6</v>
+        <v>124.95</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.0916992611907866</v>
+        <v>0.08604954367666237</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-22 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/10/2026 19:06</t>
+          <t>22/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>50.3</v>
+        <v>50.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02424830261881668</v>
+        <v>-0.01454898157129001</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.16</v>
+        <v>25.1</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.0270688321732405</v>
+        <v>-0.02938901778808964</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.885</v>
+        <v>1.817</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.06738391845979615</v>
+        <v>0.02887882219705545</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.4</v>
+        <v>32.05</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.03184713375796178</v>
+        <v>0.02070063694267512</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.7</v>
+        <v>56.15</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.006211180124223627</v>
+        <v>-0.00354924578527068</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>173.8</v>
+        <v>174.6</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.03947368421052645</v>
+        <v>0.04425837320574166</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>80.77</v>
+        <v>81.38</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.0007434023045471723</v>
+        <v>0.008301325734109797</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>32.05</v>
+        <v>31.69</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01080246913580251</v>
+        <v>-0.0219135802469135</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,10 +18833,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.083</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0277777777777778</v>
+        <v>-0.0624999999999999</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>13.7</v>
+        <v>13.26</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.05647382920110195</v>
+        <v>-0.08677685950413222</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.03240740740740754</v>
+        <v>-0.04166666666666676</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>423.4</v>
+        <v>419.4</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0226223453370268</v>
+        <v>-0.03185595567867039</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.63</v>
+        <v>1.596</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.05433376455368684</v>
+        <v>0.03234152652005177</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.81</v>
+        <v>5.82</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.05065359477124191</v>
+        <v>-0.04901960784313723</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>28.95</v>
+        <v>28.85</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01401050788091063</v>
+        <v>0.01050788091068304</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>59</v>
+        <v>58.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0</v>
+        <v>-0.01016949152542375</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>9.279999999999999</v>
+        <v>9.1</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1047619047619046</v>
+        <v>0.08333333333333325</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>5.43</v>
+        <v>4.72</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.05565217391304353</v>
+        <v>-0.1791304347826087</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19340,10 +19340,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.978</v>
+        <v>0.97</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.05507246376811589</v>
+        <v>-0.06280193236714972</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19369,10 +19369,10 @@
         <v>15.8</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.006329113924050722</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>24.4</v>
+        <v>24</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.0161290322580646</v>
+        <v>-0.03225806451612906</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.89</v>
+        <v>3.85</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.007653061224489746</v>
+        <v>-0.01785714285714282</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19486,10 +19486,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>2</v>
+        <v>1.95</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01960784313725492</v>
+        <v>-0.04411764705882357</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19515,10 +19515,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>26.2</v>
+        <v>26.5</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06428571428571431</v>
+        <v>-0.05357142857142857</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19544,10 +19544,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22.7</v>
+        <v>22.05</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.006564551422319567</v>
+        <v>-0.03501094091903723</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19573,10 +19573,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.256</v>
+        <v>0.253</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.03396226415094342</v>
+        <v>-0.04528301886792457</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>66.40000000000001</v>
+        <v>66</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01190476190476186</v>
+        <v>-0.0178571428571429</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>88.8</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.002247191011235987</v>
+        <v>-0.01573033707865175</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>26.62</v>
+        <v>26.36</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1141430948419301</v>
+        <v>-0.1227953410981698</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.37</v>
+        <v>19.51</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.009379885356956733</v>
+        <v>0.0166753517457009</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>14.87</v>
+        <v>14.7</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03378817413905142</v>
+        <v>-0.04483430799220281</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>34.88</v>
+        <v>34.26</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.07455329636475667</v>
+        <v>0.05545286506469492</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>13.475</v>
+        <v>13.225</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.03405017921146951</v>
+        <v>-0.05197132616487453</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.71</v>
+        <v>5.69</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.001754385964912243</v>
+        <v>-0.001754385964912243</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>152.3</v>
+        <v>152.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02214765100671149</v>
+        <v>0.02550335570469806</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>21/10/2026 19:06</t>
+          <t>22/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21274,10 +21274,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.08</v>
+        <v>15.06</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.007894736842105211</v>
+        <v>-0.009210526315789395</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.164999999999999</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.001833740831295913</v>
+        <v>0.002444987775061073</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>26.62</v>
+        <v>26.36</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05769911504424775</v>
+        <v>-0.06690265486725666</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.16</v>
+        <v>25.1</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02276422764227637</v>
+        <v>0.02032520325203252</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>80.77</v>
+        <v>81.38</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02852413090538641</v>
+        <v>0.03629186298229969</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>230</v>
+        <v>230.5</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0128755364806867</v>
+        <v>-0.01072961373390558</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.566</v>
+        <v>1.561</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.07702888583218714</v>
+        <v>0.07359009628610728</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21514,10 +21514,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.08661417322834646</v>
+        <v>0.09606299212598425</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>204.2</v>
+        <v>203.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05637707948244</v>
+        <v>-0.05822550831792973</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21676,10 +21676,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.525</v>
+        <v>9.345000000000001</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.02056555269922872</v>
+        <v>-0.03907455012853461</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21706,10 +21706,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.072</v>
+        <v>2.06</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02905342080599805</v>
+        <v>-0.03467666354264285</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.885</v>
+        <v>1.817</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.3659420289855074</v>
+        <v>0.3166666666666667</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>26.1</v>
+        <v>24.94</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.2334593572778829</v>
+        <v>0.1786389413988658</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>14</v>
+        <v>13.8</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.09523809523809533</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>57.95</v>
+        <v>57.6</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.05077062556663652</v>
+        <v>0.04442429737080694</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.453</v>
+        <v>0.44</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.02721088435374152</v>
+        <v>-0.002267573696145127</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>34.88</v>
+        <v>34.26</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1413612565445027</v>
+        <v>0.1210732984293194</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.5</v>
+        <v>14.44</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.0006901311249137189</v>
+        <v>-0.003450655624568717</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.300000000000001</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.06060606060606057</v>
+        <v>-0.07676767676767675</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22079,10 +22079,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.153</v>
+        <v>0.149</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03164556962025319</v>
+        <v>-0.05696202531645574</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22108,10 +22108,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.24</v>
+        <v>1.205</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04615384615384619</v>
+        <v>-0.07307692307692305</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22137,10 +22137,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.208</v>
+        <v>0.207</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1369294605809129</v>
+        <v>-0.1410788381742739</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.380000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.0749506903353057</v>
+        <v>-0.08185404339250493</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22195,10 +22195,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.4</v>
+        <v>18.7</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06598984771573609</v>
+        <v>-0.05076142131979695</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.25</v>
+        <v>4.295</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.2481644640234949</v>
+        <v>0.2613803230543319</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22282,10 +22282,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.02</v>
+        <v>4.03</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.15850144092219</v>
+        <v>0.1613832853025937</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>214.8</v>
+        <v>216.4</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.009398496240601503</v>
+        <v>0.01691729323308268</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22817,10 +22817,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>15.08</v>
+        <v>15.06</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.007894736842105211</v>
+        <v>-0.009210526315789395</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22847,10 +22847,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>44.8</v>
+        <v>46</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.1181102362204725</v>
+        <v>-0.0944881889763779</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22877,10 +22877,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>146.5</v>
+        <v>145</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03618421052631579</v>
+        <v>-0.04605263157894737</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>230</v>
+        <v>230.5</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.0128755364806867</v>
+        <v>-0.01072961373390558</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>34.88</v>
+        <v>34.26</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.1413612565445027</v>
+        <v>0.1210732984293194</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>79.7</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.0270618556701032</v>
+        <v>-0.00257731958762872</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>27.65</v>
+        <v>27.6</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.1037924151696606</v>
+        <v>0.1017964071856288</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>80.77</v>
+        <v>81.38</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.02852413090538641</v>
+        <v>0.03629186298229969</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>124.95</v>
+        <v>125.1</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.08604954367666237</v>
+        <v>0.08735332464146021</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-22 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/10/2026 13:00</t>
+          <t>22/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>50.8</v>
+        <v>51.75</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01454898157129001</v>
+        <v>0.003879728419010725</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.1</v>
+        <v>25.18</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02938901778808964</v>
+        <v>-0.02629543696829079</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.817</v>
+        <v>1.81</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02887882219705545</v>
+        <v>0.02491506228765574</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.05</v>
+        <v>32.2</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02070063694267512</v>
+        <v>0.02547770700636956</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.15</v>
+        <v>56.65</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>-0.00354924578527068</v>
+        <v>0.005323868677905894</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>174.6</v>
+        <v>177.5</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.04425837320574166</v>
+        <v>0.0616028708133972</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>81.38</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.008301325734109797</v>
+        <v>-0.006566720356832945</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>31.69</v>
+        <v>31.83</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0219135802469135</v>
+        <v>-0.0175925925925926</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,10 +18833,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.082</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02439024390243905</v>
+        <v>0</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.7</v>
+        <v>2.76</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.0624999999999999</v>
+        <v>-0.04166666666666671</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>13.26</v>
+        <v>14</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.08677685950413222</v>
+        <v>-0.03581267217630851</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -18995,10 +18995,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.04166666666666676</v>
+        <v>-0.05092592592592599</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>419.4</v>
+        <v>424</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.03185595567867039</v>
+        <v>-0.02123730378578021</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.596</v>
+        <v>1.606</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03234152652005177</v>
+        <v>0.03880983182406213</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.82</v>
+        <v>6.08</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.04901960784313723</v>
+        <v>-0.006535947712418306</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>28.85</v>
+        <v>28.8</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.01050788091068304</v>
+        <v>0.008756567425569177</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.4</v>
+        <v>58.2</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01016949152542375</v>
+        <v>-0.01355932203389826</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>125.6</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>125.3</v>
+        <v>125.2</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.002388535031847111</v>
+        <v>-0.00318471337579611</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>9.1</v>
+        <v>8.98</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.08333333333333325</v>
+        <v>0.06904761904761905</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>4.72</v>
+        <v>4.352</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.1791304347826087</v>
+        <v>-0.2431304347826087</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19340,10 +19340,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.06280193236714972</v>
+        <v>-0.05314009661835743</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.03225806451612906</v>
+        <v>-0.04435483870967748</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.85</v>
+        <v>3.82</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01785714285714282</v>
+        <v>-0.02551020408163268</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19544,10 +19544,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22.05</v>
+        <v>22.25</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03501094091903723</v>
+        <v>-0.02625820568927796</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19573,10 +19573,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.253</v>
+        <v>0.25</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.04528301886792457</v>
+        <v>-0.05660377358490571</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19602,10 +19602,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05882352941176468</v>
+        <v>-0.05476673427991878</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>66</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.0178571428571429</v>
+        <v>-0.01636904761904774</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>87.59999999999999</v>
+        <v>87.55</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01573033707865175</v>
+        <v>-0.01629213483146071</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>26.36</v>
+        <v>26.75</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1227953410981698</v>
+        <v>-0.1098169717138103</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.51</v>
+        <v>19.57</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.0166753517457009</v>
+        <v>0.01980198019801975</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>14.7</v>
+        <v>14.98</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.04483430799220281</v>
+        <v>-0.02664067576348279</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>34.26</v>
+        <v>34.46</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.05545286506469492</v>
+        <v>0.06161429451632779</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>13.225</v>
+        <v>12.83</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.05197132616487453</v>
+        <v>-0.08028673835125442</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.69</v>
+        <v>5.72</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>-0.001754385964912243</v>
+        <v>0.003508771929824486</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>152.8</v>
+        <v>152.6</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02550335570469806</v>
+        <v>0.02416107382550332</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/10/2026 13:00</t>
+          <t>22/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -21274,10 +21274,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>15.06</v>
+        <v>14.98</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.009210526315789395</v>
+        <v>-0.01447368421052624</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>8.199999999999999</v>
+        <v>7.92</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>0.002444987775061073</v>
+        <v>-0.03178484107579459</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>26.36</v>
+        <v>26.75</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.06690265486725666</v>
+        <v>-0.05309734513274336</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.1</v>
+        <v>25.18</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02032520325203252</v>
+        <v>0.02357723577235765</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21394,10 +21394,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>87.25</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.08385093167701864</v>
+        <v>0.09192546583850938</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>81.38</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.03629186298229969</v>
+        <v>0.02101107856869993</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>230.5</v>
+        <v>228.5</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01072961373390558</v>
+        <v>-0.01931330472103004</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.561</v>
+        <v>1.579</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.07359009628610728</v>
+        <v>0.0859697386519945</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21514,10 +21514,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.09606299212598425</v>
+        <v>0.09921259842519685</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>203.8</v>
+        <v>198.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.05822550831792973</v>
+        <v>-0.08133086876155265</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21646,10 +21646,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125.3</v>
+        <v>125.2</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.004006410256410257</v>
+        <v>0.003205128205128251</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21676,10 +21676,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.345000000000001</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.03907455012853461</v>
+        <v>-0.06118251928020554</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.817</v>
+        <v>1.81</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.3166666666666667</v>
+        <v>0.3115942028985509</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>24.94</v>
+        <v>24</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1786389413988658</v>
+        <v>0.1342155009451796</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.8</v>
+        <v>13.84</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.09523809523809533</v>
+        <v>0.09841269841269844</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>57.6</v>
+        <v>56</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.04442429737080694</v>
+        <v>0.01541251133272895</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.44</v>
+        <v>0.443</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.002267573696145127</v>
+        <v>0.004535147392290253</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>34.26</v>
+        <v>34.46</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1210732984293194</v>
+        <v>0.1276178010471205</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.44</v>
+        <v>14.57</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.003450655624568717</v>
+        <v>0.005521048999309873</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22021,10 +22021,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1375</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.140000000000001</v>
+        <v>9</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.07676767676767675</v>
+        <v>-0.09090909090909094</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22108,10 +22108,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.205</v>
+        <v>1.27</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.07307692307692305</v>
+        <v>-0.0230769230769231</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22137,10 +22137,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.207</v>
+        <v>0.211</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1410788381742739</v>
+        <v>-0.1244813278008299</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.31</v>
+        <v>9.17</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.08185404339250493</v>
+        <v>-0.09566074950690341</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22195,10 +22195,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.7</v>
+        <v>18.4</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05076142131979695</v>
+        <v>-0.06598984771573609</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.295</v>
+        <v>4.225</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.2613803230543319</v>
+        <v>0.2408223201174743</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22282,10 +22282,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1613832853025937</v>
+        <v>0.1642651296829971</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>216.4</v>
+        <v>213.2</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.01691729323308268</v>
+        <v>0.001879699248120194</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22817,10 +22817,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>15.06</v>
+        <v>14.98</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.009210526315789395</v>
+        <v>-0.01447368421052624</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>230.5</v>
+        <v>228.5</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01072961373390558</v>
+        <v>-0.01931330472103004</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>34.26</v>
+        <v>34.46</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.1210732984293194</v>
+        <v>0.1276178010471205</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>77.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>-0.00257731958762872</v>
+        <v>0.003865979381443446</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>27.6</v>
+        <v>27.9</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.1017964071856288</v>
+        <v>0.1137724550898203</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>81.38</v>
+        <v>80.18000000000001</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.03629186298229969</v>
+        <v>0.02101107856869993</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>125.1</v>
+        <v>126.65</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.08735332464146021</v>
+        <v>0.1008257279443721</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-23 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/10/2026 19:05</t>
+          <t>23/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>51.75</v>
+        <v>52.05</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.003879728419010725</v>
+        <v>0.009699321047526674</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.18</v>
+        <v>24.94</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02629543696829079</v>
+        <v>-0.03557617942768748</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.81</v>
+        <v>1.738</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.02491506228765574</v>
+        <v>-0.01585503963759911</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.2</v>
+        <v>31.7</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02547770700636956</v>
+        <v>0.009554140127388559</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>56.65</v>
+        <v>60.05</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.005323868677905894</v>
+        <v>0.06566104702750658</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>177.5</v>
+        <v>175.5</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0616028708133972</v>
+        <v>0.04964114832535892</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>80.18000000000001</v>
+        <v>81.84999999999999</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.006566720356832945</v>
+        <v>0.01412464378639575</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>31.83</v>
+        <v>31.85</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0175925925925926</v>
+        <v>-0.01697530864197522</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,10 +18833,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.082</v>
+        <v>0.081</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0</v>
+        <v>-0.01219512195121952</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.76</v>
+        <v>2.82</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.04166666666666671</v>
+        <v>-0.02083333333333335</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>14</v>
+        <v>14.44</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.03581267217630851</v>
+        <v>-0.005509641873278242</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>424</v>
+        <v>419.4</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02123730378578021</v>
+        <v>-0.03185595567867039</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.606</v>
+        <v>1.6</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03880983182406213</v>
+        <v>0.03492884864165591</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.08</v>
+        <v>6.01</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.006535947712418306</v>
+        <v>-0.01797385620915038</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>28.8</v>
+        <v>29.15</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.008756567425569177</v>
+        <v>0.02101576182136595</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.2</v>
+        <v>58.5</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01355932203389826</v>
+        <v>-0.008474576271186441</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19175,10 +19175,10 @@
         <v>125.6</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>125.2</v>
+        <v>125.4</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.00318471337579611</v>
+        <v>-0.001592356687897999</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.98</v>
+        <v>8.68</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.06904761904761905</v>
+        <v>0.03333333333333326</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>4.352</v>
+        <v>4.01</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2431304347826087</v>
+        <v>-0.302608695652174</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>23.7</v>
+        <v>23.2</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.04435483870967748</v>
+        <v>-0.06451612903225812</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.82</v>
+        <v>3.83</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02551020408163268</v>
+        <v>-0.02295918367346935</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19515,10 +19515,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>26.5</v>
+        <v>26.3</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.05357142857142857</v>
+        <v>-0.06071428571428569</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19544,10 +19544,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22.25</v>
+        <v>22.05</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02625820568927796</v>
+        <v>-0.03501094091903723</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19573,10 +19573,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.25</v>
+        <v>0.242</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.05660377358490571</v>
+        <v>-0.08679245283018876</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19602,10 +19602,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>23.3</v>
+        <v>22.7</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.05476673427991878</v>
+        <v>-0.07910750507099389</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>66.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.01636904761904774</v>
+        <v>-0.02529761904761909</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>87.55</v>
+        <v>87</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01629213483146071</v>
+        <v>-0.02247191011235955</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>26.75</v>
+        <v>26.12</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1098169717138103</v>
+        <v>-0.1307820299500832</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.57</v>
+        <v>19.52</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.01980198019801975</v>
+        <v>0.01719645648775395</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>14.98</v>
+        <v>14.86</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.02664067576348279</v>
+        <v>-0.03443794671864855</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>34.46</v>
+        <v>34.6</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.06161429451632779</v>
+        <v>0.06592729513247075</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>12.83</v>
+        <v>11.655</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.08028673835125442</v>
+        <v>-0.1645161290322581</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.72</v>
+        <v>5.71</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.003508771929824486</v>
+        <v>0.001754385964912243</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>152.6</v>
+        <v>152.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02416107382550332</v>
+        <v>0.02550335570469806</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>22/10/2026 19:05</t>
+          <t>23/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21274,10 +21274,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.98</v>
+        <v>14.92</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01447368421052624</v>
+        <v>-0.01842105263157891</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>7.92</v>
+        <v>7.975</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03178484107579459</v>
+        <v>-0.02506112469437654</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>26.75</v>
+        <v>26.12</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.05309734513274336</v>
+        <v>-0.07539823008849554</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>25.18</v>
+        <v>24.94</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.02357723577235765</v>
+        <v>0.01382113821138211</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21394,10 +21394,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>87.90000000000001</v>
+        <v>85.65000000000001</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.09192546583850938</v>
+        <v>0.06397515527950318</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>80.18000000000001</v>
+        <v>81.84999999999999</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.02101107856869993</v>
+        <v>0.0422768368776263</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>228.5</v>
+        <v>230</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.01931330472103004</v>
+        <v>-0.0128755364806867</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.579</v>
+        <v>1.571</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.0859697386519945</v>
+        <v>0.08046767537826685</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21514,10 +21514,10 @@
         <v>317.5</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>349</v>
+        <v>347.5</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.09921259842519685</v>
+        <v>0.09448818897637795</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>198.8</v>
+        <v>200.8</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.08133086876155265</v>
+        <v>-0.07208872458410348</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21646,10 +21646,10 @@
         <v>124.8</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>125.2</v>
+        <v>125.4</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.003205128205128251</v>
+        <v>0.004807692307692376</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21676,10 +21676,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.130000000000001</v>
+        <v>9.125</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.06118251928020554</v>
+        <v>-0.06169665809768634</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21706,10 +21706,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.06</v>
+        <v>2.018</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.03467666354264285</v>
+        <v>-0.05435801312089977</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.81</v>
+        <v>1.738</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.3115942028985509</v>
+        <v>0.2594202898550725</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>24</v>
+        <v>24.12</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1342155009451796</v>
+        <v>0.1398865784499055</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.84</v>
+        <v>13.9</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.09841269841269844</v>
+        <v>0.1031746031746032</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>56</v>
+        <v>54.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.01541251133272895</v>
+        <v>-0.01359927470534905</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.443</v>
+        <v>0.437</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.004535147392290253</v>
+        <v>-0.009070294784580506</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>34.46</v>
+        <v>34.6</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1276178010471205</v>
+        <v>0.1321989528795812</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.57</v>
+        <v>14.53</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.005521048999309873</v>
+        <v>0.002760524499654876</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9</v>
+        <v>9.34</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.09090909090909094</v>
+        <v>-0.05656565656565661</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.17</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.09566074950690341</v>
+        <v>-0.1084812623274163</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.225</v>
+        <v>4.05</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.2408223201174743</v>
+        <v>0.1894273127753304</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22282,10 +22282,10 @@
         <v>3.47</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>4.04</v>
+        <v>4.02</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0.1642651296829971</v>
+        <v>0.15850144092219</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>213.2</v>
+        <v>211.8</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>0.001879699248120194</v>
+        <v>-0.004699248120300752</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22817,10 +22817,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>14.98</v>
+        <v>14.92</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.01447368421052624</v>
+        <v>-0.01842105263157891</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22847,10 +22847,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>46</v>
+        <v>45.6</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.0944881889763779</v>
+        <v>-0.1023622047244094</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22877,10 +22877,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.04605263157894737</v>
+        <v>-0.03947368421052631</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>228.5</v>
+        <v>230</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.01931330472103004</v>
+        <v>-0.0128755364806867</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>34.46</v>
+        <v>34.6</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.1276178010471205</v>
+        <v>0.1321989528795812</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>77.90000000000001</v>
+        <v>78.8</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.003865979381443446</v>
+        <v>0.01546391752577323</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>27.9</v>
+        <v>26.05</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.1137724550898203</v>
+        <v>0.03992015968063872</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>80.18000000000001</v>
+        <v>81.84999999999999</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.02101107856869993</v>
+        <v>0.0422768368776263</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>126.65</v>
+        <v>123.55</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.1008257279443721</v>
+        <v>0.07388092133854846</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-23 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18566,7 +18566,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/10/2026 13:00</t>
+          <t>23/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -18593,10 +18593,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>52.05</v>
+        <v>52</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.009699321047526674</v>
+        <v>0.008729388942774061</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18623,10 +18623,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>24.94</v>
+        <v>24.86</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03557617942768748</v>
+        <v>-0.03866976024748647</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18653,10 +18653,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.738</v>
+        <v>1.769</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.01585503963759911</v>
+        <v>0.001698754246885556</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18683,10 +18683,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>31.7</v>
+        <v>31.9</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.009554140127388559</v>
+        <v>0.01592356687898089</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18713,10 +18713,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>60.05</v>
+        <v>60</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06566104702750658</v>
+        <v>0.06477373558118897</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18743,10 +18743,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>175.5</v>
+        <v>177.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.04964114832535892</v>
+        <v>0.05980861244019139</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18773,10 +18773,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>81.84999999999999</v>
+        <v>83.73</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.01412464378639575</v>
+        <v>0.03741791599553972</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18803,10 +18803,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>31.85</v>
+        <v>32.06</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.01697530864197522</v>
+        <v>-0.01049382716049371</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18833,10 +18833,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.081</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.01219512195121952</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18863,10 +18863,10 @@
         <v>2.88</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2.82</v>
+        <v>2.84</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.02083333333333335</v>
+        <v>-0.0138888888888889</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18965,10 +18965,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>14.44</v>
+        <v>15.72</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.005509641873278242</v>
+        <v>0.08264462809917363</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19025,10 +19025,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>419.4</v>
+        <v>418.4</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.03185595567867039</v>
+        <v>-0.03416435826408128</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19055,10 +19055,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.6</v>
+        <v>1.598</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03492884864165591</v>
+        <v>0.03363518758085385</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19085,10 +19085,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>6.01</v>
+        <v>5.99</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.01797385620915038</v>
+        <v>-0.02124183006535946</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19115,10 +19115,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>29.15</v>
+        <v>29.3</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.02101576182136595</v>
+        <v>0.02626970227670753</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19145,10 +19145,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.5</v>
+        <v>58.4</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.008474576271186441</v>
+        <v>-0.01016949152542375</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19205,10 +19205,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.68</v>
+        <v>8.65</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03333333333333326</v>
+        <v>0.02976190476190476</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19235,10 +19235,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>4.01</v>
+        <v>3.876</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.302608695652174</v>
+        <v>-0.3259130434782609</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19340,10 +19340,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.98</v>
+        <v>0.93</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.05314009661835743</v>
+        <v>-0.1014492753623187</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19369,10 +19369,10 @@
         <v>15.8</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0</v>
+        <v>-0.006329113924050722</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19398,10 +19398,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>23.2</v>
+        <v>23.4</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.06451612903225812</v>
+        <v>-0.05645161290322589</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19427,10 +19427,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.83</v>
+        <v>3.73</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.02295918367346935</v>
+        <v>-0.04846938775510203</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19486,10 +19486,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.95</v>
+        <v>2</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.04411764705882357</v>
+        <v>-0.01960784313725492</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19515,10 +19515,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>26.3</v>
+        <v>27</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06071428571428569</v>
+        <v>-0.03571428571428571</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19573,10 +19573,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.242</v>
+        <v>0.239</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.08679245283018876</v>
+        <v>-0.09811320754716989</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19602,10 +19602,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>22.7</v>
+        <v>22.5</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.07910750507099389</v>
+        <v>-0.08722109533468554</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19728,10 +19728,10 @@
         <v>67.2</v>
       </c>
       <c r="F44" s="12" t="n">
-        <v>65.5</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="G44" s="13" t="n">
-        <v>-0.02529761904761909</v>
+        <v>-0.01934523809523805</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" thickBot="1">
@@ -19757,10 +19757,10 @@
         <v>89</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>87</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.02247191011235955</v>
+        <v>-0.01797752808988758</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19786,10 +19786,10 @@
         <v>30.05</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>26.12</v>
+        <v>25.75</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>-0.1307820299500832</v>
+        <v>-0.1430948419301165</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19815,10 +19815,10 @@
         <v>19.19</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>19.52</v>
+        <v>19.45</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.01719645648775395</v>
+        <v>0.01354872329338187</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19844,10 +19844,10 @@
         <v>15.39</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>14.86</v>
+        <v>14.92</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.03443794671864855</v>
+        <v>-0.03053931124106567</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19873,10 +19873,10 @@
         <v>32.46</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>34.6</v>
+        <v>34.3</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.06592729513247075</v>
+        <v>0.05668515095502145</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19902,10 +19902,10 @@
         <v>13.95</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>11.655</v>
+        <v>11.465</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>-0.1645161290322581</v>
+        <v>-0.1781362007168459</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19931,10 +19931,10 @@
         <v>5.7</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>5.71</v>
+        <v>5.79</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.001754385964912243</v>
+        <v>0.0157894736842105</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19960,10 +19960,10 @@
         <v>149</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>152.8</v>
+        <v>151.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02550335570469806</v>
+        <v>0.01879194630872491</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21247,7 +21247,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>23/10/2026 13:00</t>
+          <t>23/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -21274,10 +21274,10 @@
         <v>15.2</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>14.92</v>
+        <v>14.94</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.01842105263157891</v>
+        <v>-0.01710526315789472</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21304,10 +21304,10 @@
         <v>8.18</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>7.975</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.02506112469437654</v>
+        <v>-0.01283618581907096</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21334,10 +21334,10 @@
         <v>28.25</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>26.12</v>
+        <v>25.75</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.07539823008849554</v>
+        <v>-0.08849557522123894</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21364,10 +21364,10 @@
         <v>24.6</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>24.94</v>
+        <v>24.86</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.01382113821138211</v>
+        <v>0.01056910569105683</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21394,10 +21394,10 @@
         <v>80.5</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>85.65000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.06397515527950318</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21424,10 +21424,10 @@
         <v>78.53</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>81.84999999999999</v>
+        <v>83.73</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.0422768368776263</v>
+        <v>0.06621673245893293</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21454,10 +21454,10 @@
         <v>233</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>-0.0128755364806867</v>
+        <v>0.004291845493562232</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21484,10 +21484,10 @@
         <v>1.454</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>1.571</v>
+        <v>1.554</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.08046767537826685</v>
+        <v>0.06877579092159566</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21544,10 +21544,10 @@
         <v>216.4</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>200.8</v>
+        <v>204.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>-0.07208872458410348</v>
+        <v>-0.05452865064695014</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -21676,10 +21676,10 @@
         <v>9.725</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>9.125</v>
+        <v>9.085000000000001</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.06169665809768634</v>
+        <v>-0.06580976863753202</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21706,10 +21706,10 @@
         <v>2.134</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>2.018</v>
+        <v>1.991</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.05435801312089977</v>
+        <v>-0.06701030927835042</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21736,10 +21736,10 @@
         <v>1.38</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.738</v>
+        <v>1.769</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.2594202898550725</v>
+        <v>0.2818840579710145</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21766,10 +21766,10 @@
         <v>21.16</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>24.12</v>
+        <v>23.54</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.1398865784499055</v>
+        <v>0.1124763705103969</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21796,10 +21796,10 @@
         <v>12.6</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.1031746031746032</v>
+        <v>0.1111111111111111</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21826,10 +21826,10 @@
         <v>55.15</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>54.4</v>
+        <v>53.7</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01359927470534905</v>
+        <v>-0.02629193109700808</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21856,10 +21856,10 @@
         <v>0.441</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>0.437</v>
+        <v>0.442</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.009070294784580506</v>
+        <v>0.002267573696145127</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21886,10 +21886,10 @@
         <v>30.56</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>34.6</v>
+        <v>34.3</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.1321989528795812</v>
+        <v>0.1223821989528795</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21916,10 +21916,10 @@
         <v>14.49</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>14.53</v>
+        <v>14.61</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>0.002760524499654876</v>
+        <v>0.008281573498964748</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22021,10 +22021,10 @@
         <v>0.08</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.068</v>
+        <v>0.067</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.15</v>
+        <v>-0.1625</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22050,10 +22050,10 @@
         <v>9.9</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>9.34</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>-0.05656565656565661</v>
+        <v>-0.07070707070707082</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -22079,10 +22079,10 @@
         <v>0.158</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>0.149</v>
+        <v>0.151</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.05696202531645574</v>
+        <v>-0.04430379746835447</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22108,10 +22108,10 @@
         <v>1.3</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>1.27</v>
+        <v>1.26</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.0230769230769231</v>
+        <v>-0.0307692307692308</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22137,10 +22137,10 @@
         <v>0.241</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.211</v>
+        <v>0.206</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.1244813278008299</v>
+        <v>-0.1452282157676349</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -22166,10 +22166,10 @@
         <v>10.14</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>9.039999999999999</v>
+        <v>9</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.1084812623274163</v>
+        <v>-0.1124260355029586</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22195,10 +22195,10 @@
         <v>19.7</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>18.4</v>
+        <v>18.15</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.06598984771573609</v>
+        <v>-0.07868020304568532</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22224,10 +22224,10 @@
         <v>3.405</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>4.05</v>
+        <v>4.075</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>0.1894273127753304</v>
+        <v>0.1967694566813511</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22787,10 +22787,10 @@
         <v>212.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>211.8</v>
+        <v>212.4</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.004699248120300752</v>
+        <v>-0.001879699248120327</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22817,10 +22817,10 @@
         <v>15.2</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>14.92</v>
+        <v>14.94</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>-0.01842105263157891</v>
+        <v>-0.01710526315789472</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22847,10 +22847,10 @@
         <v>50.8</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>45.6</v>
+        <v>46</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>-0.1023622047244094</v>
+        <v>-0.0944881889763779</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22877,10 +22877,10 @@
         <v>152</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03947368421052631</v>
+        <v>-0.04605263157894737</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22907,10 +22907,10 @@
         <v>233</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>-0.0128755364806867</v>
+        <v>0.004291845493562232</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22937,10 +22937,10 @@
         <v>30.56</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>34.6</v>
+        <v>34.3</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>0.1321989528795812</v>
+        <v>0.1223821989528795</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22967,10 +22967,10 @@
         <v>77.59999999999999</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>78.8</v>
+        <v>79.5</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.01546391752577323</v>
+        <v>0.0244845360824743</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22997,10 +22997,10 @@
         <v>25.05</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>26.05</v>
+        <v>27.75</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>0.03992015968063872</v>
+        <v>0.1077844311377245</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23027,10 +23027,10 @@
         <v>78.53</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>81.84999999999999</v>
+        <v>83.73</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>0.0422768368776263</v>
+        <v>0.06621673245893293</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23057,10 +23057,10 @@
         <v>115.05</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>123.55</v>
+        <v>124.1</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>0.07388092133854846</v>
+        <v>0.07866145154280746</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-26 19:05
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18574,7 +18574,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>26/10/2026 13:00</t>
+          <t>26/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -18601,10 +18601,10 @@
         <v>59.95</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>58.6</v>
+        <v>59.75</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.02251876563803172</v>
+        <v>-0.003336113427856594</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -18631,10 +18631,10 @@
         <v>233.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>231.5</v>
+        <v>230</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.008565310492505354</v>
+        <v>-0.01498929336188437</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18661,10 +18661,10 @@
         <v>83.45</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>82.91</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>-0.006470940683043814</v>
+        <v>0.004074295985620173</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18691,10 +18691,10 @@
         <v>32.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.45</v>
+        <v>32.4</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.001543209876543342</v>
+        <v>0</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18721,10 +18721,10 @@
         <v>185</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>186.2</v>
+        <v>185.2</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.006486486486486425</v>
+        <v>0.00108108108108102</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18751,10 +18751,10 @@
         <v>35.96</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>35.18</v>
+        <v>35.22</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.02169076751946611</v>
+        <v>-0.02057842046718582</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18781,10 +18781,10 @@
         <v>5.83</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.84</v>
+        <v>5.83</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.001715265866209226</v>
+        <v>0</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18811,10 +18811,10 @@
         <v>93.7</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>93.65000000000001</v>
+        <v>95.8</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.000533617929562403</v>
+        <v>0.02241195304162214</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18841,10 +18841,10 @@
         <v>24.44</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>24.27</v>
+        <v>24.52</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>-0.006955810147299579</v>
+        <v>0.003273322422258522</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18871,10 +18871,10 @@
         <v>11.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>11.75</v>
+        <v>11.55</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.03982300884955746</v>
+        <v>0.02212389380530973</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18973,10 +18973,10 @@
         <v>0.549</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.54</v>
+        <v>0.534</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.01639344262295083</v>
+        <v>-0.02732240437158472</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19003,10 +19003,10 @@
         <v>72.59999999999999</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>73.90000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.01790633608815443</v>
+        <v>0.01515151515151527</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19033,10 +19033,10 @@
         <v>33.74</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>34.7</v>
+        <v>34.26</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.028452874925904</v>
+        <v>0.01541197391819787</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19063,10 +19063,10 @@
         <v>0.047</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0.049</v>
+        <v>0.047</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.04255319148936174</v>
+        <v>0</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -19093,10 +19093,10 @@
         <v>3.554</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.67</v>
+        <v>3.679</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.03263927968486216</v>
+        <v>0.03517163759144626</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19123,10 +19123,10 @@
         <v>1.61</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>1.622</v>
+        <v>1.604</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.007453416149068329</v>
+        <v>-0.003726708074534164</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19153,10 +19153,10 @@
         <v>4.322</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>4.345</v>
+        <v>4.295</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>0.005321610365571422</v>
+        <v>-0.006247107820453525</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19183,10 +19183,10 @@
         <v>9.369999999999999</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>9.630000000000001</v>
+        <v>9.52</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.0277481323372467</v>
+        <v>0.01600853788687304</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19213,10 +19213,10 @@
         <v>8.038</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.568</v>
+        <v>8.406000000000001</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.06593680019905442</v>
+        <v>0.04578253296840014</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19243,10 +19243,10 @@
         <v>3.965</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>3.88</v>
+        <v>3.83</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.02143757881462799</v>
+        <v>-0.03404791929382088</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>0.124</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.121</v>
+        <v>0.118</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.02419354838709679</v>
+        <v>-0.04838709677419359</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>0.71</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.723</v>
+        <v>0.733</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.01830985915492959</v>
+        <v>0.03239436619718313</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>6.021</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.773</v>
+        <v>5.74</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.04118917123401432</v>
+        <v>-0.0466699883740242</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>3.5</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.68</v>
+        <v>3.44</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>0.05142857142857148</v>
+        <v>-0.01714285714285716</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19464,10 +19464,10 @@
         <v>0.046</v>
       </c>
       <c r="F34" s="12" t="n">
-        <v>0.043</v>
+        <v>0.044</v>
       </c>
       <c r="G34" s="13" t="n">
-        <v>-0.06521739130434788</v>
+        <v>-0.04347826086956526</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" thickBot="1">
@@ -19493,10 +19493,10 @@
         <v>1.315</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.295</v>
+        <v>1.275</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.01520912547528518</v>
+        <v>-0.03041825095057037</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.787</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.832</v>
+        <v>1.809</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.025181869054281</v>
+        <v>0.0123111359820929</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19551,10 +19551,10 @@
         <v>96</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.01041666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -19580,10 +19580,10 @@
         <v>3.3</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>3.29</v>
+        <v>3.24</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.003030303030302966</v>
+        <v>-0.01818181818181806</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19609,10 +19609,10 @@
         <v>68</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>67.5</v>
+        <v>68</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.007352941176470588</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19765,10 +19765,10 @@
         <v>0.97</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>0.952</v>
+        <v>0.956</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01855670103092785</v>
+        <v>-0.01443298969072166</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19823,10 +19823,10 @@
         <v>80.58</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>81.38</v>
+        <v>81.16</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.009928021841648017</v>
+        <v>0.007197815835194817</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19852,10 +19852,10 @@
         <v>174.68</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>174.64</v>
+        <v>175.14</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>-0.0002289901534235199</v>
+        <v>0.002633386764369015</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19881,10 +19881,10 @@
         <v>87.65000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>89.65000000000001</v>
+        <v>89.8</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.02281802624073018</v>
+        <v>0.02452937820878484</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19910,10 +19910,10 @@
         <v>436.3</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>439.35</v>
+        <v>437.5</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.006990602796241144</v>
+        <v>0.002750401100160414</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19939,10 +19939,10 @@
         <v>23.5</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>23.7</v>
+        <v>23.5</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0.008510638297872309</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19968,10 +19968,10 @@
         <v>79.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>81.09999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.01756587202007517</v>
+        <v>0.02634880803011285</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21235,7 +21235,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>26/10/2026 13:00</t>
+          <t>26/10/2026 19:05</t>
         </is>
       </c>
     </row>
@@ -21262,10 +21262,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>51.25</v>
+        <v>51.8</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>-0.005819592628515949</v>
+        <v>0.004849660523763337</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21292,10 +21292,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.16</v>
+        <v>25.02</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.0270688321732405</v>
+        <v>-0.03248259860788863</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21322,10 +21322,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.915</v>
+        <v>1.925</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.08437146092865233</v>
+        <v>0.09003397508493773</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21352,10 +21352,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>31.55</v>
+        <v>31.6</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.004777070063694336</v>
+        <v>0.006369426751592447</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21382,10 +21382,10 @@
         <v>56.35</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>58.6</v>
+        <v>59.75</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.03992901508429458</v>
+        <v>0.06033717834960068</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -21412,10 +21412,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>176.7</v>
+        <v>176.9</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.05681818181818182</v>
+        <v>0.05801435406698575</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21442,10 +21442,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>82.91</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.02725808450006199</v>
+        <v>0.03816131830008689</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21472,10 +21472,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>32.38</v>
+        <v>32.54</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>-0.0006172839506171612</v>
+        <v>0.004320987654321005</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21502,10 +21502,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.083</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.01219512195121952</v>
+        <v>0.02439024390243905</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21634,10 +21634,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>16.58</v>
+        <v>17.24</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.1418732782369145</v>
+        <v>0.18732782369146</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21664,10 +21664,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>20.4</v>
+        <v>20.3</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.05555555555555568</v>
+        <v>-0.06018518518518522</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21694,10 +21694,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>420.4</v>
+        <v>419.6</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.02954755309325949</v>
+        <v>-0.0313942751615881</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21724,10 +21724,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.622</v>
+        <v>1.604</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.0491591203104787</v>
+        <v>0.03751617076326006</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21754,10 +21754,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.97</v>
+        <v>5.96</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02450980392156869</v>
+        <v>-0.02614379084967322</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21784,10 +21784,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>29.75</v>
+        <v>29.55</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.04203152364273202</v>
+        <v>0.03502626970227671</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21814,10 +21814,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.5</v>
+        <v>58.3</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.008474576271186441</v>
+        <v>-0.01186440677966107</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21844,10 +21844,10 @@
         <v>125.6</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>125.4</v>
+        <v>125.5</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.001592356687897999</v>
+        <v>-0.0007961783439489994</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21874,10 +21874,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.74</v>
+        <v>8.69</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.04047619047619046</v>
+        <v>0.03452380952380942</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21904,10 +21904,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>4.104</v>
+        <v>4.14</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2862608695652174</v>
+        <v>-0.2800000000000001</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22067,10 +22067,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>23.4</v>
+        <v>23.6</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.05645161290322589</v>
+        <v>-0.04838709677419352</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22096,10 +22096,10 @@
         <v>3.92</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.76</v>
+        <v>3.79</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.04081632653061228</v>
+        <v>-0.03316326530612242</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -22155,10 +22155,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.85</v>
+        <v>1.995</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.09313725490196076</v>
+        <v>-0.02205882352941173</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22213,10 +22213,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22</v>
+        <v>22.2</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.03719912472647709</v>
+        <v>-0.02844638949671782</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22242,10 +22242,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.24</v>
+        <v>0.236</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.09433962264150951</v>
+        <v>-0.109433962264151</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22776,10 +22776,10 @@
         <v>57.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>53.1</v>
+        <v>52.95</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.08131487889273349</v>
+        <v>-0.08391003460207604</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22806,10 +22806,10 @@
         <v>121.35</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>125.2</v>
+        <v>124.35</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.03172641120725182</v>
+        <v>0.02472187886279357</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22836,10 +22836,10 @@
         <v>31.4</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>31.55</v>
+        <v>31.6</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.004777070063694336</v>
+        <v>0.006369426751592447</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22866,10 +22866,10 @@
         <v>36.62</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>35.44</v>
+        <v>35.28</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03222282905516111</v>
+        <v>-0.03659202621518286</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22896,10 +22896,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>82.91</v>
+        <v>83.79000000000001</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.02725808450006199</v>
+        <v>0.03816131830008689</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22926,10 +22926,10 @@
         <v>102.45</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>101.05</v>
+        <v>99.5</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.01366520253782338</v>
+        <v>-0.0287945339189849</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22956,10 +22956,10 @@
         <v>84</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>89.65000000000001</v>
+        <v>89.8</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.06726190476190483</v>
+        <v>0.06904761904761901</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22986,10 +22986,10 @@
         <v>18.99</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>18.26</v>
+        <v>18.08</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.03844128488678236</v>
+        <v>-0.04791995787256452</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23016,10 +23016,10 @@
         <v>15.39</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>14.64</v>
+        <v>14.44</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.04873294346978557</v>
+        <v>-0.06172839506172846</v>
       </c>
       <c r="H77" s="6" t="n"/>
     </row>
@@ -23046,10 +23046,10 @@
         <v>18.985</v>
       </c>
       <c r="F78" s="12" t="n">
-        <v>18.165</v>
+        <v>18.59</v>
       </c>
       <c r="G78" s="37" t="n">
-        <v>-0.04319199367922046</v>
+        <v>-0.0208058993942586</v>
       </c>
       <c r="H78" s="6" t="n"/>
     </row>

</xml_diff>

<commit_message>
Mise à jour cours (Snapshot) - 2026-10-27 13:00
</commit_message>
<xml_diff>
--- a/Twitter_Donnees.xlsx
+++ b/Twitter_Donnees.xlsx
@@ -18574,7 +18574,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>26/10/2026 19:05</t>
+          <t>27/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -18631,10 +18631,10 @@
         <v>233.5</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.01498929336188437</v>
+        <v>-0.01070663811563169</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -18661,10 +18661,10 @@
         <v>83.45</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>83.79000000000001</v>
+        <v>83.03</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.004074295985620173</v>
+        <v>-0.005032953864589595</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -18691,10 +18691,10 @@
         <v>32.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>32.4</v>
+        <v>32.35</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0</v>
+        <v>-0.001543209876543122</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -18721,10 +18721,10 @@
         <v>185</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>185.2</v>
+        <v>187</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>0.00108108108108102</v>
+        <v>0.01081081081081081</v>
       </c>
       <c r="H6" s="6" t="n"/>
     </row>
@@ -18751,10 +18751,10 @@
         <v>35.96</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>35.22</v>
+        <v>35.4</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>-0.02057842046718582</v>
+        <v>-0.01557285873192442</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -18781,10 +18781,10 @@
         <v>5.83</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>5.83</v>
+        <v>5.89</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0</v>
+        <v>0.01029159519725551</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -18811,10 +18811,10 @@
         <v>93.7</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>95.8</v>
+        <v>95.3</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.02241195304162214</v>
+        <v>0.0170757737459978</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -18841,10 +18841,10 @@
         <v>24.44</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>24.52</v>
+        <v>24.62</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.003273322422258522</v>
+        <v>0.007364975450081821</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -18871,10 +18871,10 @@
         <v>11.3</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>11.55</v>
+        <v>11.6</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>0.02212389380530973</v>
+        <v>0.02654867256637158</v>
       </c>
       <c r="H11" s="6" t="n"/>
     </row>
@@ -18973,10 +18973,10 @@
         <v>0.549</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>0.534</v>
+        <v>0.538</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>-0.02732240437158472</v>
+        <v>-0.02003642987249546</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -19003,10 +19003,10 @@
         <v>72.59999999999999</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>73.7</v>
+        <v>73.8</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>0.01515151515151527</v>
+        <v>0.01652892561983475</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -19033,10 +19033,10 @@
         <v>33.74</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>34.26</v>
+        <v>33.98</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>0.01541197391819787</v>
+        <v>0.007113218731475841</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -19093,10 +19093,10 @@
         <v>3.554</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>3.679</v>
+        <v>3.659</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>0.03517163759144626</v>
+        <v>0.02954417557681485</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -19123,10 +19123,10 @@
         <v>1.61</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>1.604</v>
+        <v>1.652</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>-0.003726708074534164</v>
+        <v>0.02608695652173901</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -19153,10 +19153,10 @@
         <v>4.322</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>4.295</v>
+        <v>4.44</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.006247107820453525</v>
+        <v>0.02730217491901905</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -19183,10 +19183,10 @@
         <v>9.369999999999999</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>9.52</v>
+        <v>10.04</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>0.01600853788687304</v>
+        <v>0.07150480256136606</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -19213,10 +19213,10 @@
         <v>8.038</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.406000000000001</v>
+        <v>8.238</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.04578253296840014</v>
+        <v>0.02488181139586953</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -19243,10 +19243,10 @@
         <v>3.965</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>3.83</v>
+        <v>3.765</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.03404791929382088</v>
+        <v>-0.05044136191677169</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -19348,10 +19348,10 @@
         <v>0.124</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.118</v>
+        <v>0.126</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.04838709677419359</v>
+        <v>0.01612903225806453</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -19377,10 +19377,10 @@
         <v>0.71</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>0.733</v>
+        <v>0.735</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>0.03239436619718313</v>
+        <v>0.03521126760563384</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" thickBot="1">
@@ -19406,10 +19406,10 @@
         <v>6.021</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>5.74</v>
+        <v>5.73</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.0466699883740242</v>
+        <v>-0.04833084205281506</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -19435,10 +19435,10 @@
         <v>3.5</v>
       </c>
       <c r="F33" s="12" t="n">
-        <v>3.44</v>
+        <v>3.36</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>-0.01714285714285716</v>
+        <v>-0.04000000000000004</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" thickBot="1">
@@ -19493,10 +19493,10 @@
         <v>1.315</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.275</v>
+        <v>1.285</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.03041825095057037</v>
+        <v>-0.02281368821292778</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -19522,10 +19522,10 @@
         <v>1.787</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>1.809</v>
+        <v>1.805</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>0.0123111359820929</v>
+        <v>0.01007274762171238</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -19580,10 +19580,10 @@
         <v>3.3</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>3.24</v>
+        <v>3.15</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.01818181818181806</v>
+        <v>-0.04545454545454543</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -19609,10 +19609,10 @@
         <v>68</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>0</v>
+        <v>-0.02941176470588235</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -19706,11 +19706,10 @@
         <v>62.2</v>
       </c>
       <c r="F43" s="12" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="G43" s="13">
-        <f>(F43/E43-1)</f>
-        <v/>
+        <v>62.5</v>
+      </c>
+      <c r="G43" s="13" t="n">
+        <v>0.004823151125401884</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" thickBot="1">
@@ -19765,10 +19764,10 @@
         <v>0.97</v>
       </c>
       <c r="F45" s="12" t="n">
-        <v>0.956</v>
+        <v>0.95</v>
       </c>
       <c r="G45" s="13" t="n">
-        <v>-0.01443298969072166</v>
+        <v>-0.02061855670103095</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" thickBot="1">
@@ -19794,10 +19793,10 @@
         <v>84.7</v>
       </c>
       <c r="F46" s="12" t="n">
-        <v>85.98</v>
+        <v>85.56</v>
       </c>
       <c r="G46" s="13" t="n">
-        <v>0.01511216056670603</v>
+        <v>0.0101534828807556</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" thickBot="1">
@@ -19823,10 +19822,10 @@
         <v>80.58</v>
       </c>
       <c r="F47" s="12" t="n">
-        <v>81.16</v>
+        <v>81</v>
       </c>
       <c r="G47" s="13" t="n">
-        <v>0.007197815835194817</v>
+        <v>0.005212211466865248</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" thickBot="1">
@@ -19852,10 +19851,10 @@
         <v>174.68</v>
       </c>
       <c r="F48" s="12" t="n">
-        <v>175.14</v>
+        <v>175.1</v>
       </c>
       <c r="G48" s="13" t="n">
-        <v>0.002633386764369015</v>
+        <v>0.002404396610945658</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" thickBot="1">
@@ -19881,10 +19880,10 @@
         <v>87.65000000000001</v>
       </c>
       <c r="F49" s="12" t="n">
-        <v>89.8</v>
+        <v>88</v>
       </c>
       <c r="G49" s="13" t="n">
-        <v>0.02452937820878484</v>
+        <v>0.003993154592127715</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" thickBot="1">
@@ -19910,10 +19909,10 @@
         <v>436.3</v>
       </c>
       <c r="F50" s="12" t="n">
-        <v>437.5</v>
+        <v>434.3</v>
       </c>
       <c r="G50" s="13" t="n">
-        <v>0.002750401100160414</v>
+        <v>-0.004584001833600733</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" thickBot="1">
@@ -19939,10 +19938,10 @@
         <v>23.5</v>
       </c>
       <c r="F51" s="12" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>0</v>
+        <v>0.004255319148936231</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" thickBot="1">
@@ -19968,10 +19967,10 @@
         <v>79.7</v>
       </c>
       <c r="F52" s="12" t="n">
-        <v>81.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="G52" s="13" t="n">
-        <v>0.02634880803011285</v>
+        <v>0.008782936010037677</v>
       </c>
     </row>
     <row r="53" ht="15.45" customHeight="1" thickBot="1">
@@ -21235,7 +21234,7 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>26/10/2026 19:05</t>
+          <t>27/10/2026 13:00</t>
         </is>
       </c>
     </row>
@@ -21262,10 +21261,10 @@
         <v>51.55</v>
       </c>
       <c r="F2" s="12" t="n">
-        <v>51.8</v>
+        <v>50.55</v>
       </c>
       <c r="G2" s="13" t="n">
-        <v>0.004849660523763337</v>
+        <v>-0.01939864209505335</v>
       </c>
       <c r="H2" s="14" t="n"/>
     </row>
@@ -21292,10 +21291,10 @@
         <v>25.86</v>
       </c>
       <c r="F3" s="12" t="n">
-        <v>25.02</v>
+        <v>25.08</v>
       </c>
       <c r="G3" s="13" t="n">
-        <v>-0.03248259860788863</v>
+        <v>-0.03016241299303949</v>
       </c>
       <c r="H3" s="6" t="n"/>
     </row>
@@ -21322,10 +21321,10 @@
         <v>1.766</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>1.925</v>
+        <v>1.949</v>
       </c>
       <c r="G4" s="13" t="n">
-        <v>0.09003397508493773</v>
+        <v>0.1036240090600227</v>
       </c>
       <c r="H4" s="6" t="n"/>
     </row>
@@ -21352,10 +21351,10 @@
         <v>31.4</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>0.006369426751592447</v>
+        <v>0.003184713375796224</v>
       </c>
       <c r="H5" s="6" t="n"/>
     </row>
@@ -21412,10 +21411,10 @@
         <v>167.2</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>176.9</v>
+        <v>177.2</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>0.05801435406698575</v>
+        <v>0.05980861244019139</v>
       </c>
       <c r="H7" s="6" t="n"/>
     </row>
@@ -21442,10 +21441,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>83.79000000000001</v>
+        <v>83.03</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>0.03816131830008689</v>
+        <v>0.02874488910915633</v>
       </c>
       <c r="H8" s="6" t="n"/>
     </row>
@@ -21472,10 +21471,10 @@
         <v>32.4</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>32.54</v>
+        <v>32.52</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>0.004320987654321005</v>
+        <v>0.003703703703703844</v>
       </c>
       <c r="H9" s="6" t="n"/>
     </row>
@@ -21502,10 +21501,10 @@
         <v>0.082</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>0.02439024390243905</v>
+        <v>0.01219512195121952</v>
       </c>
       <c r="H10" s="6" t="n"/>
     </row>
@@ -21634,10 +21633,10 @@
         <v>14.52</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>17.24</v>
+        <v>17.4</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>0.18732782369146</v>
+        <v>0.1983471074380165</v>
       </c>
       <c r="H16" s="47" t="n"/>
     </row>
@@ -21664,10 +21663,10 @@
         <v>21.6</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>20.3</v>
+        <v>19.95</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>-0.06018518518518522</v>
+        <v>-0.07638888888888898</v>
       </c>
       <c r="H17" s="6" t="n"/>
     </row>
@@ -21694,10 +21693,10 @@
         <v>433.2</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>419.6</v>
+        <v>420.6</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-0.0313942751615881</v>
+        <v>-0.02908587257617721</v>
       </c>
       <c r="H18" s="6" t="n"/>
     </row>
@@ -21724,10 +21723,10 @@
         <v>1.546</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>1.604</v>
+        <v>1.652</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>0.03751617076326006</v>
+        <v>0.06856403622250962</v>
       </c>
       <c r="H19" s="6" t="n"/>
     </row>
@@ -21754,10 +21753,10 @@
         <v>6.12</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>5.96</v>
+        <v>5.93</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>-0.02614379084967322</v>
+        <v>-0.03104575163398699</v>
       </c>
       <c r="H20" s="6" t="n"/>
     </row>
@@ -21784,10 +21783,10 @@
         <v>28.55</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>29.55</v>
+        <v>29.5</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>0.03502626970227671</v>
+        <v>0.03327495621716284</v>
       </c>
       <c r="H21" s="6" t="n"/>
     </row>
@@ -21814,10 +21813,10 @@
         <v>59</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>58.3</v>
+        <v>59.2</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-0.01186440677966107</v>
+        <v>0.003389830508474624</v>
       </c>
       <c r="H22" s="6" t="n"/>
     </row>
@@ -21844,10 +21843,10 @@
         <v>125.6</v>
       </c>
       <c r="F23" s="12" t="n">
-        <v>125.5</v>
+        <v>125.3</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>-0.0007961783439489994</v>
+        <v>-0.002388535031847111</v>
       </c>
       <c r="H23" s="6" t="n"/>
     </row>
@@ -21874,10 +21873,10 @@
         <v>8.4</v>
       </c>
       <c r="F24" s="12" t="n">
-        <v>8.69</v>
+        <v>9.9</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>0.03452380952380942</v>
+        <v>0.1785714285714286</v>
       </c>
       <c r="H24" s="6" t="n"/>
     </row>
@@ -21904,10 +21903,10 @@
         <v>5.75</v>
       </c>
       <c r="F25" s="12" t="n">
-        <v>4.14</v>
+        <v>4.1</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>-0.2800000000000001</v>
+        <v>-0.2869565217391305</v>
       </c>
       <c r="H25" s="6" t="n"/>
     </row>
@@ -22009,10 +22008,10 @@
         <v>1.035</v>
       </c>
       <c r="F30" s="12" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>-0.1014492753623187</v>
+        <v>-0.111111111111111</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" thickBot="1">
@@ -22067,10 +22066,10 @@
         <v>24.8</v>
       </c>
       <c r="F32" s="12" t="n">
-        <v>23.6</v>
+        <v>23.5</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>-0.04838709677419352</v>
+        <v>-0.05241935483870971</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" thickBot="1">
@@ -22155,10 +22154,10 @@
         <v>2.04</v>
       </c>
       <c r="F35" s="12" t="n">
-        <v>1.995</v>
+        <v>2</v>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-0.02205882352941173</v>
+        <v>-0.01960784313725492</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" thickBot="1">
@@ -22184,10 +22183,10 @@
         <v>28</v>
       </c>
       <c r="F36" s="12" t="n">
-        <v>27</v>
+        <v>26.82</v>
       </c>
       <c r="G36" s="13" t="n">
-        <v>-0.03571428571428571</v>
+        <v>-0.04214285714285713</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" thickBot="1">
@@ -22213,10 +22212,10 @@
         <v>22.85</v>
       </c>
       <c r="F37" s="12" t="n">
-        <v>22.2</v>
+        <v>22.3</v>
       </c>
       <c r="G37" s="13" t="n">
-        <v>-0.02844638949671782</v>
+        <v>-0.0240700218818381</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" thickBot="1">
@@ -22242,10 +22241,10 @@
         <v>0.265</v>
       </c>
       <c r="F38" s="12" t="n">
-        <v>0.236</v>
+        <v>0.244</v>
       </c>
       <c r="G38" s="13" t="n">
-        <v>-0.109433962264151</v>
+        <v>-0.07924528301886799</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" thickBot="1">
@@ -22271,10 +22270,10 @@
         <v>24.65</v>
       </c>
       <c r="F39" s="12" t="n">
-        <v>22.4</v>
+        <v>22.95</v>
       </c>
       <c r="G39" s="13" t="n">
-        <v>-0.09127789046653144</v>
+        <v>-0.06896551724137928</v>
       </c>
     </row>
     <row r="40" ht="15.45" customHeight="1" thickBot="1">
@@ -22776,10 +22775,10 @@
         <v>57.8</v>
       </c>
       <c r="F69" s="12" t="n">
-        <v>52.95</v>
+        <v>54.3</v>
       </c>
       <c r="G69" s="37" t="n">
-        <v>-0.08391003460207604</v>
+        <v>-0.06055363321799308</v>
       </c>
       <c r="H69" s="6" t="n"/>
     </row>
@@ -22806,10 +22805,10 @@
         <v>121.35</v>
       </c>
       <c r="F70" s="12" t="n">
-        <v>124.35</v>
+        <v>124.8</v>
       </c>
       <c r="G70" s="37" t="n">
-        <v>0.02472187886279357</v>
+        <v>0.02843016069221263</v>
       </c>
       <c r="H70" s="6" t="n"/>
     </row>
@@ -22836,10 +22835,10 @@
         <v>31.4</v>
       </c>
       <c r="F71" s="12" t="n">
-        <v>31.6</v>
+        <v>31.5</v>
       </c>
       <c r="G71" s="37" t="n">
-        <v>0.006369426751592447</v>
+        <v>0.003184713375796224</v>
       </c>
       <c r="H71" s="6" t="n"/>
     </row>
@@ -22866,10 +22865,10 @@
         <v>36.62</v>
       </c>
       <c r="F72" s="12" t="n">
-        <v>35.28</v>
+        <v>35.4</v>
       </c>
       <c r="G72" s="37" t="n">
-        <v>-0.03659202621518286</v>
+        <v>-0.03331512834516655</v>
       </c>
       <c r="H72" s="6" t="n"/>
     </row>
@@ -22896,10 +22895,10 @@
         <v>80.70999999999999</v>
       </c>
       <c r="F73" s="12" t="n">
-        <v>83.79000000000001</v>
+        <v>83.03</v>
       </c>
       <c r="G73" s="37" t="n">
-        <v>0.03816131830008689</v>
+        <v>0.02874488910915633</v>
       </c>
       <c r="H73" s="6" t="n"/>
     </row>
@@ -22926,10 +22925,10 @@
         <v>102.45</v>
       </c>
       <c r="F74" s="12" t="n">
-        <v>99.5</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="G74" s="37" t="n">
-        <v>-0.0287945339189849</v>
+        <v>-0.02430453879941444</v>
       </c>
       <c r="H74" s="6" t="n"/>
     </row>
@@ -22956,10 +22955,10 @@
         <v>84</v>
       </c>
       <c r="F75" s="12" t="n">
-        <v>89.8</v>
+        <v>88</v>
       </c>
       <c r="G75" s="37" t="n">
-        <v>0.06904761904761901</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="H75" s="6" t="n"/>
     </row>
@@ -22986,10 +22985,10 @@
         <v>18.99</v>
       </c>
       <c r="F76" s="12" t="n">
-        <v>18.08</v>
+        <v>18.36</v>
       </c>
       <c r="G76" s="37" t="n">
-        <v>-0.04791995787256452</v>
+        <v>-0.03317535545023691</v>
       </c>
       <c r="H76" s="6" t="n"/>
     </row>
@@ -23016,10 +23015,10 @@
         <v>15.39</v>
       </c>
       <c r="F77" s="12" t="n">
-        <v>14.44</v>
+        <v>14.55</v>
       </c>
       <c r="G77" s="37" t="n">
-        <v>-0.06172839506172846</v>
+        <v>-0.05458089668615983</v>
       </c>
       <c r="H77" s